<commit_message>
feat: add itinerary top seven priorities
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Re5e99390bdc94a2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R301cc00e6f564dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rf58b383e14be4f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R4289b1b4127c422a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R02fbdc4cad9e4544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rfa9914b0fca64ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R07175963f04e4a25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R8f65b37b68eb4e10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R453f66920a6f43e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Ra04e0d8eb27a4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rb8c68f0ee24d4e78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R1b131257e0da4c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R3012353b0f9f43c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rad7397d127334f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rc53c270299194bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R87bd75f5741c4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Rb002b84d39da4b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R4d913d966dae4d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R48fb8b64353f4dfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +25,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -63,8 +64,20 @@
       <x:color rgb="FF0F766E"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0B7F75"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,8 +109,23 @@
         <x:fgColor rgb="FFF5F8F6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B7F75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B7F75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B7F75"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -109,11 +137,25 @@
         <x:color rgb="FF9BC8BC"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DED9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7DED9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DED9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DED9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -222,6 +264,33 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -536,100 +605,62 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="23" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">day_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">day_label</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">date</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">weekday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">city</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lat</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lon</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">title</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">focus</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lodging</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">climate_note</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">clothing_note</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cover_image_url</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cover_image_alt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">leave_by</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lodging_resource_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">primary_resource_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ticket_resource_id</x:t>
-        </x:is>
+      <x:c r="A1" t="str">
+        <x:v>day_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>day_label</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>weekday</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>city</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>lat</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>lon</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>focus</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>lodging</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>climate_note</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>clothing_note</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>cover_image_url</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>cover_image_alt</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>transport</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>leave_by</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>lodging_resource_id</x:v>
+      </x:c>
+      <x:c r="R1" t="str">
+        <x:v>primary_resource_id</x:v>
+      </x:c>
+      <x:c r="S1" t="str">
+        <x:v>ticket_resource_id</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -773,10 +804,10 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>墨尔本近郊：Puffing Billy、Sassafras 与 Fitzroy</x:v>
+        <x:v>墨尔本近郊：Puffing Billy 与 Sassafras</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>上午乘 Puffing Billy 穿行山林，下午在 Fitzroy 看街区与小店。</x:v>
+        <x:v>上午乘 Puffing Billy 穿行山林；返城后若时间和体力合适，再去 Fitzroy 走走。</x:v>
       </x:c>
       <x:c r="J4" t="str">
         <x:v>Oaks Melbourne on Market Hotel</x:v>
@@ -891,10 +922,10 @@
         <x:v>142.9956</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>大洋路海岸：雨林、十二使徒岩与 Loch Ard Gorge</x:v>
+        <x:v>红杉林到海岸：The Redwoods、十二使徒岩与 Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="I6" t="str">
-        <x:v>从雨林步道驶向十二使徒岩，在 Loch Ard Gorge 慢慢看海岸地貌。</x:v>
+        <x:v>先走进 The Redwoods Otways，再回到海岸看十二使徒岩、Loch Ard Gorge 与 The Razorback。</x:v>
       </x:c>
       <x:c r="J6" t="str">
         <x:v>Southern Ocean Villas</x:v>
@@ -915,13 +946,13 @@
         <x:v>自驾 · 大洋路海岸段</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>08:30 前离开 Apollo Bay</x:v>
+        <x:v>07:45 前离开 Apollo Bay</x:v>
       </x:c>
       <x:c r="Q6" t="str">
         <x:v>southern-ocean-villas-map</x:v>
       </x:c>
       <x:c r="R6" t="str">
-        <x:v>maits-rest-map</x:v>
+        <x:v>redwoods-otways-map</x:v>
       </x:c>
       <x:c r="S6" t="str">
         <x:v>no-fixed-ticket</x:v>
@@ -1363,10 +1394,10 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>悉尼经典一日：歌剧院、The Rocks Weekend Market、植物园与 QVB</x:v>
+        <x:v>悉尼经典一日：歌剧院、The Rocks Markets、植物园与 QVB</x:v>
       </x:c>
       <x:c r="I14" t="str">
-        <x:v>从歌剧院中文导览出发，逛 The Rocks 周末市集，再沿植物园走到经典海港机位与 QVB。</x:v>
+        <x:v>从歌剧院中文导览出发，逛 The Rocks Markets，再沿植物园走到经典海港机位与 QVB。</x:v>
       </x:c>
       <x:c r="J14" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
@@ -1633,6 +1664,183 @@
       </x:c>
       <x:c r="S18" t="str">
         <x:v>trs-official</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="61" t="str">
+        <x:v>rank</x:v>
+      </x:c>
+      <x:c r="B1" s="61" t="str">
+        <x:v>day_id</x:v>
+      </x:c>
+      <x:c r="C1" s="61" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="D1" s="61" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="E1" s="61" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="F1" s="61" t="str">
+        <x:v>resource_id</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="54" t="str">
+        <x:v>d1</x:v>
+      </x:c>
+      <x:c r="C2" s="54" t="str">
+        <x:v>QVM Winter Night Market</x:v>
+      </x:c>
+      <x:c r="D2" s="55" t="str">
+        <x:v>必去</x:v>
+      </x:c>
+      <x:c r="E2" s="54" t="str">
+        <x:v>周三限定夜市，晚餐边逛边吃</x:v>
+      </x:c>
+      <x:c r="F2" s="54" t="str">
+        <x:v>qvm-winter-night-market-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="53" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="54" t="str">
+        <x:v>d4</x:v>
+      </x:c>
+      <x:c r="C3" s="54" t="str">
+        <x:v>The Redwoods Otways</x:v>
+      </x:c>
+      <x:c r="D3" s="55" t="str">
+        <x:v>必去</x:v>
+      </x:c>
+      <x:c r="E3" s="54" t="str">
+        <x:v>红杉林慢走 30–45 分钟</x:v>
+      </x:c>
+      <x:c r="F3" s="54" t="str">
+        <x:v>redwoods-otways-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="53" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="54" t="str">
+        <x:v>d2</x:v>
+      </x:c>
+      <x:c r="C4" s="54" t="str">
+        <x:v>Fitzroy</x:v>
+      </x:c>
+      <x:c r="D4" s="55" t="str">
+        <x:v>备选</x:v>
+      </x:c>
+      <x:c r="E4" s="54" t="str">
+        <x:v>半日团准时返城且体力合适再去</x:v>
+      </x:c>
+      <x:c r="F4" s="54" t="str">
+        <x:v>fitzroy-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="53" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="54" t="str">
+        <x:v>d10</x:v>
+      </x:c>
+      <x:c r="C5" s="54" t="str">
+        <x:v>Palm Cove</x:v>
+      </x:c>
+      <x:c r="D5" s="55" t="str">
+        <x:v>必去</x:v>
+      </x:c>
+      <x:c r="E5" s="54" t="str">
+        <x:v>傍晚沿海滨散步、喝咖啡</x:v>
+      </x:c>
+      <x:c r="F5" s="54" t="str">
+        <x:v>palm-cove-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="53" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="54" t="str">
+        <x:v>d11</x:v>
+      </x:c>
+      <x:c r="C6" s="54" t="str">
+        <x:v>Barangaroo Reserve</x:v>
+      </x:c>
+      <x:c r="D6" s="55" t="str">
+        <x:v>必去</x:v>
+      </x:c>
+      <x:c r="E6" s="54" t="str">
+        <x:v>转场日下午沿 Wulugul Walk 慢走</x:v>
+      </x:c>
+      <x:c r="F6" s="54" t="str">
+        <x:v>barangaroo-reserve-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="53" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="54" t="str">
+        <x:v>d12</x:v>
+      </x:c>
+      <x:c r="C7" s="54" t="str">
+        <x:v>The Rocks Markets</x:v>
+      </x:c>
+      <x:c r="D7" s="55" t="str">
+        <x:v>必去</x:v>
+      </x:c>
+      <x:c r="E7" s="54" t="str">
+        <x:v>中文导览后步行前往，停留 45–60 分钟</x:v>
+      </x:c>
+      <x:c r="F7" s="54" t="str">
+        <x:v>the-rocks-market-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="53" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="54" t="str">
+        <x:v>d4</x:v>
+      </x:c>
+      <x:c r="C8" s="54" t="str">
+        <x:v>The Razorback</x:v>
+      </x:c>
+      <x:c r="D8" s="55" t="str">
+        <x:v>必去</x:v>
+      </x:c>
+      <x:c r="E8" s="54" t="str">
+        <x:v>Loch Ard Gorge 景区内沿 Geology Walk 前往</x:v>
+      </x:c>
+      <x:c r="F8" s="54" t="str">
+        <x:v>razorback-map</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2156,19 +2364,19 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>备选 · 下午后段</x:v>
       </x:c>
       <x:c r="D20" t="str">
         <x:v>Fitzroy: Brunswick Street → Gertrude Street</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>半日团返城后前往 Fitzroy，完成街区漫步、独立小店和咖啡</x:v>
+        <x:v>若半日团准时返城且体力充足，再沿 Brunswick Street / Gertrude Street 随意走走。</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>街头艺术、老建筑与本地生活版墨尔本</x:v>
+        <x:v>街区小店、咖啡与旧工业街景</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>预留约 90 分钟，从 Brunswick Street 走到 Gertrude Street；18:00 左右回酒店整理行李。</x:v>
+        <x:v>把 Fitzroy 当作加分项；返城较晚或需要休息时直接回酒店。</x:v>
       </x:c>
       <x:c r="H20" t="str">
         <x:v>fitzroy-map,russell-343-map</x:v>
@@ -2220,7 +2428,7 @@
         <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>集合前吃得简单些；返城后在 Fitzroy / CBD 轻松晚餐，留出整理行李的时间。</x:v>
+        <x:v>Fitzroy 仅作返城后的备选；不去时直接在 CBD 用餐。</x:v>
       </x:c>
       <x:c r="H22" t="str">
         <x:v>russell-343-map,emerald-lake-park-map,sassafras-map,southbank-map</x:v>
@@ -2598,19 +2806,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>上午</x:v>
+        <x:v>备选 · 清晨</x:v>
       </x:c>
       <x:c r="D37" t="str">
         <x:v>Maits Rest Rainforest Walk</x:v>
       </x:c>
       <x:c r="E37" t="str">
-        <x:v>雨林短步道</x:v>
+        <x:v>若 07:45 前离开 Apollo Bay 且时间充裕，可先走一段雨林环线。</x:v>
       </x:c>
       <x:c r="F37" t="str">
         <x:v>冬日湿润雨林，非常有氛围</x:v>
       </x:c>
       <x:c r="G37" t="str">
-        <x:v>步道轻松，适合作为早晨活动；注意地面湿滑</x:v>
+        <x:v>只有早出发且时间充裕时再停，约 30 分钟。</x:v>
       </x:c>
       <x:c r="H37" t="str">
         <x:v>maits-rest-map</x:v>
@@ -2624,22 +2832,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>中午前后</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D38" t="str">
-        <x:v>Gibson Steps</x:v>
+        <x:v>The Redwoods Otways</x:v>
       </x:c>
       <x:c r="E38" t="str">
-        <x:v>下到海滩看悬崖与海蚀柱</x:v>
+        <x:v>从北侧 Binns Road 进入红杉林，沿 Aire River 林间步道慢走约 30–45 分钟。</x:v>
       </x:c>
       <x:c r="F38" t="str">
-        <x:v>人物比例感很强，比单纯观景台更有沉浸感</x:v>
+        <x:v>高大的加州红杉、林下光影与安静的河谷氛围</x:v>
       </x:c>
       <x:c r="G38" t="str">
-        <x:v>看开放情况和风浪；风大时不要太靠近海浪</x:v>
+        <x:v>林区无手机信号，地面可能湿滑；出发前查看 Parks Victoria 路况与现场标识。</x:v>
       </x:c>
       <x:c r="H38" t="str">
-        <x:v>gibson-steps-map</x:v>
+        <x:v>redwoods-otways-map,redwoods-otways-official</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2650,22 +2858,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午前后</x:v>
       </x:c>
       <x:c r="D39" t="str">
-        <x:v>Twelve Apostles</x:v>
+        <x:v>Gibson Steps</x:v>
       </x:c>
       <x:c r="E39" t="str">
-        <x:v>十二使徒岩主观景台</x:v>
+        <x:v>下到海滩看悬崖与海蚀柱</x:v>
       </x:c>
       <x:c r="F39" t="str">
-        <x:v>大洋路最具代表性的海岸地貌</x:v>
+        <x:v>人物比例感很强，比单纯观景台更有沉浸感</x:v>
       </x:c>
       <x:c r="G39" t="str">
-        <x:v>左侧平台更适合拍海岸线纵深；如果人多，不要停太久</x:v>
+        <x:v>看开放情况和风浪；风大时不要太靠近海浪</x:v>
       </x:c>
       <x:c r="H39" t="str">
-        <x:v>twelve-apostles-map</x:v>
+        <x:v>gibson-steps-map</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2679,19 +2887,19 @@
         <x:v>下午</x:v>
       </x:c>
       <x:c r="D40" t="str">
-        <x:v>Loch Ard Gorge</x:v>
+        <x:v>Twelve Apostles</x:v>
       </x:c>
       <x:c r="E40" t="str">
-        <x:v>峡谷、海湾、海蚀地貌</x:v>
+        <x:v>十二使徒岩主观景台</x:v>
       </x:c>
       <x:c r="F40" t="str">
-        <x:v>峡谷、海湾与沉船海岸故事</x:v>
+        <x:v>大洋路最具代表性的海岸地貌</x:v>
       </x:c>
       <x:c r="G40" t="str">
-        <x:v>这里要认真留时间，不要只拍一张就走</x:v>
+        <x:v>左侧平台更适合拍海岸线纵深；如果人多，不要停太久</x:v>
       </x:c>
       <x:c r="H40" t="str">
-        <x:v>loch-ard-map</x:v>
+        <x:v>twelve-apostles-map</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2705,19 +2913,19 @@
         <x:v>下午</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Tom and Eva</x:v>
+        <x:v>Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>Loch Ard Gorge 附近短停</x:v>
+        <x:v>在主观景区看峡湾与沉船故事，再接 Geology Walk。</x:v>
       </x:c>
       <x:c r="F41" t="str">
-        <x:v>两个海蚀柱，和沉船故事相关</x:v>
+        <x:v>峡湾地貌、沉船历史与悬崖顶观景</x:v>
       </x:c>
       <x:c r="G41" t="str">
-        <x:v>作为 Loch Ard Gorge 区域顺路点，不需要额外绕路</x:v>
+        <x:v>至少预留 1 小时；海滩下行台阶关闭，按现场标识走崖顶步道。</x:v>
       </x:c>
       <x:c r="H41" t="str">
-        <x:v>tom-eva-map,loch-ard-map</x:v>
+        <x:v>loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2725,25 +2933,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B42" t="n">
-        <x:v>60</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>The Razorback</x:v>
+        <x:v>Tom and Eva</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>看狭长海蚀岩脊</x:v>
+        <x:v>Loch Ard Gorge 附近短停</x:v>
       </x:c>
       <x:c r="F42" t="str">
-        <x:v>形状特别，层次感强</x:v>
+        <x:v>两个海蚀柱，和沉船故事相关</x:v>
       </x:c>
       <x:c r="G42" t="str">
-        <x:v>适合短停拍照；风大时注意安全</x:v>
+        <x:v>作为 Loch Ard Gorge 区域顺路点，不需要额外绕路</x:v>
       </x:c>
       <x:c r="H42" t="str">
-        <x:v>razorback-map</x:v>
+        <x:v>tom-eva-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2751,25 +2959,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B43" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>The Razorback</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>抵达入住 Southern Ocean Villas</x:v>
+        <x:v>从 Loch Ard Gorge 主停车场走 900 米往返 Geology Walk，经 Island Arch 到 The Razorback 观景台。</x:v>
       </x:c>
       <x:c r="F43" t="str">
-        <x:v>方便第二天清晨补拍</x:v>
+        <x:v>同一景区内的狭长海蚀岩脊与悬崖顶视角</x:v>
       </x:c>
       <x:c r="G43" t="str">
-        <x:v>不要天黑后还在海岸小路上赶</x:v>
+        <x:v>步行往返约 30–40 分钟；不需要另开一段车程。</x:v>
       </x:c>
       <x:c r="H43" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>razorback-map</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2777,22 +2985,22 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B44" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D44" t="str">
         <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>抵达后按天气选择公共电烤炉 BBQ、villa 厨房自炊或附近餐厅</x:v>
+        <x:v>抵达入住 Southern Ocean Villas</x:v>
       </x:c>
       <x:c r="F44" t="str">
-        <x:v>灵活完成 BBQ-style dinner</x:v>
+        <x:v>方便第二天清晨补拍</x:v>
       </x:c>
       <x:c r="G44" t="str">
-        <x:v>Southern Ocean Villas 没有自带 BBQ，但附近有两处免费 electric BBQ；villa 厨房备有油、盐、胡椒和锡纸。</x:v>
+        <x:v>不要天黑后还在海岸小路上赶</x:v>
       </x:c>
       <x:c r="H44" t="str">
         <x:v>port-campbell-map</x:v>
@@ -2803,51 +3011,51 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B45" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：在 Apollo Bay 买好食材，抵达后按天气选择公共 electric BBQ 或 villa 厨房自炊</x:v>
+        <x:v>抵达后按天气选择公共电烤炉 BBQ、villa 厨房自炊或附近餐厅</x:v>
       </x:c>
       <x:c r="F45" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>灵活完成 BBQ-style dinner</x:v>
       </x:c>
       <x:c r="G45" t="str">
-        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
+        <x:v>Southern Ocean Villas 没有自带 BBQ，但附近有两处免费 electric BBQ；villa 厨房备有油、盐、胡椒和锡纸。</x:v>
       </x:c>
       <x:c r="H45" t="str">
-        <x:v>apollo-map,port-campbell-map</x:v>
+        <x:v>port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
-        <x:v>d5</x:v>
+        <x:v>d4</x:v>
       </x:c>
       <x:c r="B46" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>早上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>清晨再看一处海岸景点</x:v>
+        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：在 Apollo Bay 买好食材，抵达后按天气选择公共 electric BBQ 或 villa 厨房自炊</x:v>
       </x:c>
       <x:c r="F46" t="str">
-        <x:v>光线柔和，人相对少</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G46" t="str">
-        <x:v>若前一天下雨，可在十二使徒岩或 Loch Ard Gorge 中选一处重访；天气好则按时间择一。</x:v>
+        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
       </x:c>
       <x:c r="H46" t="str">
-        <x:v>twelve-apostles-map,loch-ard-map</x:v>
+        <x:v>apollo-map,port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2855,25 +3063,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B47" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>上午</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>早餐、退房</x:v>
+        <x:v>清晨再看一处海岸景点</x:v>
       </x:c>
       <x:c r="F47" t="str">
-        <x:v>海边小镇慢节奏</x:v>
+        <x:v>光线柔和，人相对少</x:v>
       </x:c>
       <x:c r="G47" t="str">
-        <x:v>不要拖太晚，今天还要回机场</x:v>
+        <x:v>若前一天下雨，可在十二使徒岩或 Loch Ard Gorge 中选一处重访；天气好则按时间择一。</x:v>
       </x:c>
       <x:c r="H47" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>twelve-apostles-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2881,25 +3089,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B48" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>London Bridge / London Arch</x:v>
+        <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>看海蚀拱门</x:v>
+        <x:v>早餐、退房</x:v>
       </x:c>
       <x:c r="F48" t="str">
-        <x:v>Port Campbell 以西经典点</x:v>
+        <x:v>海边小镇慢节奏</x:v>
       </x:c>
       <x:c r="G48" t="str">
-        <x:v>顺路短停，很适合加</x:v>
+        <x:v>不要拖太晚，今天还要回机场</x:v>
       </x:c>
       <x:c r="H48" t="str">
-        <x:v>london-arch-map,port-campbell-map</x:v>
+        <x:v>port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2907,25 +3115,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B49" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>中午前后</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>The Grotto</x:v>
+        <x:v>London Bridge / London Arch</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>看海蚀洞和海水窗口</x:v>
+        <x:v>看海蚀拱门</x:v>
       </x:c>
       <x:c r="F49" t="str">
-        <x:v>洞穴 + 海景构图</x:v>
+        <x:v>Port Campbell 以西经典点</x:v>
       </x:c>
       <x:c r="G49" t="str">
-        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
+        <x:v>顺路短停，很适合加</x:v>
       </x:c>
       <x:c r="H49" t="str">
-        <x:v>grotto-map</x:v>
+        <x:v>london-arch-map,port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2933,25 +3141,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B50" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>中午 / 下午</x:v>
+        <x:v>中午前后</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Bay of Islands</x:v>
+        <x:v>The Grotto</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>时间充裕时延伸</x:v>
+        <x:v>看海蚀洞和海水窗口</x:v>
       </x:c>
       <x:c r="F50" t="str">
-        <x:v>更开阔、更荒凉的海蚀柱群</x:v>
+        <x:v>洞穴 + 海景构图</x:v>
       </x:c>
       <x:c r="G50" t="str">
-        <x:v>天气好、时间宽裕再去；如果要赶机场就跳过</x:v>
+        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
       </x:c>
       <x:c r="H50" t="str">
-        <x:v>bay-islands-map</x:v>
+        <x:v>grotto-map</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2959,25 +3167,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B51" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午 / 下午</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Colac</x:v>
+        <x:v>Bay of Islands</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>午餐、加油、休息</x:v>
+        <x:v>时间充裕时延伸</x:v>
       </x:c>
       <x:c r="F51" t="str">
-        <x:v>内陆牧场风光</x:v>
+        <x:v>更开阔、更荒凉的海蚀柱群</x:v>
       </x:c>
       <x:c r="G51" t="str">
-        <x:v>回程中段休息点</x:v>
+        <x:v>天气好、时间宽裕再去；如果要赶机场就跳过</x:v>
       </x:c>
       <x:c r="H51" t="str">
-        <x:v>colac-map</x:v>
+        <x:v>bay-islands-map</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2985,25 +3193,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B52" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>Colac</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
+        <x:v>午餐、加油、休息</x:v>
       </x:c>
       <x:c r="F52" t="str">
-        <x:v>大洋路自驾收尾</x:v>
+        <x:v>内陆牧场风光</x:v>
       </x:c>
       <x:c r="G52" t="str">
-        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
+        <x:v>回程中段休息点</x:v>
       </x:c>
       <x:c r="H52" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>colac-map</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -3011,25 +3219,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B53" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Holiday Inn Melbourne Airport</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>入住、整理行李</x:v>
+        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
       </x:c>
       <x:c r="F53" t="str">
-        <x:v>为次日早班机准备</x:v>
+        <x:v>大洋路自驾收尾</x:v>
       </x:c>
       <x:c r="G53" t="str">
-        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
+        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
       </x:c>
       <x:c r="H53" t="str">
-        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
+        <x:v>mel-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3037,51 +3245,51 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B54" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Holiday Inn Melbourne Airport</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>早餐：Port Campbell café；午餐：Colac / Timboon Ice Cream；晚餐：机场酒店简餐</x:v>
+        <x:v>入住、整理行李</x:v>
       </x:c>
       <x:c r="F54" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>为次日早班机准备</x:v>
       </x:c>
       <x:c r="G54" t="str">
-        <x:v>Timboon Ice Cream 可作为回程中的小惊喜；抵达机场后简单用餐并整理行李。</x:v>
+        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
       </x:c>
       <x:c r="H54" t="str">
-        <x:v>colac-map,timboon-icecream-map,port-campbell-map,holiday-inn-airport-map</x:v>
+        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B55" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>飞往凯恩斯</x:v>
+        <x:v>早餐：Port Campbell café；午餐：Colac / Timboon Ice Cream；晚餐：机场酒店简餐</x:v>
       </x:c>
       <x:c r="F55" t="str">
-        <x:v>气候切换非常明显</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G55" t="str">
-        <x:v>国内航班建议预留行李额</x:v>
+        <x:v>Timboon Ice Cream 可作为回程中的小惊喜；抵达机场后简单用餐并整理行李。</x:v>
       </x:c>
       <x:c r="H55" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>colac-map,timboon-icecream-map,port-campbell-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3089,75 +3297,75 @@
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B56" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>打车 / Uber 到酒店</x:v>
+        <x:v>飞往凯恩斯</x:v>
       </x:c>
       <x:c r="F56" t="str">
-        <x:v>不租车，降低疲劳</x:v>
+        <x:v>气候切换非常明显</x:v>
       </x:c>
       <x:c r="G56" t="str">
-        <x:v>酒店可先寄存行李</x:v>
-      </x:c>
-      <x:c r="H56"/>
+        <x:v>国内航班建议预留行李额</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" t="str">
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B57" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Esplanade Lagoon</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>免费泻湖泳池、海滨散步</x:v>
+        <x:v>打车 / Uber 到酒店</x:v>
       </x:c>
       <x:c r="F57" t="str">
-        <x:v>度假感拉满</x:v>
+        <x:v>不租车，降低疲劳</x:v>
       </x:c>
       <x:c r="G57" t="str">
-        <x:v>泳衣可提前放随身包</x:v>
-      </x:c>
-      <x:c r="H57" t="str">
-        <x:v>cairns-lagoon-map</x:v>
-      </x:c>
+        <x:v>酒店可先寄存行李</x:v>
+      </x:c>
+      <x:c r="H57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="str">
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B58" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>晚上</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Cairns Night Markets</x:v>
+        <x:v>Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>夜市、简餐、纪念品</x:v>
+        <x:v>免费泻湖泳池、海滨散步</x:v>
       </x:c>
       <x:c r="F58" t="str">
-        <x:v>热闹轻松</x:v>
+        <x:v>度假感拉满</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+        <x:v>泳衣可提前放随身包</x:v>
       </x:c>
       <x:c r="H58" t="str">
-        <x:v>cairns-night-market-map</x:v>
+        <x:v>cairns-lagoon-map</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3165,75 +3373,75 @@
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B59" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
+        <x:v>夜市、简餐、纪念品</x:v>
       </x:c>
       <x:c r="F59" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>热闹轻松</x:v>
       </x:c>
       <x:c r="G59" t="str">
-        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
-      </x:c>
-      <x:c r="H59"/>
+        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>cairns-night-market-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B60" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>早上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>凯恩斯码头</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Reef Magic check-in，登船出海</x:v>
+        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>前往外礁平台</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
-      </x:c>
-      <x:c r="H60" t="str">
-        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
-      </x:c>
+        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
+      </x:c>
+      <x:c r="H60"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="str">
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B61" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>全天</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Outer Reef Pontoon</x:v>
+        <x:v>凯恩斯码头</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
+        <x:v>Reef Magic check-in，登船出海</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
+        <x:v>前往外礁平台</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
+        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -3241,22 +3449,22 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B62" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>中午</x:v>
+        <x:v>全天</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>船上 / 平台</x:v>
+        <x:v>Outer Reef Pontoon</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>外礁平台午餐</x:v>
+        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
       </x:c>
       <x:c r="F62" t="str">
-        <x:v>轻松补给</x:v>
+        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
       </x:c>
       <x:c r="G62" t="str">
-        <x:v>不要吃太撑，避免晕船</x:v>
+        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
       </x:c>
       <x:c r="H62" t="str">
         <x:v>reef-magic-official</x:v>
@@ -3267,25 +3475,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B63" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>船上 / 平台</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>下船休息</x:v>
+        <x:v>外礁平台午餐</x:v>
       </x:c>
       <x:c r="F63" t="str">
-        <x:v>通常会比较疲惫</x:v>
+        <x:v>轻松补给</x:v>
       </x:c>
       <x:c r="G63" t="str">
-        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
+        <x:v>不要吃太撑，避免晕船</x:v>
       </x:c>
       <x:c r="H63" t="str">
-        <x:v>reef-fleet-terminal-map</x:v>
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3293,25 +3501,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B64" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>晚上</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>码头附近</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
+        <x:v>下船休息</x:v>
       </x:c>
       <x:c r="F64" t="str">
-        <x:v>海边晚餐</x:v>
+        <x:v>通常会比较疲惫</x:v>
       </x:c>
       <x:c r="G64" t="str">
-        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
+        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H64" t="str">
-        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
+        <x:v>reef-fleet-terminal-map</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3319,25 +3527,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B65" t="n">
-        <x:v>80</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>提醒</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>今日提醒</x:v>
+        <x:v>码头附近</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
+        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
       </x:c>
       <x:c r="F65" t="str">
-        <x:v>舒适与安全比拍摄数量更重要</x:v>
+        <x:v>海边晚餐</x:v>
       </x:c>
       <x:c r="G65" t="str">
-        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
       </x:c>
       <x:c r="H65" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3345,151 +3553,151 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B66" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>饮食</x:v>
+        <x:v>提醒</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>今日提醒</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
+        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>舒适与安全比拍摄数量更重要</x:v>
       </x:c>
       <x:c r="G66" t="str">
-        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
       </x:c>
       <x:c r="H66" t="str">
-        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B67" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>清晨</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
+        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="F67" t="str">
-        <x:v>不用自驾，沿途可休息看风景</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G67" t="str">
-        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
-      </x:c>
-      <x:c r="H67"/>
+        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B68" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>上午</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Daintree River / Rainforest</x:v>
+        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>鳄鱼游船、雨林步道</x:v>
+        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
       </x:c>
       <x:c r="F68" t="str">
-        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
+        <x:v>不用自驾，沿途可休息看风景</x:v>
       </x:c>
       <x:c r="G68" t="str">
-        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
-      </x:c>
-      <x:c r="H68" t="str">
-        <x:v>daintree-river-map</x:v>
-      </x:c>
+        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
+      </x:c>
+      <x:c r="H68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B69" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Daintree Rainforest</x:v>
+        <x:v>Daintree River / Rainforest</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>团含午餐</x:v>
+        <x:v>鳄鱼游船、雨林步道</x:v>
       </x:c>
       <x:c r="F69" t="str">
-        <x:v>不用自己找餐厅</x:v>
+        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
       </x:c>
       <x:c r="G69" t="str">
-        <x:v>如有忌口提前告知</x:v>
-      </x:c>
-      <x:c r="H69"/>
+        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>daintree-river-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B70" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Cape Tribulation</x:v>
+        <x:v>Daintree Rainforest</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>雨林入海、海滩短停留</x:v>
+        <x:v>团含午餐</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>雨林与海洋在这里交会</x:v>
+        <x:v>不用自己找餐厅</x:v>
       </x:c>
       <x:c r="G70" t="str">
-        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
-      </x:c>
-      <x:c r="H70" t="str">
-        <x:v>cape-trib-map</x:v>
-      </x:c>
+        <x:v>如有忌口提前告知</x:v>
+      </x:c>
+      <x:c r="H70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B71" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Daintree Ferry / Ice Cream</x:v>
+        <x:v>Cape Tribulation</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>渡河、热带水果冰淇淋</x:v>
+        <x:v>雨林入海、海滩短停留</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>丹翠地区很有代表性的热带味道</x:v>
+        <x:v>雨林与海洋在这里交会</x:v>
       </x:c>
       <x:c r="G71" t="str">
-        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
+        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
       </x:c>
       <x:c r="H71" t="str">
-        <x:v>daintree-icecream-map</x:v>
+        <x:v>cape-trib-map</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3497,75 +3705,75 @@
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B72" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Daintree Ferry / Ice Cream</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>18:30 后回到市区</x:v>
+        <x:v>渡河、热带水果冰淇淋</x:v>
       </x:c>
       <x:c r="F72" t="str">
-        <x:v>回程可休息</x:v>
+        <x:v>丹翠地区很有代表性的热带味道</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
-      </x:c>
-      <x:c r="H72"/>
+        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>daintree-icecream-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B73" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>饮食</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>18:30 后回到市区</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>回程可休息</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
-      </x:c>
-      <x:c r="H73" t="str">
-        <x:v>daintree-icecream-map</x:v>
-      </x:c>
+        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
+      </x:c>
+      <x:c r="H73"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B74" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>早上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>凯恩斯 → Lake Eacham</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
+        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F74" t="str">
-        <x:v>从热带海边城市进入清凉高原</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
+        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
       </x:c>
       <x:c r="H74" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>daintree-icecream-map</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -3573,22 +3781,22 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B75" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>上午</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Lake Eacham</x:v>
+        <x:v>凯恩斯 → Lake Eacham</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>火山湖散步、看湖景</x:v>
+        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>安静、清凉、湖水和雨林包围感</x:v>
+        <x:v>从热带海边城市进入清凉高原</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
       </x:c>
       <x:c r="H75" t="str">
         <x:v>lake-eacham-map</x:v>
@@ -3599,25 +3807,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B76" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Curtain Fig Tree</x:v>
+        <x:v>Lake Eacham</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>看巨型帘状无花果树</x:v>
+        <x:v>火山湖散步、看湖景</x:v>
       </x:c>
       <x:c r="F76" t="str">
-        <x:v>像热带森林里的巨大自然装置</x:v>
+        <x:v>安静、清凉、湖水和雨林包围感</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>停留 20–30 分钟即可</x:v>
+        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
       </x:c>
       <x:c r="H76" t="str">
-        <x:v>curtain-fig-map</x:v>
+        <x:v>lake-eacham-map</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -3625,25 +3833,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B77" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Yungaburra / Gallo Dairyland</x:v>
+        <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
+        <x:v>看巨型帘状无花果树</x:v>
       </x:c>
       <x:c r="F77" t="str">
-        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
+        <x:v>像热带森林里的巨大自然装置</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
+        <x:v>停留 20–30 分钟即可</x:v>
       </x:c>
       <x:c r="H77" t="str">
-        <x:v>yungaburra-map,gallo-map</x:v>
+        <x:v>curtain-fig-map</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -3651,25 +3859,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B78" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
+        <x:v>Yungaburra / Gallo Dairyland</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>瀑布短停留、拍照</x:v>
+        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>雨林瀑布与高原绿意</x:v>
+        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
       </x:c>
       <x:c r="H78" t="str">
-        <x:v>millaa-map,ellinjaa-map</x:v>
+        <x:v>yungaburra-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -3677,46 +3885,48 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B79" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>下山回市区，还车或次日早还</x:v>
+        <x:v>瀑布短停留、拍照</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>完成高原自然线</x:v>
+        <x:v>雨林瀑布与高原绿意</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
-      </x:c>
-      <x:c r="H79"/>
+        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>millaa-map,ellinjaa-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="str">
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B80" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>简单晚餐</x:v>
+        <x:v>下山回市区，还车或次日早还</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>回城后轻松晚餐</x:v>
+        <x:v>完成高原自然线</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>下山后就近用餐，早点休息。</x:v>
+        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
       </x:c>
       <x:c r="H80"/>
     </x:row>
@@ -3725,51 +3935,49 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B81" t="n">
-        <x:v>900</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>简单晚餐</x:v>
       </x:c>
       <x:c r="F81" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>回城后轻松晚餐</x:v>
       </x:c>
       <x:c r="G81" t="str">
-        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
-      </x:c>
-      <x:c r="H81" t="str">
-        <x:v>millaa-map,gallo-map</x:v>
-      </x:c>
+        <x:v>下山后就近用餐，早点休息。</x:v>
+      </x:c>
+      <x:c r="H81"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B82" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F82" t="str">
-        <x:v>周五正好开市，适合补水果和轻食</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G82" t="str">
-        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
+        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H82" t="str">
-        <x:v>rustys-map</x:v>
+        <x:v>millaa-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -3777,25 +3985,25 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B83" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="F83" t="str">
-        <x:v>热带城市躺平感</x:v>
+        <x:v>周五正好开市，适合补水果和轻食</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
+        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
       </x:c>
       <x:c r="H83" t="str">
-        <x:v>cairns-lagoon-map</x:v>
+        <x:v>rustys-map</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -3803,75 +4011,75 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B84" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="F84" t="str">
-        <x:v>为次日清晨航班做准备</x:v>
+        <x:v>热带城市躺平感</x:v>
       </x:c>
       <x:c r="G84" t="str">
-        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
-      </x:c>
-      <x:c r="H84"/>
+        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>cairns-lagoon-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" t="str">
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B85" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>下午 / 傍晚</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Palm Cove</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
+        <x:v>为次日清晨航班做准备</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
-      </x:c>
-      <x:c r="H85" t="str">
-        <x:v>palm-cove-map</x:v>
-      </x:c>
+        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
+      </x:c>
+      <x:c r="H85"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" t="str">
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B86" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>晚上</x:v>
+        <x:v>下午 / 傍晚</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Palm Cove</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>海鲜或轻松简餐</x:v>
+        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>早点吃，早点睡</x:v>
+        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
       </x:c>
       <x:c r="H86" t="str">
-        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
+        <x:v>palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -3879,51 +4087,51 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B87" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海鲜或轻松简餐</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
+        <x:v>早点吃，早点睡</x:v>
       </x:c>
       <x:c r="H87" t="str">
-        <x:v>rustys-map,prawn-star-map</x:v>
+        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B88" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>清晨</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>cairns-airport-map</x:v>
+        <x:v>rustys-map,prawn-star-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -3931,75 +4139,75 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B89" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>上午</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>凯恩斯 → 悉尼</x:v>
+        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H89"/>
+        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>cairns-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B90" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>从热带切换回冬季海港城市</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
-      </x:c>
-      <x:c r="H90" t="str">
-        <x:v>oaks-sydney-map</x:v>
-      </x:c>
+        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
+      </x:c>
+      <x:c r="H90"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B91" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>下午</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>悉尼 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>4人 + 行李，打车最省心</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>如不能入住，先寄存行李</x:v>
       </x:c>
       <x:c r="H91" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -4007,25 +4215,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B92" t="n">
-        <x:v>45</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>Darling Harbour / 酒店周边</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -4033,25 +4241,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B93" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4059,25 +4267,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B94" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>circular-quay-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4085,51 +4293,51 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B95" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>歌剧院、海港大桥夜景</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H95" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B96" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H96" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4137,25 +4345,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>08:15–08:30</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>抵达海港区</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>Ferry、海港桥、歌剧院远景</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4163,25 +4371,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B98" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>08:30–09:10</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>悉尼核心地标</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4189,25 +4397,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B99" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Weekend Market</x:v>
+        <x:v>中文内部导览已订</x:v>
       </x:c>
       <x:c r="F99" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>建筑故事、内部空间、剧院结构</x:v>
       </x:c>
       <x:c r="G99" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4215,25 +4423,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B100" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>10:30–10:50</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>The Rocks Weekend Market</x:v>
+        <x:v>Opera House → The Rocks</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>逛手作摊位、老街与周末市集</x:v>
+        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
       </x:c>
       <x:c r="F100" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景和本地周末氛围</x:v>
+        <x:v>海港步行衔接悉尼老城区</x:v>
       </x:c>
       <x:c r="G100" t="str">
-        <x:v>周日 10:00–17:00 开放；停留约 45–60 分钟，不必赶着逛完所有摊位</x:v>
+        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
       </x:c>
       <x:c r="H100" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -4241,25 +4449,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B101" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>10:50–11:50</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
       </x:c>
       <x:c r="F101" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
       </x:c>
       <x:c r="G101" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
       </x:c>
       <x:c r="H101" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -4267,25 +4475,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B102" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>11:50–12:40</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Royal Botanic Garden</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
       </x:c>
       <x:c r="F102" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>就地补体力，不为午餐绕路</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -4293,25 +4501,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B103" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>12:40–14:10</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>植物园海港步道</x:v>
       </x:c>
       <x:c r="F103" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G103" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H103" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>botanic-garden-map</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -4319,25 +4527,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B104" t="n">
-        <x:v>90</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>歌剧院 + 海港大桥同框</x:v>
       </x:c>
       <x:c r="F104" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>悉尼最经典机位</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
       </x:c>
       <x:c r="H104" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>mrs-macquarie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -4345,25 +4553,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B105" t="n">
-        <x:v>100</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>晚上</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>购物、室内休息</x:v>
       </x:c>
       <x:c r="F105" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>建筑漂亮，适合逛</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
       </x:c>
       <x:c r="H105" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -4371,51 +4579,51 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B106" t="n">
-        <x:v>900</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>CBD / Darling Harbour</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>Hello Auntie / CBD 晚餐</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H106" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B107" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>08:00</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F107" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H107" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -4423,25 +4631,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B108" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>09:15</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F108" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G108" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H108" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>royal-national-park-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -4449,25 +4657,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B109" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>10:00</x:v>
+        <x:v>09:15</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F109" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>南海岸第一处全景</x:v>
       </x:c>
       <x:c r="G109" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
       </x:c>
       <x:c r="H109" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>bald-hill-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -4475,25 +4683,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B110" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>11:15</x:v>
+        <x:v>10:00</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>贴着太平洋的公路画面</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>不要在桥上或路肩危险停车</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -4501,25 +4709,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B111" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>12:00</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>Wollongong / 南海岸补给</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>短停咖啡或直接通过</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H111" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>wollongong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -4527,25 +4735,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B112" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>Kiama Blowhole</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>看喷潮洞、灯塔与海边</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>Kiama 代表性海岸地貌</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -4553,25 +4761,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B113" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>13:30</x:v>
+        <x:v>12:30–13:30</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>海边小镇节奏</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -4579,25 +4787,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>13:30</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Kiama → Gerringong</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>沿海继续南下</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>kiama-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -4605,25 +4813,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>90</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>14:40</x:v>
+        <x:v>13:45–14:40</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -4631,25 +4839,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>100</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>14:40</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>Gerringong</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>判断是否延伸 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>时间、天气与体力闸门</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>gerringong-map,kangaroo-valley-map</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -4657,25 +4865,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>110</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>可选 15:30–16:15</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>看历史桥、山谷与小镇</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -4683,51 +4891,51 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>900</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>饮食</x:v>
+        <x:v>16:15 前</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>环线收束</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -4735,25 +4943,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>08:30–09:00</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -4761,25 +4969,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>09:15 左右</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -4787,25 +4995,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>09:30–13:30</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -4813,25 +5021,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>13:30–14:30</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>F2 返回市区后前往 Bondi</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>动物园切换到悉尼海岸</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -4839,25 +5047,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>18:30</x:v>
+        <x:v>14:30–17:45</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>海滩散步并走一段 Coastal Walk</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -4865,51 +5073,51 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>饮食</x:v>
+        <x:v>18:30</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -4917,25 +5125,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>oaks-sydney-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -4943,25 +5151,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>可选 09:30 左右</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Circular Quay → Manly</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>搭乘公共 F1 Manly Ferry</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>circular-quay-map,manly-ferry-map</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -4969,25 +5177,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>可选 10:00–12:45</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>Manly Beach / The Corso</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>海边散步、咖啡或早午餐</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -4995,25 +5203,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>13:00–13:30</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>Manly → Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>最晚搭船回市区</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -5021,25 +5229,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>14:00–15:30</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>酒店</x:v>
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>最后采购</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>药妆、保健品、伴手礼</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -5047,25 +5255,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>16:40</x:v>
+        <x:v>15:30–16:20</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>酒店</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>整理 TRS 物品和返程行李</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>为 D16 机场退税做准备</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>oaks-sydney-map,trs-official</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -5073,25 +5281,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>17:30</x:v>
+        <x:v>16:40</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>前往 Cafe Sydney</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>避免迟到</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -5099,51 +5307,51 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>饮食</x:v>
+        <x:v>17:30</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Cafe Sydney</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海港景观 + 澳洲最后一晚</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" t="str">
-        <x:v>d16</x:v>
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -5151,24 +5359,50 @@
         <x:v>d16</x:v>
       </x:c>
       <x:c r="B136" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F136" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G136" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H136" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B137" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C136" t="str">
+      <x:c r="C137" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D136" t="str">
+      <x:c r="D137" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E136" t="str">
+      <x:c r="E137" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F136" t="str">
+      <x:c r="F137" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G136" t="str">
+      <x:c r="G137" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H136"/>
+      <x:c r="H137"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6109,7 +6343,7 @@
         <x:v>the-rocks-market-official</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>The Rocks Weekend Market</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="C49" t="str">
         <x:v>official</x:v>
@@ -7759,6 +7993,44 @@
       </x:c>
       <x:c r="G135" t="str">
         <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>redwoods-otways-map</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>The Redwoods Otways</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=The+Redwoods+Otways+Beech+Forest+VIC</x:v>
+      </x:c>
+      <x:c r="E136" t="str"/>
+      <x:c r="F136" t="str"/>
+      <x:c r="G136" t="str">
+        <x:v>Google Maps · Binns Road, Beech Forest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>redwoods-otways-official</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>Aire Valley Reserve (Red Woods) · Parks Victoria</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>https://www.parks.vic.gov.au/places-to-see/sites/aire-valley-reserve-%28red-woods%29-day-visitor-area</x:v>
+      </x:c>
+      <x:c r="E137" t="str"/>
+      <x:c r="F137" t="str"/>
+      <x:c r="G137" t="str">
+        <x:v>Parks Victoria · 行前查看开放、路况与安全提示</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8913,30 +9185,20 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="23" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Day</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">午餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">晚餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">备注（执行重点）</x:t>
-        </x:is>
+      <x:c r="A1" s="1" t="str">
+        <x:v>Day</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="str">
+        <x:v>早餐</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="str">
+        <x:v>午餐</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="str">
+        <x:v>晚餐</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="str">
+        <x:v>备注（执行重点）</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -8970,7 +9232,7 @@
         <x:v>CBD / Southbank 轻松晚餐</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>集合前吃得简单些；返城后在 Fitzroy / CBD 轻松晚餐，留出整理行李的时间。</x:v>
+        <x:v>Fitzroy 仅作返城后的备选；不去时直接在 CBD 用餐。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
feat: reschedule delayed Melbourne arrival
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rdc8cd11382154c58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R7387639da2d6462f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R0fb52b2b1ed9457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R2a0bb2b4ba4e4109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R761947537f3f425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R0ee3268cad8d424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R009e33f1b3bc4f9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R5380afbfbf964f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R24eb1b66297e47ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R427168c2822445cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R3f31334ec7e4435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R663cd1c4fd3340f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Red1aeccf44b44e3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Redbebfcca78a4cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rc6424f5386344169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rcf49b295d11041e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rf1094558fe274ac3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R17729438aeb54e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Re06e224c17ab4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R848562c4b3ba465b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -745,10 +745,10 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>初到墨尔本：CBD、Carlton 与 QVM 冬季夜市</x:v>
+        <x:v>延误抵达墨尔本：QVM 冬季夜市</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>抵达后慢慢恢复，逛过 CBD 与 Carlton，晚上去 QVM 冬季夜市吃晚餐。</x:v>
+        <x:v>15:15 抵达 MEL；入境、进城并入住后，只安排 QVM Winter Night Market，夜市用餐后回酒店休息。</x:v>
       </x:c>
       <x:c r="J3" t="str">
         <x:v>Oaks Melbourne on Market Hotel</x:v>
@@ -766,16 +766,16 @@
         <x:v>墨尔本清晨城市街景</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>机场接送 + 步行 / 市内交通</x:v>
+        <x:v>机场接送 + rideshare / 步行</x:v>
       </x:c>
       <x:c r="P3" t="str">
-        <x:v>05:55 抵达；入境后直接前往 CBD</x:v>
+        <x:v>15:15 抵达；预计 18:15 左右前往 QVM</x:v>
       </x:c>
       <x:c r="Q3" t="str">
         <x:v>oaks-market-map</x:v>
       </x:c>
       <x:c r="R3" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>qvm-winter-night-market-official</x:v>
       </x:c>
       <x:c r="S3" t="str">
         <x:v>no-fixed-ticket</x:v>
@@ -804,10 +804,10 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>墨尔本近郊：Puffing Billy 与 Sassafras</x:v>
+        <x:v>墨尔本 City Walk + Puffing Billy + Fitzroy</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>上午乘 Puffing Billy 穿行山林；返城后若时间和体力合适，再去 Fitzroy 走走。</x:v>
+        <x:v>上午完成 Degraves Lane、Flinders Street、Hosier Lane 与 State Library 精华 city walk；11:30–17:00 参加 Puffing Billy + Sassafras 半日团，返城后去 Fitzroy 晚餐。</x:v>
       </x:c>
       <x:c r="J4" t="str">
         <x:v>Oaks Melbourne on Market Hotel</x:v>
@@ -825,10 +825,10 @@
         <x:v>Puffing Billy 蒸汽小火车穿过 Dandenong Ranges 森林</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>半日团接驳车 + Puffing Billy 蒸汽火车</x:v>
+        <x:v>步行 + 半日团接驳车 + Puffing Billy + rideshare</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>按通知的集合时间，提前 15 分钟到 343 Russell Street</x:v>
+        <x:v>08:45 酒店出发；11:15 抵达 343 Russell Street</x:v>
       </x:c>
       <x:c r="Q4" t="str">
         <x:v>oaks-market-map</x:v>
@@ -1754,10 +1754,10 @@
         <x:v>Fitzroy</x:v>
       </x:c>
       <x:c r="D4" s="55" t="str">
-        <x:v>备选</x:v>
+        <x:v>必去</x:v>
       </x:c>
       <x:c r="E4" s="54" t="str">
-        <x:v>半日团准时返城且体力合适再去</x:v>
+        <x:v>17:00 返城后前往；若团车延误则缩短停留，保留回酒店整理时间</x:v>
       </x:c>
       <x:c r="F4" s="54" t="str">
         <x:v>fitzroy-map</x:v>
@@ -1922,22 +1922,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>早上</x:v>
+        <x:v>15:15</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>墨尔本机场 → CBD</x:v>
+        <x:v>墨尔本机场 (MEL)</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>入境、取行李，打车 / Uber 或 SkyBus 进城</x:v>
+        <x:v>航班延误后抵达墨尔本</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>初到澳洲，适应南半球冬天</x:v>
+        <x:v>正式落地澳洲</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>4 人加行李较多，打车 / Uber 更舒服；从机场到 CBD 的沿途就是旅程的第一眼。</x:v>
+        <x:v>预留 60–90 分钟办理入境、取行李和会合；流程更快时，把多出的时间留给酒店休息。</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>mel-airport-map,flight-cathay</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1948,22 +1948,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>上午</x:v>
+        <x:v>15:15–17:30 预计</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>CBD / 酒店附近</x:v>
+        <x:v>MEL → Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>酒店寄存行李 + 咖啡早餐</x:v>
+        <x:v>入境、取行李后四人打车 / Uber 进城</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>墨尔本咖啡文化开场</x:v>
+        <x:v>减少延误后的转场消耗</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>先寄存行李，找一家街角 café 吃早餐，让身体慢慢进入墨尔本节奏。</x:v>
+        <x:v>4 人加多件行李，rideshare / taxi 最省力；CBD 城市步行集中放到 D2 上午。</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>oaks-market-map,oaks-market-booking,operator25-map</x:v>
+        <x:v>mel-airport-map,oaks-market-map,oaks-market-booking</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1974,22 +1974,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>中午</x:v>
+        <x:v>17:30–18:10 预计</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Degraves Lane / Flinders Street 一带</x:v>
+        <x:v>Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>轻量午餐 / café / laneway walk</x:v>
+        <x:v>入住、放行李、换衣服，短暂休息</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>墨尔本巷弄文化</x:v>
+        <x:v>夜市前快速恢复</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>体力一般时走 Degraves Lane 与 Flinders Street 已经很充实；有余力再继续。</x:v>
+        <x:v>如果到店较晚，就缩短夜市停留，保证睡眠。</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>degraves-map,flinders-street-map</x:v>
+        <x:v>oaks-market-map,oaks-market-booking</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2000,22 +2000,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>下午</x:v>
+        <x:v>18:15–20:30</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>State Library of Victoria</x:v>
+        <x:v>Queen Victoria Market</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>参观经典阅览室</x:v>
+        <x:v>QVM Winter Night Market：边逛边吃晚餐</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>历史建筑 + 圆顶阅览室</x:v>
+        <x:v>冬季周三限定夜市</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>在圆顶阅览室停留片刻即可，六楼俯拍视角最完整。</x:v>
+        <x:v>周三 17:00–22:00，免费入场、免预约；实际到达可随入境与路况顺延。</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>state-library-map</x:v>
+        <x:v>qvm-map,qvm-winter-night-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2023,25 +2023,25 @@
         <x:v>d1</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>下午</x:v>
+        <x:v>20:30–21:00</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Carlton / Lygon Street (Little Italy)</x:v>
+        <x:v>QVM → Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>从 State Library 向北前往 Carlton，沿 Lygon Street 散步，安排咖啡或 gelato</x:v>
+        <x:v>返回酒店、洗漱休息</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>墨尔本意大利移民街区 + café culture</x:v>
+        <x:v>给 D2 上午 city walk 留足体力</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>建议预留 60–90 分钟，在 Lygon Street 喝咖啡或吃 gelato；抵达较晚时可略过 NGV。</x:v>
+        <x:v>夜市结束后直接回酒店，早点休息。</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>carlton-lygon-map</x:v>
+        <x:v>qvm-map,oaks-market-map,qvm-winter-night-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2049,155 +2049,155 @@
         <x:v>d1</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>Hosier Lane</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>涂鸦巷拍照</x:v>
+        <x:v>早餐 / 午餐：航班与机场按实际情况；晚餐：QVM Winter Night Market 街头热食</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>街头艺术 + 文艺墨尔本</x:v>
+        <x:v>落地日餐食</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>预留 20–30 分钟，选一面喜欢的涂鸦墙慢慢拍。</x:v>
+        <x:v>不预订正式餐厅，夜市边逛边吃最轻松。</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>hosier-map</x:v>
+        <x:v>qvm-map,qvm-winter-night-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>d1</x:v>
+        <x:v>d2</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:v>60</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>可选</x:v>
+        <x:v>08:45</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>NGV</x:v>
+        <x:v>Oaks Melbourne on Market → Degraves Street</x:v>
       </x:c>
       <x:c r="E9" t="str">
-        <x:v>天气冷 / 想室内休息时进入</x:v>
+        <x:v>步行出发，开始集合前的精华 city walk</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>冬天避风避寒</x:v>
+        <x:v>用一个上午补上墨尔本城市经典</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>天气冷或想在室内休息时再去；时间有限可直接前往 Carlton。</x:v>
+        <x:v>随身只带轻便小包；各站按时间收口。</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>ngv-map</x:v>
+        <x:v>oaks-market-map,degraves-map</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>d1</x:v>
+        <x:v>d2</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>65</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>天气与体力备选</x:v>
+        <x:v>09:00–09:20</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Point Ormond Reserve / Lookout</x:v>
+        <x:v>Degraves Street</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>16:00 查看雷达与云量；条件合适时四人 rideshare 前往 Elwood，沿既有步道与 lookout 看海湾黄昏，再直接去 QVM</x:v>
+        <x:v>快速早餐 / Flat White + 巷弄短拍</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>Port Phillip Bay 日落 + 墨尔本城市轮廓</x:v>
+        <x:v>墨尔本 laneway 与 café culture</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>约 16:20-16:30 从 CBD 出发，16:50-17:40 停留，18:15 左右抵达 QVM；阴雨、风大或落地疲惫时直接跳过，穿防风防水层并留在有照明的步道和观景区。</x:v>
+        <x:v>停留约 20 分钟，早餐以快速出餐为主。</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>point-ormond-map,point-ormond-official</x:v>
+        <x:v>degraves-map</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>d1</x:v>
+        <x:v>d2</x:v>
       </x:c>
       <x:c r="B11" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>09:20–09:40</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>Queen Victoria Market</x:v>
+        <x:v>Flinders Street Station / Federation Square</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>17:30-19:30 QVM Winter Night Market</x:v>
+        <x:v>拍车站外观和广场城市景观</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>冬季周三限定夜市</x:v>
+        <x:v>经典墨尔本地标</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>开放时间 17:00-22:00，免费入场、免预约；建议 17:30 左右到，按体力逛 30–120 分钟。</x:v>
+        <x:v>以外观和街景为主，09:40 前前往 Hosier Lane。</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>qvm-map,qvm-winter-night-market-official</x:v>
+        <x:v>flinders-street-map</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>d1</x:v>
+        <x:v>d2</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>晚上</x:v>
+        <x:v>09:40–10:00</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>QVM → Oaks Melbourne on Market Hotel</x:v>
+        <x:v>Hosier Lane</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>夜市用餐后直接回酒店休息</x:v>
+        <x:v>涂鸦巷短停拍照</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>落地日收尾</x:v>
+        <x:v>街头艺术 + 文艺墨尔本</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>在夜市吃过晚餐就回酒店休息；体力有限时逛 30–60 分钟也很合适。</x:v>
+        <x:v>控制在 20 分钟，随后直接前往 State Library。</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>qvm-map,oaks-market-map,qvm-winter-night-market-official</x:v>
+        <x:v>hosier-map</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>d1</x:v>
+        <x:v>d2</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>饮食</x:v>
+        <x:v>10:10–10:45</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>State Library of Victoria</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>早餐：CBD café / Operator25（可选 Brunch）；午餐：Degraves Lane / CBD 简餐 / Pho Tùng（可选）；Carlton：咖啡或 gelato；晚餐：QVM Winter Night Market 街头热食（主）/ CBD 简餐（体力不足）</x:v>
+        <x:v>重点看 La Trobe Reading Room 与六楼俯拍视角</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>历史建筑 + 圆顶阅览室</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>Carlton 适合用一杯咖啡或 gelato 稍作休息；晚餐就在 QVM 冬季夜市边逛边吃。</x:v>
+        <x:v>10:45 离开；遇到开馆或排队变化时，以 11:15 抵达集合点为准。</x:v>
       </x:c>
       <x:c r="H13" t="str">
-        <x:v>qvm-map,qvm-winter-night-market-official,operator25-map,pho-tung-map,degraves-map</x:v>
+        <x:v>state-library-map</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2205,25 +2205,25 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>10</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>早上</x:v>
+        <x:v>10:45–11:15</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>Oaks Melbourne on Market → 343 Russell Street</x:v>
+        <x:v>State Library → 343 Russell Street</x:v>
       </x:c>
       <x:c r="E14" t="str">
-        <x:v>前往 Klook / Oznara 集合点</x:v>
+        <x:v>步行到集合点，留出签到与洗手间时间</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>集合点在 CBD 内</x:v>
+        <x:v>提前 15 分钟到场</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>从酒店打车约 7-12 分钟，步行约 20-25 分钟；建议打车</x:v>
+        <x:v>11:15 是硬截止；city walk 任一站超时，优先保证准时集合。</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>oaks-market-map,russell-343-map,klook-oznara-puffing-billy-note</x:v>
+        <x:v>state-library-map,russell-343-map,klook-oznara-puffing-billy-note</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2231,22 +2231,22 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B15" t="n">
-        <x:v>20</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>上午</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D15" t="str">
         <x:v>343 Russell Street</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>Klook / Oznara 半日团集合</x:v>
+        <x:v>Klook / Oznara 半日团签到</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>Puffing Billy + Sassafras 行程开始</x:v>
+        <x:v>11:30 准时开始 Puffing Billy + Sassafras 行程</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>具体 pickup 时间以前一天通知为准；提前 10-15 分钟到</x:v>
+        <x:v>已确认团期 11:30–17:00；当天细节以 operator 通知为准。</x:v>
       </x:c>
       <x:c r="H15" t="str">
         <x:v>russell-343-map,klook-oznara-puffing-billy-note</x:v>
@@ -2257,25 +2257,25 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B16" t="n">
-        <x:v>30</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>上午</x:v>
+        <x:v>11:30–17:00</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>Melbourne CBD → Belgrave</x:v>
+        <x:v>Puffing Billy + Sassafras 半日团</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>乘团车前往 Puffing Billy Railway</x:v>
+        <x:v>随团前往 Belgrave，乘 Puffing Billy，游览 Lakeside / Emerald Lake Park 与 Sassafras 后返城</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>进入 Dandenong Ranges 近郊</x:v>
+        <x:v>蒸汽火车、Dandenong Ranges 山林与小镇</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>路上可休息，不用自己研究公共交通</x:v>
+        <x:v>11:30–17:00 为完整团期；注意保暖，团内节点以向导安排为准。</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>puffing-billy-map,puffing-billy-official,klook-oznara-puffing-billy-note</x:v>
+        <x:v>russell-343-map,puffing-billy-map,puffing-billy-official,lakeside-station-map,sassafras-map,klook-oznara-puffing-billy-note</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2283,22 +2283,22 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B17" t="n">
-        <x:v>40</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>团内</x:v>
       </x:c>
       <x:c r="D17" t="str">
         <x:v>Puffing Billy Railway</x:v>
       </x:c>
       <x:c r="E17" t="str">
-        <x:v>Belgrave-Lakeside 往返蒸汽小火车体验</x:v>
+        <x:v>Belgrave–Lakeside 往返蒸汽小火车体验</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>复古蒸汽火车、森林、木桥、Dandenong Ranges 山林氛围</x:v>
+        <x:v>复古蒸汽火车、森林与木桥</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>注意保暖，车厢和山林会冷</x:v>
+        <x:v>车厢和山林会冷，防风外套放在手边。</x:v>
       </x:c>
       <x:c r="H17" t="str">
         <x:v>puffing-billy-map,puffing-billy-official,lakeside-station-map</x:v>
@@ -2309,22 +2309,22 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B18" t="n">
-        <x:v>50</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>中午 / 下午</x:v>
+        <x:v>团内</x:v>
       </x:c>
       <x:c r="D18" t="str">
         <x:v>Lakeside / Emerald Lake Park</x:v>
       </x:c>
       <x:c r="E18" t="str">
-        <x:v>湖边短停 / visitor centre / café / 简单休息</x:v>
+        <x:v>湖边、游客中心与 café 短停</x:v>
       </x:c>
       <x:c r="F18" t="str">
-        <x:v>湖边公园、游客中心、火车站台氛围</x:v>
+        <x:v>火车站台与湖边公园氛围</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>沿湖边和游客中心轻松走走，留出返程时间。</x:v>
+        <x:v>沿湖轻松走走，跟随向导掌握集合时间。</x:v>
       </x:c>
       <x:c r="H18" t="str">
         <x:v>emerald-lake-park-map,lakeside-station-map</x:v>
@@ -2335,22 +2335,22 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B19" t="n">
-        <x:v>60</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>中午 / 下午</x:v>
+        <x:v>团内</x:v>
       </x:c>
       <x:c r="D19" t="str">
         <x:v>Sassafras</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>小镇短停</x:v>
+        <x:v>小镇短停，逛店或喝热饮</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>茶屋、糖果店、Dandenong Ranges 小镇感</x:v>
+        <x:v>Dandenong Ranges 小镇感</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>逛一两家小店、喝杯热饮即可，注意返程集合时间。</x:v>
+        <x:v>停留时长由团队安排，按时回到集合点。</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>sassafras-map</x:v>
@@ -2361,25 +2361,25 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B20" t="n">
-        <x:v>70</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>下午</x:v>
+        <x:v>17:00 预计</x:v>
       </x:c>
       <x:c r="D20" t="str">
         <x:v>返回 343 Russell Street</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>半日团结束，回到 CBD</x:v>
+        <x:v>半日团结束，直接转场 Fitzroy</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>返城后继续 Fitzroy 街区漫步</x:v>
+        <x:v>从近郊自然切回本地街区</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>半日团结束后直接前往 Fitzroy；保持约 90 分钟街区时间</x:v>
+        <x:v>团车延误时缩短 Fitzroy 停留，保留回酒店整理行李的时间。</x:v>
       </x:c>
       <x:c r="H20" t="str">
-        <x:v>russell-343-map</x:v>
+        <x:v>russell-343-map,fitzroy-map</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2387,22 +2387,22 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B21" t="n">
-        <x:v>80</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>备选 · 下午后段</x:v>
+        <x:v>17:15–19:30</x:v>
       </x:c>
       <x:c r="D21" t="str">
         <x:v>Fitzroy: Brunswick Street → Gertrude Street</x:v>
       </x:c>
       <x:c r="E21" t="str">
-        <x:v>若半日团准时返城且体力充足，再沿 Brunswick Street / Gertrude Street 随意走走。</x:v>
+        <x:v>rideshare 前往 Fitzroy，沿街散步并吃晚餐</x:v>
       </x:c>
       <x:c r="F21" t="str">
-        <x:v>街区小店、咖啡与旧工业街景</x:v>
+        <x:v>街头艺术、老建筑与本地生活版墨尔本</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>把 Fitzroy 当作加分项；返城较晚或需要休息时直接回酒店。</x:v>
+        <x:v>以街区漫步和晚餐为主；19:30 左右返程。</x:v>
       </x:c>
       <x:c r="H21" t="str">
         <x:v>fitzroy-map,russell-343-map</x:v>
@@ -2413,25 +2413,25 @@
         <x:v>d2</x:v>
       </x:c>
       <x:c r="B22" t="n">
-        <x:v>90</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>晚上</x:v>
+        <x:v>19:30–21:00</x:v>
       </x:c>
       <x:c r="D22" t="str">
-        <x:v>酒店 / CBD</x:v>
+        <x:v>Fitzroy → Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E22" t="str">
-        <x:v>简单晚餐 + 整理大洋路行李</x:v>
+        <x:v>回酒店整理大洋路登机箱和随身包</x:v>
       </x:c>
       <x:c r="F22" t="str">
-        <x:v>为次日大洋路做好准备</x:v>
+        <x:v>为 D3 机场取车做好准备</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>大件行李寄存，只带登机箱和随身包上大洋路；早点睡</x:v>
+        <x:v>21:00 前回酒店；大件行李寄存，只带登机箱和随身包上大洋路。</x:v>
       </x:c>
       <x:c r="H22" t="str">
-        <x:v>oaks-market-map,southbank-map</x:v>
+        <x:v>fitzroy-map,oaks-market-map</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2448,16 +2448,16 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E23" t="str">
-        <x:v>早餐：酒店附近 café / 集合前简单吃；午餐：Lakeside / Emerald Lake Park café 或团中简餐；晚餐：CBD / Southbank 轻松晚餐</x:v>
+        <x:v>早餐：Degraves Street café / Flat White；午餐：Lakeside / 团中简餐；晚餐：Fitzroy</x:v>
       </x:c>
       <x:c r="F23" t="str">
         <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>Fitzroy 仅作返城后的备选；不去时直接在 CBD 用餐。</x:v>
+        <x:v>早餐要快，午餐服从团内节奏；晚餐放在 Fitzroy，回酒店后只整理行李。</x:v>
       </x:c>
       <x:c r="H23" t="str">
-        <x:v>russell-343-map,emerald-lake-park-map,sassafras-map,southbank-map</x:v>
+        <x:v>degraves-map,emerald-lake-park-map,sassafras-map,fitzroy-map</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -8380,7 +8380,7 @@
         <x:v>¥2,352</x:v>
       </x:c>
       <x:c r="F2" s="28" t="str">
-        <x:v>D2 使用；Klook / Oznara 半日团，343 Russell Street 集合，含 Puffing Billy 与 Sassafras</x:v>
+        <x:v>D2 11:30–17:00 使用；Klook / Oznara 半日团，343 Russell Street 集合，含 Puffing Billy 与 Sassafras。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="23" customFormat="1" ht="26.399999618530273" customHeight="1">
@@ -8673,10 +8673,8 @@
           <x:t xml:space="preserve">Melbourne CBD / 市中心</x:t>
         </x:is>
       </x:c>
-      <x:c r="H2" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">适合 D1 恢复、D2 市区步行、D3 市区提车出发大洋路；靠近 Yarra River、Southbank、Flinders Street 一带</x:t>
-        </x:is>
+      <x:c r="H2" s="28" t="str">
+        <x:v>适合 D1 延误抵达后入住并前往 QVM；D2 上午 CBD city walk、11:30–17:00 Puffing Billy 半日团，返城后去 Fitzroy；D3 退房后前往机场取车。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9177,16 +9175,16 @@
         <x:v>D1 墨尔本</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>CBD café / Operator25（可选Brunch）</x:v>
+        <x:v>航班 / 机场按实际情况</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Degraves Lane / CBD 简餐 / Pho Tùng（可选）</x:v>
+        <x:v>航班 / 机场按实际情况</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>QVM Winter Night Market 街头热食（主）/ Carlton / Lygon Street café 或 gelato / CBD 简餐（体力不足）</x:v>
+        <x:v>QVM Winter Night Market 街头热食</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>Carlton 适合用一杯咖啡或 gelato 稍作休息；晚餐就在 QVM 冬季夜市边逛边吃。</x:v>
+        <x:v>15:15 抵达；酒店入住后只去 QVM，夜市用餐后回酒店休息。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9194,16 +9192,16 @@
         <x:v>D2 墨尔本 + Puffing Billy / Sassafras</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>酒店附近 café / 集合前简单吃</x:v>
+        <x:v>Degraves Street café / Flat White</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Lakeside / Emerald Lake Park café 或团中简餐</x:v>
+        <x:v>Lakeside / 团中简餐</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>CBD / Southbank 轻松晚餐</x:v>
+        <x:v>Fitzroy 晚餐</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>Fitzroy 仅作返城后的备选；不去时直接在 CBD 用餐。</x:v>
+        <x:v>08:45 开始 city walk；11:15 到 343 Russell Street；11:30–17:00 参加半日团；Fitzroy 后 21:00 前回酒店。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
refine Melbourne day copy
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R3f31334ec7e4435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R663cd1c4fd3340f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Red1aeccf44b44e3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Redbebfcca78a4cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rc6424f5386344169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rcf49b295d11041e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rf1094558fe274ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R17729438aeb54e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Re06e224c17ab4a8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R848562c4b3ba465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R73ad8c33bf994673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R787c33d346004b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R41862d9a24f74128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R8ea84605e4724396"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R50e470a307ca4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R633f3e2f87804860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rdc447f2d6bdf488a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R540d7fb6de794640"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Rd1d00d772725456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Rc152a1542a9c4987"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -745,10 +745,10 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>延误抵达墨尔本：QVM 冬季夜市</x:v>
+        <x:v>初到墨尔本：QVM 冬季夜市</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>15:15 抵达 MEL；入境、进城并入住后，只安排 QVM Winter Night Market，夜市用餐后回酒店休息。</x:v>
+        <x:v>下午抵达墨尔本，入住稍作休整，晚上在 QVM Winter Night Market 边逛边吃，轻松开启南半球旅程。</x:v>
       </x:c>
       <x:c r="J3" t="str">
         <x:v>Oaks Melbourne on Market Hotel</x:v>
@@ -763,13 +763,13 @@
         <x:v>/itinerary/melbourne-city-morning.png</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>墨尔本清晨城市街景</x:v>
+        <x:v>墨尔本冬日城市街景</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>机场接送 + rideshare / 步行</x:v>
+        <x:v>机场出租车 / Uber + 市区步行</x:v>
       </x:c>
       <x:c r="P3" t="str">
-        <x:v>15:15 抵达；预计 18:15 左右前往 QVM</x:v>
+        <x:v>15:15 抵达 MEL；约 18:15 从酒店前往 QVM</x:v>
       </x:c>
       <x:c r="Q3" t="str">
         <x:v>oaks-market-map</x:v>
@@ -795,7 +795,7 @@
         <x:v>周四</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>墨尔本 + Belgrave</x:v>
+        <x:v>墨尔本 + Dandenong Ranges</x:v>
       </x:c>
       <x:c r="F4" t="n">
         <x:v>-37.8136</x:v>
@@ -804,10 +804,10 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>墨尔本 City Walk + Puffing Billy + Fitzroy</x:v>
+        <x:v>从城市巷弄到山林：Puffing Billy 与 Fitzroy</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>上午完成 Degraves Lane、Flinders Street、Hosier Lane 与 State Library 精华 city walk；11:30–17:00 参加 Puffing Billy + Sassafras 半日团，返城后去 Fitzroy 晚餐。</x:v>
+        <x:v>上午走过 Degraves Street、Flinders Street 与 Hosier Lane，在州立图书馆俯瞰圆顶阅览室；午后乘 Puffing Billy 穿行山林，返城后去 Fitzroy 散步吃晚餐。</x:v>
       </x:c>
       <x:c r="J4" t="str">
         <x:v>Oaks Melbourne on Market Hotel</x:v>
@@ -825,10 +825,10 @@
         <x:v>Puffing Billy 蒸汽小火车穿过 Dandenong Ranges 森林</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>步行 + 半日团接驳车 + Puffing Billy + rideshare</x:v>
+        <x:v>市区步行 + 半日团接驳 + Puffing Billy + Uber</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>08:45 酒店出发；11:15 抵达 343 Russell Street</x:v>
+        <x:v>08:45 从酒店出发；11:15 抵达 343 Russell Street</x:v>
       </x:c>
       <x:c r="Q4" t="str">
         <x:v>oaks-market-map</x:v>
@@ -1757,7 +1757,7 @@
         <x:v>必去</x:v>
       </x:c>
       <x:c r="E4" s="54" t="str">
-        <x:v>17:00 返城后前往；若团车延误则缩短停留，保留回酒店整理时间</x:v>
+        <x:v>17:00 左右返城后前往，沿 Brunswick Street 与 Gertrude Street 散步吃晚餐</x:v>
       </x:c>
       <x:c r="F4" s="54" t="str">
         <x:v>fitzroy-map</x:v>
@@ -1928,13 +1928,13 @@
         <x:v>墨尔本机场 (MEL)</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>航班延误后抵达墨尔本</x:v>
+        <x:v>抵达墨尔本，办理入境并领取行李</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>正式落地澳洲</x:v>
+        <x:v>南半球旅程正式开始</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>预留 60–90 分钟办理入境、取行李和会合；流程更快时，把多出的时间留给酒店休息。</x:v>
+        <x:v>预留 60–90 分钟办理入境、取行李并与同行人会合；落地日不必赶行程。</x:v>
       </x:c>
       <x:c r="H3" t="str">
         <x:v>mel-airport-map,flight-cathay</x:v>
@@ -1954,13 +1954,13 @@
         <x:v>MEL → Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>入境、取行李后四人打车 / Uber 进城</x:v>
+        <x:v>乘出租车 / Uber 前往酒店</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>减少延误后的转场消耗</x:v>
+        <x:v>从机场驶入冬日墨尔本</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>4 人加多件行李，rideshare / taxi 最省力；CBD 城市步行集中放到 D2 上午。</x:v>
+        <x:v>四人带多件行李，出租车 / Uber 更省心；车上看看窗外，让身体慢慢适应新的城市。</x:v>
       </x:c>
       <x:c r="H4" t="str">
         <x:v>mel-airport-map,oaks-market-map,oaks-market-booking</x:v>
@@ -1980,13 +1980,13 @@
         <x:v>Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>入住、放行李、换衣服，短暂休息</x:v>
+        <x:v>入住、放下行李，换好保暖衣物后稍作休息</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>夜市前快速恢复</x:v>
+        <x:v>在出门前缓一缓</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>如果到店较晚，就缩短夜市停留，保证睡眠。</x:v>
+        <x:v>如果到店稍晚，就少逛一会儿夜市，按照自己的状态安排。</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>oaks-market-map,oaks-market-booking</x:v>
@@ -2006,13 +2006,13 @@
         <x:v>Queen Victoria Market</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>QVM Winter Night Market：边逛边吃晚餐</x:v>
+        <x:v>逛 QVM Winter Night Market，边走边吃晚餐</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>冬季周三限定夜市</x:v>
+        <x:v>灯光、热食、现场音乐与墨尔本冬夜</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>周三 17:00–22:00，免费入场、免预约；实际到达可随入境与路况顺延。</x:v>
+        <x:v>周三 17:00–22:00，免费入场、免预约；入境或路况较慢也不用着急，夜市会营业到 22:00。</x:v>
       </x:c>
       <x:c r="H6" t="str">
         <x:v>qvm-map,qvm-winter-night-market-official</x:v>
@@ -2032,13 +2032,13 @@
         <x:v>QVM → Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>返回酒店、洗漱休息</x:v>
+        <x:v>散步或打车回酒店，洗漱休息</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>给 D2 上午 city walk 留足体力</x:v>
+        <x:v>冬夜里的轻松收尾</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>夜市结束后直接回酒店，早点休息。</x:v>
+        <x:v>吃饱后直接回酒店，早点休息。</x:v>
       </x:c>
       <x:c r="H7" t="str">
         <x:v>qvm-map,oaks-market-map,qvm-winter-night-market-official</x:v>
@@ -2058,13 +2058,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>早餐 / 午餐：航班与机场按实际情况；晚餐：QVM Winter Night Market 街头热食</x:v>
+        <x:v>早餐 / 午餐：随航班安排；晚餐：QVM Winter Night Market 街头热食</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>落地日餐食</x:v>
+        <x:v>从一顿热腾腾的夜市晚餐开始</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>不预订正式餐厅，夜市边逛边吃最轻松。</x:v>
+        <x:v>把胃口留给夜市，热食、甜点和热饮可以边走边选。</x:v>
       </x:c>
       <x:c r="H8" t="str">
         <x:v>qvm-map,qvm-winter-night-market-official</x:v>
@@ -2084,13 +2084,13 @@
         <x:v>Oaks Melbourne on Market → Degraves Street</x:v>
       </x:c>
       <x:c r="E9" t="str">
-        <x:v>步行出发，开始集合前的精华 city walk</x:v>
+        <x:v>从酒店步行到 Degraves Street，开始上午的城市漫步</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>用一个上午补上墨尔本城市经典</x:v>
+        <x:v>墨尔本清晨的街道与巷弄</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>随身只带轻便小包；各站按时间收口。</x:v>
+        <x:v>随身带轻便小包，城市漫步结束后直接步行去 Russell Street 集合。</x:v>
       </x:c>
       <x:c r="H9" t="str">
         <x:v>oaks-market-map,degraves-map</x:v>
@@ -2110,13 +2110,13 @@
         <x:v>Degraves Street</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>快速早餐 / Flat White + 巷弄短拍</x:v>
+        <x:v>在巷弄 café 吃早餐，点一杯 Flat White</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>墨尔本 laneway 与 café culture</x:v>
+        <x:v>墨尔本巷弄与咖啡文化</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>停留约 20 分钟，早餐以快速出餐为主。</x:v>
+        <x:v>选一家出餐快的店，边吃边感受巷子醒来的样子。</x:v>
       </x:c>
       <x:c r="H10" t="str">
         <x:v>degraves-map</x:v>
@@ -2136,13 +2136,13 @@
         <x:v>Flinders Street Station / Federation Square</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>拍车站外观和广场城市景观</x:v>
+        <x:v>看看 Flinders Street Station 外观，顺路走过 Federation Square</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>经典墨尔本地标</x:v>
+        <x:v>红砖钟楼与现代广场的城市对照</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>以外观和街景为主，09:40 前前往 Hosier Lane。</x:v>
+        <x:v>在车站对面拍一张全景，再沿 Flinders Street 走向 Hosier Lane。</x:v>
       </x:c>
       <x:c r="H11" t="str">
         <x:v>flinders-street-map</x:v>
@@ -2162,13 +2162,13 @@
         <x:v>Hosier Lane</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>涂鸦巷短停拍照</x:v>
+        <x:v>走进涂鸦巷，看看不断变化的墙面</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>街头艺术 + 文艺墨尔本</x:v>
+        <x:v>色彩密集的墨尔本街头艺术</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>控制在 20 分钟，随后直接前往 State Library。</x:v>
+        <x:v>停留约 20 分钟，选几面喜欢的墙拍照，再步行去州立图书馆。</x:v>
       </x:c>
       <x:c r="H12" t="str">
         <x:v>hosier-map</x:v>
@@ -2188,13 +2188,13 @@
         <x:v>State Library of Victoria</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>重点看 La Trobe Reading Room 与六楼俯拍视角</x:v>
+        <x:v>走进 La Trobe Reading Room，从六楼俯瞰圆顶阅览室</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>历史建筑 + 圆顶阅览室</x:v>
+        <x:v>白色书桌、穹顶与安静的阅读空间</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>10:45 离开；遇到开馆或排队变化时，以 11:15 抵达集合点为准。</x:v>
+        <x:v>10:45 左右离开，给步行到集合点和签到留足时间。</x:v>
       </x:c>
       <x:c r="H13" t="str">
         <x:v>state-library-map</x:v>
@@ -2214,13 +2214,13 @@
         <x:v>State Library → 343 Russell Street</x:v>
       </x:c>
       <x:c r="E14" t="str">
-        <x:v>步行到集合点，留出签到与洗手间时间</x:v>
+        <x:v>沿 Russell Street 步行到半日团集合点</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>提前 15 分钟到场</x:v>
+        <x:v>从城市漫步走向下一段旅程</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>11:15 是硬截止；city walk 任一站超时，优先保证准时集合。</x:v>
+        <x:v>建议 11:15 前抵达，可先使用洗手间并办理签到。</x:v>
       </x:c>
       <x:c r="H14" t="str">
         <x:v>state-library-map,russell-343-map,klook-oznara-puffing-billy-note</x:v>
@@ -2240,13 +2240,13 @@
         <x:v>343 Russell Street</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>Klook / Oznara 半日团签到</x:v>
+        <x:v>与团队会合，办理签到</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>11:30 准时开始 Puffing Billy + Sassafras 行程</x:v>
+        <x:v>Dandenong Ranges 山林之旅即将开始</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>已确认团期 11:30–17:00；当天细节以 operator 通知为准。</x:v>
+        <x:v>团车 11:30 出发，当天细节以运营方通知为准。</x:v>
       </x:c>
       <x:c r="H15" t="str">
         <x:v>russell-343-map,klook-oznara-puffing-billy-note</x:v>
@@ -2266,13 +2266,13 @@
         <x:v>Puffing Billy + Sassafras 半日团</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>随团前往 Belgrave，乘 Puffing Billy，游览 Lakeside / Emerald Lake Park 与 Sassafras 后返城</x:v>
+        <x:v>乘团车前往 Belgrave，搭乘 Puffing Billy，游览 Lakeside 与 Sassafras 后返回市区</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>蒸汽火车、Dandenong Ranges 山林与小镇</x:v>
+        <x:v>蒸汽火车、山林、湖畔与小镇</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>11:30–17:00 为完整团期；注意保暖，团内节点以向导安排为准。</x:v>
+        <x:v>山里比市区更凉，防风外套放在手边；沿途留意向导的集合时间。</x:v>
       </x:c>
       <x:c r="H16" t="str">
         <x:v>russell-343-map,puffing-billy-map,puffing-billy-official,lakeside-station-map,sassafras-map,klook-oznara-puffing-billy-note</x:v>
@@ -2292,13 +2292,13 @@
         <x:v>Puffing Billy Railway</x:v>
       </x:c>
       <x:c r="E17" t="str">
-        <x:v>Belgrave–Lakeside 往返蒸汽小火车体验</x:v>
+        <x:v>乘复古蒸汽火车从 Belgrave 穿行至 Lakeside</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>复古蒸汽火车、森林与木桥</x:v>
+        <x:v>开放式车厢、森林与木桥</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>车厢和山林会冷，防风外套放在手边。</x:v>
+        <x:v>靠窗能更贴近山林；注意防风保暖，并遵守现场安全提示。</x:v>
       </x:c>
       <x:c r="H17" t="str">
         <x:v>puffing-billy-map,puffing-billy-official,lakeside-station-map</x:v>
@@ -2318,13 +2318,13 @@
         <x:v>Lakeside / Emerald Lake Park</x:v>
       </x:c>
       <x:c r="E18" t="str">
-        <x:v>湖边、游客中心与 café 短停</x:v>
+        <x:v>在湖边散步，看看游客中心与火车站台</x:v>
       </x:c>
       <x:c r="F18" t="str">
-        <x:v>火车站台与湖边公园氛围</x:v>
+        <x:v>湖水、树林与复古车站</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>沿湖轻松走走，跟随向导掌握集合时间。</x:v>
+        <x:v>轻松走一小段即可，留意向导通知的集合时间。</x:v>
       </x:c>
       <x:c r="H18" t="str">
         <x:v>emerald-lake-park-map,lakeside-station-map</x:v>
@@ -2344,13 +2344,13 @@
         <x:v>Sassafras</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>小镇短停，逛店或喝热饮</x:v>
+        <x:v>逛一两家小店，喝杯热饮</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>Dandenong Ranges 小镇感</x:v>
+        <x:v>茶屋、糖果店与山间小镇气息</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>停留时长由团队安排，按时回到集合点。</x:v>
+        <x:v>冬日下午适合慢慢看看橱窗，记得按集合时间返回。</x:v>
       </x:c>
       <x:c r="H19" t="str">
         <x:v>sassafras-map</x:v>
@@ -2370,13 +2370,13 @@
         <x:v>返回 343 Russell Street</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>半日团结束，直接转场 Fitzroy</x:v>
+        <x:v>回到市区后，乘 Uber 前往 Fitzroy</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>从近郊自然切回本地街区</x:v>
+        <x:v>从山林切换到墨尔本街区夜色</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>团车延误时缩短 Fitzroy 停留，保留回酒店整理行李的时间。</x:v>
+        <x:v>如果返程稍晚，就把 Fitzroy 留给散步和晚餐，不必再赶更多地方。</x:v>
       </x:c>
       <x:c r="H20" t="str">
         <x:v>russell-343-map,fitzroy-map</x:v>
@@ -2396,13 +2396,13 @@
         <x:v>Fitzroy: Brunswick Street → Gertrude Street</x:v>
       </x:c>
       <x:c r="E21" t="str">
-        <x:v>rideshare 前往 Fitzroy，沿街散步并吃晚餐</x:v>
+        <x:v>沿 Brunswick Street 走到 Gertrude Street，逛小店、看街头艺术并吃晚餐</x:v>
       </x:c>
       <x:c r="F21" t="str">
-        <x:v>街头艺术、老建筑与本地生活版墨尔本</x:v>
+        <x:v>独立店铺、老建筑与本地街区氛围</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>以街区漫步和晚餐为主；19:30 左右返程。</x:v>
+        <x:v>不用逐店打卡，边走边选一家喜欢的餐厅即可。</x:v>
       </x:c>
       <x:c r="H21" t="str">
         <x:v>fitzroy-map,russell-343-map</x:v>
@@ -2422,13 +2422,13 @@
         <x:v>Fitzroy → Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E22" t="str">
-        <x:v>回酒店整理大洋路登机箱和随身包</x:v>
+        <x:v>回酒店，整理大洋路随身行李</x:v>
       </x:c>
       <x:c r="F22" t="str">
-        <x:v>为 D3 机场取车做好准备</x:v>
+        <x:v>把冬装和摄影设备装进登机箱</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>21:00 前回酒店；大件行李寄存，只带登机箱和随身包上大洋路。</x:v>
+        <x:v>四个大箱留在酒店，只带登机箱和随身包上路；早点休息。</x:v>
       </x:c>
       <x:c r="H22" t="str">
         <x:v>fitzroy-map,oaks-market-map</x:v>
@@ -2451,10 +2451,10 @@
         <x:v>早餐：Degraves Street café / Flat White；午餐：Lakeside / 团中简餐；晚餐：Fitzroy</x:v>
       </x:c>
       <x:c r="F23" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>从巷弄咖啡到街区晚餐</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>早餐要快，午餐服从团内节奏；晚餐放在 Fitzroy，回酒店后只整理行李。</x:v>
+        <x:v>早餐简单一点，午餐跟随团队安排，晚餐留给 Fitzroy。</x:v>
       </x:c>
       <x:c r="H23" t="str">
         <x:v>degraves-map,emerald-lake-park-map,sassafras-map,fitzroy-map</x:v>
@@ -8380,7 +8380,7 @@
         <x:v>¥2,352</x:v>
       </x:c>
       <x:c r="F2" s="28" t="str">
-        <x:v>D2 11:30–17:00 使用；Klook / Oznara 半日团，343 Russell Street 集合，含 Puffing Billy 与 Sassafras。</x:v>
+        <x:v>7/30 使用；11:15 于 343 Russell Street 集合，11:30–17:00 随团体验 Puffing Billy 与 Sassafras。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="23" customFormat="1" ht="26.399999618530273" customHeight="1">
@@ -8674,7 +8674,7 @@
         </x:is>
       </x:c>
       <x:c r="H2" s="28" t="str">
-        <x:v>适合 D1 延误抵达后入住并前往 QVM；D2 上午 CBD city walk、11:30–17:00 Puffing Billy 半日团，返城后去 Fitzroy；D3 退房后前往机场取车。</x:v>
+        <x:v>位于 CBD，入住后前往 QVM 方便；次日清晨可步行串联 Degraves Street、Flinders Street、Hosier Lane 与州立图书馆，返城后去 Fitzroy 也顺路。大洋路出发当天再打车前往机场取车。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9024,30 +9024,20 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">天气触发</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Melbourne Skydeck</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D2 傍晚可选</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">看天气决定，不提前买不可退票。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">晴天、能见度高、体力够再去。</x:t>
-        </x:is>
+      <x:c r="A4" s="28" t="str">
+        <x:v>已订</x:v>
+      </x:c>
+      <x:c r="B4" s="28" t="str">
+        <x:v>Puffing Billy + Sassafras 半日团</x:v>
+      </x:c>
+      <x:c r="C4" s="28" t="str">
+        <x:v>D2｜7/30</x:v>
+      </x:c>
+      <x:c r="D4" s="28" t="str">
+        <x:v>11:15 在 343 Russell Street 集合。</x:v>
+      </x:c>
+      <x:c r="E4" s="28" t="str">
+        <x:v>11:30–17:00 随团前往 Belgrave，乘坐 Puffing Billy，并游览 Lakeside 与 Sassafras；山里较凉，随身带防风外套。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -9175,16 +9165,16 @@
         <x:v>D1 墨尔本</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>航班 / 机场按实际情况</x:v>
+        <x:v>随航班安排</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>航班 / 机场按实际情况</x:v>
+        <x:v>随航班安排</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>QVM Winter Night Market 街头热食</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>15:15 抵达；酒店入住后只去 QVM，夜市用餐后回酒店休息。</x:v>
+        <x:v>15:15 抵达墨尔本；入住稍作休整，晚上去 QVM 逛夜市、吃晚餐。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9201,7 +9191,7 @@
         <x:v>Fitzroy 晚餐</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>08:45 开始 city walk；11:15 到 343 Russell Street；11:30–17:00 参加半日团；Fitzroy 后 21:00 前回酒店。</x:v>
+        <x:v>上午城市漫步；11:15 到 343 Russell Street 集合，11:30–17:00 随团前往 Puffing Billy 与 Sassafras，返城后去 Fitzroy。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
update D3 Great Ocean Road route
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R73ad8c33bf994673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R787c33d346004b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R41862d9a24f74128"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R8ea84605e4724396"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R50e470a307ca4b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R633f3e2f87804860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rdc447f2d6bdf488a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R540d7fb6de794640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Rd1d00d772725456f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Rc152a1542a9c4987"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R5600eec9f2f544b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Re18bc379b6f44bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rd7eb818db6b4401a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Rc3a77d811bcc4603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rb1ae6760a3884181"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R3bb2c7dfd0b1467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R051c54a6442e4bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R09ab85c4bb2f4f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Redf070c216b647fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Rc95da86ce33a4e15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -854,7 +854,7 @@
         <x:v>周五</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>墨尔本机场 → Apollo Bay</x:v>
+        <x:v>墨尔本 CBD → 墨尔本机场 → Apollo Bay</x:v>
       </x:c>
       <x:c r="F5" t="n">
         <x:v>-38.7599</x:v>
@@ -863,10 +863,10 @@
         <x:v>143.6692</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>驶上大洋路：Torquay、Lorne 到 Apollo Bay</x:v>
+        <x:v>驶上大洋路：从 Torquay 海岸到 Apollo Bay</x:v>
       </x:c>
       <x:c r="I5" t="str">
-        <x:v>机场取车后沿海向西，途经 Torquay、Lorne，傍晚住进 Apollo Bay。</x:v>
+        <x:v>把大箱寄存在机场，取车后到 Torquay 买好今晚的 BBQ 食材，再沿海经过 Bells Beach、Lorne 与 Kennett River，傍晚抵达 Apollo Bay。</x:v>
       </x:c>
       <x:c r="J5" t="str">
         <x:v>Seaview Motel &amp; Apartments</x:v>
@@ -884,10 +884,10 @@
         <x:v>大洋路早段海岸公路与灯塔</x:v>
       </x:c>
       <x:c r="O5" t="str">
-        <x:v>自驾 · 墨尔本机场取车</x:v>
+        <x:v>Uber / Taxi 到机场 · 取车后自驾</x:v>
       </x:c>
       <x:c r="P5" t="str">
-        <x:v>08:00 前退房出发，预留机场取车时间</x:v>
+        <x:v>08:00 从 Oaks 退房出发；09:30 从机场启程驶向 Torquay</x:v>
       </x:c>
       <x:c r="Q5" t="str">
         <x:v>seaview-motel-map</x:v>
@@ -2428,7 +2428,7 @@
         <x:v>把冬装和摄影设备装进登机箱</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>四个大箱留在酒店，只带登机箱和随身包上路；早点休息。</x:v>
+        <x:v>把四个大箱与大洋路小箱分开整理，第二天一起带到机场；寄存后只带小箱上路。</x:v>
       </x:c>
       <x:c r="H22" t="str">
         <x:v>fitzroy-map,oaks-market-map</x:v>
@@ -2468,22 +2468,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C24" t="str">
-        <x:v>上午</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D24" t="str">
-        <x:v>墨尔本 CBD → 墨尔本机场</x:v>
+        <x:v>Oaks Melbourne on Market Hotel</x:v>
       </x:c>
       <x:c r="E24" t="str">
-        <x:v>前往机场取车，确认车辆、保险、第二驾驶人、导航和行李安排</x:v>
+        <x:v>退房，把四个大箱与大洋路小箱分开，只带小箱上路</x:v>
       </x:c>
       <x:c r="F24" t="str">
-        <x:v>从机场取车，正式驶上大洋路</x:v>
+        <x:v>轻装开启大洋路</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>从机场取车能避开 CBD 复杂路况；出发前先设置导航和语音提示，让右舵适应更从容。</x:v>
+        <x:v>出门前确认护照、驾照、租车订单与随身设备都已带齐。</x:v>
       </x:c>
       <x:c r="H24" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>oaks-market-map</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2494,22 +2494,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>上午</x:v>
+        <x:v>08:40 左右</x:v>
       </x:c>
       <x:c r="D25" t="str">
-        <x:v>墨尔本机场 → Torquay</x:v>
+        <x:v>Holiday Inn Melbourne Airport</x:v>
       </x:c>
       <x:c r="E25" t="str">
-        <x:v>从机场出发，经 Geelong Bypass 前往 Torquay</x:v>
+        <x:v>把 4 个大箱交给前台寄存，确认领取安排后整理随身物品</x:v>
       </x:c>
       <x:c r="F25" t="str">
-        <x:v>右舵适应第一段</x:v>
+        <x:v>大件行李留在机场酒店</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>经过 Geelong 外围即可，刚开始适应右舵时把安全放在第一位。</x:v>
+        <x:v>把寄存标签和领取凭证拍照留存，再带着大洋路小箱前往租车门店。</x:v>
       </x:c>
       <x:c r="H25" t="str">
-        <x:v>mel-airport-map,torquay-map</x:v>
+        <x:v>holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2520,22 +2520,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>上午</x:v>
+        <x:v>08:40–09:30</x:v>
       </x:c>
       <x:c r="D26" t="str">
-        <x:v>Torquay</x:v>
+        <x:v>Melbourne Airport Car Rental Branch</x:v>
       </x:c>
       <x:c r="E26" t="str">
-        <x:v>咖啡 / 短暂停留 / 进入海岸线节奏</x:v>
+        <x:v>办理取车，检查车身划痕、轮毂、挡风玻璃与油量</x:v>
       </x:c>
       <x:c r="F26" t="str">
-        <x:v>大洋路氛围开始</x:v>
+        <x:v>设好 Google Maps，熟悉右舵车位</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>把 Torquay 作为第一处完整休息点，喝杯咖啡再进入海岸线。</x:v>
+        <x:v>启程前拍一圈车辆视频，调整座椅、后视镜和导航语音，再确认第二驾驶人。</x:v>
       </x:c>
       <x:c r="H26" t="str">
-        <x:v>torquay-map</x:v>
+        <x:v>mel-airport-car-rental-map,mel-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2546,22 +2546,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>上午</x:v>
+        <x:v>09:30–10:45</x:v>
       </x:c>
       <x:c r="D27" t="str">
-        <x:v>Bells Beach</x:v>
+        <x:v>墨尔本机场 → Torquay</x:v>
       </x:c>
       <x:c r="E27" t="str">
-        <x:v>冲浪海岸停靠</x:v>
+        <x:v>经 M80、M1 与 Geelong Bypass 驶向 Torquay</x:v>
       </x:c>
       <x:c r="F27" t="str">
-        <x:v>经典冲浪海滩 + 悬崖海浪</x:v>
+        <x:v>第一段以高速路为主，慢慢适应右舵</x:v>
       </x:c>
       <x:c r="G27" t="str">
-        <x:v>风大，10分钟左右即可</x:v>
+        <x:v>导航先设为 Coles Torquay；经过 Geelong 外围即可，不进市区。</x:v>
       </x:c>
       <x:c r="H27" t="str">
-        <x:v>bells-map</x:v>
+        <x:v>mel-airport-map,coles-torquay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2572,22 +2572,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>上午</x:v>
+        <x:v>10:45–11:15</x:v>
       </x:c>
       <x:c r="D28" t="str">
-        <x:v>Split Point Lighthouse</x:v>
+        <x:v>Coles Torquay</x:v>
       </x:c>
       <x:c r="E28" t="str">
-        <x:v>Aireys Inlet 灯塔</x:v>
+        <x:v>采购 Apollo Bay BBQ 晚餐食材与车上饮水</x:v>
       </x:c>
       <x:c r="F28" t="str">
-        <x:v>白色灯塔 + 海岸线开阔视野</x:v>
+        <x:v>牛排、香肠或鸡腿，搭配玉米、蘑菇、彩椒与洋葱</x:v>
       </x:c>
       <x:c r="G28" t="str">
-        <x:v>建议停，是大洋路第一个清晰记忆点</x:v>
+        <x:v>再拿 Garlic Bread、Salad Kit、面包、酱料、啤酒或葡萄酒与饮用水；冷藏食材集中装好。</x:v>
       </x:c>
       <x:c r="H28" t="str">
-        <x:v>split-point-map</x:v>
+        <x:v>coles-torquay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2598,22 +2598,22 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>11:20–11:45</x:v>
       </x:c>
       <x:c r="D29" t="str">
-        <x:v>Memorial Arch</x:v>
+        <x:v>Bells Beach</x:v>
       </x:c>
       <x:c r="E29" t="str">
-        <x:v>大洋路纪念拱门</x:v>
+        <x:v>从观景台看冲浪海岸与悬崖海浪</x:v>
       </x:c>
       <x:c r="F29" t="str">
-        <x:v>Great Ocean Road 标志入口</x:v>
+        <x:v>大洋路的第一段开阔海景</x:v>
       </x:c>
       <x:c r="G29" t="str">
-        <x:v>5–10分钟拍照即可</x:v>
+        <x:v>沿正式停车位步行到 Bells Beach Lookout，风大时在高处拍完就继续上路。</x:v>
       </x:c>
       <x:c r="H29" t="str">
-        <x:v>memorial-arch-map</x:v>
+        <x:v>bells-map</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2624,22 +2624,22 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>中午前后</x:v>
+        <x:v>12:00–12:30</x:v>
       </x:c>
       <x:c r="D30" t="str">
-        <x:v>Teddy's Lookout</x:v>
+        <x:v>Split Point Lighthouse</x:v>
       </x:c>
       <x:c r="E30" t="str">
-        <x:v>S型海岸 + 河口入海</x:v>
+        <x:v>步行看白色灯塔与 Eagle Rock Lookout</x:v>
       </x:c>
       <x:c r="F30" t="str">
-        <x:v>全路段最经典构图点之一</x:v>
+        <x:v>灯塔、礁石与 Aireys Inlet 海岸线</x:v>
       </x:c>
       <x:c r="G30" t="str">
-        <x:v>必停，但不需要久留</x:v>
+        <x:v>留约 30 分钟，沿步道走到观景点再原路返回。</x:v>
       </x:c>
       <x:c r="H30" t="str">
-        <x:v>teddys-map</x:v>
+        <x:v>split-point-map</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2650,22 +2650,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>中午</x:v>
+        <x:v>12:40–12:50</x:v>
       </x:c>
       <x:c r="D31" t="str">
-        <x:v>Lorne</x:v>
+        <x:v>Great Ocean Road Memorial Arch</x:v>
       </x:c>
       <x:c r="E31" t="str">
-        <x:v>午餐 + 补给</x:v>
+        <x:v>在纪念拱门前合影，正式进入大洋路</x:v>
       </x:c>
       <x:c r="F31" t="str">
-        <x:v>最舒服海滨小镇之一</x:v>
+        <x:v>Great Ocean Road 标志性入口</x:v>
       </x:c>
       <x:c r="G31" t="str">
-        <x:v>在 Lorne 慢慢吃午餐、补给并休息，不必赶时间。</x:v>
+        <x:v>停留约 10 分钟，拍完继续前往 Lorne 吃午餐。</x:v>
       </x:c>
       <x:c r="H31" t="str">
-        <x:v>lorne-map</x:v>
+        <x:v>memorial-arch-map</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2676,22 +2676,22 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>下午</x:v>
+        <x:v>13:00–14:00</x:v>
       </x:c>
       <x:c r="D32" t="str">
-        <x:v>Kennett River</x:v>
+        <x:v>Lorne</x:v>
       </x:c>
       <x:c r="E32" t="str">
-        <x:v>找考拉</x:v>
+        <x:v>在海边小镇吃午餐，沿海边走一走，再喝杯咖啡</x:v>
       </x:c>
       <x:c r="F32" t="str">
-        <x:v>桉树 + 野生考拉体验</x:v>
+        <x:v>在驾驶中段坐下来休息</x:v>
       </x:c>
       <x:c r="G32" t="str">
-        <x:v>抬头看树，不保证但高概率；不要为拍照打扰动物</x:v>
+        <x:v>留 45–60 分钟，吃饱但不过量，下午还有多段海岸弯道。</x:v>
       </x:c>
       <x:c r="H32" t="str">
-        <x:v>kennett-map</x:v>
+        <x:v>lorne-map,snow-monkey-ramen-map</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2702,22 +2702,22 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>下午</x:v>
+        <x:v>14:15–14:35</x:v>
       </x:c>
       <x:c r="D33" t="str">
-        <x:v>Cape Patton Lookout</x:v>
+        <x:v>Teddy's Lookout</x:v>
       </x:c>
       <x:c r="E33" t="str">
-        <x:v>海岸远景观景</x:v>
+        <x:v>从高处看 Saint George River 入海与 S 形海岸公路</x:v>
       </x:c>
       <x:c r="F33" t="str">
-        <x:v>高位俯瞰 Apollo Bay 海岸线</x:v>
+        <x:v>Lorne 一带最经典的纵深视角</x:v>
       </x:c>
       <x:c r="G33" t="str">
-        <x:v>顺路短停即可</x:v>
+        <x:v>停车后步行到观景台，留 15–20 分钟。</x:v>
       </x:c>
       <x:c r="H33" t="str">
-        <x:v>cape-patton-map,apollo-map</x:v>
+        <x:v>teddys-map</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2728,22 +2728,22 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>15:30–16:00</x:v>
       </x:c>
       <x:c r="D34" t="str">
-        <x:v>Marriners Lookout（可选）</x:v>
+        <x:v>Kennett River / Grey River Road</x:v>
       </x:c>
       <x:c r="E34" t="str">
-        <x:v>Apollo Bay 俯瞰</x:v>
+        <x:v>沿 Grey River Road 慢慢找树冠里的野生考拉</x:v>
       </x:c>
       <x:c r="F34" t="str">
-        <x:v>半月海湾 + 小镇全景</x:v>
+        <x:v>桉树林里的野生动物时刻</x:v>
       </x:c>
       <x:c r="G34" t="str">
-        <x:v>天气好、不累、时间够才去</x:v>
+        <x:v>抬头观察树冠，也留意路边鸟类；保持距离，不喂食、不追逐。</x:v>
       </x:c>
       <x:c r="H34" t="str">
-        <x:v>marriners-map,apollo-map</x:v>
+        <x:v>grey-river-road-map,kennett-map</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2754,22 +2754,22 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>16:15–16:25</x:v>
       </x:c>
       <x:c r="D35" t="str">
-        <x:v>Apollo Bay</x:v>
+        <x:v>Cape Patton Lookout</x:v>
       </x:c>
       <x:c r="E35" t="str">
-        <x:v>入住</x:v>
+        <x:v>从高处回望弯曲海岸，望向 Apollo Bay 方向</x:v>
       </x:c>
       <x:c r="F35" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>抵达小镇前的最后一段海岸全景</x:v>
       </x:c>
       <x:c r="G35" t="str">
-        <x:v>日落前抵达最佳</x:v>
+        <x:v>停留 5–10 分钟，随后继续前往住宿。</x:v>
       </x:c>
       <x:c r="H35" t="str">
-        <x:v>apollo-map</x:v>
+        <x:v>cape-patton-map,apollo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2780,22 +2780,22 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>晚上</x:v>
+        <x:v>17:00</x:v>
       </x:c>
       <x:c r="D36" t="str">
-        <x:v>Apollo Bay</x:v>
+        <x:v>Seaview Motel &amp; Apartments</x:v>
       </x:c>
       <x:c r="E36" t="str">
-        <x:v>Fishermen's Co-op / seafood café 晚餐</x:v>
+        <x:v>办理入住，把冷藏食材放好，稍作休息</x:v>
       </x:c>
       <x:c r="F36" t="str">
-        <x:v>海边渔港氛围</x:v>
+        <x:v>日落前住进 Apollo Bay</x:v>
       </x:c>
       <x:c r="G36" t="str">
-        <x:v>到 Apollo Bay 后吃 fish &amp; chips 或海鲜，早点休息。</x:v>
+        <x:v>先确认 BBQ 设施位置与使用方式，再整理晚餐食材。</x:v>
       </x:c>
       <x:c r="H36" t="str">
-        <x:v>apollo-map,fishermens-coop-map</x:v>
+        <x:v>seaview-motel-map,apollo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2803,51 +2803,51 @@
         <x:v>d3</x:v>
       </x:c>
       <x:c r="B37" t="n">
-        <x:v>900</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D37" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Seaview Motel &amp; Apartments</x:v>
       </x:c>
       <x:c r="E37" t="str">
-        <x:v>早餐：出发咖啡；午餐：Lorne café / Snow Monkey Ramen（备选）；晚餐：Apollo Bay Fishermen's Co-op / seafood café</x:v>
+        <x:v>用上午采购的食材准备 BBQ 晚餐</x:v>
       </x:c>
       <x:c r="F37" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>牛排、香肠与蔬菜，为第一天海岸自驾收尾</x:v>
       </x:c>
       <x:c r="G37" t="str">
-        <x:v>海岸驾驶日以轻松好吃为主，Apollo Bay 的 fish &amp; chips / 海鲜正合适。</x:v>
+        <x:v>吃完把次日随身物品整理好，早点休息。</x:v>
       </x:c>
       <x:c r="H37" t="str">
-        <x:v>lorne-map,snow-monkey-ramen-map,apollo-map,fishermens-coop-map</x:v>
+        <x:v>seaview-motel-map,coles-torquay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
-        <x:v>d4</x:v>
+        <x:v>d3</x:v>
       </x:c>
       <x:c r="B38" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>备选 · 清晨</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D38" t="str">
-        <x:v>Maits Rest Rainforest Walk</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E38" t="str">
-        <x:v>若 07:45 前离开 Apollo Bay 且时间充裕，可先走一段雨林环线。</x:v>
+        <x:v>早餐：出发咖啡；午餐：Lorne café / Snow Monkey Ramen；晚餐：Seaview Motel BBQ</x:v>
       </x:c>
       <x:c r="F38" t="str">
-        <x:v>冬日湿润雨林，非常有氛围</x:v>
+        <x:v>从海边午餐到住处 BBQ</x:v>
       </x:c>
       <x:c r="G38" t="str">
-        <x:v>只有早出发且时间充裕时再停，约 30 分钟。</x:v>
+        <x:v>上午在 Torquay 买好晚餐食材，Lorne 坐下来吃午餐，抵达 Apollo Bay 后在住处准备晚餐。</x:v>
       </x:c>
       <x:c r="H38" t="str">
-        <x:v>maits-rest-map</x:v>
+        <x:v>lorne-map,snow-monkey-ramen-map,seaview-motel-map,coles-torquay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2855,25 +2855,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B39" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>上午</x:v>
+        <x:v>备选 · 清晨</x:v>
       </x:c>
       <x:c r="D39" t="str">
-        <x:v>The Redwoods Otways</x:v>
+        <x:v>Maits Rest Rainforest Walk</x:v>
       </x:c>
       <x:c r="E39" t="str">
-        <x:v>从北侧 Binns Road 进入红杉林，沿 Aire River 林间步道慢走约 30–45 分钟。</x:v>
+        <x:v>若 07:45 前离开 Apollo Bay 且时间充裕，可先走一段雨林环线。</x:v>
       </x:c>
       <x:c r="F39" t="str">
-        <x:v>高大的加州红杉、林下光影与安静的河谷氛围</x:v>
+        <x:v>冬日湿润雨林，非常有氛围</x:v>
       </x:c>
       <x:c r="G39" t="str">
-        <x:v>林区无手机信号，地面可能湿滑；出发前查看 Parks Victoria 路况与现场标识。</x:v>
+        <x:v>只有早出发且时间充裕时再停，约 30 分钟。</x:v>
       </x:c>
       <x:c r="H39" t="str">
-        <x:v>redwoods-otways-map,redwoods-otways-official</x:v>
+        <x:v>maits-rest-map</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2881,25 +2881,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B40" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>中午前后</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D40" t="str">
-        <x:v>Gibson Steps</x:v>
+        <x:v>The Redwoods Otways</x:v>
       </x:c>
       <x:c r="E40" t="str">
-        <x:v>下到海滩看悬崖与海蚀柱</x:v>
+        <x:v>从北侧 Binns Road 进入红杉林，沿 Aire River 林间步道慢走约 30–45 分钟。</x:v>
       </x:c>
       <x:c r="F40" t="str">
-        <x:v>人物比例感很强，比单纯观景台更有沉浸感</x:v>
+        <x:v>高大的加州红杉、林下光影与安静的河谷氛围</x:v>
       </x:c>
       <x:c r="G40" t="str">
-        <x:v>看开放情况和风浪；风大时不要太靠近海浪</x:v>
+        <x:v>林区无手机信号，地面可能湿滑；出发前查看 Parks Victoria 路况与现场标识。</x:v>
       </x:c>
       <x:c r="H40" t="str">
-        <x:v>gibson-steps-map</x:v>
+        <x:v>redwoods-otways-map,redwoods-otways-official</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2907,25 +2907,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B41" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午前后</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Twelve Apostles</x:v>
+        <x:v>Gibson Steps</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>十二使徒岩主观景台</x:v>
+        <x:v>下到海滩看悬崖与海蚀柱</x:v>
       </x:c>
       <x:c r="F41" t="str">
-        <x:v>大洋路最具代表性的海岸地貌</x:v>
+        <x:v>人物比例感很强，比单纯观景台更有沉浸感</x:v>
       </x:c>
       <x:c r="G41" t="str">
-        <x:v>左侧平台更适合拍海岸线纵深；如果人多，不要停太久</x:v>
+        <x:v>看开放情况和风浪；风大时不要太靠近海浪</x:v>
       </x:c>
       <x:c r="H41" t="str">
-        <x:v>twelve-apostles-map</x:v>
+        <x:v>gibson-steps-map</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2933,25 +2933,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B42" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C42" t="str">
         <x:v>下午</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Loch Ard Gorge</x:v>
+        <x:v>Twelve Apostles</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>在主观景区看峡湾与沉船故事，再接 Geology Walk。</x:v>
+        <x:v>十二使徒岩主观景台</x:v>
       </x:c>
       <x:c r="F42" t="str">
-        <x:v>峡湾地貌、沉船历史与悬崖顶观景</x:v>
+        <x:v>大洋路最具代表性的海岸地貌</x:v>
       </x:c>
       <x:c r="G42" t="str">
-        <x:v>至少预留 1 小时；海滩下行台阶关闭，按现场标识走崖顶步道。</x:v>
+        <x:v>左侧平台更适合拍海岸线纵深；如果人多，不要停太久</x:v>
       </x:c>
       <x:c r="H42" t="str">
-        <x:v>loch-ard-map</x:v>
+        <x:v>twelve-apostles-map</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2959,25 +2959,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B43" t="n">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C43" t="str">
         <x:v>下午</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Tom and Eva</x:v>
+        <x:v>Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>Loch Ard Gorge 附近短停</x:v>
+        <x:v>在主观景区看峡湾与沉船故事，再接 Geology Walk。</x:v>
       </x:c>
       <x:c r="F43" t="str">
-        <x:v>两个海蚀柱，和沉船故事相关</x:v>
+        <x:v>峡湾地貌、沉船历史与悬崖顶观景</x:v>
       </x:c>
       <x:c r="G43" t="str">
-        <x:v>作为 Loch Ard Gorge 区域顺路点，不需要额外绕路</x:v>
+        <x:v>至少预留 1 小时；海滩下行台阶关闭，按现场标识走崖顶步道。</x:v>
       </x:c>
       <x:c r="H43" t="str">
-        <x:v>tom-eva-map,loch-ard-map</x:v>
+        <x:v>loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2985,25 +2985,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B44" t="n">
-        <x:v>60</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>The Razorback</x:v>
+        <x:v>Tom and Eva</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>从 Loch Ard Gorge 主停车场走 900 米往返 Geology Walk，经 Island Arch 到 The Razorback 观景台。</x:v>
+        <x:v>Loch Ard Gorge 附近短停</x:v>
       </x:c>
       <x:c r="F44" t="str">
-        <x:v>同一景区内的狭长海蚀岩脊与悬崖顶视角</x:v>
+        <x:v>两个海蚀柱，和沉船故事相关</x:v>
       </x:c>
       <x:c r="G44" t="str">
-        <x:v>步行往返约 30–40 分钟；不需要另开一段车程。</x:v>
+        <x:v>作为 Loch Ard Gorge 区域顺路点，不需要额外绕路</x:v>
       </x:c>
       <x:c r="H44" t="str">
-        <x:v>razorback-map</x:v>
+        <x:v>tom-eva-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3011,25 +3011,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B45" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>The Razorback</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>抵达入住 Southern Ocean Villas</x:v>
+        <x:v>从 Loch Ard Gorge 主停车场走 900 米往返 Geology Walk，经 Island Arch 到 The Razorback 观景台。</x:v>
       </x:c>
       <x:c r="F45" t="str">
-        <x:v>方便第二天清晨补拍</x:v>
+        <x:v>同一景区内的狭长海蚀岩脊与悬崖顶视角</x:v>
       </x:c>
       <x:c r="G45" t="str">
-        <x:v>不要天黑后还在海岸小路上赶</x:v>
+        <x:v>步行往返约 30–40 分钟；不需要另开一段车程。</x:v>
       </x:c>
       <x:c r="H45" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>razorback-map</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -3037,22 +3037,22 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B46" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D46" t="str">
         <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>抵达后按天气选择公共电烤炉 BBQ、villa 厨房自炊或附近餐厅</x:v>
+        <x:v>抵达入住 Southern Ocean Villas</x:v>
       </x:c>
       <x:c r="F46" t="str">
-        <x:v>灵活完成 BBQ-style dinner</x:v>
+        <x:v>方便第二天清晨补拍</x:v>
       </x:c>
       <x:c r="G46" t="str">
-        <x:v>Southern Ocean Villas 没有自带 BBQ，但附近有两处免费 electric BBQ；villa 厨房备有油、盐、胡椒和锡纸。</x:v>
+        <x:v>不要天黑后还在海岸小路上赶</x:v>
       </x:c>
       <x:c r="H46" t="str">
         <x:v>port-campbell-map</x:v>
@@ -3063,51 +3063,51 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B47" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：在 Apollo Bay 买好食材，抵达后按天气选择公共 electric BBQ 或 villa 厨房自炊</x:v>
+        <x:v>抵达后按天气选择公共电烤炉 BBQ、villa 厨房自炊或附近餐厅</x:v>
       </x:c>
       <x:c r="F47" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>灵活完成 BBQ-style dinner</x:v>
       </x:c>
       <x:c r="G47" t="str">
-        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
+        <x:v>Southern Ocean Villas 没有自带 BBQ，但附近有两处免费 electric BBQ；villa 厨房备有油、盐、胡椒和锡纸。</x:v>
       </x:c>
       <x:c r="H47" t="str">
-        <x:v>apollo-map,port-campbell-map</x:v>
+        <x:v>port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="str">
-        <x:v>d5</x:v>
+        <x:v>d4</x:v>
       </x:c>
       <x:c r="B48" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>07:00-07:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>退房、装车并简单早餐</x:v>
+        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：在 Apollo Bay 买好食材，抵达后按天气选择公共 electric BBQ 或 villa 厨房自炊</x:v>
       </x:c>
       <x:c r="F48" t="str">
-        <x:v>小镇清晨 + 返程准备</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G48" t="str">
-        <x:v>把行李装车、早餐和退房一次完成；07:30 左右驶离住宿。</x:v>
+        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
       </x:c>
       <x:c r="H48" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>apollo-map,port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -3115,25 +3115,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B49" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>天气补拍备选 · 07:30-08:10</x:v>
+        <x:v>07:00-07:30</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
+        <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>若前一日受天气影响，在两处中只选一处清晨补拍；若已看够则直接前往 The Grotto</x:v>
+        <x:v>退房、装车并简单早餐</x:v>
       </x:c>
       <x:c r="F49" t="str">
-        <x:v>柔和晨光 + 较少游客</x:v>
+        <x:v>小镇清晨 + 返程准备</x:v>
       </x:c>
       <x:c r="G49" t="str">
-        <x:v>只选一处，08:10 最晚离开；这段是天气补拍，不影响 10:00 后进入 Wildlife Park。</x:v>
+        <x:v>把行李装车、早餐和退房一次完成；07:30 左右驶离住宿。</x:v>
       </x:c>
       <x:c r="H49" t="str">
-        <x:v>twelve-apostles-map,loch-ard-map</x:v>
+        <x:v>port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -3141,25 +3141,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B50" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>08:35 左右</x:v>
+        <x:v>天气补拍备选 · 07:30-08:10</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>The Grotto</x:v>
+        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>看海蚀洞和海水窗口</x:v>
+        <x:v>若前一日受天气影响，在两处中只选一处清晨补拍；若已看够则直接前往 The Grotto</x:v>
       </x:c>
       <x:c r="F50" t="str">
-        <x:v>洞穴 + 海景构图</x:v>
+        <x:v>柔和晨光 + 较少游客</x:v>
       </x:c>
       <x:c r="G50" t="str">
-        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
+        <x:v>只选一处，08:10 最晚离开；这段是天气补拍，不影响 10:00 后进入 Wildlife Park。</x:v>
       </x:c>
       <x:c r="H50" t="str">
-        <x:v>grotto-map</x:v>
+        <x:v>twelve-apostles-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -3167,25 +3167,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B51" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>09:10 左右</x:v>
+        <x:v>08:35 左右</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>London Bridge / London Arch</x:v>
+        <x:v>The Grotto</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>看海蚀拱门</x:v>
+        <x:v>看海蚀洞和海水窗口</x:v>
       </x:c>
       <x:c r="F51" t="str">
-        <x:v>Port Campbell 以西经典点</x:v>
+        <x:v>洞穴 + 海景构图</x:v>
       </x:c>
       <x:c r="G51" t="str">
-        <x:v>顺路短停，很适合加</x:v>
+        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
       </x:c>
       <x:c r="H51" t="str">
-        <x:v>london-arch-map,port-campbell-map</x:v>
+        <x:v>grotto-map</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -3193,25 +3193,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B52" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>10:15-11:30</x:v>
+        <x:v>09:10 左右</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Great Ocean Road Wildlife Park</x:v>
+        <x:v>London Bridge / London Arch</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>购买普通门票进入互动区和 sanctuary，近距离看袋鼠、沙袋鼠等澳洲本土动物；游园和可选购饲料喂食合计预留 60-75 分钟</x:v>
+        <x:v>看海蚀拱门</x:v>
       </x:c>
       <x:c r="F52" t="str">
-        <x:v>大洋路沿线的澳洲本土动物互动体验</x:v>
+        <x:v>Port Campbell 以西经典点</x:v>
       </x:c>
       <x:c r="G52" t="str">
-        <x:v>普通门票建议提前在线购买；动物饲料和 close-up encounters 另付费。步道多为未铺装地面，穿防滑包脚鞋；11:45 前离园，为 Colac 午餐、加油和机场还车保留缓冲。</x:v>
+        <x:v>顺路短停，很适合加</x:v>
       </x:c>
       <x:c r="H52" t="str">
-        <x:v>great-ocean-road-wildlife-park-map,great-ocean-road-wildlife-park-official,great-ocean-road-wildlife-park-booking</x:v>
+        <x:v>london-arch-map,port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -3219,25 +3219,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B53" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>下午</x:v>
+        <x:v>10:15-11:30</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Colac</x:v>
+        <x:v>Great Ocean Road Wildlife Park</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>午餐、加油、休息</x:v>
+        <x:v>购买普通门票进入互动区和 sanctuary，近距离看袋鼠、沙袋鼠等澳洲本土动物；游园和可选购饲料喂食合计预留 60-75 分钟</x:v>
       </x:c>
       <x:c r="F53" t="str">
-        <x:v>内陆牧场风光</x:v>
+        <x:v>大洋路沿线的澳洲本土动物互动体验</x:v>
       </x:c>
       <x:c r="G53" t="str">
-        <x:v>回程中段休息点</x:v>
+        <x:v>普通门票建议提前在线购买；动物饲料和 close-up encounters 另付费。步道多为未铺装地面，穿防滑包脚鞋；11:45 前离园，为 Colac 午餐、加油和机场还车保留缓冲。</x:v>
       </x:c>
       <x:c r="H53" t="str">
-        <x:v>colac-map</x:v>
+        <x:v>great-ocean-road-wildlife-park-map,great-ocean-road-wildlife-park-official,great-ocean-road-wildlife-park-booking</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3245,25 +3245,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B54" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>Colac</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
+        <x:v>午餐、加油、休息</x:v>
       </x:c>
       <x:c r="F54" t="str">
-        <x:v>大洋路自驾收尾</x:v>
+        <x:v>内陆牧场风光</x:v>
       </x:c>
       <x:c r="G54" t="str">
-        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
+        <x:v>回程中段休息点</x:v>
       </x:c>
       <x:c r="H54" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>colac-map</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3271,25 +3271,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B55" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Holiday Inn Melbourne Airport</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>入住、整理行李</x:v>
+        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
       </x:c>
       <x:c r="F55" t="str">
-        <x:v>为次日早班机准备</x:v>
+        <x:v>大洋路自驾收尾</x:v>
       </x:c>
       <x:c r="G55" t="str">
-        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
+        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
       </x:c>
       <x:c r="H55" t="str">
-        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
+        <x:v>mel-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3297,51 +3297,51 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B56" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Holiday Inn Melbourne Airport</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>早餐：Port Campbell café；午餐：离开 Great Ocean Road Wildlife Park 后在 Colac 简餐；晚餐：机场酒店简餐</x:v>
+        <x:v>入住、整理行李</x:v>
       </x:c>
       <x:c r="F56" t="str">
-        <x:v>野生动物体验 + 内陆返程补给</x:v>
+        <x:v>为次日早班机准备</x:v>
       </x:c>
       <x:c r="G56" t="str">
-        <x:v>Colac 作为返程主休息点，把午餐、加油和休息一次完成；抵达机场后简单用餐并整理行李。</x:v>
+        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
       </x:c>
       <x:c r="H56" t="str">
-        <x:v>great-ocean-road-wildlife-park-map,colac-map,holiday-inn-airport-map</x:v>
+        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B57" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>飞往凯恩斯</x:v>
+        <x:v>早餐：Port Campbell café；午餐：离开 Great Ocean Road Wildlife Park 后在 Colac 简餐；晚餐：机场酒店简餐</x:v>
       </x:c>
       <x:c r="F57" t="str">
-        <x:v>气候切换非常明显</x:v>
+        <x:v>野生动物体验 + 内陆返程补给</x:v>
       </x:c>
       <x:c r="G57" t="str">
-        <x:v>国内航班建议预留行李额</x:v>
+        <x:v>Colac 作为返程主休息点，把午餐、加油和休息一次完成；抵达机场后简单用餐并整理行李。</x:v>
       </x:c>
       <x:c r="H57" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>great-ocean-road-wildlife-park-map,colac-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3349,75 +3349,75 @@
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B58" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>打车 / Uber 到酒店</x:v>
+        <x:v>飞往凯恩斯</x:v>
       </x:c>
       <x:c r="F58" t="str">
-        <x:v>不租车，降低疲劳</x:v>
+        <x:v>气候切换非常明显</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>酒店可先寄存行李</x:v>
-      </x:c>
-      <x:c r="H58"/>
+        <x:v>国内航班建议预留行李额</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" t="str">
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B59" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Esplanade Lagoon</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>免费泻湖泳池、海滨散步</x:v>
+        <x:v>打车 / Uber 到酒店</x:v>
       </x:c>
       <x:c r="F59" t="str">
-        <x:v>度假感拉满</x:v>
+        <x:v>不租车，降低疲劳</x:v>
       </x:c>
       <x:c r="G59" t="str">
-        <x:v>泳衣可提前放随身包</x:v>
-      </x:c>
-      <x:c r="H59" t="str">
-        <x:v>cairns-lagoon-map</x:v>
-      </x:c>
+        <x:v>酒店可先寄存行李</x:v>
+      </x:c>
+      <x:c r="H59"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="str">
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B60" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>晚上</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Cairns Night Markets</x:v>
+        <x:v>Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>夜市、简餐、纪念品</x:v>
+        <x:v>免费泻湖泳池、海滨散步</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>热闹轻松</x:v>
+        <x:v>度假感拉满</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+        <x:v>泳衣可提前放随身包</x:v>
       </x:c>
       <x:c r="H60" t="str">
-        <x:v>cairns-night-market-map</x:v>
+        <x:v>cairns-lagoon-map</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -3425,75 +3425,75 @@
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B61" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
+        <x:v>夜市、简餐、纪念品</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>热闹轻松</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
-      </x:c>
-      <x:c r="H61"/>
+        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>cairns-night-market-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B62" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>早上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>凯恩斯码头</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Reef Magic check-in，登船出海</x:v>
+        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F62" t="str">
-        <x:v>前往外礁平台</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G62" t="str">
-        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
-      </x:c>
-      <x:c r="H62" t="str">
-        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
-      </x:c>
+        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
+      </x:c>
+      <x:c r="H62"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" t="str">
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B63" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>全天</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Outer Reef Pontoon</x:v>
+        <x:v>凯恩斯码头</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
+        <x:v>Reef Magic check-in，登船出海</x:v>
       </x:c>
       <x:c r="F63" t="str">
-        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
+        <x:v>前往外礁平台</x:v>
       </x:c>
       <x:c r="G63" t="str">
-        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
+        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
       </x:c>
       <x:c r="H63" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3501,22 +3501,22 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B64" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>中午</x:v>
+        <x:v>全天</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>船上 / 平台</x:v>
+        <x:v>Outer Reef Pontoon</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>外礁平台午餐</x:v>
+        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
       </x:c>
       <x:c r="F64" t="str">
-        <x:v>轻松补给</x:v>
+        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
       </x:c>
       <x:c r="G64" t="str">
-        <x:v>不要吃太撑，避免晕船</x:v>
+        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
       </x:c>
       <x:c r="H64" t="str">
         <x:v>reef-magic-official</x:v>
@@ -3527,25 +3527,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B65" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>船上 / 平台</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>下船休息</x:v>
+        <x:v>外礁平台午餐</x:v>
       </x:c>
       <x:c r="F65" t="str">
-        <x:v>通常会比较疲惫</x:v>
+        <x:v>轻松补给</x:v>
       </x:c>
       <x:c r="G65" t="str">
-        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
+        <x:v>不要吃太撑，避免晕船</x:v>
       </x:c>
       <x:c r="H65" t="str">
-        <x:v>reef-fleet-terminal-map</x:v>
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3553,25 +3553,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B66" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>晚上</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>码头附近</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
+        <x:v>下船休息</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>海边晚餐</x:v>
+        <x:v>通常会比较疲惫</x:v>
       </x:c>
       <x:c r="G66" t="str">
-        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
+        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H66" t="str">
-        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
+        <x:v>reef-fleet-terminal-map</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3579,25 +3579,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B67" t="n">
-        <x:v>80</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>提醒</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>今日提醒</x:v>
+        <x:v>码头附近</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
+        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
       </x:c>
       <x:c r="F67" t="str">
-        <x:v>舒适与安全比拍摄数量更重要</x:v>
+        <x:v>海边晚餐</x:v>
       </x:c>
       <x:c r="G67" t="str">
-        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
       </x:c>
       <x:c r="H67" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3605,151 +3605,151 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B68" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>饮食</x:v>
+        <x:v>提醒</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>今日提醒</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
+        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
       </x:c>
       <x:c r="F68" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>舒适与安全比拍摄数量更重要</x:v>
       </x:c>
       <x:c r="G68" t="str">
-        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
       </x:c>
       <x:c r="H68" t="str">
-        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B69" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>清晨</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
+        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="F69" t="str">
-        <x:v>不用自驾，沿途可休息看风景</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G69" t="str">
-        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
-      </x:c>
-      <x:c r="H69"/>
+        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B70" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>上午</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Daintree River / Rainforest</x:v>
+        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>鳄鱼游船、雨林步道</x:v>
+        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
+        <x:v>不用自驾，沿途可休息看风景</x:v>
       </x:c>
       <x:c r="G70" t="str">
-        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
-      </x:c>
-      <x:c r="H70" t="str">
-        <x:v>daintree-river-map</x:v>
-      </x:c>
+        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
+      </x:c>
+      <x:c r="H70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B71" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Daintree Rainforest</x:v>
+        <x:v>Daintree River / Rainforest</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>团含午餐</x:v>
+        <x:v>鳄鱼游船、雨林步道</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>不用自己找餐厅</x:v>
+        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
       </x:c>
       <x:c r="G71" t="str">
-        <x:v>如有忌口提前告知</x:v>
-      </x:c>
-      <x:c r="H71"/>
+        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>daintree-river-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B72" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Cape Tribulation</x:v>
+        <x:v>Daintree Rainforest</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>雨林入海、海滩短停留</x:v>
+        <x:v>团含午餐</x:v>
       </x:c>
       <x:c r="F72" t="str">
-        <x:v>雨林与海洋在这里交会</x:v>
+        <x:v>不用自己找餐厅</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
-      </x:c>
-      <x:c r="H72" t="str">
-        <x:v>cape-trib-map</x:v>
-      </x:c>
+        <x:v>如有忌口提前告知</x:v>
+      </x:c>
+      <x:c r="H72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B73" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Daintree Ferry / Ice Cream</x:v>
+        <x:v>Cape Tribulation</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>渡河、热带水果冰淇淋</x:v>
+        <x:v>雨林入海、海滩短停留</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>丹翠地区很有代表性的热带味道</x:v>
+        <x:v>雨林与海洋在这里交会</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
+        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
       </x:c>
       <x:c r="H73" t="str">
-        <x:v>daintree-icecream-map</x:v>
+        <x:v>cape-trib-map</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3757,75 +3757,75 @@
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B74" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Daintree Ferry / Ice Cream</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>18:30 后回到市区</x:v>
+        <x:v>渡河、热带水果冰淇淋</x:v>
       </x:c>
       <x:c r="F74" t="str">
-        <x:v>回程可休息</x:v>
+        <x:v>丹翠地区很有代表性的热带味道</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
-      </x:c>
-      <x:c r="H74"/>
+        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>daintree-icecream-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B75" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>饮食</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>18:30 后回到市区</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>回程可休息</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
-      </x:c>
-      <x:c r="H75" t="str">
-        <x:v>daintree-icecream-map</x:v>
-      </x:c>
+        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
+      </x:c>
+      <x:c r="H75"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B76" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>早上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>凯恩斯 → Lake Eacham</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
+        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F76" t="str">
-        <x:v>从热带海边城市进入清凉高原</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
+        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
       </x:c>
       <x:c r="H76" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>daintree-icecream-map</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -3833,22 +3833,22 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B77" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>上午</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Lake Eacham</x:v>
+        <x:v>凯恩斯 → Lake Eacham</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>火山湖散步、看湖景</x:v>
+        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
       </x:c>
       <x:c r="F77" t="str">
-        <x:v>安静、清凉、湖水和雨林包围感</x:v>
+        <x:v>从热带海边城市进入清凉高原</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
       </x:c>
       <x:c r="H77" t="str">
         <x:v>lake-eacham-map</x:v>
@@ -3859,25 +3859,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B78" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Curtain Fig Tree</x:v>
+        <x:v>Lake Eacham</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>看巨型帘状无花果树</x:v>
+        <x:v>火山湖散步、看湖景</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>像热带森林里的巨大自然装置</x:v>
+        <x:v>安静、清凉、湖水和雨林包围感</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>停留 20–30 分钟即可</x:v>
+        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
       </x:c>
       <x:c r="H78" t="str">
-        <x:v>curtain-fig-map</x:v>
+        <x:v>lake-eacham-map</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -3885,25 +3885,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B79" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Yungaburra / Gallo Dairyland</x:v>
+        <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
+        <x:v>看巨型帘状无花果树</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
+        <x:v>像热带森林里的巨大自然装置</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
+        <x:v>停留 20–30 分钟即可</x:v>
       </x:c>
       <x:c r="H79" t="str">
-        <x:v>yungaburra-map,gallo-map</x:v>
+        <x:v>curtain-fig-map</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -3911,25 +3911,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B80" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
+        <x:v>Yungaburra / Gallo Dairyland</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>瀑布短停留、拍照</x:v>
+        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>雨林瀑布与高原绿意</x:v>
+        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
       </x:c>
       <x:c r="H80" t="str">
-        <x:v>millaa-map,ellinjaa-map</x:v>
+        <x:v>yungaburra-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -3937,46 +3937,48 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B81" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>下山回市区，还车或次日早还</x:v>
+        <x:v>瀑布短停留、拍照</x:v>
       </x:c>
       <x:c r="F81" t="str">
-        <x:v>完成高原自然线</x:v>
+        <x:v>雨林瀑布与高原绿意</x:v>
       </x:c>
       <x:c r="G81" t="str">
-        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
-      </x:c>
-      <x:c r="H81"/>
+        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>millaa-map,ellinjaa-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="str">
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B82" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>简单晚餐</x:v>
+        <x:v>下山回市区，还车或次日早还</x:v>
       </x:c>
       <x:c r="F82" t="str">
-        <x:v>回城后轻松晚餐</x:v>
+        <x:v>完成高原自然线</x:v>
       </x:c>
       <x:c r="G82" t="str">
-        <x:v>下山后就近用餐，早点休息。</x:v>
+        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
       </x:c>
       <x:c r="H82"/>
     </x:row>
@@ -3985,51 +3987,49 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B83" t="n">
-        <x:v>900</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>简单晚餐</x:v>
       </x:c>
       <x:c r="F83" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>回城后轻松晚餐</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
-      </x:c>
-      <x:c r="H83" t="str">
-        <x:v>millaa-map,gallo-map</x:v>
-      </x:c>
+        <x:v>下山后就近用餐，早点休息。</x:v>
+      </x:c>
+      <x:c r="H83"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B84" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F84" t="str">
-        <x:v>周五正好开市，适合补水果和轻食</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G84" t="str">
-        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
+        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H84" t="str">
-        <x:v>rustys-map</x:v>
+        <x:v>millaa-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -4037,25 +4037,25 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B85" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>热带城市躺平感</x:v>
+        <x:v>周五正好开市，适合补水果和轻食</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
+        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
       </x:c>
       <x:c r="H85" t="str">
-        <x:v>cairns-lagoon-map</x:v>
+        <x:v>rustys-map</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -4063,75 +4063,75 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B86" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>下午</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>为次日清晨航班做准备</x:v>
+        <x:v>热带城市躺平感</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
-      </x:c>
-      <x:c r="H86"/>
+        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>cairns-lagoon-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="str">
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B87" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>下午 / 傍晚</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Palm Cove</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
+        <x:v>为次日清晨航班做准备</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
-      </x:c>
-      <x:c r="H87" t="str">
-        <x:v>palm-cove-map</x:v>
-      </x:c>
+        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
+      </x:c>
+      <x:c r="H87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="str">
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B88" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>晚上</x:v>
+        <x:v>下午 / 傍晚</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Palm Cove</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>海鲜或轻松简餐</x:v>
+        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>早点吃，早点睡</x:v>
+        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
+        <x:v>palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4139,51 +4139,51 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B89" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海鲜或轻松简餐</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
+        <x:v>早点吃，早点睡</x:v>
       </x:c>
       <x:c r="H89" t="str">
-        <x:v>rustys-map,prawn-star-map</x:v>
+        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B90" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>清晨</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
       </x:c>
       <x:c r="H90" t="str">
-        <x:v>cairns-airport-map</x:v>
+        <x:v>rustys-map,prawn-star-map</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -4191,75 +4191,75 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B91" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>上午</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>凯恩斯 → 悉尼</x:v>
+        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H91"/>
+        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>cairns-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B92" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>从热带切换回冬季海港城市</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
-      </x:c>
-      <x:c r="H92" t="str">
-        <x:v>oaks-sydney-map</x:v>
-      </x:c>
+        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
+      </x:c>
+      <x:c r="H92"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B93" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>下午</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>悉尼 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>4人 + 行李，打车最省心</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>如不能入住，先寄存行李</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4267,25 +4267,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B94" t="n">
-        <x:v>45</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>Darling Harbour / 酒店周边</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4293,25 +4293,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B95" t="n">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H95" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -4319,25 +4319,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B96" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>晚上</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H96" t="str">
-        <x:v>circular-quay-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4345,51 +4345,51 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>歌剧院、海港大桥夜景</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B98" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4397,25 +4397,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B99" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>08:15–08:30</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>抵达海港区</x:v>
       </x:c>
       <x:c r="F99" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>Ferry、海港桥、歌剧院远景</x:v>
       </x:c>
       <x:c r="G99" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4423,25 +4423,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B100" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>08:30–09:10</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F100" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>悉尼核心地标</x:v>
       </x:c>
       <x:c r="G100" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
       </x:c>
       <x:c r="H100" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -4449,25 +4449,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B101" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
+        <x:v>中文内部导览已订</x:v>
       </x:c>
       <x:c r="F101" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>建筑故事、内部空间、剧院结构</x:v>
       </x:c>
       <x:c r="G101" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
       </x:c>
       <x:c r="H101" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -4475,25 +4475,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B102" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>10:30–10:50</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>Opera House → The Rocks</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
+        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
       </x:c>
       <x:c r="F102" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
+        <x:v>海港步行衔接悉尼老城区</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
+        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -4501,25 +4501,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B103" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>10:50–11:50</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
       </x:c>
       <x:c r="F103" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
       </x:c>
       <x:c r="G103" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
       </x:c>
       <x:c r="H103" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -4527,25 +4527,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B104" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>11:50–12:40</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Royal Botanic Garden</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
       </x:c>
       <x:c r="F104" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>就地补体力，不为午餐绕路</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
       </x:c>
       <x:c r="H104" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -4553,25 +4553,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B105" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>12:40–14:10</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>植物园海港步道</x:v>
       </x:c>
       <x:c r="F105" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H105" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>botanic-garden-map</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -4579,25 +4579,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B106" t="n">
-        <x:v>90</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>歌剧院 + 海港大桥同框</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>悉尼最经典机位</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
       </x:c>
       <x:c r="H106" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>mrs-macquarie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -4605,25 +4605,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B107" t="n">
-        <x:v>100</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>晚上</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>购物、室内休息</x:v>
       </x:c>
       <x:c r="F107" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>建筑漂亮，适合逛</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
       </x:c>
       <x:c r="H107" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -4631,51 +4631,51 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B108" t="n">
-        <x:v>900</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>饮食</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>CBD / Darling Harbour</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>Hello Auntie / CBD 晚餐</x:v>
       </x:c>
       <x:c r="F108" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G108" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H108" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B109" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>08:00</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F109" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G109" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H109" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -4683,25 +4683,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B110" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>09:15</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>royal-national-park-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -4709,25 +4709,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B111" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>10:00</x:v>
+        <x:v>09:15</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>南海岸第一处全景</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
       </x:c>
       <x:c r="H111" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>bald-hill-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -4735,25 +4735,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B112" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>11:15</x:v>
+        <x:v>10:00</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>贴着太平洋的公路画面</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>不要在桥上或路肩危险停车</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -4761,25 +4761,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B113" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>12:00</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>Wollongong / 南海岸补给</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>短停咖啡或直接通过</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>wollongong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -4787,25 +4787,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>Kiama Blowhole</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>看喷潮洞、灯塔与海边</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>Kiama 代表性海岸地貌</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -4813,25 +4813,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>13:30</x:v>
+        <x:v>12:30–13:30</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>海边小镇节奏</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -4839,25 +4839,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>13:30</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Kiama → Gerringong</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>沿海继续南下</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>kiama-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -4865,25 +4865,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>90</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>14:40</x:v>
+        <x:v>13:45–14:40</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -4891,25 +4891,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>100</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>14:40</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>Gerringong</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>判断是否延伸 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>时间、天气与体力闸门</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>gerringong-map,kangaroo-valley-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -4917,25 +4917,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>110</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>可选 15:30–16:15</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>看历史桥、山谷与小镇</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -4943,51 +4943,51 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>900</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>饮食</x:v>
+        <x:v>16:15 前</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>环线收束</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -4995,25 +4995,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>08:30–09:00</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -5021,25 +5021,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>09:15 左右</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -5047,25 +5047,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>09:30–13:30</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -5073,25 +5073,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>13:30–14:30</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>F2 返回市区后前往 Bondi</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>动物园切换到悉尼海岸</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -5099,25 +5099,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>18:30</x:v>
+        <x:v>14:30–17:45</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>海滩散步并走一段 Coastal Walk</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -5125,51 +5125,51 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>饮食</x:v>
+        <x:v>18:30</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -5177,25 +5177,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>oaks-sydney-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -5203,25 +5203,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>可选 09:30 左右</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Circular Quay → Manly</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>搭乘公共 F1 Manly Ferry</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>circular-quay-map,manly-ferry-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -5229,25 +5229,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>可选 10:00–12:45</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>Manly Beach / The Corso</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>海边散步、咖啡或早午餐</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -5255,25 +5255,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>13:00–13:30</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>Manly → Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>最晚搭船回市区</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -5281,25 +5281,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>14:00–15:30</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>酒店</x:v>
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>最后采购</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>药妆、保健品、伴手礼</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -5307,25 +5307,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>16:40</x:v>
+        <x:v>15:30–16:20</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>酒店</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>整理 TRS 物品和返程行李</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>为 D16 机场退税做准备</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>oaks-sydney-map,trs-official</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -5333,25 +5333,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>17:30</x:v>
+        <x:v>16:40</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>前往 Cafe Sydney</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>避免迟到</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -5359,51 +5359,51 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B136" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>饮食</x:v>
+        <x:v>17:30</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Cafe Sydney</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海港景观 + 澳洲最后一晚</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" t="str">
-        <x:v>d16</x:v>
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B137" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>上午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D137" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
       </x:c>
       <x:c r="F137" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -5411,24 +5411,50 @@
         <x:v>d16</x:v>
       </x:c>
       <x:c r="B138" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F138" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G138" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H138" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B139" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C138" t="str">
+      <x:c r="C139" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D138" t="str">
+      <x:c r="D139" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E138" t="str">
+      <x:c r="E139" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F138" t="str">
+      <x:c r="F139" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G138" t="str">
+      <x:c r="G139" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H138"/>
+      <x:c r="H139"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8152,6 +8178,63 @@
       <x:c r="F142" t="str"/>
       <x:c r="G142" t="str">
         <x:v>Official booking · general admission; prices and availability can change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>mel-airport-car-rental-map</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>Melbourne Airport Car Rental Branch</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Melbourne+Airport+Car+Rental</x:v>
+      </x:c>
+      <x:c r="E143"/>
+      <x:c r="F143"/>
+      <x:c r="G143" t="str">
+        <x:v>Google Maps · 按租车订单确认具体门店与接驳方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>coles-torquay-map</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>Coles Torquay</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Coles+Torquay+41+Bristol+Road+Torquay+VIC+3228</x:v>
+      </x:c>
+      <x:c r="E144"/>
+      <x:c r="F144"/>
+      <x:c r="G144" t="str">
+        <x:v>Google Maps · 41 Bristol Road, Torquay VIC 3228</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>grey-river-road-map</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>Grey River Road · Kennett River</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Grey+River+Road+Kennett+River+VIC</x:v>
+      </x:c>
+      <x:c r="E145"/>
+      <x:c r="F145"/>
+      <x:c r="G145" t="str">
+        <x:v>Google Maps · Kennett River 野生考拉观察路段</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9202,14 +9285,15 @@
         <x:v>出发咖啡</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Lorne café / Snow Monkey Ramen（备选）</x:v>
+        <x:v>Lorne café / Snow Monkey Ramen</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>Apollo Bay Fishermen's Co-op / seafood café</x:v>
+        <x:v>Seaview Motel BBQ</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>海岸驾驶日以轻松好吃为主，Apollo Bay 的 fish &amp; chips / 海鲜正合适。</x:v>
-      </x:c>
+        <x:v>上午在 Torquay 买好 BBQ 食材；Lorne 坐下来吃午餐，抵达 Apollo Bay 后在住处准备晚餐。</x:v>
+      </x:c>
+      <x:c r="F4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">

</xml_diff>

<commit_message>
use hotel as D3 first navigation stop
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R5600eec9f2f544b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Re18bc379b6f44bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rd7eb818db6b4401a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Rc3a77d811bcc4603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rb1ae6760a3884181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R3bb2c7dfd0b1467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R051c54a6442e4bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R09ab85c4bb2f4f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Redf070c216b647fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Rc95da86ce33a4e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R4e96de5bf0a54883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rc45f147ba9484eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R65f9af8492c94ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Rd2ade096a08b489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R7eed740a57084703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R5406cca3cef04901"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R557ba610ee6746f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R2a614fa8102641e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R2fe97a2cfb444590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Red2f13b699784805"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -893,7 +893,7 @@
         <x:v>seaview-motel-map</x:v>
       </x:c>
       <x:c r="R5" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>holiday-inn-airport-map</x:v>
       </x:c>
       <x:c r="S5" t="str">
         <x:v>no-fixed-ticket</x:v>

</xml_diff>

<commit_message>
update D4 Great Ocean Road route
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R4e96de5bf0a54883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rc45f147ba9484eff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R65f9af8492c94ee9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Rd2ade096a08b489d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R7eed740a57084703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R5406cca3cef04901"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R557ba610ee6746f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R2a614fa8102641e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R2fe97a2cfb444590"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Red2f13b699784805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R9e1190e64c734ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Re3405e473edb4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R075fecd285a941cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R90befce99880404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rccf875f4ea7443a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R17a534f1032d4db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R0f514ac1b7ba431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R20afad91d096442c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R2eab2ccd79a44fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R00f25b10372e4bca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -922,19 +922,19 @@
         <x:v>142.9956</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>红杉林到海岸：The Redwoods、十二使徒岩与 Loch Ard Gorge</x:v>
+        <x:v>从雨林走向海岸：The Redwoods、十二使徒岩与 Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="I6" t="str">
-        <x:v>先走进 The Redwoods Otways，再回到海岸看十二使徒岩、Loch Ard Gorge 与 The Razorback。</x:v>
+        <x:v>上午从 Apollo Bay 补给出发，走进 Maits Rest 与 The Redwoods；下午回到 Gibson Steps、十二使徒岩和 Loch Ard Gorge 的海岸线，傍晚在 Port Campbell 收住这一天。</x:v>
       </x:c>
       <x:c r="J6" t="str">
         <x:v>Southern Ocean Villas</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>海岸风大，步道和台阶雨后湿滑。</x:v>
+        <x:v>林区早上湿冷，下午海岸风大；步道和台阶雨后容易湿滑。</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>防风外套、防水鞋；拍照时不要太靠近海浪。</x:v>
+        <x:v>长袖打底、中层与防风防水外套；穿防滑鞋，帽子和薄手套放车里。</x:v>
       </x:c>
       <x:c r="M6" t="str">
         <x:v>/itinerary/d4-twelve-apostles-gorge.png</x:v>
@@ -943,16 +943,16 @@
         <x:v>十二使徒岩与峡谷海岸</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>自驾 · 大洋路海岸段</x:v>
+        <x:v>自驾 · 雨林山路 + 大洋路海岸段</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>07:45 前离开 Apollo Bay</x:v>
+        <x:v>08:30 退房启程；09:15 后离开 Apollo Bay 时，从 Maits Rest 直接前往 Castle Cove</x:v>
       </x:c>
       <x:c r="Q6" t="str">
         <x:v>southern-ocean-villas-map</x:v>
       </x:c>
       <x:c r="R6" t="str">
-        <x:v>redwoods-otways-map</x:v>
+        <x:v>d4-full-route-map</x:v>
       </x:c>
       <x:c r="S6" t="str">
         <x:v>no-fixed-ticket</x:v>
@@ -2858,22 +2858,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>备选 · 清晨</x:v>
+        <x:v>08:30</x:v>
       </x:c>
       <x:c r="D39" t="str">
-        <x:v>Maits Rest Rainforest Walk</x:v>
+        <x:v>Seaview Motel &amp; Apartments</x:v>
       </x:c>
       <x:c r="E39" t="str">
-        <x:v>若 07:45 前离开 Apollo Bay 且时间充裕，可先走一段雨林环线。</x:v>
+        <x:v>早餐后退房，检查昨晚食材、垃圾与冰袋，带好水和零食</x:v>
       </x:c>
       <x:c r="F39" t="str">
-        <x:v>冬日湿润雨林，非常有氛围</x:v>
+        <x:v>从 Apollo Bay 开始雨林与海岸的一天</x:v>
       </x:c>
       <x:c r="G39" t="str">
-        <x:v>只有早出发且时间充裕时再停，约 30 分钟。</x:v>
+        <x:v>计划 08:30–09:00 离开；防风外套放在手边，停车下车时随时可穿。</x:v>
       </x:c>
       <x:c r="H39" t="str">
-        <x:v>maits-rest-map</x:v>
+        <x:v>seaview-motel-map,d4-full-route-map,d4-direct-coast-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2884,22 +2884,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>上午</x:v>
+        <x:v>08:45</x:v>
       </x:c>
       <x:c r="D40" t="str">
-        <x:v>The Redwoods Otways</x:v>
+        <x:v>Apollo Bay 镇中心补给</x:v>
       </x:c>
       <x:c r="E40" t="str">
-        <x:v>从北侧 Binns Road 进入红杉林，沿 Aire River 林间步道慢走约 30–45 分钟。</x:v>
+        <x:v>在 FoodWorks 或 IGA 买咖啡、水、面包、三明治、水果和午间轻食</x:v>
       </x:c>
       <x:c r="F40" t="str">
-        <x:v>高大的加州红杉、林下光影与安静的河谷氛围</x:v>
+        <x:v>离开小镇前完成当天补给</x:v>
       </x:c>
       <x:c r="G40" t="str">
-        <x:v>林区无手机信号，地面可能湿滑；出发前查看 Parks Victoria 路况与现场标识。</x:v>
+        <x:v>十二使徒岩一带餐饮选择少，午餐按轻食 / picnic 准备。</x:v>
       </x:c>
       <x:c r="H40" t="str">
-        <x:v>redwoods-otways-map,redwoods-otways-official</x:v>
+        <x:v>foodworks-apollo-bay-map,apollo-bay-iga-map,d4-full-route-map,d4-direct-coast-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2910,22 +2910,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>中午前后</x:v>
+        <x:v>09:15–10:00</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Gibson Steps</x:v>
+        <x:v>Maits Rest Rainforest Walk</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>下到海滩看悬崖与海蚀柱</x:v>
+        <x:v>沿雨林环线走进树蕨、苔藓与高大古树之间</x:v>
       </x:c>
       <x:c r="F41" t="str">
-        <x:v>人物比例感很强，比单纯观景台更有沉浸感</x:v>
+        <x:v>阴天也很有层次的温带雨林</x:v>
       </x:c>
       <x:c r="G41" t="str">
-        <x:v>看开放情况和风浪；风大时不要太靠近海浪</x:v>
+        <x:v>环线约 30–45 分钟；雨后木栈道湿滑，穿防滑鞋。</x:v>
       </x:c>
       <x:c r="H41" t="str">
-        <x:v>gibson-steps-map</x:v>
+        <x:v>maits-rest-map</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2936,22 +2936,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>下午</x:v>
+        <x:v>10:20–11:10</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Twelve Apostles</x:v>
+        <x:v>The Redwoods Otways</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>十二使徒岩主观景台</x:v>
+        <x:v>沿 Binns Road 前往红杉林，在高大树干、小溪与苔藓间慢走拍照</x:v>
       </x:c>
       <x:c r="F42" t="str">
-        <x:v>大洋路最具代表性的海岸地貌</x:v>
+        <x:v>安静的红杉林与河谷光影</x:v>
       </x:c>
       <x:c r="G42" t="str">
-        <x:v>左侧平台更适合拍海岸线纵深；如果人多，不要停太久</x:v>
+        <x:v>如果 09:15 后才离开 Apollo Bay，或走完 Maits Rest 已觉疲惫，就沿主路前往 Castle Cove，让下午的海岸段更从容；入林前查看 Parks Victoria 与现场标识。</x:v>
       </x:c>
       <x:c r="H42" t="str">
-        <x:v>twelve-apostles-map</x:v>
+        <x:v>redwoods-otways-map,redwoods-otways-official,d4-direct-coast-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2962,22 +2962,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>下午</x:v>
+        <x:v>12:10</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Loch Ard Gorge</x:v>
+        <x:v>Castle Cove Lookout</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>在主观景区看峡湾与沉船故事，再接 Geology Walk。</x:v>
+        <x:v>从高处俯看海岸与悬崖，在离开森林后重新迎向南大洋</x:v>
       </x:c>
       <x:c r="F43" t="str">
-        <x:v>峡湾地貌、沉船历史与悬崖顶观景</x:v>
+        <x:v>雨林转回海岸的第一眼</x:v>
       </x:c>
       <x:c r="G43" t="str">
-        <x:v>至少预留 1 小时；海滩下行台阶关闭，按现场标识走崖顶步道。</x:v>
+        <x:v>停留 5–10 分钟，快速拍照后继续前往 Gibson Steps。</x:v>
       </x:c>
       <x:c r="H43" t="str">
-        <x:v>loch-ard-map</x:v>
+        <x:v>castle-cove-lookout-map</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2985,25 +2985,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B44" t="n">
-        <x:v>55</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>下午</x:v>
+        <x:v>12:45–13:25</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>Tom and Eva</x:v>
+        <x:v>Gibson Steps</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>Loch Ard Gorge 附近短停</x:v>
+        <x:v>从崖顶看海蚀柱；台阶开放且海况平稳时走到沙滩</x:v>
       </x:c>
       <x:c r="F44" t="str">
-        <x:v>两个海蚀柱，和沉船故事相关</x:v>
+        <x:v>在海平面感受悬崖与岩柱的尺度</x:v>
       </x:c>
       <x:c r="G44" t="str">
-        <x:v>作为 Loch Ard Gorge 区域顺路点，不需要额外绕路</x:v>
+        <x:v>停留 25–40 分钟；遵守关闭标识，风浪大时留在上方观景。</x:v>
       </x:c>
       <x:c r="H44" t="str">
-        <x:v>tom-eva-map,loch-ard-map</x:v>
+        <x:v>gibson-steps-map</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3011,25 +3011,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B45" t="n">
-        <x:v>60</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>13:40–14:40</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>The Razorback</x:v>
+        <x:v>Twelve Apostles</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>从 Loch Ard Gorge 主停车场走 900 米往返 Geology Walk，经 Island Arch 到 The Razorback 观景台。</x:v>
+        <x:v>走过主观景台与木栈道，看十二使徒岩和海岸纵深</x:v>
       </x:c>
       <x:c r="F45" t="str">
-        <x:v>同一景区内的狭长海蚀岩脊与悬崖顶视角</x:v>
+        <x:v>大洋路最经典的南大洋画面</x:v>
       </x:c>
       <x:c r="G45" t="str">
-        <x:v>步行往返约 30–40 分钟；不需要另开一段车程。</x:v>
+        <x:v>预留 45–60 分钟；下午光线好时慢一点，不必只拍一张就走。</x:v>
       </x:c>
       <x:c r="H45" t="str">
-        <x:v>razorback-map</x:v>
+        <x:v>twelve-apostles-map</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -3037,25 +3037,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B46" t="n">
-        <x:v>70</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>15:00–15:50</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>抵达入住 Southern Ocean Villas</x:v>
+        <x:v>沿上方观景区看峡谷、海湾与沉船故事相关地貌</x:v>
       </x:c>
       <x:c r="F46" t="str">
-        <x:v>方便第二天清晨补拍</x:v>
+        <x:v>峡湾、黄岩悬崖与沉船历史</x:v>
       </x:c>
       <x:c r="G46" t="str">
-        <x:v>不要天黑后还在海岸小路上赶</x:v>
+        <x:v>海滩下行台阶目前因地质不稳定关闭；按现场标识走崖顶步道，预留 40–60 分钟。</x:v>
       </x:c>
       <x:c r="H46" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>loch-ard-map,loch-ard-official</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -3063,25 +3063,25 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B47" t="n">
-        <x:v>80</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>晚上</x:v>
+        <x:v>15:50–16:05</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>Tom and Eva Lookout</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>抵达后按天气选择公共电烤炉 BBQ、villa 厨房自炊或附近餐厅</x:v>
+        <x:v>沿 Loch Ard Gorge 步道看 Tom and Eva 两座海蚀柱</x:v>
       </x:c>
       <x:c r="F47" t="str">
-        <x:v>灵活完成 BBQ-style dinner</x:v>
+        <x:v>沉船故事里的两座海蚀柱</x:v>
       </x:c>
       <x:c r="G47" t="str">
-        <x:v>Southern Ocean Villas 没有自带 BBQ，但附近有两处免费 electric BBQ；villa 厨房备有油、盐、胡椒和锡纸。</x:v>
+        <x:v>停留 10–15 分钟，与 Loch Ard Gorge 连在一起步行完成。</x:v>
       </x:c>
       <x:c r="H47" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>tom-eva-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -3089,129 +3089,129 @@
         <x:v>d4</x:v>
       </x:c>
       <x:c r="B48" t="n">
-        <x:v>900</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>饮食</x:v>
+        <x:v>16:10–16:35</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>The Razorback Lookout</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：在 Apollo Bay 买好食材，抵达后按天气选择公共 electric BBQ 或 villa 厨房自炊</x:v>
+        <x:v>沿 Loch Ard Gorge 同一景区步道前往观景台，看狭长岩脊与岩层纹理</x:v>
       </x:c>
       <x:c r="F48" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>低角度光线下更有层次的海蚀岩脊</x:v>
       </x:c>
       <x:c r="G48" t="str">
-        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
+        <x:v>与 Tom and Eva、Loch Ard Gorge 同一片区域，实际步行按现场标识和体力安排。</x:v>
       </x:c>
       <x:c r="H48" t="str">
-        <x:v>apollo-map,port-campbell-map</x:v>
+        <x:v>razorback-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
-        <x:v>d5</x:v>
+        <x:v>d4</x:v>
       </x:c>
       <x:c r="B49" t="n">
-        <x:v>10</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>07:00-07:30</x:v>
+        <x:v>16:45</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>Port Campbell Foreshore</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>退房、装车并简单早餐</x:v>
+        <x:v>到镇上后沿海湾短走，看看防波堤与傍晚海面</x:v>
       </x:c>
       <x:c r="F49" t="str">
-        <x:v>小镇清晨 + 返程准备</x:v>
+        <x:v>用小镇海湾结束当天海岸线</x:v>
       </x:c>
       <x:c r="G49" t="str">
-        <x:v>把行李装车、早餐和退房一次完成；07:30 左右驶离住宿。</x:v>
+        <x:v>停留 15–30 分钟；如果风冷或天色已暗，就先去办理入住。</x:v>
       </x:c>
       <x:c r="H49" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>port-campbell-foreshore-map</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" t="str">
-        <x:v>d5</x:v>
+        <x:v>d4</x:v>
       </x:c>
       <x:c r="B50" t="n">
-        <x:v>20</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>天气补拍备选 · 07:30-08:10</x:v>
+        <x:v>17:00</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
+        <x:v>Southern Ocean Villas</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>若前一日受天气影响，在两处中只选一处清晨补拍；若已看够则直接前往 The Grotto</x:v>
+        <x:v>办理入住，洗澡换衣，稍作休息</x:v>
       </x:c>
       <x:c r="F50" t="str">
-        <x:v>柔和晨光 + 较少游客</x:v>
+        <x:v>在 Port Campbell 安顿下来</x:v>
       </x:c>
       <x:c r="G50" t="str">
-        <x:v>只选一处，08:10 最晚离开；这段是天气补拍，不影响 10:00 后进入 Wildlife Park。</x:v>
+        <x:v>放好行李后，于 18:00–18:30 前往晚餐。</x:v>
       </x:c>
       <x:c r="H50" t="str">
-        <x:v>twelve-apostles-map,loch-ard-map</x:v>
+        <x:v>southern-ocean-villas-map</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
-        <x:v>d5</x:v>
+        <x:v>d4</x:v>
       </x:c>
       <x:c r="B51" t="n">
-        <x:v>30</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>08:35 左右</x:v>
+        <x:v>18:00–18:30</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>The Grotto</x:v>
+        <x:v>Port Campbell 晚餐</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>看海蚀洞和海水窗口</x:v>
+        <x:v>首选 Port Campbell Hotel；想吃海鲜可去 12 Rocks，想轻松外带可选 REAL Pizza，想配精酿啤酒可去 Sow &amp; Piglets</x:v>
       </x:c>
       <x:c r="F51" t="str">
-        <x:v>洞穴 + 海景构图</x:v>
+        <x:v>热餐、海鲜、披萨或精酿，按当晚状态选择</x:v>
       </x:c>
       <x:c r="G51" t="str">
-        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
+        <x:v>尽量 18:30 前开始晚餐；到镇前确认营业时间，需要时提前订位或下单。</x:v>
       </x:c>
       <x:c r="H51" t="str">
-        <x:v>grotto-map</x:v>
+        <x:v>port-campbell-map,port-campbell-hotel-map,twelve-rocks-map,real-pizza-port-campbell-map,sow-piglets-map</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" t="str">
-        <x:v>d5</x:v>
+        <x:v>d4</x:v>
       </x:c>
       <x:c r="B52" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>09:10 左右</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>London Bridge / London Arch</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>看海蚀拱门</x:v>
+        <x:v>早餐：Apollo Bay café；午餐：提前准备的轻食 / picnic；晚餐：Port Campbell Hotel / 12 Rocks / REAL Pizza / Sow &amp; Piglets</x:v>
       </x:c>
       <x:c r="F52" t="str">
-        <x:v>Port Campbell 以西经典点</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G52" t="str">
-        <x:v>顺路短停，很适合加</x:v>
+        <x:v>咖啡、水和午间轻食离开 Apollo Bay 前买好；晚餐尽量 18:00–18:30 入座。</x:v>
       </x:c>
       <x:c r="H52" t="str">
-        <x:v>london-arch-map,port-campbell-map</x:v>
+        <x:v>foodworks-apollo-bay-map,apollo-bay-iga-map,port-campbell-hotel-map,twelve-rocks-map,real-pizza-port-campbell-map,sow-piglets-map</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -3219,25 +3219,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B53" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>10:15-11:30</x:v>
+        <x:v>07:00-07:30</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Great Ocean Road Wildlife Park</x:v>
+        <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>购买普通门票进入互动区和 sanctuary，近距离看袋鼠、沙袋鼠等澳洲本土动物；游园和可选购饲料喂食合计预留 60-75 分钟</x:v>
+        <x:v>退房、装车并简单早餐</x:v>
       </x:c>
       <x:c r="F53" t="str">
-        <x:v>大洋路沿线的澳洲本土动物互动体验</x:v>
+        <x:v>小镇清晨 + 返程准备</x:v>
       </x:c>
       <x:c r="G53" t="str">
-        <x:v>普通门票建议提前在线购买；动物饲料和 close-up encounters 另付费。步道多为未铺装地面，穿防滑包脚鞋；11:45 前离园，为 Colac 午餐、加油和机场还车保留缓冲。</x:v>
+        <x:v>把行李装车、早餐和退房一次完成；07:30 左右驶离住宿。</x:v>
       </x:c>
       <x:c r="H53" t="str">
-        <x:v>great-ocean-road-wildlife-park-map,great-ocean-road-wildlife-park-official,great-ocean-road-wildlife-park-booking</x:v>
+        <x:v>port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3245,25 +3245,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B54" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>下午</x:v>
+        <x:v>天气补拍备选 · 07:30-08:10</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Colac</x:v>
+        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>午餐、加油、休息</x:v>
+        <x:v>若前一日受天气影响，在两处中只选一处清晨补拍；若已看够则直接前往 The Grotto</x:v>
       </x:c>
       <x:c r="F54" t="str">
-        <x:v>内陆牧场风光</x:v>
+        <x:v>柔和晨光 + 较少游客</x:v>
       </x:c>
       <x:c r="G54" t="str">
-        <x:v>回程中段休息点</x:v>
+        <x:v>只选一处，08:10 最晚离开；这段是天气补拍，不影响 10:00 后进入 Wildlife Park。</x:v>
       </x:c>
       <x:c r="H54" t="str">
-        <x:v>colac-map</x:v>
+        <x:v>twelve-apostles-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3271,25 +3271,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B55" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>08:35 左右</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>The Grotto</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
+        <x:v>看海蚀洞和海水窗口</x:v>
       </x:c>
       <x:c r="F55" t="str">
-        <x:v>大洋路自驾收尾</x:v>
+        <x:v>洞穴 + 海景构图</x:v>
       </x:c>
       <x:c r="G55" t="str">
-        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
+        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
       </x:c>
       <x:c r="H55" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>grotto-map</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3297,25 +3297,25 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B56" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>晚上</x:v>
+        <x:v>09:10 左右</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Holiday Inn Melbourne Airport</x:v>
+        <x:v>London Bridge / London Arch</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>入住、整理行李</x:v>
+        <x:v>看海蚀拱门</x:v>
       </x:c>
       <x:c r="F56" t="str">
-        <x:v>为次日早班机准备</x:v>
+        <x:v>Port Campbell 以西经典点</x:v>
       </x:c>
       <x:c r="G56" t="str">
-        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
+        <x:v>顺路短停，很适合加</x:v>
       </x:c>
       <x:c r="H56" t="str">
-        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
+        <x:v>london-arch-map,port-campbell-map</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3323,127 +3323,129 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B57" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>饮食</x:v>
+        <x:v>10:15-11:30</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Great Ocean Road Wildlife Park</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>早餐：Port Campbell café；午餐：离开 Great Ocean Road Wildlife Park 后在 Colac 简餐；晚餐：机场酒店简餐</x:v>
+        <x:v>购买普通门票进入互动区和 sanctuary，近距离看袋鼠、沙袋鼠等澳洲本土动物；游园和可选购饲料喂食合计预留 60-75 分钟</x:v>
       </x:c>
       <x:c r="F57" t="str">
-        <x:v>野生动物体验 + 内陆返程补给</x:v>
+        <x:v>大洋路沿线的澳洲本土动物互动体验</x:v>
       </x:c>
       <x:c r="G57" t="str">
-        <x:v>Colac 作为返程主休息点，把午餐、加油和休息一次完成；抵达机场后简单用餐并整理行李。</x:v>
+        <x:v>普通门票建议提前在线购买；动物饲料和 close-up encounters 另付费。步道多为未铺装地面，穿防滑包脚鞋；11:45 前离园，为 Colac 午餐、加油和机场还车保留缓冲。</x:v>
       </x:c>
       <x:c r="H57" t="str">
-        <x:v>great-ocean-road-wildlife-park-map,colac-map,holiday-inn-airport-map</x:v>
+        <x:v>great-ocean-road-wildlife-park-map,great-ocean-road-wildlife-park-official,great-ocean-road-wildlife-park-booking</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B58" t="n">
-        <x:v>10</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>Colac</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>飞往凯恩斯</x:v>
+        <x:v>午餐、加油、休息</x:v>
       </x:c>
       <x:c r="F58" t="str">
-        <x:v>气候切换非常明显</x:v>
+        <x:v>内陆牧场风光</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>国内航班建议预留行李额</x:v>
+        <x:v>回程中段休息点</x:v>
       </x:c>
       <x:c r="H58" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>colac-map</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B59" t="n">
-        <x:v>20</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>中午</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>打车 / Uber 到酒店</x:v>
+        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
       </x:c>
       <x:c r="F59" t="str">
-        <x:v>不租车，降低疲劳</x:v>
+        <x:v>大洋路自驾收尾</x:v>
       </x:c>
       <x:c r="G59" t="str">
-        <x:v>酒店可先寄存行李</x:v>
-      </x:c>
-      <x:c r="H59"/>
+        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B60" t="n">
-        <x:v>30</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>下午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Esplanade Lagoon</x:v>
+        <x:v>Holiday Inn Melbourne Airport</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>免费泻湖泳池、海滨散步</x:v>
+        <x:v>入住、整理行李</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>度假感拉满</x:v>
+        <x:v>为次日早班机准备</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>泳衣可提前放随身包</x:v>
+        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
       </x:c>
       <x:c r="H60" t="str">
-        <x:v>cairns-lagoon-map</x:v>
+        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B61" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>晚上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Cairns Night Markets</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>夜市、简餐、纪念品</x:v>
+        <x:v>早餐：Port Campbell café；午餐：离开 Great Ocean Road Wildlife Park 后在 Colac 简餐；晚餐：机场酒店简餐</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>热闹轻松</x:v>
+        <x:v>野生动物体验 + 内陆返程补给</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+        <x:v>Colac 作为返程主休息点，把午餐、加油和休息一次完成；抵达机场后简单用餐并整理行李。</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>cairns-night-market-map</x:v>
+        <x:v>great-ocean-road-wildlife-park-map,colac-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -3451,153 +3453,151 @@
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B62" t="n">
-        <x:v>900</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>饮食</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
+        <x:v>飞往凯恩斯</x:v>
       </x:c>
       <x:c r="F62" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>气候切换非常明显</x:v>
       </x:c>
       <x:c r="G62" t="str">
-        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
-      </x:c>
-      <x:c r="H62"/>
+        <x:v>国内航班建议预留行李额</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B63" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>早上</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>凯恩斯码头</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Reef Magic check-in，登船出海</x:v>
+        <x:v>打车 / Uber 到酒店</x:v>
       </x:c>
       <x:c r="F63" t="str">
-        <x:v>前往外礁平台</x:v>
+        <x:v>不租车，降低疲劳</x:v>
       </x:c>
       <x:c r="G63" t="str">
-        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
-      </x:c>
-      <x:c r="H63" t="str">
-        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
-      </x:c>
+        <x:v>酒店可先寄存行李</x:v>
+      </x:c>
+      <x:c r="H63"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B64" t="n">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>全天</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Outer Reef Pontoon</x:v>
+        <x:v>Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
+        <x:v>免费泻湖泳池、海滨散步</x:v>
       </x:c>
       <x:c r="F64" t="str">
-        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
+        <x:v>度假感拉满</x:v>
       </x:c>
       <x:c r="G64" t="str">
-        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
+        <x:v>泳衣可提前放随身包</x:v>
       </x:c>
       <x:c r="H64" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>cairns-lagoon-map</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B65" t="n">
-        <x:v>30</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>中午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>船上 / 平台</x:v>
+        <x:v>Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>外礁平台午餐</x:v>
+        <x:v>夜市、简餐、纪念品</x:v>
       </x:c>
       <x:c r="F65" t="str">
-        <x:v>轻松补给</x:v>
+        <x:v>热闹轻松</x:v>
       </x:c>
       <x:c r="G65" t="str">
-        <x:v>不要吃太撑，避免晕船</x:v>
+        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
       </x:c>
       <x:c r="H65" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>cairns-night-market-map</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B66" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>下午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>下船休息</x:v>
+        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>通常会比较疲惫</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G66" t="str">
-        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
-      </x:c>
-      <x:c r="H66" t="str">
-        <x:v>reef-fleet-terminal-map</x:v>
-      </x:c>
+        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
+      </x:c>
+      <x:c r="H66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B67" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>晚上</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>码头附近</x:v>
+        <x:v>凯恩斯码头</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
+        <x:v>Reef Magic check-in，登船出海</x:v>
       </x:c>
       <x:c r="F67" t="str">
-        <x:v>海边晚餐</x:v>
+        <x:v>前往外礁平台</x:v>
       </x:c>
       <x:c r="G67" t="str">
-        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
+        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
       </x:c>
       <x:c r="H67" t="str">
-        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
+        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3605,22 +3605,22 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B68" t="n">
-        <x:v>80</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>提醒</x:v>
+        <x:v>全天</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>今日提醒</x:v>
+        <x:v>Outer Reef Pontoon</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
+        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
       </x:c>
       <x:c r="F68" t="str">
-        <x:v>舒适与安全比拍摄数量更重要</x:v>
+        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
       </x:c>
       <x:c r="G68" t="str">
-        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
       </x:c>
       <x:c r="H68" t="str">
         <x:v>reef-magic-official</x:v>
@@ -3631,125 +3631,129 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B69" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>船上 / 平台</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
+        <x:v>外礁平台午餐</x:v>
       </x:c>
       <x:c r="F69" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>轻松补给</x:v>
       </x:c>
       <x:c r="G69" t="str">
-        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+        <x:v>不要吃太撑，避免晕船</x:v>
       </x:c>
       <x:c r="H69" t="str">
-        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B70" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>清晨</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
+        <x:v>下船休息</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>不用自驾，沿途可休息看风景</x:v>
+        <x:v>通常会比较疲惫</x:v>
       </x:c>
       <x:c r="G70" t="str">
-        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
-      </x:c>
-      <x:c r="H70"/>
+        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>reef-fleet-terminal-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B71" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>上午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Daintree River / Rainforest</x:v>
+        <x:v>码头附近</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>鳄鱼游船、雨林步道</x:v>
+        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
+        <x:v>海边晚餐</x:v>
       </x:c>
       <x:c r="G71" t="str">
-        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
       </x:c>
       <x:c r="H71" t="str">
-        <x:v>daintree-river-map</x:v>
+        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B72" t="n">
-        <x:v>30</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>中午</x:v>
+        <x:v>提醒</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Daintree Rainforest</x:v>
+        <x:v>今日提醒</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>团含午餐</x:v>
+        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
       </x:c>
       <x:c r="F72" t="str">
-        <x:v>不用自己找餐厅</x:v>
+        <x:v>舒适与安全比拍摄数量更重要</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>如有忌口提前告知</x:v>
-      </x:c>
-      <x:c r="H72"/>
+        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>reef-magic-official</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B73" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>下午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Cape Tribulation</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>雨林入海、海滩短停留</x:v>
+        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>雨林与海洋在这里交会</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
+        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
       </x:c>
       <x:c r="H73" t="str">
-        <x:v>cape-trib-map</x:v>
+        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3757,179 +3761,175 @@
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B74" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Daintree Ferry / Ice Cream</x:v>
+        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>渡河、热带水果冰淇淋</x:v>
+        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
       </x:c>
       <x:c r="F74" t="str">
-        <x:v>丹翠地区很有代表性的热带味道</x:v>
+        <x:v>不用自驾，沿途可休息看风景</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
-      </x:c>
-      <x:c r="H74" t="str">
-        <x:v>daintree-icecream-map</x:v>
-      </x:c>
+        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
+      </x:c>
+      <x:c r="H74"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B75" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Daintree River / Rainforest</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>18:30 后回到市区</x:v>
+        <x:v>鳄鱼游船、雨林步道</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>回程可休息</x:v>
+        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
-      </x:c>
-      <x:c r="H75"/>
+        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>daintree-river-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B76" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Daintree Rainforest</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>团含午餐</x:v>
       </x:c>
       <x:c r="F76" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>不用自己找餐厅</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
-      </x:c>
-      <x:c r="H76" t="str">
-        <x:v>daintree-icecream-map</x:v>
-      </x:c>
+        <x:v>如有忌口提前告知</x:v>
+      </x:c>
+      <x:c r="H76"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B77" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>早上</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>凯恩斯 → Lake Eacham</x:v>
+        <x:v>Cape Tribulation</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
+        <x:v>雨林入海、海滩短停留</x:v>
       </x:c>
       <x:c r="F77" t="str">
-        <x:v>从热带海边城市进入清凉高原</x:v>
+        <x:v>雨林与海洋在这里交会</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
+        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
       </x:c>
       <x:c r="H77" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>cape-trib-map</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B78" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Lake Eacham</x:v>
+        <x:v>Daintree Ferry / Ice Cream</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>火山湖散步、看湖景</x:v>
+        <x:v>渡河、热带水果冰淇淋</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>安静、清凉、湖水和雨林包围感</x:v>
+        <x:v>丹翠地区很有代表性的热带味道</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
       </x:c>
       <x:c r="H78" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>daintree-icecream-map</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B79" t="n">
-        <x:v>30</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Curtain Fig Tree</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>看巨型帘状无花果树</x:v>
+        <x:v>18:30 后回到市区</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>像热带森林里的巨大自然装置</x:v>
+        <x:v>回程可休息</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>停留 20–30 分钟即可</x:v>
-      </x:c>
-      <x:c r="H79" t="str">
-        <x:v>curtain-fig-map</x:v>
-      </x:c>
+        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
+      </x:c>
+      <x:c r="H79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B80" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>中午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Yungaburra / Gallo Dairyland</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
+        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
+        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
       </x:c>
       <x:c r="H80" t="str">
-        <x:v>yungaburra-map,gallo-map</x:v>
+        <x:v>daintree-icecream-map</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -3937,25 +3937,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B81" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>下午</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
+        <x:v>凯恩斯 → Lake Eacham</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>瀑布短停留、拍照</x:v>
+        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
       </x:c>
       <x:c r="F81" t="str">
-        <x:v>雨林瀑布与高原绿意</x:v>
+        <x:v>从热带海边城市进入清凉高原</x:v>
       </x:c>
       <x:c r="G81" t="str">
-        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
       </x:c>
       <x:c r="H81" t="str">
-        <x:v>millaa-map,ellinjaa-map</x:v>
+        <x:v>lake-eacham-map</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -3963,175 +3963,177 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B82" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Lake Eacham</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>下山回市区，还车或次日早还</x:v>
+        <x:v>火山湖散步、看湖景</x:v>
       </x:c>
       <x:c r="F82" t="str">
-        <x:v>完成高原自然线</x:v>
+        <x:v>安静、清凉、湖水和雨林包围感</x:v>
       </x:c>
       <x:c r="G82" t="str">
-        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
-      </x:c>
-      <x:c r="H82"/>
+        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>lake-eacham-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" t="str">
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B83" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>简单晚餐</x:v>
+        <x:v>看巨型帘状无花果树</x:v>
       </x:c>
       <x:c r="F83" t="str">
-        <x:v>回城后轻松晚餐</x:v>
+        <x:v>像热带森林里的巨大自然装置</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>下山后就近用餐，早点休息。</x:v>
-      </x:c>
-      <x:c r="H83"/>
+        <x:v>停留 20–30 分钟即可</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>curtain-fig-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" t="str">
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B84" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Yungaburra / Gallo Dairyland</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
       </x:c>
       <x:c r="F84" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
       </x:c>
       <x:c r="G84" t="str">
-        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
+        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
       </x:c>
       <x:c r="H84" t="str">
-        <x:v>millaa-map,gallo-map</x:v>
+        <x:v>yungaburra-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B85" t="n">
-        <x:v>10</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>瀑布短停留、拍照</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>周五正好开市，适合补水果和轻食</x:v>
+        <x:v>雨林瀑布与高原绿意</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
+        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
       </x:c>
       <x:c r="H85" t="str">
-        <x:v>rustys-map</x:v>
+        <x:v>millaa-map,ellinjaa-map</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B86" t="n">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>中午</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>下山回市区，还车或次日早还</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>热带城市躺平感</x:v>
+        <x:v>完成高原自然线</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
-      </x:c>
-      <x:c r="H86" t="str">
-        <x:v>cairns-lagoon-map</x:v>
-      </x:c>
+        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
+      </x:c>
+      <x:c r="H86"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B87" t="n">
-        <x:v>30</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>下午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>简单晚餐</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>为次日清晨航班做准备</x:v>
+        <x:v>回城后轻松晚餐</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
+        <x:v>下山后就近用餐，早点休息。</x:v>
       </x:c>
       <x:c r="H87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B88" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>下午 / 傍晚</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Palm Cove</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
+        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
+        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>palm-cove-map</x:v>
+        <x:v>millaa-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4139,25 +4141,25 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B89" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>海鲜或轻松简餐</x:v>
+        <x:v>周五正好开市，适合补水果和轻食</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>早点吃，早点睡</x:v>
+        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
       </x:c>
       <x:c r="H89" t="str">
-        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
+        <x:v>rustys-map</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4165,127 +4167,127 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B90" t="n">
-        <x:v>900</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>热带城市躺平感</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
+        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
       </x:c>
       <x:c r="H90" t="str">
-        <x:v>rustys-map,prawn-star-map</x:v>
+        <x:v>cairns-lagoon-map</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B91" t="n">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>清晨</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>为次日清晨航班做准备</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
-      </x:c>
-      <x:c r="H91" t="str">
-        <x:v>cairns-airport-map</x:v>
-      </x:c>
+        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
+      </x:c>
+      <x:c r="H91"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B92" t="n">
-        <x:v>20</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午 / 傍晚</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>凯恩斯 → 悉尼</x:v>
+        <x:v>Palm Cove</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H92"/>
+        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>palm-cove-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B93" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>海鲜或轻松简餐</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
+        <x:v>早点吃，早点睡</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>oaks-sydney-map</x:v>
+        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B94" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>下午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>rustys-map,prawn-star-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4293,25 +4295,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B95" t="n">
-        <x:v>45</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
       </x:c>
       <x:c r="H95" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>cairns-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -4319,51 +4321,49 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B96" t="n">
-        <x:v>50</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>从热带切换回冬季海港城市</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
-      </x:c>
-      <x:c r="H96" t="str">
-        <x:v>the-rocks-map</x:v>
-      </x:c>
+        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
+      </x:c>
+      <x:c r="H96"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>60</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>悉尼 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>4人 + 行李，打车最省心</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
+        <x:v>如不能入住，先寄存行李</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>circular-quay-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4371,129 +4371,129 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B98" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>饮食</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Darling Harbour / 酒店周边</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B99" t="n">
-        <x:v>10</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
       </x:c>
       <x:c r="F99" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G99" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B100" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F100" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G100" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H100" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B101" t="n">
-        <x:v>30</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>歌剧院、海港大桥夜景</x:v>
       </x:c>
       <x:c r="F101" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G101" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H101" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B102" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
+        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F102" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -4501,25 +4501,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B103" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>08:15–08:30</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
+        <x:v>抵达海港区</x:v>
       </x:c>
       <x:c r="F103" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
+        <x:v>Ferry、海港桥、歌剧院远景</x:v>
       </x:c>
       <x:c r="G103" t="str">
-        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
+        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
       </x:c>
       <x:c r="H103" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -4527,25 +4527,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B104" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>08:30–09:10</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F104" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>悉尼核心地标</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
       </x:c>
       <x:c r="H104" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -4553,25 +4553,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B105" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Royal Botanic Garden</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>中文内部导览已订</x:v>
       </x:c>
       <x:c r="F105" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>建筑故事、内部空间、剧院结构</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
       </x:c>
       <x:c r="H105" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -4579,25 +4579,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B106" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>10:30–10:50</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Opera House → The Rocks</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>海港步行衔接悉尼老城区</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
       </x:c>
       <x:c r="H106" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -4605,25 +4605,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B107" t="n">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>10:50–11:50</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
       </x:c>
       <x:c r="F107" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
       </x:c>
       <x:c r="H107" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -4631,25 +4631,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B108" t="n">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>晚上</x:v>
+        <x:v>11:50–12:40</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
       </x:c>
       <x:c r="F108" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>就地补体力，不为午餐绕路</x:v>
       </x:c>
       <x:c r="G108" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
       </x:c>
       <x:c r="H108" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -4657,129 +4657,129 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B109" t="n">
-        <x:v>900</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>饮食</x:v>
+        <x:v>12:40–14:10</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>植物园海港步道</x:v>
       </x:c>
       <x:c r="F109" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G109" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H109" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>botanic-garden-map</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B110" t="n">
-        <x:v>10</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>08:00</x:v>
+        <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>歌剧院 + 海港大桥同框</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>悉尼最经典机位</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>mrs-macquarie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B111" t="n">
-        <x:v>20</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>09:15</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>购物、室内休息</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>建筑漂亮，适合逛</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
       </x:c>
       <x:c r="H111" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B112" t="n">
-        <x:v>30</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>10:00</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>CBD / Darling Harbour</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>Hello Auntie / CBD 晚餐</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B113" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>11:15</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -4787,25 +4787,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>12:00</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>royal-national-park-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -4813,25 +4813,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>09:15</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>南海岸第一处全景</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>bald-hill-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -4839,25 +4839,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>13:30</x:v>
+        <x:v>10:00</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>贴着太平洋的公路画面</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>不要在桥上或路肩危险停车</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -4865,25 +4865,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Wollongong / 南海岸补给</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>短停咖啡或直接通过</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>wollongong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -4891,25 +4891,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>14:40</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Kiama Blowhole</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>看喷潮洞、灯塔与海边</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>Kiama 代表性海岸地貌</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -4917,25 +4917,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>12:30–13:30</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>海边小镇节奏</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -4943,25 +4943,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>110</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>13:30</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Kiama → Gerringong</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>沿海继续南下</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kiama-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -4969,129 +4969,129 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>饮食</x:v>
+        <x:v>13:45–14:40</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>10</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>14:40</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Gerringong</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>判断是否延伸 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>时间、天气与体力闸门</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>gerringong-map,kangaroo-valley-map</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>20</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>可选 15:30–16:15</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>看历史桥、山谷与小镇</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>16:15 前</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>环线收束</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -5099,25 +5099,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>08:30–09:00</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -5125,25 +5125,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>18:30</x:v>
+        <x:v>09:15 左右</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -5151,129 +5151,129 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>饮食</x:v>
+        <x:v>09:30–13:30</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>上午</x:v>
+        <x:v>13:30–14:30</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>F2 返回市区后前往 Bondi</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>动物园切换到悉尼海岸</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>14:30–17:45</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>海滩散步并走一段 Coastal Walk</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>30</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>18:30</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -5281,25 +5281,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>oaks-sydney-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -5307,25 +5307,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>可选 09:30 左右</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>酒店</x:v>
+        <x:v>Circular Quay → Manly</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>搭乘公共 F1 Manly Ferry</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>circular-quay-map,manly-ferry-map</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -5333,25 +5333,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>16:40</x:v>
+        <x:v>可选 10:00–12:45</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Manly Beach / The Corso</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>海边散步、咖啡或早午餐</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -5359,25 +5359,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B136" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>17:30</x:v>
+        <x:v>13:00–13:30</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>Manly → Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>最晚搭船回市区</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -5385,76 +5385,180 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B137" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>饮食</x:v>
+        <x:v>14:00–15:30</x:v>
       </x:c>
       <x:c r="D137" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>最后采购</x:v>
       </x:c>
       <x:c r="F137" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>药妆、保健品、伴手礼</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" t="str">
-        <x:v>d16</x:v>
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B138" t="n">
-        <x:v>10</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>上午</x:v>
+        <x:v>15:30–16:20</x:v>
       </x:c>
       <x:c r="D138" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>酒店</x:v>
       </x:c>
       <x:c r="E138" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>整理 TRS 物品和返程行李</x:v>
       </x:c>
       <x:c r="F138" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>为 D16 机场退税做准备</x:v>
       </x:c>
       <x:c r="G138" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
       </x:c>
       <x:c r="H138" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>oaks-sydney-map,trs-official</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B139" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C139" t="str">
+        <x:v>16:40</x:v>
+      </x:c>
+      <x:c r="D139" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E139" t="str">
+        <x:v>前往 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>避免迟到</x:v>
+      </x:c>
+      <x:c r="G139" t="str">
+        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+      </x:c>
+      <x:c r="H139" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B140" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C140" t="str">
+        <x:v>17:30</x:v>
+      </x:c>
+      <x:c r="D140" t="str">
+        <x:v>Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="E140" t="str">
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+      </x:c>
+      <x:c r="F140" t="str">
+        <x:v>海港景观 + 澳洲最后一晚</x:v>
+      </x:c>
+      <x:c r="G140" t="str">
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+      </x:c>
+      <x:c r="H140" t="str">
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B141" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>当天餐食节奏</x:v>
+      </x:c>
+      <x:c r="G141" t="str">
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+      </x:c>
+      <x:c r="H141" t="str">
+        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
         <x:v>d16</x:v>
       </x:c>
-      <x:c r="B139" t="n">
+      <x:c r="B142" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G142" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H142" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B143" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C139" t="str">
+      <x:c r="C143" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D139" t="str">
+      <x:c r="D143" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E139" t="str">
+      <x:c r="E143" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F139" t="str">
+      <x:c r="F143" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G139" t="str">
+      <x:c r="G143" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H139"/>
+      <x:c r="H143"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6927,16 +7031,16 @@
         <x:v>twelve-rocks-map</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>12 Rocks Cafe</x:v>
+        <x:v>12 Rocks Beach Cafe &amp; Bar</x:v>
       </x:c>
       <x:c r="C77" t="str">
         <x:v>restaurant</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=12+Rocks+Cafe+Port+Campbell</x:v>
-      </x:c>
-      <x:c r="E77"/>
-      <x:c r="F77"/>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=12+Rocks+Beach+Cafe+%26+Bar+Port+Campbell+VIC</x:v>
+      </x:c>
+      <x:c r="E77" t="str"/>
+      <x:c r="F77" t="str"/>
       <x:c r="G77" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8098,8 +8202,8 @@
       <x:c r="D138" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Point+Ormond+Reserve+Elwood+Melbourne</x:v>
       </x:c>
-      <x:c r="E138" t="str"/>
-      <x:c r="F138" t="str"/>
+      <x:c r="E138"/>
+      <x:c r="F138"/>
       <x:c r="G138" t="str">
         <x:v>Google Maps · Marine Parade, Elwood</x:v>
       </x:c>
@@ -8117,8 +8221,8 @@
       <x:c r="D139" t="str">
         <x:v>https://www.portphillip.vic.gov.au/explore-the-city/beaches-parks-and-playgrounds/find-parks-and-playgrounds/point-ormond-reserve/</x:v>
       </x:c>
-      <x:c r="E139" t="str"/>
-      <x:c r="F139" t="str"/>
+      <x:c r="E139"/>
+      <x:c r="F139"/>
       <x:c r="G139" t="str">
         <x:v>City of Port Phillip · location, paths and facilities</x:v>
       </x:c>
@@ -8136,8 +8240,8 @@
       <x:c r="D140" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Great+Ocean+Road+Wildlife+Park+Gellibrand+Lower+VIC</x:v>
       </x:c>
-      <x:c r="E140" t="str"/>
-      <x:c r="F140" t="str"/>
+      <x:c r="E140"/>
+      <x:c r="F140"/>
       <x:c r="G140" t="str">
         <x:v>Google Maps · 29 The Boulevarde, Gellibrand Lower</x:v>
       </x:c>
@@ -8155,8 +8259,8 @@
       <x:c r="D141" t="str">
         <x:v>https://greatoceanroadwildlifepark.com.au/visitor-information/</x:v>
       </x:c>
-      <x:c r="E141" t="str"/>
-      <x:c r="F141" t="str"/>
+      <x:c r="E141"/>
+      <x:c r="F141"/>
       <x:c r="G141" t="str">
         <x:v>Official · daily 10:00-17:00; recheck hours before travel</x:v>
       </x:c>
@@ -8174,8 +8278,8 @@
       <x:c r="D142" t="str">
         <x:v>https://fareharbor.com/embeds/book/greatoceanroadwildlifepark/?flow=1586423&amp;full-items=yes</x:v>
       </x:c>
-      <x:c r="E142" t="str"/>
-      <x:c r="F142" t="str"/>
+      <x:c r="E142"/>
+      <x:c r="F142"/>
       <x:c r="G142" t="str">
         <x:v>Official booking · general admission; prices and availability can change</x:v>
       </x:c>
@@ -8235,6 +8339,196 @@
       <x:c r="F145"/>
       <x:c r="G145" t="str">
         <x:v>Google Maps · Kennett River 野生考拉观察路段</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>d4-full-route-map</x:v>
+      </x:c>
+      <x:c r="B146" t="str">
+        <x:v>D4 全程导航（含 The Redwoods）</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Seaview+Motel+%26+Apartments%2C+Apollo+Bay+VIC&amp;destination=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;travelmode=driving&amp;waypoints=FoodWorks+Apollo+Bay+VIC%7CMaits+Rest+Rainforest+Walk+VIC%7CThe+Redwoods+Otways%2C+Beech+Forest+VIC%7CCastle+Cove+Lookout+VIC%7CGibson+Steps+VIC%7CTwelve+Apostles+VIC%7CLoch+Ard+Gorge+VIC%7CPort+Campbell+Foreshore+VIC</x:v>
+      </x:c>
+      <x:c r="E146" t="str"/>
+      <x:c r="F146" t="str"/>
+      <x:c r="G146" t="str">
+        <x:v>Google Maps · Apollo Bay 至 Port Campbell</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>d4-direct-coast-route-map</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>D4 沿海导航（跳过 The Redwoods）</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Seaview+Motel+%26+Apartments%2C+Apollo+Bay+VIC&amp;destination=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;travelmode=driving&amp;waypoints=FoodWorks+Apollo+Bay+VIC%7CMaits+Rest+Rainforest+Walk+VIC%7CCastle+Cove+Lookout+VIC%7CGibson+Steps+VIC%7CTwelve+Apostles+VIC%7CLoch+Ard+Gorge+VIC%7CPort+Campbell+Foreshore+VIC</x:v>
+      </x:c>
+      <x:c r="E147" t="str"/>
+      <x:c r="F147" t="str"/>
+      <x:c r="G147" t="str">
+        <x:v>Google Maps · 09:15 后离开 Apollo Bay 时使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>foodworks-apollo-bay-map</x:v>
+      </x:c>
+      <x:c r="B148" t="str">
+        <x:v>FoodWorks Apollo Bay</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=FoodWorks+Apollo+Bay+VIC</x:v>
+      </x:c>
+      <x:c r="E148" t="str"/>
+      <x:c r="F148" t="str"/>
+      <x:c r="G148" t="str">
+        <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>apollo-bay-iga-map</x:v>
+      </x:c>
+      <x:c r="B149" t="str">
+        <x:v>Apollo Bay IGA</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Apollo+Bay+IGA+VIC</x:v>
+      </x:c>
+      <x:c r="E149" t="str"/>
+      <x:c r="F149" t="str"/>
+      <x:c r="G149" t="str">
+        <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>castle-cove-lookout-map</x:v>
+      </x:c>
+      <x:c r="B150" t="str">
+        <x:v>Castle Cove Lookout</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Castle+Cove+Lookout+VIC</x:v>
+      </x:c>
+      <x:c r="E150" t="str"/>
+      <x:c r="F150" t="str"/>
+      <x:c r="G150" t="str">
+        <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
+        <x:v>port-campbell-foreshore-map</x:v>
+      </x:c>
+      <x:c r="B151" t="str">
+        <x:v>Port Campbell Foreshore</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Port+Campbell+Foreshore+VIC</x:v>
+      </x:c>
+      <x:c r="E151" t="str"/>
+      <x:c r="F151" t="str"/>
+      <x:c r="G151" t="str">
+        <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>loch-ard-official</x:v>
+      </x:c>
+      <x:c r="B152" t="str">
+        <x:v>Loch Ard Gorge · Parks Victoria</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>https://www.parks.vic.gov.au/places-to-see/parks/port-campbell-national-park/things-to-do/loch-ard-gorge</x:v>
+      </x:c>
+      <x:c r="E152" t="str"/>
+      <x:c r="F152" t="str"/>
+      <x:c r="G152" t="str">
+        <x:v>Parks Victoria · 行前查看开放与安全提示</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>port-campbell-hotel-map</x:v>
+      </x:c>
+      <x:c r="B153" t="str">
+        <x:v>Port Campbell Hotel</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Port+Campbell+Hotel+VIC</x:v>
+      </x:c>
+      <x:c r="E153" t="str"/>
+      <x:c r="F153" t="str"/>
+      <x:c r="G153" t="str">
+        <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>real-pizza-port-campbell-map</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>REAL Pizza Pasta Salads</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=REAL+Pizza+Pasta+Salads+Port+Campbell+VIC</x:v>
+      </x:c>
+      <x:c r="E154" t="str"/>
+      <x:c r="F154" t="str"/>
+      <x:c r="G154" t="str">
+        <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>sow-piglets-map</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>Sow &amp; Piglets Brew Pub</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>restaurant</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Sow+%26+Piglets+Brew+Pub+Port+Campbell+VIC</x:v>
+      </x:c>
+      <x:c r="E155" t="str"/>
+      <x:c r="F155" t="str"/>
+      <x:c r="G155" t="str">
+        <x:v>Google Maps</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9300,16 +9594,16 @@
         <x:v>D4 大洋路</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Apollo Bay café</x:v>
+        <x:v>Apollo Bay café / 镇中心补给</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>轻食 / picnic</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Apollo Bay 主采购食材 → 抵达 Southern Ocean Villas 后看天气和时间：可去附近 public electric BBQ；不行就 villa 厨房自炊</x:v>
+        <x:v>Port Campbell 18:00–18:30</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
+        <x:v>早上在 Apollo Bay 买好水和轻食；晚餐首选 Port Campbell Hotel，备选 12 Rocks / REAL Pizza / Sow &amp; Piglets。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>

<commit_message>
update D5 Port Campbell return route
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R9e1190e64c734ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Re3405e473edb4873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R075fecd285a941cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R90befce99880404c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rccf875f4ea7443a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R17a534f1032d4db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R0f514ac1b7ba431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R20afad91d096442c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R2eab2ccd79a44fef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R00f25b10372e4bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Ra7287dbd9d7641b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rc4de295262394320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R005fab262b674af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R00385372e1674ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R2fa09837b4e0450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R5500f194334c4118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R89562c77ca9b4a9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Rd442702503344d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R4b83c1c01f534b3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R8f38fb855c9b4166"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -981,19 +981,19 @@
         <x:v>144.841</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>海岸地貌到野生动物：大洋路返程日</x:v>
+        <x:v>晨光中的海岸：十二使徒岩、Loch Ard Gorge 与野生动物</x:v>
       </x:c>
       <x:c r="I7" t="str">
-        <x:v>清晨补看海岸，再经 The Grotto、London Arch 与 Great Ocean Road Wildlife Park 走内陆线返回机场。</x:v>
+        <x:v>清晨沿十二使徒岩、Gibson Steps 与 Loch Ard Gorge 追着晨光看海岸，回别墅早餐退房后去 Wildlife Park，午后经 Colac 返回墨尔本机场。</x:v>
       </x:c>
       <x:c r="J7" t="str">
         <x:v>Holiday Inn Melbourne Airport</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>早晨海边冷，回程时间长。</x:v>
+        <x:v>清晨海岸寒冷多风，午后内陆相对温和；沿途天气变化快。</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>早上防风保暖，下午回机场前预留加油和还车时间。</x:v>
+        <x:v>清晨穿轻薄羽绒和防风外套，帽子、手套随身；动物园穿防滑包脚鞋。</x:v>
       </x:c>
       <x:c r="M7" t="str">
         <x:v>/itinerary/d5-port-campbell-morning.png</x:v>
@@ -1002,16 +1002,16 @@
         <x:v>Port Campbell 清晨海岸</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>自驾 · 内陆回墨尔本机场</x:v>
+        <x:v>自驾 · 清晨海岸环线 + 内陆返回墨尔本机场</x:v>
       </x:c>
       <x:c r="P7" t="str">
-        <x:v>07:00 前退房；11:45 前离开 Wildlife Park，17:00 前还车</x:v>
+        <x:v>06:45 离开别墅看晨光；10:30 前退房；13:30–14:30 经 Colac 开始返程</x:v>
       </x:c>
       <x:c r="Q7" t="str">
         <x:v>holiday-inn-airport-map</x:v>
       </x:c>
       <x:c r="R7" t="str">
-        <x:v>great-ocean-road-wildlife-park-map</x:v>
+        <x:v>d5-sunrise-route-map</x:v>
       </x:c>
       <x:c r="S7" t="str">
         <x:v>great-ocean-road-wildlife-park-booking</x:v>
@@ -3222,22 +3222,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>07:00-07:30</x:v>
+        <x:v>06:30–06:45</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Port Campbell</x:v>
+        <x:v>Southern Ocean Villas</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>退房、装车并简单早餐</x:v>
+        <x:v>换好防风保暖层，带上随身小包，06:45 驾车出发</x:v>
       </x:c>
       <x:c r="F53" t="str">
-        <x:v>小镇清晨 + 返程准备</x:v>
+        <x:v>天亮前驶向十二使徒岩</x:v>
       </x:c>
       <x:c r="G53" t="str">
-        <x:v>把行李装车、早餐和退房一次完成；07:30 左右驶离住宿。</x:v>
+        <x:v>清晨只带手机、相机和保温杯；出门前先设置好第一段导航。</x:v>
       </x:c>
       <x:c r="H53" t="str">
-        <x:v>port-campbell-map</x:v>
+        <x:v>southern-ocean-villas-map,d5-sunrise-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3248,22 +3248,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>天气补拍备选 · 07:30-08:10</x:v>
+        <x:v>07:05–07:45</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
+        <x:v>Twelve Apostles</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>若前一日受天气影响，在两处中只选一处清晨补拍；若已看够则直接前往 The Grotto</x:v>
+        <x:v>沿主观景台看晨光落在海蚀柱与海岸线上</x:v>
       </x:c>
       <x:c r="F54" t="str">
-        <x:v>柔和晨光 + 较少游客</x:v>
+        <x:v>07:29 左右日出 + 清晨人少</x:v>
       </x:c>
       <x:c r="G54" t="str">
-        <x:v>只选一处，08:10 最晚离开；这段是天气补拍，不影响 10:00 后进入 Wildlife Park。</x:v>
+        <x:v>07:05–07:15 抵达较从容；风口体感冷，拍完后直接前往 Gibson Steps。</x:v>
       </x:c>
       <x:c r="H54" t="str">
-        <x:v>twelve-apostles-map,loch-ard-map</x:v>
+        <x:v>twelve-apostles-map,d5-sunrise-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3274,22 +3274,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>08:35 左右</x:v>
+        <x:v>07:50–08:10</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>The Grotto</x:v>
+        <x:v>Gibson Steps</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>看海蚀洞和海水窗口</x:v>
+        <x:v>从上方观景台看悬崖与 Gog and Magog；开放且海况安全时再下台阶</x:v>
       </x:c>
       <x:c r="F55" t="str">
-        <x:v>洞穴 + 海景构图</x:v>
+        <x:v>海平面视角下的巨大尺度</x:v>
       </x:c>
       <x:c r="G55" t="str">
-        <x:v>台阶上下，雨后注意湿滑；停留 20–30 分钟即可</x:v>
+        <x:v>海滩入口会受潮位与海浪影响，以现场标识为准；关闭时在上方短停即可。</x:v>
       </x:c>
       <x:c r="H55" t="str">
-        <x:v>grotto-map</x:v>
+        <x:v>gibson-steps-map,d5-sunrise-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3300,22 +3300,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>09:10 左右</x:v>
+        <x:v>08:20–08:40</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>London Bridge / London Arch</x:v>
+        <x:v>Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>看海蚀拱门</x:v>
+        <x:v>沿上方步道看峡谷、海湾与沉船海岸</x:v>
       </x:c>
       <x:c r="F56" t="str">
-        <x:v>Port Campbell 以西经典点</x:v>
+        <x:v>晨光中的峡谷轮廓</x:v>
       </x:c>
       <x:c r="G56" t="str">
-        <x:v>顺路短停，很适合加</x:v>
+        <x:v>海滩入口台阶目前因地质不稳定关闭；留在上方开放步道和观景台。</x:v>
       </x:c>
       <x:c r="H56" t="str">
-        <x:v>london-arch-map,port-campbell-map</x:v>
+        <x:v>loch-ard-map,loch-ard-official,d5-sunrise-route-map,d5-west-coast-loop-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3326,22 +3326,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>10:15-11:30</x:v>
+        <x:v>08:40–08:50</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Great Ocean Road Wildlife Park</x:v>
+        <x:v>Tom and Eva Lookout</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>购买普通门票进入互动区和 sanctuary，近距离看袋鼠、沙袋鼠等澳洲本土动物；游园和可选购饲料喂食合计预留 60-75 分钟</x:v>
+        <x:v>步行到观景台看两座海蚀柱与外海</x:v>
       </x:c>
       <x:c r="F57" t="str">
-        <x:v>大洋路沿线的澳洲本土动物互动体验</x:v>
+        <x:v>Loch Ard 沉船故事中的幸存者之名</x:v>
       </x:c>
       <x:c r="G57" t="str">
-        <x:v>普通门票建议提前在线购买；动物饲料和 close-up encounters 另付费。步道多为未铺装地面，穿防滑包脚鞋；11:45 前离园，为 Colac 午餐、加油和机场还车保留缓冲。</x:v>
+        <x:v>与 Loch Ard Gorge 在同一景区内，沿开放步道顺路完成。</x:v>
       </x:c>
       <x:c r="H57" t="str">
-        <x:v>great-ocean-road-wildlife-park-map,great-ocean-road-wildlife-park-official,great-ocean-road-wildlife-park-booking</x:v>
+        <x:v>tom-eva-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3352,22 +3352,22 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>下午</x:v>
+        <x:v>08:50–09:00</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Colac</x:v>
+        <x:v>The Razorback Lookout</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>午餐、加油、休息</x:v>
+        <x:v>看狭长岩脊、层理与南大洋海浪</x:v>
       </x:c>
       <x:c r="F58" t="str">
-        <x:v>内陆牧场风光</x:v>
+        <x:v>最有雕塑感的海蚀地貌</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>回程中段休息点</x:v>
+        <x:v>继续沿 Loch Ard Gorge 景区步道前往，不需要重新驾车找入口。</x:v>
       </x:c>
       <x:c r="H58" t="str">
-        <x:v>colac-map</x:v>
+        <x:v>razorback-map,loch-ard-map</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3378,22 +3378,22 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>09:15–09:25</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>London Arch</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>抵达机场、还车、取回寄存大件行李</x:v>
+        <x:v>在观景台看断开的海蚀拱门与开阔海面</x:v>
       </x:c>
       <x:c r="F59" t="str">
-        <x:v>大洋路自驾收尾</x:v>
+        <x:v>曾被称为 London Bridge 的经典地貌</x:v>
       </x:c>
       <x:c r="G59" t="str">
-        <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
+        <x:v>停留约 10 分钟，随后继续前往 The Grotto。</x:v>
       </x:c>
       <x:c r="H59" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>london-arch-map,d5-west-coast-loop-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -3404,22 +3404,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>晚上</x:v>
+        <x:v>09:30–09:40</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Holiday Inn Melbourne Airport</x:v>
+        <x:v>The Grotto</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>入住、整理行李</x:v>
+        <x:v>走下观景步道，看海蚀洞框住海面</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>为次日早班机准备</x:v>
+        <x:v>洞穴、岩池与海景同框</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>厚衣服收好，准备凯恩斯热带段；早睡</x:v>
+        <x:v>台阶雨后可能湿滑；拍完即返回别墅吃早餐。</x:v>
       </x:c>
       <x:c r="H60" t="str">
-        <x:v>mel-airport-map,holiday-inn-airport-map</x:v>
+        <x:v>grotto-map,d5-west-coast-loop-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -3427,127 +3427,129 @@
         <x:v>d5</x:v>
       </x:c>
       <x:c r="B61" t="n">
-        <x:v>900</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>饮食</x:v>
+        <x:v>09:55–10:30</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Southern Ocean Villas</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>早餐：Port Campbell café；午餐：离开 Great Ocean Road Wildlife Park 后在 Colac 简餐；晚餐：机场酒店简餐</x:v>
+        <x:v>回到别墅吃早餐、洗漱、整理行李并退房</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>野生动物体验 + 内陆返程补给</x:v>
+        <x:v>清晨海岸环线后的休整</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>Colac 作为返程主休息点，把午餐、加油和休息一次完成；抵达机场后简单用餐并整理行李。</x:v>
+        <x:v>前一晚把退房物品集中好；具体退房时间以订单或前台确认信息为准。</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>great-ocean-road-wildlife-park-map,colac-map,holiday-inn-airport-map</x:v>
+        <x:v>southern-ocean-villas-map,d5-west-coast-loop-route-map,d5-return-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B62" t="n">
-        <x:v>10</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>上午</x:v>
+        <x:v>10:50–12:20</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>Great Ocean Road Wildlife Park</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>飞往凯恩斯</x:v>
+        <x:v>在互动区近距离观察袋鼠和沙袋鼠，再沿 sanctuary 步道寻找考拉、袋熊与澳洲野犬</x:v>
       </x:c>
       <x:c r="F62" t="str">
-        <x:v>气候切换非常明显</x:v>
+        <x:v>大洋路沿线的本土动物体验</x:v>
       </x:c>
       <x:c r="G62" t="str">
-        <x:v>国内航班建议预留行李额</x:v>
+        <x:v>园区 10:00–17:00，通常 45–60 分钟可走完；这里留 75–90 分钟，动物饲料和 close-up encounters 另付费。</x:v>
       </x:c>
       <x:c r="H62" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>great-ocean-road-wildlife-park-map,great-ocean-road-wildlife-park-official,great-ocean-road-wildlife-park-booking,d5-return-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B63" t="n">
-        <x:v>20</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>中午</x:v>
+        <x:v>13:40–14:25 预计</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>Colac</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>打车 / Uber 到酒店</x:v>
+        <x:v>午餐、加油和短休，把返程补给一次完成</x:v>
       </x:c>
       <x:c r="F63" t="str">
-        <x:v>不租车，降低疲劳</x:v>
+        <x:v>内陆回程的中段休息站</x:v>
       </x:c>
       <x:c r="G63" t="str">
-        <x:v>酒店可先寄存行李</x:v>
-      </x:c>
-      <x:c r="H63"/>
+        <x:v>14:00–14:30 左右重新上路，最后一段直达墨尔本机场区域。</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>colac-map,d5-return-route-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B64" t="n">
-        <x:v>30</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>下午</x:v>
+        <x:v>16:15–17:00 预计</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Esplanade Lagoon</x:v>
+        <x:v>Holiday Inn Melbourne Airport</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>免费泻湖泳池、海滨散步</x:v>
+        <x:v>取回寄存的 4 个大箱，按租车指引完成还车，再办理入住</x:v>
       </x:c>
       <x:c r="F64" t="str">
-        <x:v>度假感拉满</x:v>
+        <x:v>大洋路自驾顺利收尾</x:v>
       </x:c>
       <x:c r="G64" t="str">
-        <x:v>泳衣可提前放随身包</x:v>
+        <x:v>进入机场区域前检查油量、车内物品和还车入口；晚上只做简单用餐和行李整理。</x:v>
       </x:c>
       <x:c r="H64" t="str">
-        <x:v>cairns-lagoon-map</x:v>
+        <x:v>holiday-inn-airport-map,mel-airport-car-rental-map,d5-return-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" t="str">
-        <x:v>d6</x:v>
+        <x:v>d5</x:v>
       </x:c>
       <x:c r="B65" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>晚上</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Cairns Night Markets</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>夜市、简餐、纪念品</x:v>
+        <x:v>早餐：回 Southern Ocean Villas 后用餐；午餐：Wildlife Park 轻食或 Colac 简餐；晚餐：机场酒店简餐</x:v>
       </x:c>
       <x:c r="F65" t="str">
-        <x:v>热闹轻松</x:v>
+        <x:v>清晨看景、午后返程的轻量餐食</x:v>
       </x:c>
       <x:c r="G65" t="str">
-        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+        <x:v>早餐食材前一晚整理好；Colac 可把午餐、加油和休息一次完成。</x:v>
       </x:c>
       <x:c r="H65" t="str">
-        <x:v>cairns-night-market-map</x:v>
+        <x:v>southern-ocean-villas-map,great-ocean-road-wildlife-park-map,colac-map,holiday-inn-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3555,153 +3557,151 @@
         <x:v>d6</x:v>
       </x:c>
       <x:c r="B66" t="n">
-        <x:v>900</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>饮食</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>墨尔本机场</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
+        <x:v>飞往凯恩斯</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>气候切换非常明显</x:v>
       </x:c>
       <x:c r="G66" t="str">
-        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
-      </x:c>
-      <x:c r="H66"/>
+        <x:v>国内航班建议预留行李额</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B67" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>早上</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>凯恩斯码头</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Reef Magic check-in，登船出海</x:v>
+        <x:v>打车 / Uber 到酒店</x:v>
       </x:c>
       <x:c r="F67" t="str">
-        <x:v>前往外礁平台</x:v>
+        <x:v>不租车，降低疲劳</x:v>
       </x:c>
       <x:c r="G67" t="str">
-        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
-      </x:c>
-      <x:c r="H67" t="str">
-        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
-      </x:c>
+        <x:v>酒店可先寄存行李</x:v>
+      </x:c>
+      <x:c r="H67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B68" t="n">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>全天</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Outer Reef Pontoon</x:v>
+        <x:v>Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
+        <x:v>免费泻湖泳池、海滨散步</x:v>
       </x:c>
       <x:c r="F68" t="str">
-        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
+        <x:v>度假感拉满</x:v>
       </x:c>
       <x:c r="G68" t="str">
-        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
+        <x:v>泳衣可提前放随身包</x:v>
       </x:c>
       <x:c r="H68" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>cairns-lagoon-map</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B69" t="n">
-        <x:v>30</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>中午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>船上 / 平台</x:v>
+        <x:v>Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>外礁平台午餐</x:v>
+        <x:v>夜市、简餐、纪念品</x:v>
       </x:c>
       <x:c r="F69" t="str">
-        <x:v>轻松补给</x:v>
+        <x:v>热闹轻松</x:v>
       </x:c>
       <x:c r="G69" t="str">
-        <x:v>不要吃太撑，避免晕船</x:v>
+        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
       </x:c>
       <x:c r="H69" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>cairns-night-market-map</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" t="str">
-        <x:v>d7</x:v>
+        <x:v>d6</x:v>
       </x:c>
       <x:c r="B70" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>下午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>下船休息</x:v>
+        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>通常会比较疲惫</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G70" t="str">
-        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
-      </x:c>
-      <x:c r="H70" t="str">
-        <x:v>reef-fleet-terminal-map</x:v>
-      </x:c>
+        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
+      </x:c>
+      <x:c r="H70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="str">
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B71" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>晚上</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>码头附近</x:v>
+        <x:v>凯恩斯码头</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
+        <x:v>Reef Magic check-in，登船出海</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>海边晚餐</x:v>
+        <x:v>前往外礁平台</x:v>
       </x:c>
       <x:c r="G71" t="str">
-        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
+        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
       </x:c>
       <x:c r="H71" t="str">
-        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
+        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3709,22 +3709,22 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B72" t="n">
-        <x:v>80</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>提醒</x:v>
+        <x:v>全天</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>今日提醒</x:v>
+        <x:v>Outer Reef Pontoon</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
+        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
       </x:c>
       <x:c r="F72" t="str">
-        <x:v>舒适与安全比拍摄数量更重要</x:v>
+        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
       </x:c>
       <x:c r="H72" t="str">
         <x:v>reef-magic-official</x:v>
@@ -3735,125 +3735,129 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B73" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>船上 / 平台</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
+        <x:v>外礁平台午餐</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>轻松补给</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+        <x:v>不要吃太撑，避免晕船</x:v>
       </x:c>
       <x:c r="H73" t="str">
-        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B74" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>清晨</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
+        <x:v>下船休息</x:v>
       </x:c>
       <x:c r="F74" t="str">
-        <x:v>不用自驾，沿途可休息看风景</x:v>
+        <x:v>通常会比较疲惫</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
-      </x:c>
-      <x:c r="H74"/>
+        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>reef-fleet-terminal-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B75" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>上午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Daintree River / Rainforest</x:v>
+        <x:v>码头附近</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>鳄鱼游船、雨林步道</x:v>
+        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
+        <x:v>海边晚餐</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
       </x:c>
       <x:c r="H75" t="str">
-        <x:v>daintree-river-map</x:v>
+        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B76" t="n">
-        <x:v>30</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>中午</x:v>
+        <x:v>提醒</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Daintree Rainforest</x:v>
+        <x:v>今日提醒</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>团含午餐</x:v>
+        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
       </x:c>
       <x:c r="F76" t="str">
-        <x:v>不用自己找餐厅</x:v>
+        <x:v>舒适与安全比拍摄数量更重要</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>如有忌口提前告知</x:v>
-      </x:c>
-      <x:c r="H76"/>
+        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>reef-magic-official</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" t="str">
-        <x:v>d8</x:v>
+        <x:v>d7</x:v>
       </x:c>
       <x:c r="B77" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>下午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Cape Tribulation</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>雨林入海、海滩短停留</x:v>
+        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="F77" t="str">
-        <x:v>雨林与海洋在这里交会</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
+        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
       </x:c>
       <x:c r="H77" t="str">
-        <x:v>cape-trib-map</x:v>
+        <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -3861,179 +3865,175 @@
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B78" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Daintree Ferry / Ice Cream</x:v>
+        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>渡河、热带水果冰淇淋</x:v>
+        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>丹翠地区很有代表性的热带味道</x:v>
+        <x:v>不用自驾，沿途可休息看风景</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
-      </x:c>
-      <x:c r="H78" t="str">
-        <x:v>daintree-icecream-map</x:v>
-      </x:c>
+        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
+      </x:c>
+      <x:c r="H78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B79" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Daintree River / Rainforest</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>18:30 后回到市区</x:v>
+        <x:v>鳄鱼游船、雨林步道</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>回程可休息</x:v>
+        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
-      </x:c>
-      <x:c r="H79"/>
+        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>daintree-river-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="str">
         <x:v>d8</x:v>
       </x:c>
       <x:c r="B80" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Daintree Rainforest</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>团含午餐</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>不用自己找餐厅</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
-      </x:c>
-      <x:c r="H80" t="str">
-        <x:v>daintree-icecream-map</x:v>
-      </x:c>
+        <x:v>如有忌口提前告知</x:v>
+      </x:c>
+      <x:c r="H80"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B81" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>早上</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>凯恩斯 → Lake Eacham</x:v>
+        <x:v>Cape Tribulation</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
+        <x:v>雨林入海、海滩短停留</x:v>
       </x:c>
       <x:c r="F81" t="str">
-        <x:v>从热带海边城市进入清凉高原</x:v>
+        <x:v>雨林与海洋在这里交会</x:v>
       </x:c>
       <x:c r="G81" t="str">
-        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
+        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
       </x:c>
       <x:c r="H81" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>cape-trib-map</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B82" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Lake Eacham</x:v>
+        <x:v>Daintree Ferry / Ice Cream</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>火山湖散步、看湖景</x:v>
+        <x:v>渡河、热带水果冰淇淋</x:v>
       </x:c>
       <x:c r="F82" t="str">
-        <x:v>安静、清凉、湖水和雨林包围感</x:v>
+        <x:v>丹翠地区很有代表性的热带味道</x:v>
       </x:c>
       <x:c r="G82" t="str">
-        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
       </x:c>
       <x:c r="H82" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>daintree-icecream-map</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B83" t="n">
-        <x:v>30</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Curtain Fig Tree</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>看巨型帘状无花果树</x:v>
+        <x:v>18:30 后回到市区</x:v>
       </x:c>
       <x:c r="F83" t="str">
-        <x:v>像热带森林里的巨大自然装置</x:v>
+        <x:v>回程可休息</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>停留 20–30 分钟即可</x:v>
-      </x:c>
-      <x:c r="H83" t="str">
-        <x:v>curtain-fig-map</x:v>
-      </x:c>
+        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
+      </x:c>
+      <x:c r="H83"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" t="str">
-        <x:v>d9</x:v>
+        <x:v>d8</x:v>
       </x:c>
       <x:c r="B84" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>中午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Yungaburra / Gallo Dairyland</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
+        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F84" t="str">
-        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G84" t="str">
-        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
+        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
       </x:c>
       <x:c r="H84" t="str">
-        <x:v>yungaburra-map,gallo-map</x:v>
+        <x:v>daintree-icecream-map</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -4041,25 +4041,25 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B85" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>下午</x:v>
+        <x:v>早上</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
+        <x:v>凯恩斯 → Lake Eacham</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>瀑布短停留、拍照</x:v>
+        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>雨林瀑布与高原绿意</x:v>
+        <x:v>从热带海边城市进入清凉高原</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
       </x:c>
       <x:c r="H85" t="str">
-        <x:v>millaa-map,ellinjaa-map</x:v>
+        <x:v>lake-eacham-map</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -4067,175 +4067,177 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B86" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Lake Eacham</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>下山回市区，还车或次日早还</x:v>
+        <x:v>火山湖散步、看湖景</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>完成高原自然线</x:v>
+        <x:v>安静、清凉、湖水和雨林包围感</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
-      </x:c>
-      <x:c r="H86"/>
+        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>lake-eacham-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="str">
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B87" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>简单晚餐</x:v>
+        <x:v>看巨型帘状无花果树</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>回城后轻松晚餐</x:v>
+        <x:v>像热带森林里的巨大自然装置</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>下山后就近用餐，早点休息。</x:v>
-      </x:c>
-      <x:c r="H87"/>
+        <x:v>停留 20–30 分钟即可</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>curtain-fig-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="str">
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B88" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Yungaburra / Gallo Dairyland</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
+        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>millaa-map,gallo-map</x:v>
+        <x:v>yungaburra-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B89" t="n">
-        <x:v>10</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>瀑布短停留、拍照</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>周五正好开市，适合补水果和轻食</x:v>
+        <x:v>雨林瀑布与高原绿意</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
+        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
       </x:c>
       <x:c r="H89" t="str">
-        <x:v>rustys-map</x:v>
+        <x:v>millaa-map,ellinjaa-map</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B90" t="n">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>中午</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>返回凯恩斯</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>下山回市区，还车或次日早还</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>热带城市躺平感</x:v>
+        <x:v>完成高原自然线</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
-      </x:c>
-      <x:c r="H90" t="str">
-        <x:v>cairns-lagoon-map</x:v>
-      </x:c>
+        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
+      </x:c>
+      <x:c r="H90"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B91" t="n">
-        <x:v>30</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>下午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>简单晚餐</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>为次日清晨航班做准备</x:v>
+        <x:v>回城后轻松晚餐</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
+        <x:v>下山后就近用餐，早点休息。</x:v>
       </x:c>
       <x:c r="H91"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B92" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>下午 / 傍晚</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Palm Cove</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
+        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
+        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>palm-cove-map</x:v>
+        <x:v>millaa-map,gallo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -4243,25 +4245,25 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B93" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>海鲜或轻松简餐</x:v>
+        <x:v>周五正好开市，适合补水果和轻食</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>早点吃，早点睡</x:v>
+        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
+        <x:v>rustys-map</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4269,127 +4271,127 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B94" t="n">
-        <x:v>900</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>饮食</x:v>
+        <x:v>中午</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
+        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>热带城市躺平感</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
+        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>rustys-map,prawn-star-map</x:v>
+        <x:v>cairns-lagoon-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B95" t="n">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>清晨</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>为次日清晨航班做准备</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
-      </x:c>
-      <x:c r="H95" t="str">
-        <x:v>cairns-airport-map</x:v>
-      </x:c>
+        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
+      </x:c>
+      <x:c r="H95"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B96" t="n">
-        <x:v>20</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>上午</x:v>
+        <x:v>下午 / 傍晚</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>凯恩斯 → 悉尼</x:v>
+        <x:v>Palm Cove</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H96"/>
+        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>palm-cove-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>海鲜或轻松简餐</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
+        <x:v>早点吃，早点睡</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>oaks-sydney-map</x:v>
+        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B98" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>下午</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>rustys-map,prawn-star-map</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4397,25 +4399,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B99" t="n">
-        <x:v>45</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F99" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G99" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>cairns-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4423,51 +4425,49 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B100" t="n">
-        <x:v>50</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F100" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>从热带切换回冬季海港城市</x:v>
       </x:c>
       <x:c r="G100" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
-      </x:c>
-      <x:c r="H100" t="str">
-        <x:v>the-rocks-map</x:v>
-      </x:c>
+        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
+      </x:c>
+      <x:c r="H100"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B101" t="n">
-        <x:v>60</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>悉尼 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F101" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>4人 + 行李，打车最省心</x:v>
       </x:c>
       <x:c r="G101" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
+        <x:v>如不能入住，先寄存行李</x:v>
       </x:c>
       <x:c r="H101" t="str">
-        <x:v>circular-quay-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -4475,129 +4475,129 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B102" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>饮食</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Darling Harbour / 酒店周边</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F102" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B103" t="n">
-        <x:v>10</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
       </x:c>
       <x:c r="F103" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G103" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H103" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B104" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F104" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H104" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B105" t="n">
-        <x:v>30</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>歌剧院、海港大桥夜景</x:v>
       </x:c>
       <x:c r="F105" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H105" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B106" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
+        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H106" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -4605,25 +4605,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B107" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>08:15–08:30</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
+        <x:v>抵达海港区</x:v>
       </x:c>
       <x:c r="F107" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
+        <x:v>Ferry、海港桥、歌剧院远景</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
+        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
       </x:c>
       <x:c r="H107" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -4631,25 +4631,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B108" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>08:30–09:10</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F108" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>悉尼核心地标</x:v>
       </x:c>
       <x:c r="G108" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
       </x:c>
       <x:c r="H108" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -4657,25 +4657,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B109" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Royal Botanic Garden</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>中文内部导览已订</x:v>
       </x:c>
       <x:c r="F109" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>建筑故事、内部空间、剧院结构</x:v>
       </x:c>
       <x:c r="G109" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
       </x:c>
       <x:c r="H109" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -4683,25 +4683,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B110" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>10:30–10:50</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Opera House → The Rocks</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>海港步行衔接悉尼老城区</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -4709,25 +4709,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B111" t="n">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>10:50–11:50</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
       </x:c>
       <x:c r="H111" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -4735,25 +4735,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B112" t="n">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>晚上</x:v>
+        <x:v>11:50–12:40</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>就地补体力，不为午餐绕路</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -4761,129 +4761,129 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B113" t="n">
-        <x:v>900</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>饮食</x:v>
+        <x:v>12:40–14:10</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>植物园海港步道</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>botanic-garden-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>10</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>08:00</x:v>
+        <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>歌剧院 + 海港大桥同框</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>悉尼最经典机位</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>mrs-macquarie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>20</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>09:15</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>购物、室内休息</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>建筑漂亮，适合逛</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>30</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>10:00</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>CBD / Darling Harbour</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>Hello Auntie / CBD 晚餐</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>11:15</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -4891,25 +4891,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>12:00</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>royal-national-park-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -4917,25 +4917,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>09:15</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>南海岸第一处全景</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>bald-hill-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -4943,25 +4943,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>13:30</x:v>
+        <x:v>10:00</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>贴着太平洋的公路画面</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>不要在桥上或路肩危险停车</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -4969,25 +4969,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Wollongong / 南海岸补给</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>短停咖啡或直接通过</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>wollongong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -4995,25 +4995,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>14:40</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Kiama Blowhole</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>看喷潮洞、灯塔与海边</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>Kiama 代表性海岸地貌</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -5021,25 +5021,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>12:30–13:30</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>海边小镇节奏</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -5047,25 +5047,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>110</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>13:30</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Kiama → Gerringong</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>沿海继续南下</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kiama-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -5073,129 +5073,129 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>饮食</x:v>
+        <x:v>13:45–14:40</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>10</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>14:40</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Gerringong</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>判断是否延伸 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>时间、天气与体力闸门</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>gerringong-map,kangaroo-valley-map</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>20</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>可选 15:30–16:15</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>看历史桥、山谷与小镇</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>16:15 前</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>环线收束</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -5203,25 +5203,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>08:30–09:00</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -5229,25 +5229,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>18:30</x:v>
+        <x:v>09:15 左右</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -5255,129 +5255,129 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>饮食</x:v>
+        <x:v>09:30–13:30</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>上午</x:v>
+        <x:v>13:30–14:30</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>F2 返回市区后前往 Bondi</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>动物园切换到悉尼海岸</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>14:30–17:45</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>海滩散步并走一段 Coastal Walk</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>30</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>18:30</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B136" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -5385,25 +5385,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B137" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D137" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F137" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>oaks-sydney-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -5411,25 +5411,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B138" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>可选 09:30 左右</x:v>
       </x:c>
       <x:c r="D138" t="str">
-        <x:v>酒店</x:v>
+        <x:v>Circular Quay → Manly</x:v>
       </x:c>
       <x:c r="E138" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>搭乘公共 F1 Manly Ferry</x:v>
       </x:c>
       <x:c r="F138" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G138" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H138" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>circular-quay-map,manly-ferry-map</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -5437,25 +5437,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B139" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>16:40</x:v>
+        <x:v>可选 10:00–12:45</x:v>
       </x:c>
       <x:c r="D139" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Manly Beach / The Corso</x:v>
       </x:c>
       <x:c r="E139" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>海边散步、咖啡或早午餐</x:v>
       </x:c>
       <x:c r="F139" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G139" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H139" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -5463,25 +5463,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B140" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C140" t="str">
-        <x:v>17:30</x:v>
+        <x:v>13:00–13:30</x:v>
       </x:c>
       <x:c r="D140" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>Manly → Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E140" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>最晚搭船回市区</x:v>
       </x:c>
       <x:c r="F140" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G140" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H140" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -5489,76 +5489,180 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B141" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C141" t="str">
-        <x:v>饮食</x:v>
+        <x:v>14:00–15:30</x:v>
       </x:c>
       <x:c r="D141" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
       </x:c>
       <x:c r="E141" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>最后采购</x:v>
       </x:c>
       <x:c r="F141" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>药妆、保健品、伴手礼</x:v>
       </x:c>
       <x:c r="G141" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
       </x:c>
       <x:c r="H141" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" t="str">
-        <x:v>d16</x:v>
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B142" t="n">
-        <x:v>10</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C142" t="str">
-        <x:v>上午</x:v>
+        <x:v>15:30–16:20</x:v>
       </x:c>
       <x:c r="D142" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>酒店</x:v>
       </x:c>
       <x:c r="E142" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>整理 TRS 物品和返程行李</x:v>
       </x:c>
       <x:c r="F142" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>为 D16 机场退税做准备</x:v>
       </x:c>
       <x:c r="G142" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
       </x:c>
       <x:c r="H142" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>oaks-sydney-map,trs-official</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B143" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>16:40</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>前往 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>避免迟到</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+      </x:c>
+      <x:c r="H143" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B144" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>17:30</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>海港景观 + 澳洲最后一晚</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B145" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>当天餐食节奏</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+      </x:c>
+      <x:c r="H145" t="str">
+        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
         <x:v>d16</x:v>
       </x:c>
-      <x:c r="B143" t="n">
+      <x:c r="B146" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G146" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H146" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B147" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C143" t="str">
+      <x:c r="C147" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D143" t="str">
+      <x:c r="D147" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E143" t="str">
+      <x:c r="E147" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F143" t="str">
+      <x:c r="F147" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G143" t="str">
+      <x:c r="G147" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H143"/>
+      <x:c r="H147"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7039,8 +7143,8 @@
       <x:c r="D77" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=12+Rocks+Beach+Cafe+%26+Bar+Port+Campbell+VIC</x:v>
       </x:c>
-      <x:c r="E77" t="str"/>
-      <x:c r="F77" t="str"/>
+      <x:c r="E77"/>
+      <x:c r="F77"/>
       <x:c r="G77" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8354,8 +8458,8 @@
       <x:c r="D146" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Seaview+Motel+%26+Apartments%2C+Apollo+Bay+VIC&amp;destination=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;travelmode=driving&amp;waypoints=FoodWorks+Apollo+Bay+VIC%7CMaits+Rest+Rainforest+Walk+VIC%7CThe+Redwoods+Otways%2C+Beech+Forest+VIC%7CCastle+Cove+Lookout+VIC%7CGibson+Steps+VIC%7CTwelve+Apostles+VIC%7CLoch+Ard+Gorge+VIC%7CPort+Campbell+Foreshore+VIC</x:v>
       </x:c>
-      <x:c r="E146" t="str"/>
-      <x:c r="F146" t="str"/>
+      <x:c r="E146"/>
+      <x:c r="F146"/>
       <x:c r="G146" t="str">
         <x:v>Google Maps · Apollo Bay 至 Port Campbell</x:v>
       </x:c>
@@ -8373,8 +8477,8 @@
       <x:c r="D147" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Seaview+Motel+%26+Apartments%2C+Apollo+Bay+VIC&amp;destination=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;travelmode=driving&amp;waypoints=FoodWorks+Apollo+Bay+VIC%7CMaits+Rest+Rainforest+Walk+VIC%7CCastle+Cove+Lookout+VIC%7CGibson+Steps+VIC%7CTwelve+Apostles+VIC%7CLoch+Ard+Gorge+VIC%7CPort+Campbell+Foreshore+VIC</x:v>
       </x:c>
-      <x:c r="E147" t="str"/>
-      <x:c r="F147" t="str"/>
+      <x:c r="E147"/>
+      <x:c r="F147"/>
       <x:c r="G147" t="str">
         <x:v>Google Maps · 09:15 后离开 Apollo Bay 时使用</x:v>
       </x:c>
@@ -8392,8 +8496,8 @@
       <x:c r="D148" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=FoodWorks+Apollo+Bay+VIC</x:v>
       </x:c>
-      <x:c r="E148" t="str"/>
-      <x:c r="F148" t="str"/>
+      <x:c r="E148"/>
+      <x:c r="F148"/>
       <x:c r="G148" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8411,8 +8515,8 @@
       <x:c r="D149" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Apollo+Bay+IGA+VIC</x:v>
       </x:c>
-      <x:c r="E149" t="str"/>
-      <x:c r="F149" t="str"/>
+      <x:c r="E149"/>
+      <x:c r="F149"/>
       <x:c r="G149" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8430,8 +8534,8 @@
       <x:c r="D150" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Castle+Cove+Lookout+VIC</x:v>
       </x:c>
-      <x:c r="E150" t="str"/>
-      <x:c r="F150" t="str"/>
+      <x:c r="E150"/>
+      <x:c r="F150"/>
       <x:c r="G150" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8449,8 +8553,8 @@
       <x:c r="D151" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Port+Campbell+Foreshore+VIC</x:v>
       </x:c>
-      <x:c r="E151" t="str"/>
-      <x:c r="F151" t="str"/>
+      <x:c r="E151"/>
+      <x:c r="F151"/>
       <x:c r="G151" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8468,8 +8572,8 @@
       <x:c r="D152" t="str">
         <x:v>https://www.parks.vic.gov.au/places-to-see/parks/port-campbell-national-park/things-to-do/loch-ard-gorge</x:v>
       </x:c>
-      <x:c r="E152" t="str"/>
-      <x:c r="F152" t="str"/>
+      <x:c r="E152"/>
+      <x:c r="F152"/>
       <x:c r="G152" t="str">
         <x:v>Parks Victoria · 行前查看开放与安全提示</x:v>
       </x:c>
@@ -8487,8 +8591,8 @@
       <x:c r="D153" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Port+Campbell+Hotel+VIC</x:v>
       </x:c>
-      <x:c r="E153" t="str"/>
-      <x:c r="F153" t="str"/>
+      <x:c r="E153"/>
+      <x:c r="F153"/>
       <x:c r="G153" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8506,8 +8610,8 @@
       <x:c r="D154" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=REAL+Pizza+Pasta+Salads+Port+Campbell+VIC</x:v>
       </x:c>
-      <x:c r="E154" t="str"/>
-      <x:c r="F154" t="str"/>
+      <x:c r="E154"/>
+      <x:c r="F154"/>
       <x:c r="G154" t="str">
         <x:v>Google Maps</x:v>
       </x:c>
@@ -8525,10 +8629,67 @@
       <x:c r="D155" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Sow+%26+Piglets+Brew+Pub+Port+Campbell+VIC</x:v>
       </x:c>
-      <x:c r="E155" t="str"/>
-      <x:c r="F155" t="str"/>
+      <x:c r="E155"/>
+      <x:c r="F155"/>
       <x:c r="G155" t="str">
         <x:v>Google Maps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>d5-sunrise-route-map</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>D5 晨光海岸路线</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;destination=Loch+Ard+Gorge%2C+VIC&amp;travelmode=driving&amp;waypoints=Twelve+Apostles%2C+VIC%7CGibson+Steps%2C+VIC</x:v>
+      </x:c>
+      <x:c r="E156" t="str"/>
+      <x:c r="F156" t="str"/>
+      <x:c r="G156" t="str">
+        <x:v>Google Maps · Southern Ocean Villas → Twelve Apostles → Gibson Steps → Loch Ard Gorge</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>d5-west-coast-loop-route-map</x:v>
+      </x:c>
+      <x:c r="B157" t="str">
+        <x:v>D5 西侧海岸环线</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D157" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Loch+Ard+Gorge%2C+VIC&amp;destination=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;travelmode=driving&amp;waypoints=London+Arch%2C+VIC%7CThe+Grotto%2C+Port+Campbell+VIC</x:v>
+      </x:c>
+      <x:c r="E157" t="str"/>
+      <x:c r="F157" t="str"/>
+      <x:c r="G157" t="str">
+        <x:v>Google Maps · Loch Ard Gorge → London Arch → The Grotto → Southern Ocean Villas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>d5-return-route-map</x:v>
+      </x:c>
+      <x:c r="B158" t="str">
+        <x:v>D5 Wildlife Park 与机场返程</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D158" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;destination=Holiday+Inn+Melbourne+Airport&amp;travelmode=driving&amp;waypoints=Great+Ocean+Road+Wildlife+Park%2C+Gellibrand+Lower+VIC%7CColac%2C+VIC</x:v>
+      </x:c>
+      <x:c r="E158" t="str"/>
+      <x:c r="F158" t="str"/>
+      <x:c r="G158" t="str">
+        <x:v>Google Maps · Southern Ocean Villas → Great Ocean Road Wildlife Park → Colac → Holiday Inn Melbourne Airport</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
update Cairns itinerary stage
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Ra7287dbd9d7641b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rc4de295262394320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R005fab262b674af5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R00385372e1674ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R2fa09837b4e0450e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R5500f194334c4118"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R89562c77ca9b4a9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Rd442702503344d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R4b83c1c01f534b3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R8f38fb855c9b4166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rbbdec6bcd99347dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R216794ce226a4c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rcccb1a42fdb54591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Rfe6719406d3c44b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R9166dea9e89e4a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R0688fcc6254e49f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R70c1f63ea10a4896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R49b094d638a04366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R1a67babebb054830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Rc4325b17e05e443c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1040,10 +1040,10 @@
         <x:v>145.7781</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>抵达凯恩斯：Esplanade Lagoon 与热带夜市</x:v>
+        <x:v>初到凯恩斯：热带花园、海滨与夜市</x:v>
       </x:c>
       <x:c r="I8" t="str">
-        <x:v>从墨尔本飞到凯恩斯，下午在 Esplanade Lagoon 放松，晚上逛夜市。</x:v>
+        <x:v>早班机抵达凯恩斯后先寄存行李与休息，午后视体力走进热带花园，再沿 Esplanade 到 Marina，晚上在 Night Markets 边逛边吃。</x:v>
       </x:c>
       <x:c r="J8" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -1061,16 +1061,16 @@
         <x:v>凯恩斯热带海岸</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>航班 / 机场转场</x:v>
+        <x:v>航班 + Uber / Taxi + 市区步行 / 短途交通</x:v>
       </x:c>
       <x:c r="P8" t="str">
-        <x:v>04:00 前从机场酒店步行或接驳至航站楼</x:v>
+        <x:v>04:45 离开 Holiday Inn 步行至航站楼；06:25 起飞，09:50 抵达凯恩斯</x:v>
       </x:c>
       <x:c r="Q8" t="str">
         <x:v>southern-cross-map</x:v>
       </x:c>
       <x:c r="R8" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>cairns-esplanade-boardwalk-map</x:v>
       </x:c>
       <x:c r="S8" t="str">
         <x:v>virgin-australia-official</x:v>
@@ -1102,7 +1102,7 @@
         <x:v>奔赴外礁：Reef Magic 大堡礁一日</x:v>
       </x:c>
       <x:c r="I9" t="str">
-        <x:v>在 Reef Magic 外礁平台体验浮潜、半潜艇与大堡礁海上风景。</x:v>
+        <x:v>在 Reef Magic 外礁平台体验浮潜、半潜艇与大堡礁海上风景，返港后到码头边吃一顿海鲜晚餐。</x:v>
       </x:c>
       <x:c r="J9" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -1123,7 +1123,7 @@
         <x:v>步行 / 打车至码头 + Reef Magic 游船</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>按船票集合时间，提前 45 分钟到 Reef Fleet Terminal</x:v>
+        <x:v>07:45–07:55 从酒店出发；08:15 开始登船，08:45 前完成登船</x:v>
       </x:c>
       <x:c r="Q9" t="str">
         <x:v>southern-cross-map</x:v>
@@ -1161,7 +1161,7 @@
         <x:v>深入丹翠：雨林、河流与 Cape Tribulation</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>沿丹翠河进入雨林，在 Cape Tribulation 看雨林与海相接。</x:v>
+        <x:v>清晨从酒店出发，沿丹翠河进入雨林，在 Cape Tribulation 看雨林与海相接，傍晚回城后简单用餐。</x:v>
       </x:c>
       <x:c r="J10" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -1182,7 +1182,7 @@
         <x:v>Billy Tea 小团接驳车</x:v>
       </x:c>
       <x:c r="P10" t="str">
-        <x:v>06:40 前到酒店门口，06:55 集合</x:v>
+        <x:v>06:45 到酒店门口等候；订单集合时间 06:55</x:v>
       </x:c>
       <x:c r="Q10" t="str">
         <x:v>southern-cross-map</x:v>
@@ -1220,7 +1220,7 @@
         <x:v>阿瑟顿高原：火山湖、巨树与瀑布</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>自驾串联 Lake Eacham、Curtain Fig Tree、高原小镇与瀑布。</x:v>
+        <x:v>从 Cairns 自驾上高原，串联 Lake Eacham、Curtain Fig Tree、Yungaburra、Gallo Dairyland 与 Millaa Millaa Falls，傍晚还车回城。</x:v>
       </x:c>
       <x:c r="J11" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -1241,13 +1241,13 @@
         <x:v>自驾 · 阿瑟顿高原</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>08:30 前取车出发</x:v>
+        <x:v>08:00–08:30 取车；08:30 启程上高原</x:v>
       </x:c>
       <x:c r="Q11" t="str">
         <x:v>southern-cross-map</x:v>
       </x:c>
       <x:c r="R11" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>d9-tablelands-route-map</x:v>
       </x:c>
       <x:c r="S11" t="str">
         <x:v>no-fixed-ticket</x:v>
@@ -1279,7 +1279,7 @@
         <x:v>慢享凯恩斯：Rusty's Market 与 Palm Cove</x:v>
       </x:c>
       <x:c r="I12" t="str">
-        <x:v>上午逛 Rusty's Market，午后休整，傍晚去 Palm Cove 看海。</x:v>
+        <x:v>上午逛 Rusty's Market，午间回酒店洗衣打包，下午沿 Palm Cove 海滨与 Jetty 散步，在蓝调时刻用一顿早晚餐收尾。</x:v>
       </x:c>
       <x:c r="J12" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -1297,10 +1297,10 @@
         <x:v>凯恩斯市场与海滨</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>步行 / 市内短途交通</x:v>
+        <x:v>步行 + Uber / Didi</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>09:00 前出门逛 Rusty's Market</x:v>
+        <x:v>08:30 去 Rusty's Market；15:00 叫车前往 Palm Cove；19:00 返程</x:v>
       </x:c>
       <x:c r="Q12" t="str">
         <x:v>southern-cross-map</x:v>
@@ -3560,22 +3560,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>上午</x:v>
+        <x:v>06:25–11:00</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>墨尔本机场</x:v>
+        <x:v>Melbourne Airport → Cairns Airport → Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>飞往凯恩斯</x:v>
+        <x:v>搭乘 06:25 航班，09:50 抵达凯恩斯；取行李后打车到公寓寄存行李或办理入住</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>气候切换非常明显</x:v>
+        <x:v>从南部冬天飞进热带</x:v>
       </x:c>
       <x:c r="G66" t="str">
-        <x:v>国内航班建议预留行李额</x:v>
+        <x:v>薄外套放在随身包里，落地后再换成轻便衣物；到公寓先确认房间与行李安排。</x:v>
       </x:c>
       <x:c r="H66" t="str">
-        <x:v>mel-airport-map</x:v>
+        <x:v>mel-airport-map,cairns-airport-map,southern-cross-map,virgin-australia-official</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3586,21 +3586,23 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>中午</x:v>
+        <x:v>11:15–14:30</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>Cairns CBD / Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>打车 / Uber 到酒店</x:v>
+        <x:v>在公寓附近吃一顿 brunch，随后回房间洗澡、补觉与整理随身物品</x:v>
       </x:c>
       <x:c r="F67" t="str">
-        <x:v>不租车，降低疲劳</x:v>
+        <x:v>给早班机后的身体留出缓冲</x:v>
       </x:c>
       <x:c r="G67" t="str">
-        <x:v>酒店可先寄存行李</x:v>
-      </x:c>
-      <x:c r="H67"/>
+        <x:v>午后先休息两小时；若房间尚未准备好，就在附近咖啡馆慢慢坐一会儿。</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>cairns-cbd-map,southern-cross-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" t="str">
@@ -3610,22 +3612,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>下午</x:v>
+        <x:v>15:00–16:30 · 可选</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Esplanade Lagoon</x:v>
+        <x:v>Cairns Botanic Gardens</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>免费泻湖泳池、海滨散步</x:v>
+        <x:v>沿 Flecker Garden 轻松散步，看热带植物、树冠与雨林景观</x:v>
       </x:c>
       <x:c r="F68" t="str">
-        <x:v>度假感拉满</x:v>
+        <x:v>抵达凯恩斯后的第一段热带绿意</x:v>
       </x:c>
       <x:c r="G68" t="str">
-        <x:v>泳衣可提前放随身包</x:v>
+        <x:v>花园免费开放；如果上午转场后仍然疲惫，就留在公寓休息，傍晚再去海滨。</x:v>
       </x:c>
       <x:c r="H68" t="str">
-        <x:v>cairns-lagoon-map</x:v>
+        <x:v>cairns-botanic-gardens-map,cairns-botanic-gardens-official</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3636,22 +3638,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>晚上</x:v>
+        <x:v>17:00–19:30</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Cairns Night Markets</x:v>
+        <x:v>Esplanade Boardwalk → Marlin Marina → Cairns Night Markets</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>夜市、简餐、纪念品</x:v>
+        <x:v>沿海滨步道慢慢走到 Marina，顺便认好次日 Reef Fleet Terminal 的方向；随后到 Night Markets 边逛边吃</x:v>
       </x:c>
       <x:c r="F69" t="str">
-        <x:v>热闹轻松</x:v>
+        <x:v>海风、码头与凯恩斯第一晚</x:v>
       </x:c>
       <x:c r="G69" t="str">
-        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
+        <x:v>Esplanade Lagoon 于 7 月 13 日至 8 月 16 日因维护关闭；今天以海滨散步和公寓泳池为主。Night Markets 摊位通常从 16:30 起营业。</x:v>
       </x:c>
       <x:c r="H69" t="str">
-        <x:v>cairns-night-market-map</x:v>
+        <x:v>cairns-esplanade-boardwalk-map,cairns-marlin-marina-map,cairns-night-market-map,cairns-night-markets-official,cairns-lagoon-closure-official</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -3668,15 +3670,17 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
+        <x:v>早餐：机场或飞机轻食；午餐：公寓附近 brunch / Overlay Coffee；晚餐：Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>用轻松餐食完成气候与节奏切换</x:v>
       </x:c>
       <x:c r="G70" t="str">
-        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
-      </x:c>
-      <x:c r="H70"/>
+        <x:v>20:00 后回公寓整理泳衣、防晒衣、薄外套和晕船用品，为次日出海早点休息。</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>cairns-cbd-map,cairns-night-market-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="str">
@@ -3686,22 +3690,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>早上</x:v>
+        <x:v>06:45–07:30</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>凯恩斯码头</x:v>
+        <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Reef Magic check-in，登船出海</x:v>
+        <x:v>吃一顿清淡早餐，检查泳衣、防晒衣、毛巾、薄外套与晕船用品</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>前往外礁平台</x:v>
+        <x:v>在出海前把身体与随身包准备好</x:v>
       </x:c>
       <x:c r="G71" t="str">
-        <x:v>提前吃晕船药；不要卡点到码头；带好泳衣、防晒衣、毛巾、薄外套</x:v>
+        <x:v>按药品说明提前服用晕船药；早餐不要空腹，也不要吃得太油腻。</x:v>
       </x:c>
       <x:c r="H71" t="str">
-        <x:v>reef-fleet-terminal-map,reef-magic-official</x:v>
+        <x:v>southern-cross-map,reef-magic-schedule-official</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3712,22 +3716,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>全天</x:v>
+        <x:v>07:45–08:45</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Outer Reef Pontoon</x:v>
+        <x:v>Southern Cross Atrium → Reef Fleet Terminal</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>浮潜、半潜艇、玻璃底船、海底观景室、可选深潜 / 海底漫步</x:v>
+        <x:v>前往码头办理 Reef Magic check-in；08:15 开始登船，最晚 08:45 完成登船</x:v>
       </x:c>
       <x:c r="F72" t="str">
-        <x:v>珊瑚、热带鱼、大堡礁平台体验</x:v>
+        <x:v>清晨从城市走向大堡礁</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>防晒衣比防晒霜更重要；船舱空调可能很冷；不下水的人也有体验</x:v>
+        <x:v>不要卡最后登船时间；到码头后先确认回程集合点、储物方式与当天海况。</x:v>
       </x:c>
       <x:c r="H72" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>southern-cross-map,reef-fleet-terminal-map,reef-magic-official,reef-magic-schedule-official</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -3738,22 +3742,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>中午</x:v>
+        <x:v>09:00–10:30</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>船上 / 平台</x:v>
+        <x:v>Cairns Marina → Outer Reef Pontoon</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>外礁平台午餐</x:v>
+        <x:v>09:00 离港，乘船前往 Moore Reef 外礁平台</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>轻松补给</x:v>
+        <x:v>海水颜色从港湾一路变成外礁蓝</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>不要吃太撑，避免晕船</x:v>
+        <x:v>船上风大且空调偏冷，薄外套放在容易拿到的位置；不舒服时尽早到船尾或室外通风处休息。</x:v>
       </x:c>
       <x:c r="H73" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>reef-fleet-terminal-map,reef-magic-official,reef-magic-schedule-official</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3764,22 +3768,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>下午</x:v>
+        <x:v>10:30–15:30</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Outer Reef Pontoon</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>下船休息</x:v>
+        <x:v>在平台体验浮潜、半潜艇、玻璃底船与海底观景室，中午享用包含在行程内的午餐</x:v>
       </x:c>
       <x:c r="F74" t="str">
-        <x:v>通常会比较疲惫</x:v>
+        <x:v>大堡礁珊瑚、热带鱼与平台活动</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
+        <x:v>先确认半潜艇和玻璃底船班次，再安排下水时间；防晒衣比反复补涂更省心。</x:v>
       </x:c>
       <x:c r="H74" t="str">
-        <x:v>reef-fleet-terminal-map</x:v>
+        <x:v>reef-magic-official,reef-magic-schedule-official</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -3790,22 +3794,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>晚上</x:v>
+        <x:v>15:30–18:15</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>码头附近</x:v>
+        <x:v>Outer Reef Pontoon → Cairns → Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
+        <x:v>15:30 离开平台，约 17:00 回到凯恩斯；下船后回公寓洗澡、换干衣并休息</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>海边晚餐</x:v>
+        <x:v>从海上慢慢回到城市节奏</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
+        <x:v>湿衣物及时分开收纳，回房后先补水；晚上只留一顿轻松的码头晚餐。</x:v>
       </x:c>
       <x:c r="H75" t="str">
-        <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
+        <x:v>reef-fleet-terminal-map,southern-cross-map,reef-magic-schedule-official</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -3813,25 +3817,25 @@
         <x:v>d7</x:v>
       </x:c>
       <x:c r="B76" t="n">
-        <x:v>80</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>提醒</x:v>
+        <x:v>18:30–20:30</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>今日提醒</x:v>
+        <x:v>Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
+        <x:v>按当晚状态在码头边吃海鲜，饭后散步回公寓</x:v>
       </x:c>
       <x:c r="F76" t="str">
-        <x:v>舒适与安全比拍摄数量更重要</x:v>
+        <x:v>用一顿轻松海鲜为外礁日收尾</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
+        <x:v>Prawn Star 更随意直接，Salt House 更适合坐下来慢慢吃；20:30 左右回到公寓。</x:v>
       </x:c>
       <x:c r="H76" t="str">
-        <x:v>reef-magic-official</x:v>
+        <x:v>prawn-star-map,salt-house-map,southern-cross-map</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -3848,13 +3852,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
+        <x:v>早餐：公寓轻食；午餐：Reef Magic 外礁平台午餐；晚餐：Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="F77" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>出海日以清淡、补水和方便为主</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
+        <x:v>随身带一瓶水和少量饼干；浮潜前后都不要一次吃得太撑。</x:v>
       </x:c>
       <x:c r="H77" t="str">
         <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
@@ -3868,21 +3872,23 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>清晨</x:v>
+        <x:v>06:10–06:55</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>凯恩斯酒店 → 丹翠方向</x:v>
+        <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>6:55am 酒店门口集合，跟团车北上</x:v>
+        <x:v>简单吃早餐并带好水、防晒、防蚊与薄外套；06:45 到酒店门口等候，订单集合时间 06:55</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>不用自驾，沿途可休息看风景</x:v>
+        <x:v>清晨跟着 Billy Tea 向北出发</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>早上提前吃一点，带水、防晒、帽子和薄外套</x:v>
-      </x:c>
-      <x:c r="H78"/>
+        <x:v>贵重物品和随身用品放在一个小包里；如有饮食禁忌，出发前再次向导游确认。</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>southern-cross-map,billy-tea-official</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
@@ -3898,16 +3904,16 @@
         <x:v>Daintree River / Rainforest</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>鳄鱼游船、雨林步道</x:v>
+        <x:v>乘坐 Daintree River Cruise 寻找鳄鱼与鸟类，再沿雨林步道观察红树林、藤蔓和热带树冠</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>野生鳄鱼、鸟类、红树林、热带雨林生态</x:v>
+        <x:v>河流与古老雨林的生态层次</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>野生动物不保证，但 Daintree River 是经典鳄鱼河道</x:v>
+        <x:v>野生动物出现看运气；船上和团车空调可能偏冷，薄外套不要放进行李舱。</x:v>
       </x:c>
       <x:c r="H79" t="str">
-        <x:v>daintree-river-map</x:v>
+        <x:v>daintree-river-map,billy-tea-official</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -3924,15 +3930,17 @@
         <x:v>Daintree Rainforest</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>团含午餐</x:v>
+        <x:v>跟随团内安排享用午餐，在雨林行程中段坐下来休息</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>不用自己找餐厅</x:v>
+        <x:v>不用另找餐厅的从容午间</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>如有忌口提前告知</x:v>
-      </x:c>
-      <x:c r="H80"/>
+        <x:v>午餐已包含在行程内；下午还有步行与海滩停留，吃到舒服即可。</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>billy-tea-official</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="str">
@@ -3948,16 +3956,16 @@
         <x:v>Cape Tribulation</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>雨林入海、海滩短停留</x:v>
+        <x:v>走到 Cape Tribulation Beach，看热带雨林一直延伸到海边</x:v>
       </x:c>
       <x:c r="F81" t="str">
-        <x:v>雨林与海洋在这里交会</x:v>
+        <x:v>丹翠最具代表性的雨林入海画面</x:v>
       </x:c>
       <x:c r="G81" t="str">
-        <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
+        <x:v>不把下海游泳列入行程；留意鳄鱼、水母与现场警示牌。</x:v>
       </x:c>
       <x:c r="H81" t="str">
-        <x:v>cape-trib-map</x:v>
+        <x:v>cape-trib-map,billy-tea-official</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -3971,19 +3979,19 @@
         <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Daintree Ferry / Ice Cream</x:v>
+        <x:v>Daintree Ferry / Daintree Ice Cream</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>渡河、热带水果冰淇淋</x:v>
+        <x:v>乘渡轮穿过丹翠河，品尝行程包含的热带水果冰淇淋</x:v>
       </x:c>
       <x:c r="F82" t="str">
-        <x:v>丹翠地区很有代表性的热带味道</x:v>
+        <x:v>雨林水果带来的独特味道</x:v>
       </x:c>
       <x:c r="G82" t="str">
-        <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
+        <x:v>留意当天口味组合，也可以顺手拍下每一种水果的名字。</x:v>
       </x:c>
       <x:c r="H82" t="str">
-        <x:v>daintree-icecream-map</x:v>
+        <x:v>daintree-icecream-map,billy-tea-official</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -3994,21 +4002,23 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>18:30–20:30</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>返回凯恩斯 / Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>18:30 后回到市区</x:v>
+        <x:v>约 18:30 回到市区，在酒店附近简餐或从 Night Markets 外带，随后回房休息</x:v>
       </x:c>
       <x:c r="F83" t="str">
-        <x:v>回程可休息</x:v>
+        <x:v>长日跟团后的轻松夜晚</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
-      </x:c>
-      <x:c r="H83"/>
+        <x:v>晚餐以方便为主，不另外安排夜间活动；20:00–20:30 回房整理次日自驾用品。</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>southern-cross-map,cairns-night-market-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" t="str">
@@ -4024,16 +4034,16 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>早餐：公寓轻食；午餐：Billy Tea 团餐；下午：Daintree Ice Cream；晚餐：酒店附近简餐 / Night Markets 外带</x:v>
       </x:c>
       <x:c r="F84" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>团内餐食与回城简餐自然衔接</x:v>
       </x:c>
       <x:c r="G84" t="str">
-        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
+        <x:v>清晨准备一份不油腻的早餐，回城较晚时以方便和早点休息为先。</x:v>
       </x:c>
       <x:c r="H84" t="str">
-        <x:v>daintree-icecream-map</x:v>
+        <x:v>billy-tea-official,daintree-icecream-map,cairns-night-market-map</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -4044,22 +4054,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>早上</x:v>
+        <x:v>08:00–08:30</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>凯恩斯 → Lake Eacham</x:v>
+        <x:v>凯恩斯取车点</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>取车后出发，开上 Atherton Tablelands</x:v>
+        <x:v>办理取车、拍下车身与轮毂状况，设置整日导航后向 Atherton Tablelands 出发</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>从热带海边城市进入清凉高原</x:v>
+        <x:v>从热带海边城市切换到清凉高原</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>不要太晚出发，8:30–9:00 比较理想</x:v>
+        <x:v>确认油量、还车时间与第二驾驶人；08:30 左右启程，山路保持从容车距。</x:v>
       </x:c>
       <x:c r="H85" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>d9-tablelands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -4070,22 +4080,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>上午</x:v>
+        <x:v>09:45–10:30</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Lake Eacham</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>火山湖散步、看湖景</x:v>
+        <x:v>沿湖边走一小段，看火山湖、雨林倒影与清晨水色</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>安静、清凉、湖水和雨林包围感</x:v>
+        <x:v>被雨林包围的安静火山湖</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>可走一小段湖边步道，不必完整绕湖</x:v>
+        <x:v>不必完整绕湖；以现场游泳警示和水况为准，今天以散步看湖为主。</x:v>
       </x:c>
       <x:c r="H86" t="str">
-        <x:v>lake-eacham-map</x:v>
+        <x:v>lake-eacham-map,d9-tablelands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4096,22 +4106,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>10:50–11:20</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>看巨型帘状无花果树</x:v>
+        <x:v>沿短步道走到巨型帘状无花果树下，观察垂落根系与森林尺度</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>像热带森林里的巨大自然装置</x:v>
+        <x:v>像天然装置艺术般的高原巨树</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>停留 20–30 分钟即可</x:v>
+        <x:v>木栈道雨后可能湿滑，停留约 20–30 分钟即可。</x:v>
       </x:c>
       <x:c r="H87" t="str">
-        <x:v>curtain-fig-map</x:v>
+        <x:v>curtain-fig-map,d9-tablelands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4122,22 +4132,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>中午</x:v>
+        <x:v>11:30–12:00</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Yungaburra / Gallo Dairyland</x:v>
+        <x:v>Yungaburra</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>小镇午餐、咖啡、奶制品、巧克力</x:v>
+        <x:v>在高原小镇老街散步，看看木屋、咖啡馆与乡村街景</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>高原小镇、牧场氛围、乡村节奏</x:v>
+        <x:v>高原生活节奏的短暂停靠</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>适合中段坐下来休息，不要午餐拖太久</x:v>
+        <x:v>先散步再前往 Gallo Dairyland 用餐，午间节奏会更顺。</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>yungaburra-map,gallo-map</x:v>
+        <x:v>yungaburra-map,d9-tablelands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4148,22 +4158,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>下午</x:v>
+        <x:v>12:15–13:15</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Millaa Millaa Falls / Ellinjaa Falls</x:v>
+        <x:v>Gallo Dairyland</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>瀑布短停留、拍照</x:v>
+        <x:v>在牧场享用午餐，尝试本地奶酪、巧克力或奶制品</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>雨林瀑布与高原绿意</x:v>
+        <x:v>阿瑟顿高原的农场味道</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
+        <x:v>留意厨房与品鉴供应时间；午餐后在 13:15 左右继续前往瀑布。</x:v>
       </x:c>
       <x:c r="H89" t="str">
-        <x:v>millaa-map,ellinjaa-map</x:v>
+        <x:v>gallo-map,d9-tablelands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4174,21 +4184,23 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>14:00–15:15</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>返回凯恩斯</x:v>
+        <x:v>Millaa Millaa Falls / Ellinjaa Falls（可选）</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>下山回市区，还车或次日早还</x:v>
+        <x:v>14:00–14:40 欣赏 Millaa Millaa Falls；路况与状态都合适时，14:50–15:15 再到 Ellinjaa Falls 短停</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>完成高原自然线</x:v>
+        <x:v>高原瀑布与热带绿意</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>尽量 15:30–16:00 开始回程，避免天黑后还在乡村路和山路上开</x:v>
-      </x:c>
-      <x:c r="H90"/>
+        <x:v>Millaa Millaa Falls 是这一段的完整停留；无论是否去 Ellinjaa Falls，都在 15:15 开始返回凯恩斯。</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>millaa-map,ellinjaa-map,d9-tablelands-route-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
@@ -4198,21 +4210,23 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>晚上</x:v>
+        <x:v>15:15–17:45</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>凯恩斯</x:v>
+        <x:v>返回 Cairns / 凯恩斯还车点</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>简单晚餐</x:v>
+        <x:v>沿山路返回凯恩斯，途中补满油并按订单时间完成还车</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>回城后轻松晚餐</x:v>
+        <x:v>在天黑前结束高原自驾</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>下山后就近用餐，早点休息。</x:v>
-      </x:c>
-      <x:c r="H91"/>
+        <x:v>15:15 开始返程，预计 17:00–17:45 完成加油与还车；下山路段留意弯道和野生动物。</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>d9-tablelands-route-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
@@ -4228,16 +4242,16 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
+        <x:v>早餐：公寓或咖啡馆；午餐：Gallo Dairyland；晚餐：18:30 左右在 Salt House 或公寓附近简餐</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>农场午餐与回城晚餐</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
+        <x:v>午餐留给高原风味，晚餐按还车后的状态轻松选择。</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>millaa-map,gallo-map</x:v>
+        <x:v>gallo-map,salt-house-map,southern-cross-map</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -4248,22 +4262,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>上午</x:v>
+        <x:v>08:30–10:30</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>Rusty's Market</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>逛热带水果、咖啡与早餐摊位，挑选当天可以吃完的水果和轻食</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>周五正好开市，适合补水果和轻食</x:v>
+        <x:v>凯恩斯周五早晨的市场气息</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
+        <x:v>买少量即可，水果在飞悉尼前吃完；现场营业情况以当天摊位为准。</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>rustys-map</x:v>
+        <x:v>rustys-map,rustys-official</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4274,22 +4288,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>中午</x:v>
+        <x:v>10:45–14:30</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>酒店休息 / 泳池 / Esplanade Lagoon</x:v>
+        <x:v>回公寓洗衣、休息、整理行李，把 Jetstar 托运行李和随身物品分装好</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>热带城市躺平感</x:v>
+        <x:v>给连续三天自然行程留出恢复时间</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
+        <x:v>午餐在附近简单解决；泳池、咖啡与午休都留在这段时间里。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>cairns-lagoon-map</x:v>
+        <x:v>southern-cross-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4300,21 +4314,23 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>下午</x:v>
+        <x:v>15:00–17:30</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>Southern Cross Atrium → Palm Cove</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>洗衣、整理行李、轻松逛街或按摩</x:v>
+        <x:v>15:00 叫 Uber / Didi，约 15:40 抵达；15:40–17:30 沿 Williams Esplanade、Palm Cove Beach 与 Palm Cove Jetty 慢慢散步</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>为次日清晨航班做准备</x:v>
+        <x:v>棕榈树、海岸与热带蓝调前的光线</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>Jetstar 行李控制在 20kg 内，提前分装</x:v>
-      </x:c>
-      <x:c r="H95"/>
+        <x:v>海滩活动以现场旗帜和警示为准；这里更适合散步与拍照，不把下海游泳作为固定安排。</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>southern-cross-map,palm-cove-map,williams-esplanade-map,palm-cove-jetty-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
@@ -4324,22 +4340,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>下午 / 傍晚</x:v>
+        <x:v>17:30–18:45</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Palm Cove</x:v>
+        <x:v>Palm Cove 早晚餐</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>前往 Palm Cove，沿棕榈树海滨大道散步、喝咖啡并看海</x:v>
+        <x:v>在 Williams Esplanade 一带选一家海滨餐厅，边吃晚餐边看天空进入蓝调时刻</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
+        <x:v>凯恩斯段最后一顿海边晚餐</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
+        <x:v>Palm Cove 面向东侧，重点是傍晚天色与棕榈树剪影；19:00 前准备返程。</x:v>
       </x:c>
       <x:c r="H96" t="str">
-        <x:v>palm-cove-map</x:v>
+        <x:v>williams-esplanade-map,palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4350,22 +4366,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>晚上</x:v>
+        <x:v>19:00–21:30</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>Palm Cove → Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prawn Star / Salt House / Cairns Night Markets</x:v>
+        <x:v>19:00 叫车返回，预计 19:30–19:45 抵达；20:00–21:00 完成行李称重、Jetstar 在线值机与次日随身包检查</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>海鲜或轻松简餐</x:v>
+        <x:v>把热带假期从容收进行李箱</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>早点吃，早点睡</x:v>
+        <x:v>闹钟、证件、薄外套和机场用物放在手边；21:15–21:30 上床休息。</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>cairns-night-market-map,prawn-star-map,salt-house-map</x:v>
+        <x:v>palm-cove-map,southern-cross-map,cairns-airport-map,jetstar-official</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4382,16 +4398,16 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
+        <x:v>早餐：Rusty's Market；午餐：公寓附近简餐；晚餐：Palm Cove 海滨早晚餐</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>市场、水果与海边晚餐组成轻松收尾</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
+        <x:v>晚餐结束后直接返回凯恩斯，不让次日清晨航班变得匆忙。</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>rustys-map,prawn-star-map</x:v>
+        <x:v>rustys-map,rustys-official,williams-esplanade-map,palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -8648,8 +8664,8 @@
       <x:c r="D156" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;destination=Loch+Ard+Gorge%2C+VIC&amp;travelmode=driving&amp;waypoints=Twelve+Apostles%2C+VIC%7CGibson+Steps%2C+VIC</x:v>
       </x:c>
-      <x:c r="E156" t="str"/>
-      <x:c r="F156" t="str"/>
+      <x:c r="E156"/>
+      <x:c r="F156"/>
       <x:c r="G156" t="str">
         <x:v>Google Maps · Southern Ocean Villas → Twelve Apostles → Gibson Steps → Loch Ard Gorge</x:v>
       </x:c>
@@ -8667,8 +8683,8 @@
       <x:c r="D157" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Loch+Ard+Gorge%2C+VIC&amp;destination=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;travelmode=driving&amp;waypoints=London+Arch%2C+VIC%7CThe+Grotto%2C+Port+Campbell+VIC</x:v>
       </x:c>
-      <x:c r="E157" t="str"/>
-      <x:c r="F157" t="str"/>
+      <x:c r="E157"/>
+      <x:c r="F157"/>
       <x:c r="G157" t="str">
         <x:v>Google Maps · Loch Ard Gorge → London Arch → The Grotto → Southern Ocean Villas</x:v>
       </x:c>
@@ -8686,10 +8702,238 @@
       <x:c r="D158" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Southern+Ocean+Villas%2C+Port+Campbell+VIC&amp;destination=Holiday+Inn+Melbourne+Airport&amp;travelmode=driving&amp;waypoints=Great+Ocean+Road+Wildlife+Park%2C+Gellibrand+Lower+VIC%7CColac%2C+VIC</x:v>
       </x:c>
-      <x:c r="E158" t="str"/>
-      <x:c r="F158" t="str"/>
+      <x:c r="E158"/>
+      <x:c r="F158"/>
       <x:c r="G158" t="str">
         <x:v>Google Maps · Southern Ocean Villas → Great Ocean Road Wildlife Park → Colac → Holiday Inn Melbourne Airport</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>cairns-lagoon-closure-official</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
+        <x:v>Cairns Esplanade Lagoon 维护公告</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>https://www.cairns.qld.gov.au/council/news-notices/news/media-releases/esplanade-lagoon-to-close-for-essential-maintenance</x:v>
+      </x:c>
+      <x:c r="E159" t="str"/>
+      <x:c r="F159" t="str"/>
+      <x:c r="G159" t="str">
+        <x:v>Cairns Regional Council · 2026 年 7 月 13 日至 8 月 16 日维护关闭</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>cairns-botanic-gardens-map</x:v>
+      </x:c>
+      <x:c r="B160" t="str">
+        <x:v>Cairns Botanic Gardens</x:v>
+      </x:c>
+      <x:c r="C160" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D160" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+Botanic+Gardens</x:v>
+      </x:c>
+      <x:c r="E160" t="str"/>
+      <x:c r="F160" t="str"/>
+      <x:c r="G160" t="str">
+        <x:v>Google Maps · Cairns Botanic Gardens</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>cairns-botanic-gardens-official</x:v>
+      </x:c>
+      <x:c r="B161" t="str">
+        <x:v>Cairns Botanic Gardens 官网</x:v>
+      </x:c>
+      <x:c r="C161" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D161" t="str">
+        <x:v>https://www.cairns.qld.gov.au/experience-cairns/botanic-gardens</x:v>
+      </x:c>
+      <x:c r="E161" t="str"/>
+      <x:c r="F161" t="str"/>
+      <x:c r="G161" t="str">
+        <x:v>Cairns Regional Council · Flecker Garden 每日 07:30–17:30 免费开放</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>cairns-cbd-map</x:v>
+      </x:c>
+      <x:c r="B162" t="str">
+        <x:v>Cairns CBD</x:v>
+      </x:c>
+      <x:c r="C162" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D162" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+CBD+Queensland</x:v>
+      </x:c>
+      <x:c r="E162" t="str"/>
+      <x:c r="F162" t="str"/>
+      <x:c r="G162" t="str">
+        <x:v>Google Maps · Cairns CBD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" t="str">
+        <x:v>cairns-esplanade-boardwalk-map</x:v>
+      </x:c>
+      <x:c r="B163" t="str">
+        <x:v>Cairns Esplanade Boardwalk</x:v>
+      </x:c>
+      <x:c r="C163" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D163" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+Esplanade+Boardwalk</x:v>
+      </x:c>
+      <x:c r="E163" t="str"/>
+      <x:c r="F163" t="str"/>
+      <x:c r="G163" t="str">
+        <x:v>Google Maps · Cairns Esplanade Boardwalk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>cairns-marlin-marina-map</x:v>
+      </x:c>
+      <x:c r="B164" t="str">
+        <x:v>Cairns Marlin Marina</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+Marlin+Marina</x:v>
+      </x:c>
+      <x:c r="E164" t="str"/>
+      <x:c r="F164" t="str"/>
+      <x:c r="G164" t="str">
+        <x:v>Google Maps · Cairns Marlin Marina</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>cairns-night-markets-official</x:v>
+      </x:c>
+      <x:c r="B165" t="str">
+        <x:v>Cairns Night Markets 官网</x:v>
+      </x:c>
+      <x:c r="C165" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D165" t="str">
+        <x:v>https://www.nightmarkets.com.au/faq</x:v>
+      </x:c>
+      <x:c r="E165" t="str"/>
+      <x:c r="F165" t="str"/>
+      <x:c r="G165" t="str">
+        <x:v>Cairns Night Markets · 市场摊位每日 16:30 起营业</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>reef-magic-schedule-official</x:v>
+      </x:c>
+      <x:c r="B166" t="str">
+        <x:v>Reef Magic 当日时刻表</x:v>
+      </x:c>
+      <x:c r="C166" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D166" t="str">
+        <x:v>https://www.reefmagic.com.au/faqs/</x:v>
+      </x:c>
+      <x:c r="E166" t="str"/>
+      <x:c r="F166" t="str"/>
+      <x:c r="G166" t="str">
+        <x:v>Reef Magic · 08:15 登船、08:45 最晚登船、09:00 离港、17:00 返回</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>d9-tablelands-route-map</x:v>
+      </x:c>
+      <x:c r="B167" t="str">
+        <x:v>D9 阿瑟顿高原完整路线</x:v>
+      </x:c>
+      <x:c r="C167" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D167" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Lake+Eacham%7CCurtain+Fig+Tree%7CYungaburra%7CGallo+Dairyland%7CMillaa+Millaa+Falls</x:v>
+      </x:c>
+      <x:c r="E167" t="str"/>
+      <x:c r="F167" t="str"/>
+      <x:c r="G167" t="str">
+        <x:v>Google Maps · Cairns → Lake Eacham → Curtain Fig Tree → Yungaburra → Gallo Dairyland → Millaa Millaa Falls → Cairns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" t="str">
+        <x:v>rustys-official</x:v>
+      </x:c>
+      <x:c r="B168" t="str">
+        <x:v>Rusty's Markets 官网</x:v>
+      </x:c>
+      <x:c r="C168" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D168" t="str">
+        <x:v>https://rustysmarkets.com.au/location/</x:v>
+      </x:c>
+      <x:c r="E168" t="str"/>
+      <x:c r="F168" t="str"/>
+      <x:c r="G168" t="str">
+        <x:v>Rusty's Markets · 周五、周六、周日开放</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" t="str">
+        <x:v>williams-esplanade-map</x:v>
+      </x:c>
+      <x:c r="B169" t="str">
+        <x:v>Williams Esplanade · Palm Cove</x:v>
+      </x:c>
+      <x:c r="C169" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D169" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Williams+Esplanade+Palm+Cove</x:v>
+      </x:c>
+      <x:c r="E169" t="str"/>
+      <x:c r="F169" t="str"/>
+      <x:c r="G169" t="str">
+        <x:v>Google Maps · Williams Esplanade, Palm Cove</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" t="str">
+        <x:v>palm-cove-jetty-map</x:v>
+      </x:c>
+      <x:c r="B170" t="str">
+        <x:v>Palm Cove Jetty</x:v>
+      </x:c>
+      <x:c r="C170" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D170" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Palm+Cove+Jetty</x:v>
+      </x:c>
+      <x:c r="E170" t="str"/>
+      <x:c r="F170" t="str"/>
+      <x:c r="G170" t="str">
+        <x:v>Google Maps · Palm Cove Jetty</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
update D9 Atherton itinerary
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rbbdec6bcd99347dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R216794ce226a4c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rcccb1a42fdb54591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Rfe6719406d3c44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R9166dea9e89e4a6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R0688fcc6254e49f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R70c1f63ea10a4896"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R49b094d638a04366"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R1a67babebb054830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Rc4325b17e05e443c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R0770be89d65e4a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R658f7356b93f4292"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Ra69ca48cab7e4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R7f5a3ee70a384c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R3f8f2ca273ca4ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rbdfcc6d86ff4481d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Ra4d6a9dd09c243c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R6cdef1af7c214b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R2c1d98f50d8746be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R6f9f43abd5084a89"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1217,19 +1217,19 @@
         <x:v>145.5831</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>阿瑟顿高原：火山湖、巨树与瀑布</x:v>
+        <x:v>穿行阿瑟顿高原：火山湖、巨树与瀑布</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>从 Cairns 自驾上高原，串联 Lake Eacham、Curtain Fig Tree、Yungaburra、Gallo Dairyland 与 Millaa Millaa Falls，傍晚还车回城。</x:v>
+        <x:v>从 Cairns 驶上阿瑟顿高原，在 Lake Eacham 看火山湖，沿 Yungaburra 与 Curtain Fig Tree 走进高原风景，午后到 Gallo Dairyland 吃午餐，再以 Millaa Millaa Falls 收尾。</x:v>
       </x:c>
       <x:c r="J11" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>高原比凯恩斯海边更清凉。</x:v>
+        <x:v>高原清晨约 10–15°C，中午约 22–26°C；天气与体感会随海拔变化。</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>短袖加薄外套，瀑布和雨林步道注意防滑。</x:v>
+        <x:v>短袖打底 + 薄外套 + 轻薄长裤 + 防滑运动鞋；车里备雨衣、帽子、墨镜与防晒。</x:v>
       </x:c>
       <x:c r="M11" t="str">
         <x:v>/itinerary/d9-atherton-tablelands-waterfall.png</x:v>
@@ -1238,16 +1238,16 @@
         <x:v>阿瑟顿高原瀑布</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>自驾 · 阿瑟顿高原</x:v>
+        <x:v>自驾 · 阿瑟顿高原环线（约 230–260 km；纯驾驶约 4–4.5 小时；全天约 9 小时）</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>08:00–08:30 取车；08:30 启程上高原</x:v>
+        <x:v>07:45 前往取车点；08:30 前驶离 Cairns；13:15 离开 Gallo；15:35 开始返程</x:v>
       </x:c>
       <x:c r="Q11" t="str">
         <x:v>southern-cross-map</x:v>
       </x:c>
       <x:c r="R11" t="str">
-        <x:v>d9-tablelands-route-map</x:v>
+        <x:v>d9-core-route-map</x:v>
       </x:c>
       <x:c r="S11" t="str">
         <x:v>no-fixed-ticket</x:v>
@@ -4054,22 +4054,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>08:00–08:30</x:v>
+        <x:v>07:15–07:45</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>凯恩斯取车点</x:v>
+        <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>办理取车、拍下车身与轮毂状况，设置整日导航后向 Atherton Tablelands 出发</x:v>
+        <x:v>吃早餐、装好饮用水，检查驾照、租车订单与充电线，并把当天区域下载到 Google Maps 离线地图</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>从热带海边城市切换到清凉高原</x:v>
+        <x:v>从一段从容准备开启高原自驾</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>确认油量、还车时间与第二驾驶人；08:30 左右启程，山路保持从容车距。</x:v>
+        <x:v>每人带约 1L 水和一份小零食；薄外套、轻薄雨衣、帽子、墨镜、防晒与纸巾放在随手可取的位置。</x:v>
       </x:c>
       <x:c r="H85" t="str">
-        <x:v>d9-tablelands-route-map</x:v>
+        <x:v>southern-cross-map,d9-core-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -4080,22 +4080,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>09:45–10:30</x:v>
+        <x:v>07:45–08:30</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Lake Eacham</x:v>
+        <x:v>凯恩斯取车点</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>沿湖边走一小段，看火山湖、雨林倒影与清晨水色</x:v>
+        <x:v>前往租车订单上的准确门店，取车后拍下车身四角、轮毂、挡风玻璃与油表，再调好座椅、后视镜和手机支架</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>被雨林包围的安静火山湖</x:v>
+        <x:v>在驶入 Gillies Highway 前熟悉车辆</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>不必完整绕湖；以现场游泳警示和水况为准，今天以散步看湖为主。</x:v>
+        <x:v>导航以订单中的准确 branch 为准；离店前再次确认还车地点、油量规则与时间，08:30 前驶离 Cairns。</x:v>
       </x:c>
       <x:c r="H86" t="str">
-        <x:v>lake-eacham-map,d9-tablelands-route-map</x:v>
+        <x:v>cairns-car-rental-search-map,d9-core-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4106,22 +4106,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>10:50–11:20</x:v>
+        <x:v>08:30–09:40</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Curtain Fig Tree</x:v>
+        <x:v>Cairns → Lake Eacham</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>沿短步道走到巨型帘状无花果树下，观察垂落根系与森林尺度</x:v>
+        <x:v>经 Gordonvale 与 Gillies Highway 驶上高原，沿铺装道路前往 Lake Eacham Day Use Area</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>像天然装置艺术般的高原巨树</x:v>
+        <x:v>海边城市逐渐切换成清凉高原</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>木栈道雨后可能湿滑，停留约 20–30 分钟即可。</x:v>
+        <x:v>Gillies Highway 弯道密集，保持舒服车距；只在安全让车区让快车通过，不跟着后车加速。</x:v>
       </x:c>
       <x:c r="H87" t="str">
-        <x:v>curtain-fig-map,d9-tablelands-route-map</x:v>
+        <x:v>d9-cairns-lake-eacham-route-map,lake-eacham-official</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4132,22 +4132,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>11:30–12:00</x:v>
+        <x:v>09:40–10:20</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Yungaburra</x:v>
+        <x:v>Lake Eacham Day Use Area</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>在高原小镇老街散步，看看木屋、咖啡馆与乡村街景</x:v>
+        <x:v>到湖边观景台看火山湖与雨林倒影，再沿湖边步道轻松走一小段</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>高原生活节奏的短暂停靠</x:v>
+        <x:v>被雨林环抱的清澈火山湖</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>先散步再前往 Gallo Dairyland 用餐，午间节奏会更顺。</x:v>
+        <x:v>今天不完整环湖，也不安排游泳；沿成形步道行走，10:20 左右继续前往 Yungaburra。</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>yungaburra-map,d9-tablelands-route-map</x:v>
+        <x:v>lake-eacham-day-use-map,lake-eacham-official,d9-core-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4158,22 +4158,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>12:15–13:15</x:v>
+        <x:v>10:30–10:55</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Gallo Dairyland</x:v>
+        <x:v>Yungaburra Village</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>在牧场享用午餐，尝试本地奶酪、巧克力或奶制品</x:v>
+        <x:v>沿老街短走，看看历史木屋、高原小店与街景，需要时买一杯咖啡</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>阿瑟顿高原的农场味道</x:v>
+        <x:v>高原小镇的安静生活感</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>留意厨房与品鉴供应时间；午餐后在 13:15 左右继续前往瀑布。</x:v>
+        <x:v>这里留给散步与咖啡，不安排长早餐；10:55 左右继续前往鸭嘴兽平台或 Curtain Fig Tree。</x:v>
       </x:c>
       <x:c r="H89" t="str">
-        <x:v>gallo-map,d9-tablelands-route-map</x:v>
+        <x:v>yungaburra-village-map,d9-core-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4184,22 +4184,22 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>14:00–15:15</x:v>
+        <x:v>10:55–11:05 · 可选</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Millaa Millaa Falls / Ellinjaa Falls（可选）</x:v>
+        <x:v>Platypus Viewing Platform Yungaburra（可选）</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>14:00–14:40 欣赏 Millaa Millaa Falls；路况与状态都合适时，14:50–15:15 再到 Ellinjaa Falls 短停</x:v>
+        <x:v>在平台安静观察水面约 10 分钟，看看是否有鸭嘴兽浮出水面</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>高原瀑布与热带绿意</x:v>
+        <x:v>一段看运气的高原动物小插曲</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>Millaa Millaa Falls 是这一段的完整停留；无论是否去 Ellinjaa Falls，都在 15:15 开始返回凯恩斯。</x:v>
+        <x:v>平台仍可使用，但通往 Other Side 的连接步道关闭；没有发现就轻松离开，不沿关闭路段继续走。</x:v>
       </x:c>
       <x:c r="H90" t="str">
-        <x:v>millaa-map,ellinjaa-map,d9-tablelands-route-map</x:v>
+        <x:v>platypus-viewing-platform-map,peterson-creek-tracks-official</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -4210,22 +4210,22 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>15:15–17:45</x:v>
+        <x:v>11:15–11:35</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>返回 Cairns / 凯恩斯还车点</x:v>
+        <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>沿山路返回凯恩斯，途中补满油并按订单时间完成还车</x:v>
+        <x:v>沿短木栈道走到巨型帘状无花果树下，观察垂落气根并拍下人与巨树的尺度</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>在天黑前结束高原自驾</x:v>
+        <x:v>像天然装置艺术般的高原巨树</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>15:15 开始返程，预计 17:00–17:45 完成加油与还车；下山路段留意弯道和野生动物。</x:v>
+        <x:v>木栈道雨后可能湿滑；慢慢绕一圈即可，11:35 左右前往 Gallo Dairyland。</x:v>
       </x:c>
       <x:c r="H91" t="str">
-        <x:v>d9-tablelands-route-map</x:v>
+        <x:v>curtain-fig-map,curtain-fig-official,d9-core-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -4233,155 +4233,155 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B92" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>饮食</x:v>
+        <x:v>11:55–13:15</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Gallo Dairyland</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>早餐：公寓或咖啡馆；午餐：Gallo Dairyland；晚餐：18:30 左右在 Salt House 或公寓附近简餐</x:v>
+        <x:v>在 BB's Café 吃午餐，分享一份奶酪拼盘，再逛逛手工巧克力与农场商店</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>农场午餐与回城晚餐</x:v>
+        <x:v>牧场风景、奶酪与巧克力组成的高原午间</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>午餐留给高原风味，晚餐按还车后的状态轻松选择。</x:v>
+        <x:v>工作日厨房热餐通常供应至 14:00；留出点单和用餐时间，13:15 左右继续向 Millaa Millaa 出发。</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>gallo-map,salt-house-map,southern-cross-map</x:v>
+        <x:v>gallo-map,gallo-hours-official,d9-waterfall-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B93" t="n">
-        <x:v>10</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>08:30–10:30</x:v>
+        <x:v>13:55–14:10</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Rusty's Market</x:v>
+        <x:v>Millaa Millaa Public Toilets</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>逛热带水果、咖啡与早餐摊位，挑选当天可以吃完的水果和轻食</x:v>
+        <x:v>先在镇中心使用公共厕所、补水并短暂舒展，再前往瀑布</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>凯恩斯周五早晨的市场气息</x:v>
+        <x:v>在进入 Waterfall Circuit 前完成实用停靠</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>买少量即可，水果在飞悉尼前吃完；现场营业情况以当天摊位为准。</x:v>
+        <x:v>Millaa Millaa Falls 现场厕所因升级施工关闭；替代公共厕所位于镇中心、Millaa Millaa Hotel 对面。</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>rustys-map,rustys-official</x:v>
+        <x:v>millaa-public-toilets-map,millaa-upgrade-official,d9-waterfall-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B94" t="n">
-        <x:v>20</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>10:45–14:30</x:v>
+        <x:v>14:15–15:00</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Southern Cross Atrium Apartments</x:v>
+        <x:v>Millaa Millaa Falls</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>回公寓洗衣、休息、整理行李，把 Jetstar 托运行李和随身物品分装好</x:v>
+        <x:v>从主观景面欣赏经典单落差瀑布，沿草坪与水潭边取景，在雨林绿意中慢慢走一圈</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>给连续三天自然行程留出恢复时间</x:v>
+        <x:v>阿瑟顿高原最经典的瀑布画面</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>午餐在附近简单解决；泳池、咖啡与午休都留在这段时间里。</x:v>
+        <x:v>停车与步行区域正在升级施工，按现场标志使用开放区域；若在这里下水，下午直接返回 Cairns 会更从容。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>southern-cross-map</x:v>
+        <x:v>millaa-map,millaa-falls-official,millaa-upgrade-official,d9-waterfall-route-map,d9-return-from-millaa-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B95" t="n">
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>15:00–17:30</x:v>
+        <x:v>15:10–15:35 · 可选</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Southern Cross Atrium → Palm Cove</x:v>
+        <x:v>Ellinjaa Falls（可选）</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>15:00 叫 Uber / Didi，约 15:40 抵达；15:40–17:30 沿 Williams Esplanade、Palm Cove Beach 与 Palm Cove Jetty 慢慢散步</x:v>
+        <x:v>从停车与野餐区沿短步道下到瀑布底部，感受更贴近雨林的水声与绿意</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>棕榈树、海岸与热带蓝调前的光线</x:v>
+        <x:v>比主瀑布更安静的第二段雨林瀑布</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>海滩活动以现场旗帜和警示为准；这里更适合散步与拍照，不把下海游泳作为固定安排。</x:v>
+        <x:v>只有在 15:00 前离开 Millaa Millaa Falls、路面与驾驶状态都舒服时前往；15:35 开始返回 Cairns。</x:v>
       </x:c>
       <x:c r="H95" t="str">
-        <x:v>southern-cross-map,palm-cove-map,williams-esplanade-map,palm-cove-jetty-map</x:v>
+        <x:v>ellinjaa-map,ellinjaa-falls-official,d9-return-from-ellinjaa-map</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B96" t="n">
-        <x:v>40</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>17:30–18:45</x:v>
+        <x:v>15:35–18:00</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Palm Cove 早晚餐</x:v>
+        <x:v>返回 Cairns / 凯恩斯还车点</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>在 Williams Esplanade 一带选一家海滨餐厅，边吃晚餐边看天空进入蓝调时刻</x:v>
+        <x:v>经 Malanda、Gillies Highway 与 Gordonvale 返回 Cairns，进城后补满油并按订单地点完成还车</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>凯恩斯段最后一顿海边晚餐</x:v>
+        <x:v>在日落前后结束高原自驾</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>Palm Cove 面向东侧，重点是傍晚天色与棕榈树剪影；19:00 前准备返程。</x:v>
+        <x:v>从 Millaa Millaa Falls 或 Ellinjaa Falls 选择对应返程地图，始终走铺装主路，不接受导航推荐的无铺装林道。Cairns 当日日落约 18:05。</x:v>
       </x:c>
       <x:c r="H96" t="str">
-        <x:v>williams-esplanade-map,palm-cove-map</x:v>
+        <x:v>d9-return-from-millaa-map,d9-return-from-ellinjaa-map,cairns-car-rental-search-map,cairns-sunset-august-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>19:00–21:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Palm Cove → Southern Cross Atrium</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>19:00 叫车返回，预计 19:30–19:45 抵达；20:00–21:00 完成行李称重、Jetstar 在线值机与次日随身包检查</x:v>
+        <x:v>早餐：公寓；午餐：Gallo Dairyland；晚餐：18:30 后在 Salt House 或公寓附近简餐</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>把热带假期从容收进行李箱</x:v>
+        <x:v>农场午餐与回城后的轻松晚餐</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>闹钟、证件、薄外套和机场用物放在手边；21:15–21:30 上床休息。</x:v>
+        <x:v>还车后先回房洗澡休息，晚上不再安排 Night Markets 或 Palm Cove。</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>palm-cove-map,southern-cross-map,cairns-airport-map,jetstar-official</x:v>
+        <x:v>gallo-map,salt-house-map,southern-cross-map</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4389,153 +4389,155 @@
         <x:v>d10</x:v>
       </x:c>
       <x:c r="B98" t="n">
-        <x:v>900</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>饮食</x:v>
+        <x:v>08:30–10:30</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Rusty's Market</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>早餐：Rusty's Market；午餐：公寓附近简餐；晚餐：Palm Cove 海滨早晚餐</x:v>
+        <x:v>逛热带水果、咖啡与早餐摊位，挑选当天可以吃完的水果和轻食</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>市场、水果与海边晚餐组成轻松收尾</x:v>
+        <x:v>凯恩斯周五早晨的市场气息</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>晚餐结束后直接返回凯恩斯，不让次日清晨航班变得匆忙。</x:v>
+        <x:v>买少量即可，水果在飞悉尼前吃完；现场营业情况以当天摊位为准。</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>rustys-map,rustys-official,williams-esplanade-map,palm-cove-map</x:v>
+        <x:v>rustys-map,rustys-official</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B99" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>清晨</x:v>
+        <x:v>10:45–14:30</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>回公寓洗衣、休息、整理行李，把 Jetstar 托运行李和随身物品分装好</x:v>
       </x:c>
       <x:c r="F99" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>给连续三天自然行程留出恢复时间</x:v>
       </x:c>
       <x:c r="G99" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+        <x:v>午餐在附近简单解决；泳池、咖啡与午休都留在这段时间里。</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>cairns-airport-map</x:v>
+        <x:v>southern-cross-map</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B100" t="n">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>上午</x:v>
+        <x:v>15:00–17:30</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>凯恩斯 → 悉尼</x:v>
+        <x:v>Southern Cross Atrium → Palm Cove</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>15:00 叫 Uber / Didi，约 15:40 抵达；15:40–17:30 沿 Williams Esplanade、Palm Cove Beach 与 Palm Cove Jetty 慢慢散步</x:v>
       </x:c>
       <x:c r="F100" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>棕榈树、海岸与热带蓝调前的光线</x:v>
       </x:c>
       <x:c r="G100" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H100"/>
+        <x:v>海滩活动以现场旗帜和警示为准；这里更适合散步与拍照，不把下海游泳作为固定安排。</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>southern-cross-map,palm-cove-map,williams-esplanade-map,palm-cove-jetty-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B101" t="n">
-        <x:v>30</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>17:30–18:45</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>Palm Cove 早晚餐</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>在 Williams Esplanade 一带选一家海滨餐厅，边吃晚餐边看天空进入蓝调时刻</x:v>
       </x:c>
       <x:c r="F101" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>凯恩斯段最后一顿海边晚餐</x:v>
       </x:c>
       <x:c r="G101" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
+        <x:v>Palm Cove 面向东侧，重点是傍晚天色与棕榈树剪影；19:00 前准备返程。</x:v>
       </x:c>
       <x:c r="H101" t="str">
-        <x:v>oaks-sydney-map</x:v>
+        <x:v>williams-esplanade-map,palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B102" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>下午</x:v>
+        <x:v>19:00–21:30</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>Palm Cove → Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>19:00 叫车返回，预计 19:30–19:45 抵达；20:00–21:00 完成行李称重、Jetstar 在线值机与次日随身包检查</x:v>
       </x:c>
       <x:c r="F102" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>把热带假期从容收进行李箱</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>闹钟、证件、薄外套和机场用物放在手边；21:15–21:30 上床休息。</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>palm-cove-map,southern-cross-map,cairns-airport-map,jetstar-official</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B103" t="n">
-        <x:v>45</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>早餐：Rusty's Market；午餐：公寓附近简餐；晚餐：Palm Cove 海滨早晚餐</x:v>
       </x:c>
       <x:c r="F103" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>市场、水果与海边晚餐组成轻松收尾</x:v>
       </x:c>
       <x:c r="G103" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>晚餐结束后直接返回凯恩斯，不让次日清晨航班变得匆忙。</x:v>
       </x:c>
       <x:c r="H103" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>rustys-map,rustys-official,williams-esplanade-map,palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -4543,25 +4545,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B104" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F104" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
+        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
       </x:c>
       <x:c r="H104" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>cairns-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -4569,181 +4571,179 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B105" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>晚上</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F105" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>从热带切换回冬季海港城市</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
-      </x:c>
-      <x:c r="H105" t="str">
-        <x:v>circular-quay-map</x:v>
-      </x:c>
+        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
+      </x:c>
+      <x:c r="H105"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" t="str">
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B106" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>饮食</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>悉尼 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>4人 + 行李，打车最省心</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
+        <x:v>如不能入住，先寄存行李</x:v>
       </x:c>
       <x:c r="H106" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B107" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>Darling Harbour / 酒店周边</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F107" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H107" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B108" t="n">
-        <x:v>20</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
       </x:c>
       <x:c r="F108" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G108" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H108" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B109" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F109" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G109" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H109" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B110" t="n">
-        <x:v>40</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
+        <x:v>歌剧院、海港大桥夜景</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B111" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
+        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H111" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -4751,25 +4751,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B112" t="n">
-        <x:v>60</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>08:15–08:30</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>抵达海港区</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>Ferry、海港桥、歌剧院远景</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -4777,25 +4777,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B113" t="n">
-        <x:v>70</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>08:30–09:10</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Royal Botanic Garden</x:v>
+        <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>悉尼核心地标</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -4803,25 +4803,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>80</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>中文内部导览已订</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>建筑故事、内部空间、剧院结构</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -4829,25 +4829,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>90</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>10:30–10:50</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>Opera House → The Rocks</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>海港步行衔接悉尼老城区</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -4855,25 +4855,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>100</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>晚上</x:v>
+        <x:v>10:50–11:50</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -4881,155 +4881,155 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>饮食</x:v>
+        <x:v>11:50–12:40</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>就地补体力，不为午餐绕路</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>10</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>08:00</x:v>
+        <x:v>12:40–14:10</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>植物园海港步道</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>botanic-garden-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>20</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>09:15</x:v>
+        <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>歌剧院 + 海港大桥同框</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>悉尼最经典机位</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>mrs-macquarie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>30</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>10:00</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>购物、室内休息</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>建筑漂亮，适合逛</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>40</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>11:15</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>CBD / Darling Harbour</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>Hello Auntie / CBD 晚餐</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>12:00</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -5037,25 +5037,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>60</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>royal-national-park-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -5063,25 +5063,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>70</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>13:30</x:v>
+        <x:v>09:15</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>南海岸第一处全景</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>bald-hill-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -5089,25 +5089,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>80</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>10:00</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>贴着太平洋的公路画面</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>不要在桥上或路肩危险停车</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -5115,25 +5115,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>90</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>14:40</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Wollongong / 南海岸补给</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>短停咖啡或直接通过</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>wollongong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -5141,25 +5141,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>100</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>Kiama Blowhole</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>看喷潮洞、灯塔与海边</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>Kiama 代表性海岸地貌</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -5167,25 +5167,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>110</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>12:30–13:30</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>海边小镇节奏</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -5193,155 +5193,155 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>900</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>饮食</x:v>
+        <x:v>13:30</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Kiama → Gerringong</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>沿海继续南下</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kiama-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>10</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>13:45–14:40</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>20</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>14:40</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>Gerringong</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>判断是否延伸 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>时间、天气与体力闸门</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>gerringong-map,kangaroo-valley-map</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>30</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>可选 15:30–16:15</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>看历史桥、山谷与小镇</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>40</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>16:15 前</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>环线收束</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -5349,25 +5349,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>60</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>18:30</x:v>
+        <x:v>08:30–09:00</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -5375,155 +5375,155 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B136" t="n">
-        <x:v>900</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>饮食</x:v>
+        <x:v>09:15 左右</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B137" t="n">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>上午</x:v>
+        <x:v>09:30–13:30</x:v>
       </x:c>
       <x:c r="D137" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F137" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B138" t="n">
-        <x:v>20</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>13:30–14:30</x:v>
       </x:c>
       <x:c r="D138" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
       </x:c>
       <x:c r="E138" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>F2 返回市区后前往 Bondi</x:v>
       </x:c>
       <x:c r="F138" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>动物园切换到悉尼海岸</x:v>
       </x:c>
       <x:c r="G138" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
       </x:c>
       <x:c r="H138" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B139" t="n">
-        <x:v>30</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>14:30–17:45</x:v>
       </x:c>
       <x:c r="D139" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E139" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>海滩散步并走一段 Coastal Walk</x:v>
       </x:c>
       <x:c r="F139" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G139" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H139" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B140" t="n">
-        <x:v>40</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C140" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>18:30</x:v>
       </x:c>
       <x:c r="D140" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E140" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F140" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G140" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
       </x:c>
       <x:c r="H140" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B141" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C141" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D141" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E141" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F141" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G141" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H141" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
@@ -5531,25 +5531,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B142" t="n">
-        <x:v>60</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C142" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D142" t="str">
-        <x:v>酒店</x:v>
+        <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E142" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F142" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G142" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H142" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>oaks-sydney-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -5557,25 +5557,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B143" t="n">
-        <x:v>70</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C143" t="str">
-        <x:v>16:40</x:v>
+        <x:v>可选 09:30 左右</x:v>
       </x:c>
       <x:c r="D143" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Circular Quay → Manly</x:v>
       </x:c>
       <x:c r="E143" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>搭乘公共 F1 Manly Ferry</x:v>
       </x:c>
       <x:c r="F143" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H143" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>circular-quay-map,manly-ferry-map</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -5583,25 +5583,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B144" t="n">
-        <x:v>80</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C144" t="str">
-        <x:v>17:30</x:v>
+        <x:v>可选 10:00–12:45</x:v>
       </x:c>
       <x:c r="D144" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>Manly Beach / The Corso</x:v>
       </x:c>
       <x:c r="E144" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>海边散步、咖啡或早午餐</x:v>
       </x:c>
       <x:c r="F144" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G144" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H144" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -5609,76 +5609,206 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B145" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C145" t="str">
-        <x:v>饮食</x:v>
+        <x:v>13:00–13:30</x:v>
       </x:c>
       <x:c r="D145" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Manly → Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E145" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>最晚搭船回市区</x:v>
       </x:c>
       <x:c r="F145" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G145" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H145" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" t="str">
-        <x:v>d16</x:v>
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B146" t="n">
-        <x:v>10</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C146" t="str">
-        <x:v>上午</x:v>
+        <x:v>14:00–15:30</x:v>
       </x:c>
       <x:c r="D146" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
       </x:c>
       <x:c r="E146" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>最后采购</x:v>
       </x:c>
       <x:c r="F146" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>药妆、保健品、伴手礼</x:v>
       </x:c>
       <x:c r="G146" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
       </x:c>
       <x:c r="H146" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B147" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>15:30–16:20</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>酒店</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>整理 TRS 物品和返程行李</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>为 D16 机场退税做准备</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>oaks-sydney-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B148" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>16:40</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E148" t="str">
+        <x:v>前往 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="F148" t="str">
+        <x:v>避免迟到</x:v>
+      </x:c>
+      <x:c r="G148" t="str">
+        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+      </x:c>
+      <x:c r="H148" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B149" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>17:30</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="E149" t="str">
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+      </x:c>
+      <x:c r="F149" t="str">
+        <x:v>海港景观 + 澳洲最后一晚</x:v>
+      </x:c>
+      <x:c r="G149" t="str">
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+      </x:c>
+      <x:c r="H149" t="str">
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B150" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E150" t="str">
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="F150" t="str">
+        <x:v>当天餐食节奏</x:v>
+      </x:c>
+      <x:c r="G150" t="str">
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+      </x:c>
+      <x:c r="H150" t="str">
+        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
         <x:v>d16</x:v>
       </x:c>
-      <x:c r="B147" t="n">
+      <x:c r="B151" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B152" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C147" t="str">
+      <x:c r="C152" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D147" t="str">
+      <x:c r="D152" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E147" t="str">
+      <x:c r="E152" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F147" t="str">
+      <x:c r="F152" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G147" t="str">
+      <x:c r="G152" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H147"/>
+      <x:c r="H152"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8721,8 +8851,8 @@
       <x:c r="D159" t="str">
         <x:v>https://www.cairns.qld.gov.au/council/news-notices/news/media-releases/esplanade-lagoon-to-close-for-essential-maintenance</x:v>
       </x:c>
-      <x:c r="E159" t="str"/>
-      <x:c r="F159" t="str"/>
+      <x:c r="E159"/>
+      <x:c r="F159"/>
       <x:c r="G159" t="str">
         <x:v>Cairns Regional Council · 2026 年 7 月 13 日至 8 月 16 日维护关闭</x:v>
       </x:c>
@@ -8740,8 +8870,8 @@
       <x:c r="D160" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+Botanic+Gardens</x:v>
       </x:c>
-      <x:c r="E160" t="str"/>
-      <x:c r="F160" t="str"/>
+      <x:c r="E160"/>
+      <x:c r="F160"/>
       <x:c r="G160" t="str">
         <x:v>Google Maps · Cairns Botanic Gardens</x:v>
       </x:c>
@@ -8759,8 +8889,8 @@
       <x:c r="D161" t="str">
         <x:v>https://www.cairns.qld.gov.au/experience-cairns/botanic-gardens</x:v>
       </x:c>
-      <x:c r="E161" t="str"/>
-      <x:c r="F161" t="str"/>
+      <x:c r="E161"/>
+      <x:c r="F161"/>
       <x:c r="G161" t="str">
         <x:v>Cairns Regional Council · Flecker Garden 每日 07:30–17:30 免费开放</x:v>
       </x:c>
@@ -8778,8 +8908,8 @@
       <x:c r="D162" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+CBD+Queensland</x:v>
       </x:c>
-      <x:c r="E162" t="str"/>
-      <x:c r="F162" t="str"/>
+      <x:c r="E162"/>
+      <x:c r="F162"/>
       <x:c r="G162" t="str">
         <x:v>Google Maps · Cairns CBD</x:v>
       </x:c>
@@ -8797,8 +8927,8 @@
       <x:c r="D163" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+Esplanade+Boardwalk</x:v>
       </x:c>
-      <x:c r="E163" t="str"/>
-      <x:c r="F163" t="str"/>
+      <x:c r="E163"/>
+      <x:c r="F163"/>
       <x:c r="G163" t="str">
         <x:v>Google Maps · Cairns Esplanade Boardwalk</x:v>
       </x:c>
@@ -8816,8 +8946,8 @@
       <x:c r="D164" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cairns+Marlin+Marina</x:v>
       </x:c>
-      <x:c r="E164" t="str"/>
-      <x:c r="F164" t="str"/>
+      <x:c r="E164"/>
+      <x:c r="F164"/>
       <x:c r="G164" t="str">
         <x:v>Google Maps · Cairns Marlin Marina</x:v>
       </x:c>
@@ -8835,8 +8965,8 @@
       <x:c r="D165" t="str">
         <x:v>https://www.nightmarkets.com.au/faq</x:v>
       </x:c>
-      <x:c r="E165" t="str"/>
-      <x:c r="F165" t="str"/>
+      <x:c r="E165"/>
+      <x:c r="F165"/>
       <x:c r="G165" t="str">
         <x:v>Cairns Night Markets · 市场摊位每日 16:30 起营业</x:v>
       </x:c>
@@ -8854,8 +8984,8 @@
       <x:c r="D166" t="str">
         <x:v>https://www.reefmagic.com.au/faqs/</x:v>
       </x:c>
-      <x:c r="E166" t="str"/>
-      <x:c r="F166" t="str"/>
+      <x:c r="E166"/>
+      <x:c r="F166"/>
       <x:c r="G166" t="str">
         <x:v>Reef Magic · 08:15 登船、08:45 最晚登船、09:00 离港、17:00 返回</x:v>
       </x:c>
@@ -8873,8 +9003,8 @@
       <x:c r="D167" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Lake+Eacham%7CCurtain+Fig+Tree%7CYungaburra%7CGallo+Dairyland%7CMillaa+Millaa+Falls</x:v>
       </x:c>
-      <x:c r="E167" t="str"/>
-      <x:c r="F167" t="str"/>
+      <x:c r="E167"/>
+      <x:c r="F167"/>
       <x:c r="G167" t="str">
         <x:v>Google Maps · Cairns → Lake Eacham → Curtain Fig Tree → Yungaburra → Gallo Dairyland → Millaa Millaa Falls → Cairns</x:v>
       </x:c>
@@ -8892,8 +9022,8 @@
       <x:c r="D168" t="str">
         <x:v>https://rustysmarkets.com.au/location/</x:v>
       </x:c>
-      <x:c r="E168" t="str"/>
-      <x:c r="F168" t="str"/>
+      <x:c r="E168"/>
+      <x:c r="F168"/>
       <x:c r="G168" t="str">
         <x:v>Rusty's Markets · 周五、周六、周日开放</x:v>
       </x:c>
@@ -8911,8 +9041,8 @@
       <x:c r="D169" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Williams+Esplanade+Palm+Cove</x:v>
       </x:c>
-      <x:c r="E169" t="str"/>
-      <x:c r="F169" t="str"/>
+      <x:c r="E169"/>
+      <x:c r="F169"/>
       <x:c r="G169" t="str">
         <x:v>Google Maps · Williams Esplanade, Palm Cove</x:v>
       </x:c>
@@ -8930,10 +9060,352 @@
       <x:c r="D170" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Palm+Cove+Jetty</x:v>
       </x:c>
-      <x:c r="E170" t="str"/>
-      <x:c r="F170" t="str"/>
+      <x:c r="E170"/>
+      <x:c r="F170"/>
       <x:c r="G170" t="str">
         <x:v>Google Maps · Palm Cove Jetty</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>cairns-car-rental-search-map</x:v>
+      </x:c>
+      <x:c r="B171" t="str">
+        <x:v>Cairns 租车门店搜索</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Car+Rental+Cairns+QLD</x:v>
+      </x:c>
+      <x:c r="E171" t="str"/>
+      <x:c r="F171" t="str"/>
+      <x:c r="G171" t="str">
+        <x:v>Google Maps · 准确门店以租车订单为准</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>d9-core-route-map</x:v>
+      </x:c>
+      <x:c r="B172" t="str">
+        <x:v>D9 阿瑟顿高原核心环线</x:v>
+      </x:c>
+      <x:c r="C172" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D172" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Lake+Eacham+Day+Use+Area%7CYungaburra+Village%7CCurtain+Fig+Tree%7CGallo+Dairyland%7CMillaa+Millaa+Public+Toilets%7CMillaa+Millaa+Falls</x:v>
+      </x:c>
+      <x:c r="E172" t="str"/>
+      <x:c r="F172" t="str"/>
+      <x:c r="G172" t="str">
+        <x:v>Google Maps · Cairns → Lake Eacham → Yungaburra → Curtain Fig → Gallo → Millaa Millaa 镇 → 主瀑布 → Cairns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" t="str">
+        <x:v>d9-cairns-lake-eacham-route-map</x:v>
+      </x:c>
+      <x:c r="B173" t="str">
+        <x:v>Cairns → Lake Eacham</x:v>
+      </x:c>
+      <x:c r="C173" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D173" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Lake+Eacham+Day+Use+Area&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E173" t="str"/>
+      <x:c r="F173" t="str"/>
+      <x:c r="G173" t="str">
+        <x:v>Google Maps · 经 Gordonvale 与 Gillies Highway</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>d9-waterfall-route-map</x:v>
+      </x:c>
+      <x:c r="B174" t="str">
+        <x:v>Gallo → Millaa Millaa 瀑布段</x:v>
+      </x:c>
+      <x:c r="C174" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D174" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Gallo+Dairyland&amp;destination=Ellinjaa+Falls&amp;travelmode=driving&amp;waypoints=Millaa+Millaa+Public+Toilets%7CMillaa+Millaa+Falls</x:v>
+      </x:c>
+      <x:c r="E174" t="str"/>
+      <x:c r="F174" t="str"/>
+      <x:c r="G174" t="str">
+        <x:v>Google Maps · Gallo → 镇中心厕所 → Millaa Millaa Falls → Ellinjaa Falls</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" t="str">
+        <x:v>d9-return-from-millaa-map</x:v>
+      </x:c>
+      <x:c r="B175" t="str">
+        <x:v>Millaa Millaa Falls → Cairns</x:v>
+      </x:c>
+      <x:c r="C175" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D175" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Millaa+Millaa+Falls&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Malanda+QLD%7CGordonvale+QLD</x:v>
+      </x:c>
+      <x:c r="E175" t="str"/>
+      <x:c r="F175" t="str"/>
+      <x:c r="G175" t="str">
+        <x:v>Google Maps · 经 Malanda、Gillies Highway 与 Gordonvale 返回</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" t="str">
+        <x:v>d9-return-from-ellinjaa-map</x:v>
+      </x:c>
+      <x:c r="B176" t="str">
+        <x:v>Ellinjaa Falls → Cairns</x:v>
+      </x:c>
+      <x:c r="C176" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D176" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Ellinjaa+Falls&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Malanda+QLD%7CGordonvale+QLD</x:v>
+      </x:c>
+      <x:c r="E176" t="str"/>
+      <x:c r="F176" t="str"/>
+      <x:c r="G176" t="str">
+        <x:v>Google Maps · 经 Malanda、Gillies Highway 与 Gordonvale 返回</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" t="str">
+        <x:v>lake-eacham-day-use-map</x:v>
+      </x:c>
+      <x:c r="B177" t="str">
+        <x:v>Lake Eacham Day Use Area</x:v>
+      </x:c>
+      <x:c r="C177" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D177" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Lake+Eacham+Day+Use+Area%2C+Lakes+Drive%2C+Lake+Eacham+QLD</x:v>
+      </x:c>
+      <x:c r="E177" t="str"/>
+      <x:c r="F177" t="str"/>
+      <x:c r="G177" t="str">
+        <x:v>Google Maps · Lakes Drive, Lake Eacham</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" t="str">
+        <x:v>lake-eacham-official</x:v>
+      </x:c>
+      <x:c r="B178" t="str">
+        <x:v>Lake Eacham Day Use Area 官方信息</x:v>
+      </x:c>
+      <x:c r="C178" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D178" t="str">
+        <x:v>https://parks.qld.gov.au/parks/crater-lakes/attractions/lake-eacham-day-use-area</x:v>
+      </x:c>
+      <x:c r="E178" t="str"/>
+      <x:c r="F178" t="str"/>
+      <x:c r="G178" t="str">
+        <x:v>Queensland Parks · 距 Cairns 约 68 km，铺装路适合普通车辆，全天开放</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" t="str">
+        <x:v>yungaburra-village-map</x:v>
+      </x:c>
+      <x:c r="B179" t="str">
+        <x:v>Yungaburra Village</x:v>
+      </x:c>
+      <x:c r="C179" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D179" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Yungaburra+Village+QLD</x:v>
+      </x:c>
+      <x:c r="E179" t="str"/>
+      <x:c r="F179" t="str"/>
+      <x:c r="G179" t="str">
+        <x:v>Google Maps · Yungaburra Village</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" t="str">
+        <x:v>platypus-viewing-platform-map</x:v>
+      </x:c>
+      <x:c r="B180" t="str">
+        <x:v>Platypus Viewing Platform Yungaburra</x:v>
+      </x:c>
+      <x:c r="C180" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D180" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Platypus+Viewing+Platform+Yungaburra</x:v>
+      </x:c>
+      <x:c r="E180" t="str"/>
+      <x:c r="F180" t="str"/>
+      <x:c r="G180" t="str">
+        <x:v>Google Maps · Peterson Creek Platypus Viewing Platform</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" t="str">
+        <x:v>peterson-creek-tracks-official</x:v>
+      </x:c>
+      <x:c r="B181" t="str">
+        <x:v>Peterson Creek 步道与平台信息</x:v>
+      </x:c>
+      <x:c r="C181" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D181" t="str">
+        <x:v>https://petersoncreek.org.au/walking-tracks/</x:v>
+      </x:c>
+      <x:c r="E181" t="str"/>
+      <x:c r="F181" t="str"/>
+      <x:c r="G181" t="str">
+        <x:v>Yungaburra Landcare Group · 平台可用，平台至 Other Side 的连接步道关闭</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" t="str">
+        <x:v>curtain-fig-official</x:v>
+      </x:c>
+      <x:c r="B182" t="str">
+        <x:v>Curtain Fig National Park 官方信息</x:v>
+      </x:c>
+      <x:c r="C182" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D182" t="str">
+        <x:v>https://parks.qld.gov.au/parks/curtain-fig</x:v>
+      </x:c>
+      <x:c r="E182" t="str"/>
+      <x:c r="F182" t="str"/>
+      <x:c r="G182" t="str">
+        <x:v>Queensland Parks · 高架木栈道环绕 Curtain Fig Tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" t="str">
+        <x:v>gallo-hours-official</x:v>
+      </x:c>
+      <x:c r="B183" t="str">
+        <x:v>Gallo Dairyland 午餐信息</x:v>
+      </x:c>
+      <x:c r="C183" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D183" t="str">
+        <x:v>https://www.athertontablelands.com.au/travel-directory/gallo-dairyland/</x:v>
+      </x:c>
+      <x:c r="E183" t="str"/>
+      <x:c r="F183" t="str"/>
+      <x:c r="G183" t="str">
+        <x:v>Tourism Atherton Tablelands · 工作日厨房热餐通常 09:30–14:00</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" t="str">
+        <x:v>millaa-public-toilets-map</x:v>
+      </x:c>
+      <x:c r="B184" t="str">
+        <x:v>Millaa Millaa Public Toilets</x:v>
+      </x:c>
+      <x:c r="C184" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D184" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Millaa+Millaa+Public+Toilets%2C+Main+Street%2C+Millaa+Millaa+QLD</x:v>
+      </x:c>
+      <x:c r="E184" t="str"/>
+      <x:c r="F184" t="str"/>
+      <x:c r="G184" t="str">
+        <x:v>Google Maps · 镇中心，Millaa Millaa Hotel 对面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" t="str">
+        <x:v>millaa-upgrade-official</x:v>
+      </x:c>
+      <x:c r="B185" t="str">
+        <x:v>Millaa Millaa Falls 施工更新</x:v>
+      </x:c>
+      <x:c r="C185" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D185" t="str">
+        <x:v>https://www.trc.qld.gov.au/our-council/projects/millaa-millaa-falls-upgrade/</x:v>
+      </x:c>
+      <x:c r="E185" t="str"/>
+      <x:c r="F185" t="str"/>
+      <x:c r="G185" t="str">
+        <x:v>Tablelands Regional Council · 2026 年 7 月起施工，停车和步行区域受影响，现场厕所停用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" t="str">
+        <x:v>millaa-falls-official</x:v>
+      </x:c>
+      <x:c r="B186" t="str">
+        <x:v>Millaa Millaa Falls 官方旅游信息</x:v>
+      </x:c>
+      <x:c r="C186" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D186" t="str">
+        <x:v>https://www.queensland.com/au/en/things-to-do/attractions/p-56b25fd67b935fbe730df3b1-millaa-millaa-falls</x:v>
+      </x:c>
+      <x:c r="E186" t="str"/>
+      <x:c r="F186" t="str"/>
+      <x:c r="G186" t="str">
+        <x:v>Tourism and Events Queensland · Waterfalls Circuit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" t="str">
+        <x:v>ellinjaa-falls-official</x:v>
+      </x:c>
+      <x:c r="B187" t="str">
+        <x:v>Ellinjaa Falls 步道信息</x:v>
+      </x:c>
+      <x:c r="C187" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D187" t="str">
+        <x:v>https://www.athertontablelands.com.au/travel-directory/elinjaa-falls-millaa-millaa/</x:v>
+      </x:c>
+      <x:c r="E187" t="str"/>
+      <x:c r="F187" t="str"/>
+      <x:c r="G187" t="str">
+        <x:v>Tourism Atherton Tablelands · 从停车与野餐区沿步道下到瀑布底部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" t="str">
+        <x:v>cairns-sunset-august-2026</x:v>
+      </x:c>
+      <x:c r="B188" t="str">
+        <x:v>Cairns 2026 年 8 月日落时间</x:v>
+      </x:c>
+      <x:c r="C188" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="D188" t="str">
+        <x:v>https://www.timeanddate.com/sun/australia/cairns?month=8</x:v>
+      </x:c>
+      <x:c r="E188" t="str"/>
+      <x:c r="F188" t="str"/>
+      <x:c r="G188" t="str">
+        <x:v>Timeanddate · 2026 年 8 月 6 日日落约 18:05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
update D9 Kuranda Skybury route
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R0770be89d65e4a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R658f7356b93f4292"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Ra69ca48cab7e4864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R7f5a3ee70a384c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R3f8f2ca273ca4ccd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rbdfcc6d86ff4481d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Ra4d6a9dd09c243c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R6cdef1af7c214b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R2c1d98f50d8746be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R6f9f43abd5084a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rc8061742401442c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R921bb94272c14fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Ra0f3b31856e048bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R28b5f28c18c3485c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rae8a01e45d5c4975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rf01a54bb81324a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Ra8bbf3ff94f5428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Re563cd4ccc284873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R5ed7e048d1d14c85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Ra0f6339450414c90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,7 +1208,7 @@
         <x:v>周四</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>阿瑟顿高原</x:v>
+        <x:v>Kuranda + 阿瑟顿高原</x:v>
       </x:c>
       <x:c r="F11" t="n">
         <x:v>-17.2706</x:v>
@@ -1217,16 +1217,16 @@
         <x:v>145.5831</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>穿行阿瑟顿高原：火山湖、巨树与瀑布</x:v>
+        <x:v>从雨林小镇到高原瀑布：Kuranda、Skybury 与 Millaa Millaa</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>从 Cairns 驶上阿瑟顿高原，在 Lake Eacham 看火山湖，沿 Yungaburra 与 Curtain Fig Tree 走进高原风景，午后到 Gallo Dairyland 吃午餐，再以 Millaa Millaa Falls 收尾。</x:v>
+        <x:v>从 Cairns 沿 Kuranda Range 北上，经过 Kuranda 与 Mareeba，在 Skybury 看咖啡园景并享用早午餐；下午走过 Lake Eacham、Yungaburra 与 Curtain Fig Tree，最后以 Millaa Millaa Falls 收尾。</x:v>
       </x:c>
       <x:c r="J11" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>高原清晨约 10–15°C，中午约 22–26°C；天气与体感会随海拔变化。</x:v>
+        <x:v>Kuranda 与高原清晨偏凉，Mareeba 白天较暖；天气和体感会随海拔与林区变化。</x:v>
       </x:c>
       <x:c r="L11" t="str">
         <x:v>短袖打底 + 薄外套 + 轻薄长裤 + 防滑运动鞋；车里备雨衣、帽子、墨镜与防晒。</x:v>
@@ -1238,10 +1238,10 @@
         <x:v>阿瑟顿高原瀑布</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>自驾 · 阿瑟顿高原环线（约 230–260 km；纯驾驶约 4–4.5 小时；全天约 9 小时）</x:v>
+        <x:v>自驾 · Kuranda / Mareeba / 阿瑟顿高原环线（约 285 km；纯驾驶约 5 小时；全天约 9.5–10 小时）</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>07:45 前往取车点；08:30 前驶离 Cairns；13:15 离开 Gallo；15:35 开始返程</x:v>
+        <x:v>08:00 左右驶离 Cairns；11:30 离开 Skybury；15:35 从 Millaa Millaa Falls 返程</x:v>
       </x:c>
       <x:c r="Q11" t="str">
         <x:v>southern-cross-map</x:v>
@@ -4054,7 +4054,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>07:15–07:45</x:v>
+        <x:v>07:15–07:35</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -4063,7 +4063,7 @@
         <x:v>吃早餐、装好饮用水，检查驾照、租车订单与充电线，并把当天区域下载到 Google Maps 离线地图</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>从一段从容准备开启高原自驾</x:v>
+        <x:v>从一段从容准备开启高原环线</x:v>
       </x:c>
       <x:c r="G85" t="str">
         <x:v>每人带约 1L 水和一份小零食；薄外套、轻薄雨衣、帽子、墨镜、防晒与纸巾放在随手可取的位置。</x:v>
@@ -4080,7 +4080,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>07:45–08:30</x:v>
+        <x:v>07:35–08:00 · 按订单时间</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>凯恩斯取车点</x:v>
@@ -4089,13 +4089,13 @@
         <x:v>前往租车订单上的准确门店，取车后拍下车身四角、轮毂、挡风玻璃与油表，再调好座椅、后视镜和手机支架</x:v>
       </x:c>
       <x:c r="F86" t="str">
-        <x:v>在驶入 Gillies Highway 前熟悉车辆</x:v>
+        <x:v>在驶入 Kuranda Range 前熟悉车辆</x:v>
       </x:c>
       <x:c r="G86" t="str">
-        <x:v>导航以订单中的准确 branch 为准；离店前再次确认还车地点、油量规则与时间，08:30 前驶离 Cairns。</x:v>
+        <x:v>实际取车时间以订单为准；能在 08:00 左右驶离 Cairns 最从容，若稍晚出发，就把 Kuranda 与 Mareeba 各控制在 15–20 分钟。</x:v>
       </x:c>
       <x:c r="H86" t="str">
-        <x:v>cairns-car-rental-search-map,d9-core-route-map</x:v>
+        <x:v>cairns-car-rental-search-map,d9-north-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4106,22 +4106,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>08:30–09:40</x:v>
+        <x:v>08:00–08:40</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Cairns → Lake Eacham</x:v>
+        <x:v>Cairns → Kuranda Village</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>经 Gordonvale 与 Gillies Highway 驶上高原，沿铺装道路前往 Lake Eacham Day Use Area</x:v>
+        <x:v>沿 Kennedy Highway 驶上 Kuranda Range，穿过雨林山路前往 Kuranda Village</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>海边城市逐渐切换成清凉高原</x:v>
+        <x:v>从海边城市缓缓进入雨林高地</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>Gillies Highway 弯道密集，保持舒服车距；只在安全让车区让快车通过，不跟着后车加速。</x:v>
+        <x:v>山路弯道较多，保持舒服车距，只在安全让车区让快车通过；司机专心驾驶，副驾负责导航。</x:v>
       </x:c>
       <x:c r="H87" t="str">
-        <x:v>d9-cairns-lake-eacham-route-map,lake-eacham-official</x:v>
+        <x:v>d9-north-route-map,kuranda-village-map</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4132,22 +4132,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>09:40–10:20</x:v>
+        <x:v>08:40–09:15</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Lake Eacham Day Use Area</x:v>
+        <x:v>Kuranda Village</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>到湖边观景台看火山湖与雨林倒影，再沿湖边步道轻松走一小段</x:v>
+        <x:v>沿 Coondoo Street 一带短走，看看雨林小镇街景、老建筑与清晨开门的小店</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>被雨林环抱的清澈火山湖</x:v>
+        <x:v>雨林包围的小镇清晨</x:v>
       </x:c>
       <x:c r="G88" t="str">
-        <x:v>今天不完整环湖，也不安排游泳；沿成形步道行走，10:20 左右继续前往 Yungaburra。</x:v>
+        <x:v>今天不安排缆车或长时间逛市场；停留约 35 分钟，把咖啡与正式用餐留给 Skybury。</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>lake-eacham-day-use-map,lake-eacham-official,d9-core-route-map</x:v>
+        <x:v>kuranda-village-map,d9-north-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4158,22 +4158,22 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>10:30–10:55</x:v>
+        <x:v>09:15–09:45</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Yungaburra Village</x:v>
+        <x:v>Kuranda → Mareeba</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>沿老街短走，看看历史木屋、高原小店与街景，需要时买一杯咖啡</x:v>
+        <x:v>沿 Kennedy Highway 继续向西北行驶，从湿润雨林逐渐进入开阔高原</x:v>
       </x:c>
       <x:c r="F89" t="str">
-        <x:v>高原小镇的安静生活感</x:v>
+        <x:v>沿途景观从雨林切换为热带草原</x:v>
       </x:c>
       <x:c r="G89" t="str">
-        <x:v>这里留给散步与咖啡，不安排长早餐；10:55 左右继续前往鸭嘴兽平台或 Curtain Fig Tree。</x:v>
+        <x:v>这一段约 28 分钟；不临时驶入小路，把 Mareeba 作为轻松的中途短停。</x:v>
       </x:c>
       <x:c r="H89" t="str">
-        <x:v>yungaburra-village-map,d9-core-route-map</x:v>
+        <x:v>d9-north-route-map,mareeba-town-map</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4184,22 +4184,22 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>10:55–11:05 · 可选</x:v>
+        <x:v>09:45–10:05</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Platypus Viewing Platform Yungaburra（可选）</x:v>
+        <x:v>Mareeba</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>在平台安静观察水面约 10 分钟，看看是否有鸭嘴兽浮出水面</x:v>
+        <x:v>在镇中心短走、使用洗手间并舒展一下，再确认油量和下一段导航</x:v>
       </x:c>
       <x:c r="F90" t="str">
-        <x:v>一段看运气的高原动物小插曲</x:v>
+        <x:v>咖啡产区入口的一段小镇停靠</x:v>
       </x:c>
       <x:c r="G90" t="str">
-        <x:v>平台仍可使用，但通往 Other Side 的连接步道关闭；没有发现就轻松离开，不沿关闭路段继续走。</x:v>
+        <x:v>这里以 20 分钟短停为主，不再安排完整早餐；10:05 左右继续前往 Skybury。</x:v>
       </x:c>
       <x:c r="H90" t="str">
-        <x:v>platypus-viewing-platform-map,peterson-creek-tracks-official</x:v>
+        <x:v>mareeba-town-map,d9-north-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -4210,22 +4210,22 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>11:15–11:35</x:v>
+        <x:v>10:05–10:20</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Curtain Fig Tree</x:v>
+        <x:v>Mareeba → Skybury</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>沿短木栈道走到巨型帘状无花果树下，观察垂落气根并拍下人与巨树的尺度</x:v>
+        <x:v>从 Mareeba 驶向 Paddys Green，沿 Ivicevic Road 前往 Skybury Cafe &amp; Roastery</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>像天然装置艺术般的高原巨树</x:v>
+        <x:v>从高原小镇进入咖啡农场风景</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>木栈道雨后可能湿滑；慢慢绕一圈即可，11:35 左右前往 Gallo Dairyland。</x:v>
+        <x:v>最后一段约 12 分钟；接近农场后放慢车速，按现场标志进入停车区。</x:v>
       </x:c>
       <x:c r="H91" t="str">
-        <x:v>curtain-fig-map,curtain-fig-official,d9-core-route-map</x:v>
+        <x:v>d9-north-route-map,skybury-map</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -4236,22 +4236,22 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>11:55–13:15</x:v>
+        <x:v>10:20–11:30</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Gallo Dairyland</x:v>
+        <x:v>Skybury Cafe &amp; Roastery</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>在 BB's Café 吃午餐，分享一份奶酪拼盘，再逛逛手工巧克力与农场商店</x:v>
+        <x:v>坐下来喝一杯本地咖啡，享用早午餐，再看看农场与高原景观</x:v>
       </x:c>
       <x:c r="F92" t="str">
-        <x:v>牧场风景、奶酪与巧克力组成的高原午间</x:v>
+        <x:v>咖啡产区最有地方感的一餐</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>工作日厨房热餐通常供应至 14:00；留出点单和用餐时间，13:15 左右继续向 Millaa Millaa 出发。</x:v>
+        <x:v>官网列周一至周五 09:00–16:00；今天留约 70 分钟，用餐后可买少量咖啡豆或木瓜产品，11:30 左右离开。</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>gallo-map,gallo-hours-official,d9-waterfall-route-map</x:v>
+        <x:v>skybury-map,skybury-official,d9-north-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -4262,22 +4262,22 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>13:55–14:10</x:v>
+        <x:v>11:30–12:20</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Millaa Millaa Public Toilets</x:v>
+        <x:v>Skybury → Lake Eacham</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>先在镇中心使用公共厕所、补水并短暂舒展，再前往瀑布</x:v>
+        <x:v>沿高原主路向南前往 Lake Eacham Day Use Area</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>在进入 Waterfall Circuit 前完成实用停靠</x:v>
+        <x:v>从开阔农场回到雨林火山湖</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>Millaa Millaa Falls 现场厕所因升级施工关闭；替代公共厕所位于镇中心、Millaa Millaa Hotel 对面。</x:v>
+        <x:v>这一段约 50 分钟；午后还有多个短停点，途中不再临时增加绕路景点。</x:v>
       </x:c>
       <x:c r="H93" t="str">
-        <x:v>millaa-public-toilets-map,millaa-upgrade-official,d9-waterfall-route-map</x:v>
+        <x:v>d9-highlands-route-map,lake-eacham-day-use-map</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4288,22 +4288,22 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>14:15–15:00</x:v>
+        <x:v>12:20–13:00</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Millaa Millaa Falls</x:v>
+        <x:v>Lake Eacham Day Use Area</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>从主观景面欣赏经典单落差瀑布，沿草坪与水潭边取景，在雨林绿意中慢慢走一圈</x:v>
+        <x:v>到湖边观景台看火山湖与雨林倒影，再沿湖边步道轻松走一小段</x:v>
       </x:c>
       <x:c r="F94" t="str">
-        <x:v>阿瑟顿高原最经典的瀑布画面</x:v>
+        <x:v>被雨林环抱的清澈火山湖</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>停车与步行区域正在升级施工，按现场标志使用开放区域；若在这里下水，下午直接返回 Cairns 会更从容。</x:v>
+        <x:v>今天不完整环湖，也不安排游泳；沿成形步道散步，13:00 左右继续前往 Yungaburra。</x:v>
       </x:c>
       <x:c r="H94" t="str">
-        <x:v>millaa-map,millaa-falls-official,millaa-upgrade-official,d9-waterfall-route-map,d9-return-from-millaa-map</x:v>
+        <x:v>lake-eacham-day-use-map,lake-eacham-official,d9-highlands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4314,22 +4314,22 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>15:10–15:35 · 可选</x:v>
+        <x:v>13:00–13:10</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Ellinjaa Falls（可选）</x:v>
+        <x:v>Lake Eacham → Yungaburra</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>从停车与野餐区沿短步道下到瀑布底部，感受更贴近雨林的水声与绿意</x:v>
+        <x:v>沿 Lakes Drive 与高原道路短途前往 Yungaburra</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>比主瀑布更安静的第二段雨林瀑布</x:v>
+        <x:v>火山湖与小镇之间的轻松转场</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>只有在 15:00 前离开 Millaa Millaa Falls、路面与驾驶状态都舒服时前往；15:35 开始返回 Cairns。</x:v>
+        <x:v>车程约 9 分钟；抵达后把车停稳，再沿老街短走。</x:v>
       </x:c>
       <x:c r="H95" t="str">
-        <x:v>ellinjaa-map,ellinjaa-falls-official,d9-return-from-ellinjaa-map</x:v>
+        <x:v>d9-highlands-route-map,yungaburra-village-map</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -4340,22 +4340,22 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>15:35–18:00</x:v>
+        <x:v>13:10–13:35</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>返回 Cairns / 凯恩斯还车点</x:v>
+        <x:v>Yungaburra Village</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>经 Malanda、Gillies Highway 与 Gordonvale 返回 Cairns，进城后补满油并按订单地点完成还车</x:v>
+        <x:v>沿老街看看历史木屋、高原小店与街景，需要时补一杯咖啡或带走小点心</x:v>
       </x:c>
       <x:c r="F96" t="str">
-        <x:v>在日落前后结束高原自驾</x:v>
+        <x:v>高原小镇安静而缓慢的午后</x:v>
       </x:c>
       <x:c r="G96" t="str">
-        <x:v>从 Millaa Millaa Falls 或 Ellinjaa Falls 选择对应返程地图，始终走铺装主路，不接受导航推荐的无铺装林道。Cairns 当日日落约 18:05。</x:v>
+        <x:v>这里停留约 25 分钟，专心看看老街与历史木屋；13:35 左右继续去 Curtain Fig Tree。</x:v>
       </x:c>
       <x:c r="H96" t="str">
-        <x:v>d9-return-from-millaa-map,d9-return-from-ellinjaa-map,cairns-car-rental-search-map,cairns-sunset-august-2026</x:v>
+        <x:v>yungaburra-village-map,d9-highlands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4363,160 +4363,160 @@
         <x:v>d9</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>900</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>饮食</x:v>
+        <x:v>13:35–13:40</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Yungaburra → Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>早餐：公寓；午餐：Gallo Dairyland；晚餐：18:30 后在 Salt House 或公寓附近简餐</x:v>
+        <x:v>沿短途高原道路前往 Curtain Fig National Park</x:v>
       </x:c>
       <x:c r="F97" t="str">
-        <x:v>农场午餐与回城后的轻松晚餐</x:v>
+        <x:v>小镇与雨林巨树之间只隔一小段车程</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>还车后先回房洗澡休息，晚上不再安排 Night Markets 或 Palm Cove。</x:v>
+        <x:v>车程约 5 分钟；按停车区标志停好车，不在路肩临时停车。</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>gallo-map,salt-house-map,southern-cross-map</x:v>
+        <x:v>d9-highlands-route-map,curtain-fig-map</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B98" t="n">
-        <x:v>10</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>08:30–10:30</x:v>
+        <x:v>13:40–14:05</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Rusty's Market</x:v>
+        <x:v>Curtain Fig Tree</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>逛热带水果、咖啡与早餐摊位，挑选当天可以吃完的水果和轻食</x:v>
+        <x:v>沿短木栈道走到巨型帘状无花果树下，观察垂落气根并拍下人与巨树的尺度</x:v>
       </x:c>
       <x:c r="F98" t="str">
-        <x:v>凯恩斯周五早晨的市场气息</x:v>
+        <x:v>像天然装置艺术般的高原巨树</x:v>
       </x:c>
       <x:c r="G98" t="str">
-        <x:v>买少量即可，水果在飞悉尼前吃完；现场营业情况以当天摊位为准。</x:v>
+        <x:v>木栈道雨后可能湿滑；慢慢绕一圈即可，14:05 左右继续向 Millaa Millaa 出发。</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>rustys-map,rustys-official</x:v>
+        <x:v>curtain-fig-map,curtain-fig-official,d9-highlands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B99" t="n">
-        <x:v>20</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>10:45–14:30</x:v>
+        <x:v>14:05–14:35</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Southern Cross Atrium Apartments</x:v>
+        <x:v>Curtain Fig Tree → Millaa Millaa</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>回公寓洗衣、休息、整理行李，把 Jetstar 托运行李和随身物品分装好</x:v>
+        <x:v>沿 Atherton–Malanda Road 与高原主路前往 Millaa Millaa 镇</x:v>
       </x:c>
       <x:c r="F99" t="str">
-        <x:v>给连续三天自然行程留出恢复时间</x:v>
+        <x:v>农场、雨林与高原道路交替展开</x:v>
       </x:c>
       <x:c r="G99" t="str">
-        <x:v>午餐在附近简单解决；泳池、咖啡与午休都留在这段时间里。</x:v>
+        <x:v>继续使用铺装主路；先到镇中心使用公共厕所，再前往瀑布。</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>southern-cross-map</x:v>
+        <x:v>d9-highlands-route-map,millaa-public-toilets-map</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B100" t="n">
-        <x:v>30</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>15:00–17:30</x:v>
+        <x:v>14:35–14:45</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Southern Cross Atrium → Palm Cove</x:v>
+        <x:v>Millaa Millaa Public Toilets</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>15:00 叫 Uber / Didi，约 15:40 抵达；15:40–17:30 沿 Williams Esplanade、Palm Cove Beach 与 Palm Cove Jetty 慢慢散步</x:v>
+        <x:v>在镇中心使用公共厕所、补水并短暂舒展，再前往瀑布</x:v>
       </x:c>
       <x:c r="F100" t="str">
-        <x:v>棕榈树、海岸与热带蓝调前的光线</x:v>
+        <x:v>在最后一处主景点前完成实用停靠</x:v>
       </x:c>
       <x:c r="G100" t="str">
-        <x:v>海滩活动以现场旗帜和警示为准；这里更适合散步与拍照，不把下海游泳作为固定安排。</x:v>
+        <x:v>Millaa Millaa Falls 现场厕所因升级施工关闭；替代公共厕所位于镇中心、Millaa Millaa Hotel 对面。</x:v>
       </x:c>
       <x:c r="H100" t="str">
-        <x:v>southern-cross-map,palm-cove-map,williams-esplanade-map,palm-cove-jetty-map</x:v>
+        <x:v>millaa-public-toilets-map,millaa-upgrade-official,d9-highlands-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B101" t="n">
-        <x:v>40</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>17:30–18:45</x:v>
+        <x:v>14:50–15:35</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Palm Cove 早晚餐</x:v>
+        <x:v>Millaa Millaa Falls</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>在 Williams Esplanade 一带选一家海滨餐厅，边吃晚餐边看天空进入蓝调时刻</x:v>
+        <x:v>从主观景面欣赏经典单落差瀑布，沿草坪与水潭边取景，在雨林绿意中慢慢走一圈</x:v>
       </x:c>
       <x:c r="F101" t="str">
-        <x:v>凯恩斯段最后一顿海边晚餐</x:v>
+        <x:v>阿瑟顿高原最经典的瀑布画面</x:v>
       </x:c>
       <x:c r="G101" t="str">
-        <x:v>Palm Cove 面向东侧，重点是傍晚天色与棕榈树剪影；19:00 前准备返程。</x:v>
+        <x:v>停车与步行区域正在升级施工，按现场标志使用开放区域；15:35 左右离开，给回 Cairns 的山路留足天光。</x:v>
       </x:c>
       <x:c r="H101" t="str">
-        <x:v>williams-esplanade-map,palm-cove-map</x:v>
+        <x:v>millaa-map,millaa-falls-official,millaa-upgrade-official,d9-highlands-route-map,d9-return-from-millaa-map</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B102" t="n">
-        <x:v>50</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>19:00–21:30</x:v>
+        <x:v>15:35–18:00</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Palm Cove → Southern Cross Atrium</x:v>
+        <x:v>返回 Cairns / 凯恩斯还车点</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>19:00 叫车返回，预计 19:30–19:45 抵达；20:00–21:00 完成行李称重、Jetstar 在线值机与次日随身包检查</x:v>
+        <x:v>按 Google Maps 的铺装主路返回 Cairns，进城后补满油并按订单地点完成还车</x:v>
       </x:c>
       <x:c r="F102" t="str">
-        <x:v>把热带假期从容收进行李箱</x:v>
+        <x:v>在傍晚前后结束完整高原环线</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>闹钟、证件、薄外套和机场用物放在手边；21:15–21:30 上床休息。</x:v>
+        <x:v>Millaa Millaa Falls 到 Cairns 约 1 小时 40 分钟；出发前再看一次实时路况，不接受导航推荐的无铺装林道。</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>palm-cove-map,southern-cross-map,cairns-airport-map,jetstar-official</x:v>
+        <x:v>d9-return-from-millaa-map,cairns-car-rental-search-map,cairns-sunset-august-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" t="str">
-        <x:v>d10</x:v>
+        <x:v>d9</x:v>
       </x:c>
       <x:c r="B103" t="n">
         <x:v>900</x:v>
@@ -4528,170 +4528,172 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>早餐：Rusty's Market；午餐：公寓附近简餐；晚餐：Palm Cove 海滨早晚餐</x:v>
+        <x:v>早餐：公寓；早午餐：Skybury Cafe &amp; Roastery；下午：Yungaburra 小点心可选；晚餐：回 Cairns 后在酒店附近简单吃</x:v>
       </x:c>
       <x:c r="F103" t="str">
-        <x:v>市场、水果与海边晚餐组成轻松收尾</x:v>
+        <x:v>农场咖啡早午餐与回城后的轻松晚餐</x:v>
       </x:c>
       <x:c r="G103" t="str">
-        <x:v>晚餐结束后直接返回凯恩斯，不让次日清晨航班变得匆忙。</x:v>
+        <x:v>Skybury 是今天的正式用餐站；回城后先洗澡休息，晚上不再安排长距离活动。</x:v>
       </x:c>
       <x:c r="H103" t="str">
-        <x:v>rustys-map,rustys-official,williams-esplanade-map,palm-cove-map</x:v>
+        <x:v>skybury-map,skybury-official,southern-cross-map</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B104" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>清晨</x:v>
+        <x:v>08:30–10:30</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>Rusty's Market</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>逛热带水果、咖啡与早餐摊位，挑选当天可以吃完的水果和轻食</x:v>
       </x:c>
       <x:c r="F104" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>凯恩斯周五早晨的市场气息</x:v>
       </x:c>
       <x:c r="G104" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+        <x:v>买少量即可，水果在飞悉尼前吃完；现场营业情况以当天摊位为准。</x:v>
       </x:c>
       <x:c r="H104" t="str">
-        <x:v>cairns-airport-map</x:v>
+        <x:v>rustys-map,rustys-official</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B105" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>上午</x:v>
+        <x:v>10:45–14:30</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>凯恩斯 → 悉尼</x:v>
+        <x:v>Southern Cross Atrium Apartments</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>回公寓洗衣、休息、整理行李，把 Jetstar 托运行李和随身物品分装好</x:v>
       </x:c>
       <x:c r="F105" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>给连续三天自然行程留出恢复时间</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H105"/>
+        <x:v>午餐在附近简单解决；泳池、咖啡与午休都留在这段时间里。</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B106" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>15:00–17:30</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>Southern Cross Atrium → Palm Cove</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>15:00 叫 Uber / Didi，约 15:40 抵达；15:40–17:30 沿 Williams Esplanade、Palm Cove Beach 与 Palm Cove Jetty 慢慢散步</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>棕榈树、海岸与热带蓝调前的光线</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
+        <x:v>海滩活动以现场旗帜和警示为准；这里更适合散步与拍照，不把下海游泳作为固定安排。</x:v>
       </x:c>
       <x:c r="H106" t="str">
-        <x:v>oaks-sydney-map</x:v>
+        <x:v>southern-cross-map,palm-cove-map,williams-esplanade-map,palm-cove-jetty-map</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B107" t="n">
         <x:v>40</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>下午</x:v>
+        <x:v>17:30–18:45</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>Palm Cove 早晚餐</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>在 Williams Esplanade 一带选一家海滨餐厅，边吃晚餐边看天空进入蓝调时刻</x:v>
       </x:c>
       <x:c r="F107" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>凯恩斯段最后一顿海边晚餐</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>Palm Cove 面向东侧，重点是傍晚天色与棕榈树剪影；19:00 前准备返程。</x:v>
       </x:c>
       <x:c r="H107" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>williams-esplanade-map,palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B108" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>19:00–21:30</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>Palm Cove → Southern Cross Atrium</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>19:00 叫车返回，预计 19:30–19:45 抵达；20:00–21:00 完成行李称重、Jetstar 在线值机与次日随身包检查</x:v>
       </x:c>
       <x:c r="F108" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>把热带假期从容收进行李箱</x:v>
       </x:c>
       <x:c r="G108" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>闹钟、证件、薄外套和机场用物放在手边；21:15–21:30 上床休息。</x:v>
       </x:c>
       <x:c r="H108" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>palm-cove-map,southern-cross-map,cairns-airport-map,jetstar-official</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" t="str">
-        <x:v>d11</x:v>
+        <x:v>d10</x:v>
       </x:c>
       <x:c r="B109" t="n">
-        <x:v>50</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>早餐：Rusty's Market；午餐：公寓附近简餐；晚餐：Palm Cove 海滨早晚餐</x:v>
       </x:c>
       <x:c r="F109" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>市场、水果与海边晚餐组成轻松收尾</x:v>
       </x:c>
       <x:c r="G109" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
+        <x:v>晚餐结束后直接返回凯恩斯，不让次日清晨航班变得匆忙。</x:v>
       </x:c>
       <x:c r="H109" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>rustys-map,rustys-official,williams-esplanade-map,palm-cove-map</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -4699,25 +4701,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B110" t="n">
-        <x:v>60</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>晚上</x:v>
+        <x:v>清晨</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
+        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>circular-quay-map</x:v>
+        <x:v>cairns-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -4725,181 +4727,179 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B111" t="n">
-        <x:v>900</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>饮食</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>从热带切换回冬季海港城市</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
-      </x:c>
-      <x:c r="H111" t="str">
-        <x:v>the-rocks-map</x:v>
-      </x:c>
+        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
+      </x:c>
+      <x:c r="H111"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B112" t="n">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>上午 / 中午</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>悉尼 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>4人 + 行李，打车最省心</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>如不能入住，先寄存行李</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B113" t="n">
-        <x:v>20</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>下午</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>Darling Harbour / 酒店周边</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>30</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>下午后段</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>傍晚</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
+        <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
+        <x:v>歌剧院、海港大桥夜景</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
+        <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>60</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>the-rocks-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -4907,25 +4907,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>70</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>08:15–08:30</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Royal Botanic Garden</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>抵达海港区</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>Ferry、海港桥、歌剧院远景</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -4933,25 +4933,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>80</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>08:30–09:10</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>悉尼核心地标</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -4959,25 +4959,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>90</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>中文内部导览已订</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>建筑故事、内部空间、剧院结构</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -4985,25 +4985,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>100</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>晚上</x:v>
+        <x:v>10:30–10:50</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>Opera House → The Rocks</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>海港步行衔接悉尼老城区</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -5011,181 +5011,181 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>900</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>饮食</x:v>
+        <x:v>10:50–11:50</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>The Rocks Markets</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>10</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>08:00</x:v>
+        <x:v>11:50–12:40</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>就地补体力，不为午餐绕路</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>20</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>09:15</x:v>
+        <x:v>12:40–14:10</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>植物园海港步道</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>botanic-garden-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>30</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>10:00</x:v>
+        <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>歌剧院 + 海港大桥同框</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>悉尼最经典机位</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>mrs-macquarie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>40</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>11:15</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>购物、室内休息</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>建筑漂亮，适合逛</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>50</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>12:00</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>CBD / Darling Harbour</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>Hello Auntie / CBD 晚餐</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>60</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -5193,25 +5193,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>70</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>13:30</x:v>
+        <x:v>08:00</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>royal-national-park-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -5219,25 +5219,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>80</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>09:15</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>南海岸第一处全景</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>bald-hill-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -5245,25 +5245,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>90</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>14:40</x:v>
+        <x:v>10:00</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>贴着太平洋的公路画面</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>不要在桥上或路肩危险停车</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -5271,25 +5271,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>100</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>11:15</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>Wollongong / 南海岸补给</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>短停咖啡或直接通过</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>wollongong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -5297,25 +5297,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>110</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Kiama Blowhole</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>看喷潮洞、灯塔与海边</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>Kiama 代表性海岸地貌</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -5323,181 +5323,181 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>饮食</x:v>
+        <x:v>12:30–13:30</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>海边小镇节奏</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>10</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>13:30</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Kiama → Gerringong</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>沿海继续南下</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>kiama-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B136" t="n">
-        <x:v>20</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>13:45–14:40</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B137" t="n">
-        <x:v>30</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>14:40</x:v>
       </x:c>
       <x:c r="D137" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>Gerringong</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>判断是否延伸 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="F137" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>时间、天气与体力闸门</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>gerringong-map,kangaroo-valley-map</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B138" t="n">
-        <x:v>40</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>可选 15:30–16:15</x:v>
       </x:c>
       <x:c r="D138" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E138" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>看历史桥、山谷与小镇</x:v>
       </x:c>
       <x:c r="F138" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G138" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H138" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B139" t="n">
-        <x:v>50</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>16:15 前</x:v>
       </x:c>
       <x:c r="D139" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
       </x:c>
       <x:c r="E139" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
       </x:c>
       <x:c r="F139" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>环线收束</x:v>
       </x:c>
       <x:c r="G139" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
       </x:c>
       <x:c r="H139" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B140" t="n">
-        <x:v>60</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C140" t="str">
-        <x:v>18:30</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D140" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E140" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F140" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G140" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H140" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -5505,181 +5505,181 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B141" t="n">
-        <x:v>900</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C141" t="str">
-        <x:v>饮食</x:v>
+        <x:v>08:30–09:00</x:v>
       </x:c>
       <x:c r="D141" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E141" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F141" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G141" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
       </x:c>
       <x:c r="H141" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B142" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C142" t="str">
-        <x:v>上午</x:v>
+        <x:v>09:15 左右</x:v>
       </x:c>
       <x:c r="D142" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E142" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F142" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
       </x:c>
       <x:c r="G142" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
       </x:c>
       <x:c r="H142" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B143" t="n">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C143" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>09:30–13:30</x:v>
       </x:c>
       <x:c r="D143" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E143" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F143" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H143" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B144" t="n">
-        <x:v>30</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C144" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>13:30–14:30</x:v>
       </x:c>
       <x:c r="D144" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
       </x:c>
       <x:c r="E144" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>F2 返回市区后前往 Bondi</x:v>
       </x:c>
       <x:c r="F144" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>动物园切换到悉尼海岸</x:v>
       </x:c>
       <x:c r="G144" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
       </x:c>
       <x:c r="H144" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B145" t="n">
-        <x:v>40</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C145" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>14:30–17:45</x:v>
       </x:c>
       <x:c r="D145" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E145" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>海滩散步并走一段 Coastal Walk</x:v>
       </x:c>
       <x:c r="F145" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G145" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H145" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B146" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C146" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>18:30</x:v>
       </x:c>
       <x:c r="D146" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E146" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F146" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G146" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
       </x:c>
       <x:c r="H146" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B147" t="n">
-        <x:v>60</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C147" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D147" t="str">
-        <x:v>酒店</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E147" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F147" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G147" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H147" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -5687,25 +5687,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B148" t="n">
-        <x:v>70</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C148" t="str">
-        <x:v>16:40</x:v>
+        <x:v>上午</x:v>
       </x:c>
       <x:c r="D148" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E148" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F148" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G148" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H148" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>oaks-sydney-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -5713,25 +5713,25 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B149" t="n">
-        <x:v>80</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C149" t="str">
-        <x:v>17:30</x:v>
+        <x:v>可选 09:30 左右</x:v>
       </x:c>
       <x:c r="D149" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>Circular Quay → Manly</x:v>
       </x:c>
       <x:c r="E149" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>搭乘公共 F1 Manly Ferry</x:v>
       </x:c>
       <x:c r="F149" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G149" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H149" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>circular-quay-map,manly-ferry-map</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -5739,76 +5739,232 @@
         <x:v>d15</x:v>
       </x:c>
       <x:c r="B150" t="n">
-        <x:v>900</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C150" t="str">
-        <x:v>饮食</x:v>
+        <x:v>可选 10:00–12:45</x:v>
       </x:c>
       <x:c r="D150" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Manly Beach / The Corso</x:v>
       </x:c>
       <x:c r="E150" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>海边散步、咖啡或早午餐</x:v>
       </x:c>
       <x:c r="F150" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G150" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H150" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" t="str">
-        <x:v>d16</x:v>
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B151" t="n">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C151" t="str">
-        <x:v>上午</x:v>
+        <x:v>13:00–13:30</x:v>
       </x:c>
       <x:c r="D151" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>Manly → Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E151" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>最晚搭船回市区</x:v>
       </x:c>
       <x:c r="F151" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G151" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H151" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
       <x:c r="A152" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B152" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>14:00–15:30</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+      </x:c>
+      <x:c r="E152" t="str">
+        <x:v>最后采购</x:v>
+      </x:c>
+      <x:c r="F152" t="str">
+        <x:v>药妆、保健品、伴手礼</x:v>
+      </x:c>
+      <x:c r="G152" t="str">
+        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+      </x:c>
+      <x:c r="H152" t="str">
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B153" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>15:30–16:20</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>酒店</x:v>
+      </x:c>
+      <x:c r="E153" t="str">
+        <x:v>整理 TRS 物品和返程行李</x:v>
+      </x:c>
+      <x:c r="F153" t="str">
+        <x:v>为 D16 机场退税做准备</x:v>
+      </x:c>
+      <x:c r="G153" t="str">
+        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+      </x:c>
+      <x:c r="H153" t="str">
+        <x:v>oaks-sydney-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B154" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>16:40</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E154" t="str">
+        <x:v>前往 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="F154" t="str">
+        <x:v>避免迟到</x:v>
+      </x:c>
+      <x:c r="G154" t="str">
+        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+      </x:c>
+      <x:c r="H154" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B155" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>17:30</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="E155" t="str">
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+      </x:c>
+      <x:c r="F155" t="str">
+        <x:v>海港景观 + 澳洲最后一晚</x:v>
+      </x:c>
+      <x:c r="G155" t="str">
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+      </x:c>
+      <x:c r="H155" t="str">
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B156" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E156" t="str">
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="F156" t="str">
+        <x:v>当天餐食节奏</x:v>
+      </x:c>
+      <x:c r="G156" t="str">
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+      </x:c>
+      <x:c r="H156" t="str">
+        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
         <x:v>d16</x:v>
       </x:c>
-      <x:c r="B152" t="n">
+      <x:c r="B157" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D157" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E157" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F157" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G157" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H157" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B158" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C152" t="str">
+      <x:c r="C158" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D152" t="str">
+      <x:c r="D158" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E152" t="str">
+      <x:c r="E158" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F152" t="str">
+      <x:c r="F158" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G152" t="str">
+      <x:c r="G158" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H152"/>
+      <x:c r="H158"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6603,12 +6759,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Curtain+Fig+Tree</x:v>
-      </x:c>
-      <x:c r="E41"/>
-      <x:c r="F41"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Curtain+Fig+Tree%2C+Fig+Tree+Road%2C+East+Barron+QLD+4883&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E41" t="str"/>
+      <x:c r="F41" t="str"/>
       <x:c r="G41" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Fig Tree Road, East Barron</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -6660,12 +6816,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Millaa+Millaa+Falls</x:v>
-      </x:c>
-      <x:c r="E44"/>
-      <x:c r="F44"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Millaa+Millaa+Falls%2C+Falls+Road%2C+Millaa+Millaa+QLD+4886&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E44" t="str"/>
+      <x:c r="F44" t="str"/>
       <x:c r="G44" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Falls Road, Millaa Millaa</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -9079,8 +9235,8 @@
       <x:c r="D171" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Car+Rental+Cairns+QLD</x:v>
       </x:c>
-      <x:c r="E171" t="str"/>
-      <x:c r="F171" t="str"/>
+      <x:c r="E171"/>
+      <x:c r="F171"/>
       <x:c r="G171" t="str">
         <x:v>Google Maps · 准确门店以租车订单为准</x:v>
       </x:c>
@@ -9090,18 +9246,18 @@
         <x:v>d9-core-route-map</x:v>
       </x:c>
       <x:c r="B172" t="str">
-        <x:v>D9 阿瑟顿高原核心环线</x:v>
+        <x:v>D9 Kuranda 与阿瑟顿高原完整环线</x:v>
       </x:c>
       <x:c r="C172" t="str">
         <x:v>map</x:v>
       </x:c>
       <x:c r="D172" t="str">
-        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Lake+Eacham+Day+Use+Area%7CYungaburra+Village%7CCurtain+Fig+Tree%7CGallo+Dairyland%7CMillaa+Millaa+Public+Toilets%7CMillaa+Millaa+Falls</x:v>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Kuranda+Village%7CMareeba+QLD%7CSkybury+Cafe+and+Roastery%7CLake+Eacham+Day+Use+Area%7CYungaburra+Village%7CCurtain+Fig+Tree%7CMillaa+Millaa+Public+Toilets%7CMillaa+Millaa+Falls</x:v>
       </x:c>
       <x:c r="E172" t="str"/>
       <x:c r="F172" t="str"/>
       <x:c r="G172" t="str">
-        <x:v>Google Maps · Cairns → Lake Eacham → Yungaburra → Curtain Fig → Gallo → Millaa Millaa 镇 → 主瀑布 → Cairns</x:v>
+        <x:v>Google Maps · Cairns → Kuranda → Mareeba → Skybury → Lake Eacham → Yungaburra → Curtain Fig → Millaa Millaa → Cairns</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -9117,8 +9273,8 @@
       <x:c r="D173" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Lake+Eacham+Day+Use+Area&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E173" t="str"/>
-      <x:c r="F173" t="str"/>
+      <x:c r="E173"/>
+      <x:c r="F173"/>
       <x:c r="G173" t="str">
         <x:v>Google Maps · 经 Gordonvale 与 Gillies Highway</x:v>
       </x:c>
@@ -9136,8 +9292,8 @@
       <x:c r="D174" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Gallo+Dairyland&amp;destination=Ellinjaa+Falls&amp;travelmode=driving&amp;waypoints=Millaa+Millaa+Public+Toilets%7CMillaa+Millaa+Falls</x:v>
       </x:c>
-      <x:c r="E174" t="str"/>
-      <x:c r="F174" t="str"/>
+      <x:c r="E174"/>
+      <x:c r="F174"/>
       <x:c r="G174" t="str">
         <x:v>Google Maps · Gallo → 镇中心厕所 → Millaa Millaa Falls → Ellinjaa Falls</x:v>
       </x:c>
@@ -9153,12 +9309,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D175" t="str">
-        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Millaa+Millaa+Falls&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Malanda+QLD%7CGordonvale+QLD</x:v>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Millaa+Millaa+Falls&amp;destination=Cairns+QLD&amp;travelmode=driving</x:v>
       </x:c>
       <x:c r="E175" t="str"/>
       <x:c r="F175" t="str"/>
       <x:c r="G175" t="str">
-        <x:v>Google Maps · 经 Malanda、Gillies Highway 与 Gordonvale 返回</x:v>
+        <x:v>Google Maps · 返程前重新打开，按实时路况使用铺装主路</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -9174,8 +9330,8 @@
       <x:c r="D176" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Ellinjaa+Falls&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Malanda+QLD%7CGordonvale+QLD</x:v>
       </x:c>
-      <x:c r="E176" t="str"/>
-      <x:c r="F176" t="str"/>
+      <x:c r="E176"/>
+      <x:c r="F176"/>
       <x:c r="G176" t="str">
         <x:v>Google Maps · 经 Malanda、Gillies Highway 与 Gordonvale 返回</x:v>
       </x:c>
@@ -9191,7 +9347,7 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D177" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Lake+Eacham+Day+Use+Area%2C+Lakes+Drive%2C+Lake+Eacham+QLD</x:v>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Lake+Eacham+Day+Use+Area%2C+Lakes+Drive%2C+Lake+Eacham+QLD+4884&amp;travelmode=driving</x:v>
       </x:c>
       <x:c r="E177" t="str"/>
       <x:c r="F177" t="str"/>
@@ -9212,8 +9368,8 @@
       <x:c r="D178" t="str">
         <x:v>https://parks.qld.gov.au/parks/crater-lakes/attractions/lake-eacham-day-use-area</x:v>
       </x:c>
-      <x:c r="E178" t="str"/>
-      <x:c r="F178" t="str"/>
+      <x:c r="E178"/>
+      <x:c r="F178"/>
       <x:c r="G178" t="str">
         <x:v>Queensland Parks · 距 Cairns 约 68 km，铺装路适合普通车辆，全天开放</x:v>
       </x:c>
@@ -9229,7 +9385,7 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D179" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Yungaburra+Village+QLD</x:v>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Yungaburra+QLD+4884&amp;travelmode=driving</x:v>
       </x:c>
       <x:c r="E179" t="str"/>
       <x:c r="F179" t="str"/>
@@ -9250,8 +9406,8 @@
       <x:c r="D180" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Platypus+Viewing+Platform+Yungaburra</x:v>
       </x:c>
-      <x:c r="E180" t="str"/>
-      <x:c r="F180" t="str"/>
+      <x:c r="E180"/>
+      <x:c r="F180"/>
       <x:c r="G180" t="str">
         <x:v>Google Maps · Peterson Creek Platypus Viewing Platform</x:v>
       </x:c>
@@ -9269,8 +9425,8 @@
       <x:c r="D181" t="str">
         <x:v>https://petersoncreek.org.au/walking-tracks/</x:v>
       </x:c>
-      <x:c r="E181" t="str"/>
-      <x:c r="F181" t="str"/>
+      <x:c r="E181"/>
+      <x:c r="F181"/>
       <x:c r="G181" t="str">
         <x:v>Yungaburra Landcare Group · 平台可用，平台至 Other Side 的连接步道关闭</x:v>
       </x:c>
@@ -9288,8 +9444,8 @@
       <x:c r="D182" t="str">
         <x:v>https://parks.qld.gov.au/parks/curtain-fig</x:v>
       </x:c>
-      <x:c r="E182" t="str"/>
-      <x:c r="F182" t="str"/>
+      <x:c r="E182"/>
+      <x:c r="F182"/>
       <x:c r="G182" t="str">
         <x:v>Queensland Parks · 高架木栈道环绕 Curtain Fig Tree</x:v>
       </x:c>
@@ -9307,8 +9463,8 @@
       <x:c r="D183" t="str">
         <x:v>https://www.athertontablelands.com.au/travel-directory/gallo-dairyland/</x:v>
       </x:c>
-      <x:c r="E183" t="str"/>
-      <x:c r="F183" t="str"/>
+      <x:c r="E183"/>
+      <x:c r="F183"/>
       <x:c r="G183" t="str">
         <x:v>Tourism Atherton Tablelands · 工作日厨房热餐通常 09:30–14:00</x:v>
       </x:c>
@@ -9324,7 +9480,7 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D184" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Millaa+Millaa+Public+Toilets%2C+Main+Street%2C+Millaa+Millaa+QLD</x:v>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Millaa+Millaa+Public+Toilets%2C+Main+Street%2C+Millaa+Millaa+QLD&amp;travelmode=driving</x:v>
       </x:c>
       <x:c r="E184" t="str"/>
       <x:c r="F184" t="str"/>
@@ -9345,8 +9501,8 @@
       <x:c r="D185" t="str">
         <x:v>https://www.trc.qld.gov.au/our-council/projects/millaa-millaa-falls-upgrade/</x:v>
       </x:c>
-      <x:c r="E185" t="str"/>
-      <x:c r="F185" t="str"/>
+      <x:c r="E185"/>
+      <x:c r="F185"/>
       <x:c r="G185" t="str">
         <x:v>Tablelands Regional Council · 2026 年 7 月起施工，停车和步行区域受影响，现场厕所停用</x:v>
       </x:c>
@@ -9364,8 +9520,8 @@
       <x:c r="D186" t="str">
         <x:v>https://www.queensland.com/au/en/things-to-do/attractions/p-56b25fd67b935fbe730df3b1-millaa-millaa-falls</x:v>
       </x:c>
-      <x:c r="E186" t="str"/>
-      <x:c r="F186" t="str"/>
+      <x:c r="E186"/>
+      <x:c r="F186"/>
       <x:c r="G186" t="str">
         <x:v>Tourism and Events Queensland · Waterfalls Circuit</x:v>
       </x:c>
@@ -9383,8 +9539,8 @@
       <x:c r="D187" t="str">
         <x:v>https://www.athertontablelands.com.au/travel-directory/elinjaa-falls-millaa-millaa/</x:v>
       </x:c>
-      <x:c r="E187" t="str"/>
-      <x:c r="F187" t="str"/>
+      <x:c r="E187"/>
+      <x:c r="F187"/>
       <x:c r="G187" t="str">
         <x:v>Tourism Atherton Tablelands · 从停车与野餐区沿步道下到瀑布底部</x:v>
       </x:c>
@@ -9402,10 +9558,124 @@
       <x:c r="D188" t="str">
         <x:v>https://www.timeanddate.com/sun/australia/cairns?month=8</x:v>
       </x:c>
-      <x:c r="E188" t="str"/>
-      <x:c r="F188" t="str"/>
+      <x:c r="E188"/>
+      <x:c r="F188"/>
       <x:c r="G188" t="str">
         <x:v>Timeanddate · 2026 年 8 月 6 日日落约 18:05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" t="str">
+        <x:v>d9-north-route-map</x:v>
+      </x:c>
+      <x:c r="B189" t="str">
+        <x:v>Cairns → Kuranda → Mareeba → Skybury</x:v>
+      </x:c>
+      <x:c r="C189" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D189" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Skybury+Cafe+and+Roastery%2C+136+Ivicevic+Road%2C+Paddys+Green+QLD+4880&amp;travelmode=driving&amp;waypoints=Kuranda+Village%7CMareeba+QLD</x:v>
+      </x:c>
+      <x:c r="E189" t="str"/>
+      <x:c r="F189" t="str"/>
+      <x:c r="G189" t="str">
+        <x:v>Google Maps · 北上段，依次经过 Kuranda 与 Mareeba</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" t="str">
+        <x:v>d9-highlands-route-map</x:v>
+      </x:c>
+      <x:c r="B190" t="str">
+        <x:v>Skybury → Lake Eacham → Millaa Millaa Falls</x:v>
+      </x:c>
+      <x:c r="C190" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D190" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Skybury+Cafe+and+Roastery%2C+136+Ivicevic+Road%2C+Paddys+Green+QLD+4880&amp;destination=Millaa+Millaa+Falls&amp;travelmode=driving&amp;waypoints=Lake+Eacham+Day+Use+Area%7CYungaburra+Village%7CCurtain+Fig+Tree%7CMillaa+Millaa+Public+Toilets</x:v>
+      </x:c>
+      <x:c r="E190" t="str"/>
+      <x:c r="F190" t="str"/>
+      <x:c r="G190" t="str">
+        <x:v>Google Maps · 高原段，依次经过火山湖、小镇、巨树与镇中心厕所</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" t="str">
+        <x:v>kuranda-village-map</x:v>
+      </x:c>
+      <x:c r="B191" t="str">
+        <x:v>Kuranda Village</x:v>
+      </x:c>
+      <x:c r="C191" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D191" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Kuranda+Village%2C+Coondoo+Street%2C+Kuranda+QLD+4881&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E191" t="str"/>
+      <x:c r="F191" t="str"/>
+      <x:c r="G191" t="str">
+        <x:v>Google Maps · Coondoo Street, Kuranda</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" t="str">
+        <x:v>mareeba-town-map</x:v>
+      </x:c>
+      <x:c r="B192" t="str">
+        <x:v>Mareeba</x:v>
+      </x:c>
+      <x:c r="C192" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D192" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Mareeba+QLD+4880&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E192" t="str"/>
+      <x:c r="F192" t="str"/>
+      <x:c r="G192" t="str">
+        <x:v>Google Maps · Mareeba 镇中心</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" t="str">
+        <x:v>skybury-map</x:v>
+      </x:c>
+      <x:c r="B193" t="str">
+        <x:v>Skybury Cafe &amp; Roastery</x:v>
+      </x:c>
+      <x:c r="C193" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D193" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Skybury+Cafe+and+Roastery%2C+136+Ivicevic+Road%2C+Paddys+Green+QLD+4880&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E193" t="str"/>
+      <x:c r="F193" t="str"/>
+      <x:c r="G193" t="str">
+        <x:v>Google Maps · 136 Ivicevic Road, Paddys Green QLD 4880</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" t="str">
+        <x:v>skybury-official</x:v>
+      </x:c>
+      <x:c r="B194" t="str">
+        <x:v>Skybury Cafe &amp; Roastery 官网</x:v>
+      </x:c>
+      <x:c r="C194" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D194" t="str">
+        <x:v>https://skybury.com.au/</x:v>
+      </x:c>
+      <x:c r="E194" t="str"/>
+      <x:c r="F194" t="str"/>
+      <x:c r="G194" t="str">
+        <x:v>Skybury · 周一至周五 09:00–16:00，公共假日关闭</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update Sydney itinerary for D11-D15
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rc8061742401442c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R921bb94272c14fb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Ra0f3b31856e048bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R28b5f28c18c3485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Rae8a01e45d5c4975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rf01a54bb81324a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Ra8bbf3ff94f5428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Re563cd4ccc284873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R5ed7e048d1d14c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="Ra0f6339450414c90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R0eb9878c2b36459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Ra349258437e0492c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rab8972202a104e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R6c376bf4de7e4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R970f6fee78a7405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rc1da6c6bf7a14a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rcb44cb5a9b0143cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Rb3d2b6738e9e4313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R36ce943256d4465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="10" r:id="R64d7b4b7111d44bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1335,19 +1335,19 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H13" t="str">
-        <x:v>初到悉尼：Barangaroo、The Rocks 与海港夜景</x:v>
+        <x:v>从热带飞抵海港：Barangaroo、The Rocks 与 Circular Quay</x:v>
       </x:c>
       <x:c r="I13" t="str">
-        <x:v>飞抵悉尼后休息片刻，沿 Barangaroo、The Rocks 走到 Circular Quay 夜景。</x:v>
+        <x:v>清晨从凯恩斯飞抵悉尼，午后充分休息，再沿 Barangaroo 与 Wulugul Walk 走进 The Rocks，在 Circular Quay 看日落与蓝调。</x:v>
       </x:c>
       <x:c r="J13" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="K13" t="str">
-        <x:v>悉尼约 9-18°C，早晚凉，海边防风。</x:v>
+        <x:v>悉尼约 9–18°C，午后海港步道和日落时段都有风。</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>薄羽绒、风衣或卫衣；从凯恩斯上飞机随身带外套。</x:v>
+        <x:v>从凯恩斯登机时把薄外套放在随身包里；海港边按长袖加防风外层穿。</x:v>
       </x:c>
       <x:c r="M13" t="str">
         <x:v>/itinerary/d11-sydney-arrival-rocks.png</x:v>
@@ -1356,16 +1356,16 @@
         <x:v>悉尼 The Rocks 夜景</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>航班 / 机场转场 + 步行</x:v>
+        <x:v>JQ953 + Uber / Taxi + 海港步行</x:v>
       </x:c>
       <x:c r="P13" t="str">
-        <x:v>按 JQ953 起飞时间，提前 2 小时到凯恩斯机场 T2</x:v>
+        <x:v>04:40–04:50 抵达凯恩斯机场 T2；15:00 左右从酒店前往 Barangaroo Reserve</x:v>
       </x:c>
       <x:c r="Q13" t="str">
         <x:v>oaks-sydney-map</x:v>
       </x:c>
       <x:c r="R13" t="str">
-        <x:v>cairns-airport-map</x:v>
+        <x:v>d11-harbour-walk-map</x:v>
       </x:c>
       <x:c r="S13" t="str">
         <x:v>jetstar-official</x:v>
@@ -1394,19 +1394,19 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>悉尼经典一日：歌剧院、The Rocks Markets、植物园与 QVB</x:v>
+        <x:v>海港晨光与城市经典：Mrs Macquarie's Chair、歌剧院与 QVB</x:v>
       </x:c>
       <x:c r="I14" t="str">
-        <x:v>从歌剧院中文导览出发，逛 The Rocks Markets，再沿植物园走到经典海港机位与 QVB。</x:v>
+        <x:v>清晨先到 Mrs Macquarie's Chair 拍下歌剧院与海港桥同框，再穿过皇家植物园参加 09:30 中文导览，午后在 QVB 与 CBD 从容逛街。</x:v>
       </x:c>
       <x:c r="J14" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="K14" t="str">
-        <x:v>悉尼冬季晴天概率较好，早晚凉。</x:v>
+        <x:v>上午后段起阵雨机会增多，海港户外机位尽量前置；下午以室内行程为主。</x:v>
       </x:c>
       <x:c r="L14" t="str">
-        <x:v>薄羽绒或风衣，海港边风大时注意保暖。</x:v>
+        <x:v>薄外套与轻便雨具随身，穿适合植物园步行和歌剧院台阶的鞋。</x:v>
       </x:c>
       <x:c r="M14" t="str">
         <x:v>/itinerary/d12-sydney-opera-garden.png</x:v>
@@ -1415,16 +1415,16 @@
         <x:v>悉尼歌剧院与植物园</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>步行 + 市内交通</x:v>
+        <x:v>Uber / Taxi + 步行 + 市内交通</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>08:45 前出门，09:15 前到 Sydney Opera House</x:v>
+        <x:v>07:30–07:45 离开酒店；09:05 前抵达 Sydney Opera House 集合区</x:v>
       </x:c>
       <x:c r="Q14" t="str">
         <x:v>oaks-sydney-map</x:v>
       </x:c>
       <x:c r="R14" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>d12-harbour-morning-walk-map</x:v>
       </x:c>
       <x:c r="S14" t="str">
         <x:v>opera-house-official</x:v>
@@ -1444,7 +1444,7 @@
         <x:v>周一</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>悉尼南海岸</x:v>
+        <x:v>悉尼｜Taronga + Bondi</x:v>
       </x:c>
       <x:c r="F15" t="n">
         <x:v>-34.6713</x:v>
@@ -1453,40 +1453,40 @@
         <x:v>150.8565</x:v>
       </x:c>
       <x:c r="H15" t="str">
-        <x:v>悉尼南海岸：Sea Cliff Bridge、Kiama 与 Gerringong</x:v>
+        <x:v>动物园与海岸：Taronga、Bondi 与 Totti's</x:v>
       </x:c>
       <x:c r="I15" t="str">
-        <x:v>沿 Grand Pacific Drive 南下，经过 Sea Cliff Bridge、Kiama 与 Gerringong，视情况延伸袋鼠谷。</x:v>
+        <x:v>上午搭 F2 渡轮前往 Taronga；下午视天气直接前往 Bondi，若风雨仍大则回酒店休息，17:30 到 Totti's Bondi 用餐。</x:v>
       </x:c>
       <x:c r="J15" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="K15" t="str">
-        <x:v>南海岸晴天最出片；沿海有风，袋鼠谷山区傍晚更凉。</x:v>
+        <x:v>动物园高处、渡轮甲板和 Bondi 海边都有风；下午是否走海岸以当天降雨和风力为准。</x:v>
       </x:c>
       <x:c r="L15" t="str">
-        <x:v>海边防风，穿舒适步行鞋；出发前检查 Royal National Park 道路警报。</x:v>
+        <x:v>穿舒适步行鞋，薄外套与轻便雨具随身；Bondi 只走到 Tamarama 的短段。</x:v>
       </x:c>
       <x:c r="M15" t="str">
-        <x:v>/itinerary/d13-south-coast-kiama-gerringong.png</x:v>
+        <x:v>/itinerary/d14-taronga-bondi.png</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>Kiama 与 Gerringong 南海岸公路</x:v>
+        <x:v>Taronga Zoo、悉尼港与 Bondi 海岸</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>自驾（南海岸）</x:v>
+        <x:v>F2 Ferry + Uber / Taxi + 步行</x:v>
       </x:c>
       <x:c r="P15" t="str">
-        <x:v>08:00 出发；14:40 在 Gerringong 决定是否延伸袋鼠谷</x:v>
+        <x:v>08:45 左右出门；14:00 从 Taronga Zoo 正门离开；17:20 前抵达 Totti's Bondi</x:v>
       </x:c>
       <x:c r="Q15" t="str">
         <x:v>oaks-sydney-map</x:v>
       </x:c>
       <x:c r="R15" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>taronga-zoo-map</x:v>
       </x:c>
       <x:c r="S15" t="str">
-        <x:v>no-fixed-ticket</x:v>
+        <x:v>taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1503,7 +1503,7 @@
         <x:v>周二</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>悉尼</x:v>
+        <x:v>悉尼南海岸</x:v>
       </x:c>
       <x:c r="F16" t="n">
         <x:v>-33.8688</x:v>
@@ -1512,40 +1512,40 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>动物园到海岸：Taronga、Bondi 与 Totti's</x:v>
+        <x:v>南海岸环线：Sea Cliff Bridge、Kiama 与 Kangaroo Valley</x:v>
       </x:c>
       <x:c r="I16" t="str">
-        <x:v>搭渡轮看 Taronga 的澳洲动物，下午走 Bondi 海岸，晚上在 Totti's 用餐。</x:v>
+        <x:v>08:00 取车后沿海岸南下，经过 Bald Hill、Sea Cliff Bridge、Kiama 与 Werri Beach，再由 Kangaroo Valley 内陆返回悉尼。</x:v>
       </x:c>
       <x:c r="J16" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>悉尼冬季早晚凉，渡轮甲板、动物园高处和 Bondi 海边都有风。</x:v>
+        <x:v>沿海观景点风大，袋鼠谷山区傍晚更凉；出发前再次查看实时道路与天气。</x:v>
       </x:c>
       <x:c r="L16" t="str">
-        <x:v>穿舒适步行鞋，薄外套随身；Bondi 海岸步道只走短段。</x:v>
+        <x:v>穿防风外套与舒适步行鞋，车里备雨具、水和零食；驾驶员避免在返程前过度停留。</x:v>
       </x:c>
       <x:c r="M16" t="str">
-        <x:v>/itinerary/d14-taronga-bondi.png</x:v>
+        <x:v>/itinerary/d13-south-coast-kiama-gerringong.png</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>Taronga Zoo、悉尼港与 Bondi 海岸</x:v>
+        <x:v>Sea Cliff Bridge、Kiama 与 Kangaroo Valley 南海岸环线</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>F2 Ferry + 打车 / 市内交通 + 步行</x:v>
+        <x:v>SIXT 自驾 · 沿海去 / 内陆回（08:00–19:00，约 330–360 km）</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>08:30–09:00 出门前往 Circular Quay；18:15 前抵达 Totti's</x:v>
+        <x:v>07:25 离开酒店；14:00 离开 Werri Beach；15:30 离开 Kangaroo Valley；18:50 前还车</x:v>
       </x:c>
       <x:c r="Q16" t="str">
         <x:v>oaks-sydney-map</x:v>
       </x:c>
       <x:c r="R16" t="str">
-        <x:v>taronga-zoo-map</x:v>
+        <x:v>d14-south-coast-loop-map</x:v>
       </x:c>
       <x:c r="S16" t="str">
-        <x:v>taronga-zoo-official</x:v>
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1571,31 +1571,31 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H17" t="str">
-        <x:v>悉尼告别日：可选 Manly、最后采购与 Cafe Sydney</x:v>
+        <x:v>悉尼告别日：Bondi 补位、Manly 备选与 Cafe Sydney</x:v>
       </x:c>
       <x:c r="I17" t="str">
-        <x:v>上午悠闲安排 Manly 或 CBD，下午采购并整理行李，傍晚在 Cafe Sydney 告别。</x:v>
+        <x:v>若 8/10 未完成 Bondi，上午优先补走 Bondi；若已完成且天气与体力都好，再选 Manly，否则留在 CBD 慢慢收尾。下午采购、整理 TRS，17:30 在 Cafe Sydney 告别。</x:v>
       </x:c>
       <x:c r="J17" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>悉尼早晚凉，若去 Manly，渡轮甲板和海边风更明显。</x:v>
+        <x:v>Bondi 与 Manly 都受海风影响；上午路线按 8/10 的实际完成情况与当天体感决定。</x:v>
       </x:c>
       <x:c r="L17" t="str">
-        <x:v>薄外套随身；晚餐换 smart casual，并给回酒店整理行李留足时间。</x:v>
+        <x:v>薄外套随身；晚餐换 smart casual，并把发票、TRS 商品与返程行李提前整理好。</x:v>
       </x:c>
       <x:c r="M17" t="str">
         <x:v>/itinerary/d15-manly-flex-farewell.png</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>Manly 渡轮与悉尼港告别黄昏</x:v>
+        <x:v>悉尼海岸、渡轮与海港告别黄昏</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>F1 Ferry（可选） + 步行 / 市内交通</x:v>
+        <x:v>Uber / 市内交通；F1 Ferry 仅在选择 Manly 时使用</x:v>
       </x:c>
       <x:c r="P17" t="str">
-        <x:v>上午按状态决定；去 Manly 则 13:00–13:30 返程；16:40 前往 Cafe Sydney</x:v>
+        <x:v>上午按 8/10 实际完成情况决定；13:30 前回到 CBD；16:15 离开酒店前往 Circular Quay</x:v>
       </x:c>
       <x:c r="Q17" t="str">
         <x:v>oaks-sydney-map</x:v>
@@ -1791,16 +1791,16 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="C6" s="54" t="str">
-        <x:v>Barangaroo Reserve</x:v>
+        <x:v>Barangaroo 至 Circular Quay 海港步行</x:v>
       </x:c>
       <x:c r="D6" s="55" t="str">
         <x:v>必去</x:v>
       </x:c>
       <x:c r="E6" s="54" t="str">
-        <x:v>转场日下午沿 Wulugul Walk 慢走</x:v>
+        <x:v>15:00 后从 Barangaroo 起步，经 The Rocks 在 Circular Quay 看日落</x:v>
       </x:c>
       <x:c r="F6" s="54" t="str">
-        <x:v>barangaroo-reserve-map</x:v>
+        <x:v>d11-harbour-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
@@ -1811,16 +1811,16 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="C7" s="54" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>Mrs Macquarie's Chair + 歌剧院中文导览</x:v>
       </x:c>
       <x:c r="D7" s="55" t="str">
         <x:v>必去</x:v>
       </x:c>
       <x:c r="E7" s="54" t="str">
-        <x:v>中文导览后步行前往，停留 45–60 分钟</x:v>
+        <x:v>清晨先走海港机位与植物园，09:30 参加已订中文导览</x:v>
       </x:c>
       <x:c r="F7" s="54" t="str">
-        <x:v>the-rocks-market-official</x:v>
+        <x:v>d12-harbour-morning-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
@@ -4704,22 +4704,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>清晨</x:v>
+        <x:v>04:40–04:50</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>凯恩斯酒店 → 凯恩斯机场 T2</x:v>
+        <x:v>凯恩斯机场 T2</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>早起退房，打车 / Uber 前往机场</x:v>
+        <x:v>抵达机场，办理托运、安检与登机手续</x:v>
       </x:c>
       <x:c r="F110" t="str">
-        <x:v>从凯恩斯启程前往悉尼</x:v>
+        <x:v>从热带清晨启程前往悉尼</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
+        <x:v>前一晚完成打包；Jetstar 托运行李按订单额度分装，薄外套留在随身包。</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>cairns-airport-map</x:v>
+        <x:v>cairns-airport-map,jetstar-official</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -4730,21 +4730,23 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>上午</x:v>
+        <x:v>06:45–09:45</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>JQ953 飞往悉尼</x:v>
+        <x:v>搭乘 JQ953 飞往悉尼</x:v>
       </x:c>
       <x:c r="F111" t="str">
-        <x:v>从热带切换回冬季海港城市</x:v>
+        <x:v>从热带暖冬切换到冬季海港</x:v>
       </x:c>
       <x:c r="G111" t="str">
-        <x:v>随身带薄外套，悉尼比凯恩斯凉</x:v>
-      </x:c>
-      <x:c r="H111"/>
+        <x:v>起降时间以 Jetstar App 与登机牌为准；落地前把外套穿好。</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>cairns-airport-map,sydney-airport-map,jetstar-official</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" t="str">
@@ -4754,22 +4756,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>上午 / 中午</x:v>
+        <x:v>09:45–10:35</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>悉尼 T2 → 酒店</x:v>
+        <x:v>悉尼机场 T2</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>抵达后打车 / Uber 前往 Oaks Sydney Goldsbrough Suites</x:v>
+        <x:v>下机、取行李并集合</x:v>
       </x:c>
       <x:c r="F112" t="str">
-        <x:v>4人 + 行李，打车最省心</x:v>
+        <x:v>旅程进入悉尼阶段</x:v>
       </x:c>
       <x:c r="G112" t="str">
-        <x:v>如不能入住，先寄存行李</x:v>
+        <x:v>取齐四人的行李后再叫车，避免司机到达后等待。</x:v>
       </x:c>
       <x:c r="H112" t="str">
-        <x:v>oaks-sydney-map</x:v>
+        <x:v>sydney-airport-map</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -4780,22 +4782,22 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>下午</x:v>
+        <x:v>10:35–11:15</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Darling Harbour / 酒店周边</x:v>
+        <x:v>悉尼机场 T2 → 酒店</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>轻松适应，简单午餐或休息</x:v>
+        <x:v>4 人带行李，搭 Uber / Taxi 前往 Oaks Sydney Goldsbrough Suites</x:v>
       </x:c>
       <x:c r="F113" t="str">
-        <x:v>在 Darling Harbour 缓一缓</x:v>
+        <x:v>一次完成机场到酒店转场</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
+        <x:v>不能提前入住时先寄存行李；车程按当天交通为准。</x:v>
       </x:c>
       <x:c r="H113" t="str">
-        <x:v>darling-harbour-map</x:v>
+        <x:v>sydney-airport-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -4803,25 +4805,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B114" t="n">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>下午后段</x:v>
+        <x:v>11:15–12:30</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
+        <x:v>酒店 / Darling Harbour</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>从 Darling Harbour 沿海滨前往 Barangaroo Reserve，再衔接 The Rocks</x:v>
+        <x:v>寄存行李并在附近简单午餐</x:v>
       </x:c>
       <x:c r="F114" t="str">
-        <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
+        <x:v>先把转场后的体力补回来</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
+        <x:v>午餐就近解决，不为餐厅专程绕路。</x:v>
       </x:c>
       <x:c r="H114" t="str">
-        <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
+        <x:v>oaks-sydney-map,darling-harbour-map</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -4829,25 +4831,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B115" t="n">
-        <x:v>50</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>傍晚</x:v>
+        <x:v>12:30–14:45</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>The Rocks</x:v>
+        <x:v>酒店</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>岩石区散步、晚餐</x:v>
+        <x:v>入住后洗澡、补觉与整理随身物品</x:v>
       </x:c>
       <x:c r="F115" t="str">
-        <x:v>砂岩老街与海港傍晚</x:v>
+        <x:v>用完整休息换一个舒服的海港傍晚</x:v>
       </x:c>
       <x:c r="G115" t="str">
-        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
+        <x:v>午后不增加景点；15:00 左右再出发。</x:v>
       </x:c>
       <x:c r="H115" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -4855,25 +4857,25 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B116" t="n">
-        <x:v>60</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>晚上</x:v>
+        <x:v>15:00–15:15</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>酒店 → Barangaroo Reserve</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>歌剧院、海港大桥夜景</x:v>
+        <x:v>体力一般时搭 Uber / Taxi 到 Barangaroo Reserve 起步</x:v>
       </x:c>
       <x:c r="F116" t="str">
-        <x:v>悉尼开场画面</x:v>
+        <x:v>从安静的海港公园开始第一段悉尼步行</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
+        <x:v>不必从 Pyrmont 全程步行过去，把脚力留给海港沿线。</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>circular-quay-map</x:v>
+        <x:v>oaks-sydney-map,barangaroo-reserve-map</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -4881,129 +4883,129 @@
         <x:v>d11</x:v>
       </x:c>
       <x:c r="B117" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>饮食</x:v>
+        <x:v>15:15–16:15</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Barangaroo Reserve / Wulugul Walk</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
+        <x:v>沿海港步道单向走向 The Rocks</x:v>
       </x:c>
       <x:c r="F117" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>原生植物、砂岩海岸与城市天际线</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
+        <x:v>沿水边慢走，途中看体力短停；这段不用赶速度。</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>the-rocks-map</x:v>
+        <x:v>barangaroo-reserve-map,the-rocks-map,d11-harbour-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B118" t="n">
-        <x:v>10</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>08:15–08:30</x:v>
+        <x:v>16:15–16:55</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Circular Quay</x:v>
+        <x:v>The Rocks</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>抵达海港区</x:v>
+        <x:v>走过砂岩老街与海港巷弄</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>Ferry、海港桥、歌剧院远景</x:v>
+        <x:v>悉尼老城区的傍晚质感</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>早到人少，光线舒服；可拍 Circular Quay 低机位 + Ferry + Opera House</x:v>
+        <x:v>以短走和拍照为主，晚餐放在日落之后。</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>circular-quay-map,opera-house-map</x:v>
+        <x:v>the-rocks-map,d11-harbour-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B119" t="n">
-        <x:v>20</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>08:30–09:10</x:v>
+        <x:v>17:00–17:45</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Opera House 外观</x:v>
+        <x:v>Circular Quay</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
+        <x:v>看歌剧院、海港大桥与日落后的蓝调</x:v>
       </x:c>
       <x:c r="F119" t="str">
-        <x:v>悉尼核心地标</x:v>
+        <x:v>悉尼第一组完整海港画面</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>导览前先拍外观，避免后面人多；重点拍帆形结构、台阶、侧面海港机位</x:v>
+        <x:v>8 月 8 日日落约 17:20；先看日落与亮灯，再去吃晚餐。</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>opera-house-map</x:v>
+        <x:v>circular-quay-map,opera-house-map,d11-harbour-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B120" t="n">
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>09:30–10:30</x:v>
+        <x:v>18:00 之后</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Sydney Opera House</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>中文内部导览已订</x:v>
+        <x:v>找一家舒服的餐厅或 pub 吃晚餐，饭后回酒店</x:v>
       </x:c>
       <x:c r="F120" t="str">
-        <x:v>建筑故事、内部空间、剧院结构</x:v>
+        <x:v>用轻松的一餐结束转场日</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>提前到集合点；导览需步行和上下台阶；允许拍摄的空间再拍，不要影响团队</x:v>
+        <x:v>不增加游船或正式大餐，吃完按体力打车或搭市内交通回酒店。</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>opera-house-map,opera-house-official</x:v>
+        <x:v>the-rocks-map,circular-quay-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" t="str">
-        <x:v>d12</x:v>
+        <x:v>d11</x:v>
       </x:c>
       <x:c r="B121" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>10:30–10:50</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Opera House → The Rocks</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>中文导览结束后沿 Circular Quay 步行前往 The Rocks Markets</x:v>
+        <x:v>早餐：机场 / 飞机简餐；午餐：Darling Harbour 就近解决；晚餐：The Rocks 或 Circular Quay</x:v>
       </x:c>
       <x:c r="F121" t="str">
-        <x:v>海港步行衔接悉尼老城区</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>步行约 15–20 分钟；沿途可拍 Ferry、Opera House 与 Harbour Bridge</x:v>
+        <x:v>转场日不追餐厅，先休息，再把晚餐接在海港日落之后。</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>opera-house-map,circular-quay-map,the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>darling-harbour-map,the-rocks-map,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -5011,25 +5013,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B122" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>10:50–11:50</x:v>
+        <x:v>07:30–07:45</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>The Rocks Markets</x:v>
+        <x:v>酒店 → Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>10:00–17:00 开放；中文导览结束后步行前往，停留约 45–60 分钟。</x:v>
+        <x:v>早餐后搭 Uber / Taxi 前往海港东侧</x:v>
       </x:c>
       <x:c r="F122" t="str">
-        <x:v>悉尼老城区、手作市集、Harbour Bridge 背景与本地周末氛围</x:v>
+        <x:v>把最重要的户外机位放在清晨</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>周日 10:00–17:00；导览后步行前往，停留 45–60 分钟。</x:v>
+        <x:v>若 08:00 前已经明显下雨，就直接前往歌剧院，在附近喝咖啡等候导览。</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official</x:v>
+        <x:v>oaks-sydney-map,mrs-macquarie-map,d12-hotel-to-mrs-map</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -5037,25 +5039,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B123" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>11:50–12:40</x:v>
+        <x:v>08:00–08:25</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>The Rocks / Circular Quay</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>市集小吃或简单午餐 / 咖啡</x:v>
+        <x:v>拍歌剧院与海港大桥同框</x:v>
       </x:c>
       <x:c r="F123" t="str">
-        <x:v>就地补体力，不为午餐绕路</x:v>
+        <x:v>清晨人少的悉尼明信片机位</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>若市集已吃饱，这里只补咖啡；给下午植物园和 QVB 留节奏</x:v>
+        <x:v>在石椅左侧与海港边各取一组构图；有雨或大风时缩短停留。</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>the-rocks-map,the-rocks-market-official,circular-quay-map</x:v>
+        <x:v>mrs-macquarie-map,d12-harbour-morning-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -5063,25 +5065,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B124" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>12:40–14:10</x:v>
+        <x:v>08:25–09:05</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Royal Botanic Garden</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>植物园海港步道</x:v>
+        <x:v>沿 Farm Cove 穿过植物园，单向步行前往歌剧院</x:v>
       </x:c>
       <x:c r="F124" t="str">
-        <x:v>海港景观非常好</x:v>
+        <x:v>晨光、草坪与海港一路相连</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>沿水边主步道前进，不在支线花园停太久；09:05 左右到歌剧院。</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>botanic-garden-map</x:v>
+        <x:v>botanic-garden-map,opera-house-map,d12-harbour-morning-walk-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -5089,25 +5091,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B125" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>14:10–15:10</x:v>
+        <x:v>09:05–09:20</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Mrs Macquarie's Chair</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>歌剧院 + 海港大桥同框</x:v>
+        <x:v>找到中文导览集合点、签到并上洗手间</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>悉尼最经典机位</x:v>
+        <x:v>为已订导览留出从容缓冲</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>晴天很好看，风大注意保暖；可在石椅机位左侧 45° 构图</x:v>
+        <x:v>把电子票和订单提前打开；09:20 前完成签到。</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>mrs-macquarie-map</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -5115,25 +5117,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B126" t="n">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>15:30–17:00</x:v>
+        <x:v>09:30–10:30</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>QVB / Westfield / CBD</x:v>
+        <x:v>Sydney Opera House</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>购物、室内休息</x:v>
+        <x:v>参加中文内部导览（已订）</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>建筑漂亮，适合逛</x:v>
+        <x:v>走进建筑内部与剧院空间</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>商店关门较早，别拖太晚；QVB 穹顶适合仰拍对称构图</x:v>
+        <x:v>导览包含步行与台阶；只在允许拍摄的区域取景。</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>qvb-map</x:v>
+        <x:v>opera-house-map,opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -5141,25 +5143,25 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B127" t="n">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>晚上</x:v>
+        <x:v>10:30–11:00</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>CBD / Darling Harbour</x:v>
+        <x:v>Opera House 周边</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Hello Auntie / CBD 晚餐</x:v>
+        <x:v>按天气补拍外观，或在附近喝咖啡休息</x:v>
       </x:c>
       <x:c r="F127" t="str">
-        <x:v>城市核心日收尾</x:v>
+        <x:v>给海港地标留一段自由时间</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
+        <x:v>天气转雨时不继续露天久走，直接进入午餐与 CBD 行程。</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>darling-harbour-map,hello-auntie-map</x:v>
+        <x:v>opera-house-map,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -5167,129 +5169,129 @@
         <x:v>d12</x:v>
       </x:c>
       <x:c r="B128" t="n">
-        <x:v>900</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>饮食</x:v>
+        <x:v>11:00–12:00</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Circular Quay / CBD</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>就近吃一顿简单午餐</x:v>
       </x:c>
       <x:c r="F128" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>不为餐厅增加折返</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
+        <x:v>午餐后直接前往 QVB / Westfield；下午主要在室内活动。</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
+        <x:v>circular-quay-map,qvb-map</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B129" t="n">
-        <x:v>10</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>08:00</x:v>
+        <x:v>12:15–15:30</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>悉尼 → Royal National Park / Bald Hill</x:v>
+        <x:v>QVB / Westfield / CBD</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>自驾南下，进入 Grand Pacific Drive</x:v>
+        <x:v>逛 QVB 建筑与商场，并提前完成大部分药妆和伴手礼采购</x:v>
       </x:c>
       <x:c r="F129" t="str">
-        <x:v>城市切换到南海岸</x:v>
+        <x:v>用室内城市漫步避开午后阵雨</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
+        <x:v>先看 QVB 穹顶与长廊，再按购物清单集中采购；保留 tax invoice。</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>royal-national-park-map,bald-hill-map</x:v>
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B130" t="n">
-        <x:v>20</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>09:15</x:v>
+        <x:v>15:30–17:00</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Bald Hill Lookout</x:v>
+        <x:v>酒店</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>俯瞰海岸线和 Sea Cliff Bridge</x:v>
+        <x:v>放下购物、休息并整理当天物品</x:v>
       </x:c>
       <x:c r="F130" t="str">
-        <x:v>南海岸第一处全景</x:v>
+        <x:v>在晚餐前留一段真正的空白</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>风大时缩短停留，优先保证后续 Kiama 与 Gerringong 时间</x:v>
+        <x:v>下午购物完成后直接回酒店，不再临时增加长距离景点。</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>bald-hill-map,sea-cliff-map</x:v>
+        <x:v>oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>30</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>10:00</x:v>
+        <x:v>晚上</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Sea Cliff Bridge</x:v>
+        <x:v>Darling Harbour / CBD</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>驶过海崖桥并在合法位置短停拍照</x:v>
+        <x:v>在 Hello Auntie 或酒店附近轻松吃晚餐</x:v>
       </x:c>
       <x:c r="F131" t="str">
-        <x:v>贴着太平洋的公路画面</x:v>
+        <x:v>用一顿舒服的城市晚餐收尾</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>不要在桥上或路肩危险停车</x:v>
+        <x:v>按大家体力选择餐厅；饭后可在 Darling Harbour 短走。</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>sea-cliff-map</x:v>
+        <x:v>darling-harbour-map,hello-auntie-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" t="str">
-        <x:v>d13</x:v>
+        <x:v>d12</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>40</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>11:15</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>Wollongong / 南海岸补给</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>短停咖啡或直接通过</x:v>
+        <x:v>早餐：酒店附近 café；午餐：Circular Quay / CBD 简餐；晚餐：Hello Auntie 或酒店附近</x:v>
       </x:c>
       <x:c r="F132" t="str">
-        <x:v>为 Kiama 留出完整窗口</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
+        <x:v>上午围绕 09:30 导览安排，午餐不绕路，晚上按体力轻松选择。</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>wollongong-map</x:v>
+        <x:v>circular-quay-map,hello-auntie-map,oaks-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -5297,25 +5299,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B133" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>12:00</x:v>
+        <x:v>08:45–09:15</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>Kiama Blowhole</x:v>
+        <x:v>酒店 → Circular Quay</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>看喷潮洞、灯塔与海边</x:v>
+        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
       </x:c>
       <x:c r="F133" t="str">
-        <x:v>Kiama 代表性海岸地貌</x:v>
+        <x:v>沿悉尼港开启动物与海岸日</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>海况决定喷潮效果；没有大浪也不必等待太久</x:v>
+        <x:v>提前查看当天 F2 船班；建议在 09:15 左右抵达码头。</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>kiama-map</x:v>
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -5323,25 +5325,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B134" t="n">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>12:30–13:30</x:v>
+        <x:v>09:20–09:45</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>Kiama</x:v>
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>午餐与短暂休息</x:v>
+        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>海边小镇节奏</x:v>
+        <x:v>从水上看歌剧院、海港桥与城市天际线</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>午餐控制在一小时左右，下午还要去 Gerringong</x:v>
+        <x:v>Opal / contactless 即可；到站后沿指示进入动物园。</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -5349,25 +5351,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B135" t="n">
-        <x:v>70</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>13:30</x:v>
+        <x:v>10:00–14:00</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>Kiama → Gerringong</x:v>
+        <x:v>Taronga Zoo</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>沿海继续南下</x:v>
+        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
       </x:c>
       <x:c r="F135" t="str">
-        <x:v>海岸逐渐转为农场与小镇</x:v>
+        <x:v>澳洲本土动物与 Harbour view</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
+        <x:v>先看最想看的澳洲动物，再按当天 keeper talk 调整；午餐在园内简单解决。</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>kiama-map,gerringong-map</x:v>
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -5375,25 +5377,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B136" t="n">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>13:45–14:40</x:v>
+        <x:v>14:00</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>Gerringong / Werri Beach</x:v>
+        <x:v>Taronga Zoo 正门</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>看海岸、草坡与小镇，短停咖啡或散步</x:v>
+        <x:v>根据海边风雨决定下一站</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>南海岸与乡村景观同框</x:v>
+        <x:v>把 Bondi 留给真正舒服的天气</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
+        <x:v>天气转好就从正门直接 Uber / Taxi 去 Bondi，不再搭船绕回 Circular Quay；若仍有明显风雨，就回酒店休息。</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>gerringong-map</x:v>
+        <x:v>d13-taronga-to-bondi-map,oaks-sydney-map,bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -5401,25 +5403,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B137" t="n">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>14:40</x:v>
+        <x:v>天气好 · 14:30–16:50</x:v>
       </x:c>
       <x:c r="D137" t="str">
-        <x:v>Gerringong</x:v>
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>判断是否延伸 Kangaroo Valley</x:v>
+        <x:v>沿海滩与 Coastal Walk 走一段短线</x:v>
       </x:c>
       <x:c r="F137" t="str">
-        <x:v>时间、天气与体力闸门</x:v>
+        <x:v>泳池、海浪与悬崖海岸线</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>若已晚于 14:45、天气转差或驾驶疲劳，直接返回悉尼</x:v>
+        <x:v>只走 Bondi–Tamarama 短段；16:50 左右离开海边，给晚餐留出转场时间。</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>gerringong-map,kangaroo-valley-map</x:v>
+        <x:v>bondi-map,icebergs-map,tamarama-map,d13-taronga-to-bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -5427,25 +5429,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B138" t="n">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>可选 15:30–16:15</x:v>
+        <x:v>天气欠佳 · 14:30–16:30</x:v>
       </x:c>
       <x:c r="D138" t="str">
-        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
+        <x:v>酒店休息</x:v>
       </x:c>
       <x:c r="E138" t="str">
-        <x:v>看历史桥、山谷与小镇</x:v>
+        <x:v>回房间休息、换装，再直接前往 Totti's Bondi</x:v>
       </x:c>
       <x:c r="F138" t="str">
-        <x:v>海岸日的乡村加餐</x:v>
+        <x:v>雨天也保留一顿从容晚餐</x:v>
       </x:c>
       <x:c r="G138" t="str">
-        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
+        <x:v>若今天没有完成 Bondi，把它留到 D15 上午，D15 的 Manly 随之取消。</x:v>
       </x:c>
       <x:c r="H138" t="str">
-        <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
+        <x:v>oaks-sydney-map,d15-bondi-fallback-route-map,tottis-bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -5453,25 +5455,25 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B139" t="n">
-        <x:v>110</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>16:15 前</x:v>
+        <x:v>16:50–17:20</x:v>
       </x:c>
       <x:c r="D139" t="str">
-        <x:v>Kangaroo Valley / Gerringong → Sydney</x:v>
+        <x:v>Bondi Beach / 酒店 → Totti's Bondi</x:v>
       </x:c>
       <x:c r="E139" t="str">
-        <x:v>返程；去了袋鼠谷优先走内陆 M31，未去则从 Gerringong 直接北返</x:v>
+        <x:v>按当天所在位置前往餐厅</x:v>
       </x:c>
       <x:c r="F139" t="str">
-        <x:v>环线收束</x:v>
+        <x:v>从海岸或酒店从容转入晚餐</x:v>
       </x:c>
       <x:c r="G139" t="str">
-        <x:v>目标 18:30 左右回城，晚餐保持简单</x:v>
+        <x:v>餐厅在 Bondi Road，不在沙滩第一排；预留叫车和堵车时间。</x:v>
       </x:c>
       <x:c r="H139" t="str">
-        <x:v>kangaroo-valley-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>bondi-map,oaks-sydney-map,tottis-bondi-map</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -5479,51 +5481,51 @@
         <x:v>d13</x:v>
       </x:c>
       <x:c r="B140" t="n">
-        <x:v>900</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C140" t="str">
-        <x:v>饮食</x:v>
+        <x:v>17:30</x:v>
       </x:c>
       <x:c r="D140" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E140" t="str">
-        <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>分享式 Italian 晚餐（已订）</x:v>
       </x:c>
       <x:c r="F140" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>puffy bread + shared plates</x:v>
       </x:c>
       <x:c r="G140" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
+        <x:v>按 17:30 的预订入座；结束后直接回酒店休息。</x:v>
       </x:c>
       <x:c r="H140" t="str">
-        <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
+        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" t="str">
-        <x:v>d14</x:v>
+        <x:v>d13</x:v>
       </x:c>
       <x:c r="B141" t="n">
-        <x:v>10</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C141" t="str">
-        <x:v>08:30–09:00</x:v>
+        <x:v>饮食</x:v>
       </x:c>
       <x:c r="D141" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E141" t="str">
-        <x:v>前往公共 F2 Taronga Zoo Ferry 码头</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食；晚餐：Totti's Bondi 17:30（已订）</x:v>
       </x:c>
       <x:c r="F141" t="str">
-        <x:v>悉尼港开启动物与海岸日</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G141" t="str">
-        <x:v>提前查看当天 Trip Planner，建议在开园前后抵达</x:v>
+        <x:v>动物园午餐简单些；无论下午是否走 Bondi，都按 17:30 的预订前往 Totti's。</x:v>
       </x:c>
       <x:c r="H141" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
+        <x:v>taronga-zoo-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
@@ -5531,25 +5533,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B142" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C142" t="str">
-        <x:v>09:15 左右</x:v>
+        <x:v>07:25–07:45</x:v>
       </x:c>
       <x:c r="D142" t="str">
-        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+        <x:v>Oaks Sydney Goldsbrough Suites → SIXT Sydney City</x:v>
       </x:c>
       <x:c r="E142" t="str">
-        <x:v>搭乘公共 F2 Ferry 前往 Taronga Zoo</x:v>
+        <x:v>打车前往 Domain Car Park 内的 SIXT 门店</x:v>
       </x:c>
       <x:c r="F142" t="str">
-        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+        <x:v>在早高峰前抵达取车点</x:v>
       </x:c>
       <x:c r="G142" t="str">
-        <x:v>Opal / contactless 即可；建议坐上层甲板</x:v>
+        <x:v>门店地址为 52 Sir John Young Crescent；直接把完整地址交给司机。</x:v>
       </x:c>
       <x:c r="H142" t="str">
-        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
+        <x:v>d14-hotel-to-sixt-map,sixt-sydney-city-map</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -5557,25 +5559,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B143" t="n">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C143" t="str">
-        <x:v>09:30–13:30</x:v>
+        <x:v>07:45–08:20</x:v>
       </x:c>
       <x:c r="D143" t="str">
-        <x:v>Taronga Zoo</x:v>
+        <x:v>SIXT Sydney City</x:v>
       </x:c>
       <x:c r="E143" t="str">
-        <x:v>优先游览 Australian Wildlife 区域与悉尼港景观</x:v>
+        <x:v>办理取车并检查车身、轮毂、挡风玻璃、油量与 CarPlay</x:v>
       </x:c>
       <x:c r="F143" t="str">
-        <x:v>澳洲本土动物 + Harbour view</x:v>
+        <x:v>08:00–19:00 的自驾窗口正式开始</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
+        <x:v>门店工作日 07:30–16:00，晚间使用 after-hours return；取车时确认还车车位和钥匙投递位置。</x:v>
       </x:c>
       <x:c r="H143" t="str">
-        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
+        <x:v>sixt-sydney-city-map,sixt-sydney-city-official,d14-south-coast-loop-map</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -5583,25 +5585,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B144" t="n">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C144" t="str">
-        <x:v>13:30–14:30</x:v>
+        <x:v>08:20–09:25</x:v>
       </x:c>
       <x:c r="D144" t="str">
-        <x:v>Taronga Zoo Wharf → Circular Quay → Bondi</x:v>
+        <x:v>SIXT Sydney City → Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E144" t="str">
-        <x:v>F2 返回市区后前往 Bondi</x:v>
+        <x:v>沿主路驶向 Otford，开始 Grand Pacific Drive</x:v>
       </x:c>
       <x:c r="F144" t="str">
-        <x:v>动物园切换到悉尼海岸</x:v>
+        <x:v>城市道路逐渐切换到南海岸</x:v>
       </x:c>
       <x:c r="G144" t="str">
-        <x:v>午餐保持轻量；回到 Circular Quay 后打车去 Bondi 更省时间</x:v>
+        <x:v>副驾负责导航；途中不临时增加 Royal National Park 支线。</x:v>
       </x:c>
       <x:c r="H144" t="str">
-        <x:v>taronga-ferry-official,circular-quay-map,bondi-map</x:v>
+        <x:v>d14-coastal-route-map,bald-hill-map</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -5609,25 +5611,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B145" t="n">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C145" t="str">
-        <x:v>14:30–17:45</x:v>
+        <x:v>09:25–09:50</x:v>
       </x:c>
       <x:c r="D145" t="str">
-        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+        <x:v>Bald Hill Lookout</x:v>
       </x:c>
       <x:c r="E145" t="str">
-        <x:v>海滩散步并走一段 Coastal Walk</x:v>
+        <x:v>俯瞰海岸线与远处的 Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="F145" t="str">
-        <x:v>泳池、海浪、悬崖海岸线</x:v>
+        <x:v>南海岸第一处开阔全景</x:v>
       </x:c>
       <x:c r="G145" t="str">
-        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
+        <x:v>风大时缩短停留；09:50 左右继续出发。</x:v>
       </x:c>
       <x:c r="H145" t="str">
-        <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
+        <x:v>bald-hill-map,d14-coastal-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -5635,25 +5637,25 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B146" t="n">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C146" t="str">
-        <x:v>18:30</x:v>
+        <x:v>09:50–10:05</x:v>
       </x:c>
       <x:c r="D146" t="str">
-        <x:v>Totti's Bondi</x:v>
+        <x:v>Bald Hill → Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E146" t="str">
-        <x:v>分享式 Italian 晚餐（已订）</x:v>
+        <x:v>沿 Lawrence Hargrave Drive 继续南下</x:v>
       </x:c>
       <x:c r="F146" t="str">
-        <x:v>puffy bread + shared plates</x:v>
+        <x:v>贴近太平洋的短途转场</x:v>
       </x:c>
       <x:c r="G146" t="str">
-        <x:v>餐厅在 Bondi Road，不在沙滩第一排；建议 18:15 前抵达</x:v>
+        <x:v>按导航通过 Stanwell Park 与 Clifton，不在弯道或路肩临时停车。</x:v>
       </x:c>
       <x:c r="H146" t="str">
-        <x:v>tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>d14-coastal-route-map,sea-cliff-map</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
@@ -5661,310 +5663,674 @@
         <x:v>d14</x:v>
       </x:c>
       <x:c r="B147" t="n">
-        <x:v>900</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C147" t="str">
-        <x:v>饮食</x:v>
+        <x:v>10:05–10:40</x:v>
       </x:c>
       <x:c r="D147" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Sea Cliff Bridge</x:v>
       </x:c>
       <x:c r="E147" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
+        <x:v>先驶过海崖桥，再在合法停车位置停好车，步行体验一小段</x:v>
       </x:c>
       <x:c r="F147" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>公路悬在海岸与山崖之间</x:v>
       </x:c>
       <x:c r="G147" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
+        <x:v>桥上不能停车；只在合法位置上下车，10:40 左右继续前往 Kiama。</x:v>
       </x:c>
       <x:c r="H147" t="str">
-        <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
+        <x:v>sea-cliff-map,d14-coastal-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B148" t="n">
-        <x:v>10</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C148" t="str">
-        <x:v>上午</x:v>
+        <x:v>10:40–11:30</x:v>
       </x:c>
       <x:c r="D148" t="str">
-        <x:v>酒店 / 悉尼市区</x:v>
+        <x:v>Sea Cliff Bridge → Kiama</x:v>
       </x:c>
       <x:c r="E148" t="str">
-        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
+        <x:v>沿海岸主路直接前往 Kiama</x:v>
       </x:c>
       <x:c r="F148" t="str">
-        <x:v>告别日从容开场</x:v>
+        <x:v>把完整午间窗口留给喷潮洞与小镇</x:v>
       </x:c>
       <x:c r="G148" t="str">
-        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
+        <x:v>今天不在 Wollongong 停留；按主路继续南下。</x:v>
       </x:c>
       <x:c r="H148" t="str">
-        <x:v>oaks-sydney-map,qvb-map</x:v>
+        <x:v>d14-coastal-route-map,kiama-map</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B149" t="n">
-        <x:v>20</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C149" t="str">
-        <x:v>可选 09:30 左右</x:v>
+        <x:v>11:30–12:05</x:v>
       </x:c>
       <x:c r="D149" t="str">
-        <x:v>Circular Quay → Manly</x:v>
+        <x:v>Kiama Blowhole / Lighthouse</x:v>
       </x:c>
       <x:c r="E149" t="str">
-        <x:v>搭乘公共 F1 Manly Ferry</x:v>
+        <x:v>看喷潮洞、灯塔与海岸线</x:v>
       </x:c>
       <x:c r="F149" t="str">
-        <x:v>悉尼港经典渡轮体验</x:v>
+        <x:v>Kiama 最具代表性的海边画面</x:v>
       </x:c>
       <x:c r="G149" t="str">
-        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
+        <x:v>喷潮效果取决于海况；无大浪时看完主视角即可，不为等待浪花拖延午餐。</x:v>
       </x:c>
       <x:c r="H149" t="str">
-        <x:v>circular-quay-map,manly-ferry-map</x:v>
+        <x:v>kiama-map,kiama-lighthouse-map,d14-coastal-route-map</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B150" t="n">
-        <x:v>30</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C150" t="str">
-        <x:v>可选 10:00–12:45</x:v>
+        <x:v>12:05–13:00</x:v>
       </x:c>
       <x:c r="D150" t="str">
-        <x:v>Manly Beach / The Corso</x:v>
+        <x:v>Kiama</x:v>
       </x:c>
       <x:c r="E150" t="str">
-        <x:v>海边散步、咖啡或早午餐</x:v>
+        <x:v>午餐与短暂休息</x:v>
       </x:c>
       <x:c r="F150" t="str">
-        <x:v>比 Bondi 更松弛</x:v>
+        <x:v>在海边小镇补充体力</x:v>
       </x:c>
       <x:c r="G150" t="str">
-        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
+        <x:v>午餐控制在一小时内，13:00 准时继续去 Werri Beach。</x:v>
       </x:c>
       <x:c r="H150" t="str">
-        <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
+        <x:v>kiama-map,kiama-hungry-monkey-map</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B151" t="n">
-        <x:v>40</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C151" t="str">
-        <x:v>13:00–13:30</x:v>
+        <x:v>13:00–13:15</x:v>
       </x:c>
       <x:c r="D151" t="str">
-        <x:v>Manly → Circular Quay / CBD</x:v>
+        <x:v>Kiama → Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E151" t="str">
-        <x:v>最晚搭船回市区</x:v>
+        <x:v>沿海短途前往 Werri Beach</x:v>
       </x:c>
       <x:c r="F151" t="str">
-        <x:v>给采购、TRS 和晚餐留余量</x:v>
+        <x:v>海岸逐渐切换为草坡与农场</x:v>
       </x:c>
       <x:c r="G151" t="str">
-        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
+        <x:v>这一段不加停靠，按导航直达海边停车区。</x:v>
       </x:c>
       <x:c r="H151" t="str">
-        <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
+        <x:v>d14-coastal-route-map,gerringong-map</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
       <x:c r="A152" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B152" t="n">
-        <x:v>50</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C152" t="str">
-        <x:v>14:00–15:30</x:v>
+        <x:v>13:15–14:00</x:v>
       </x:c>
       <x:c r="D152" t="str">
-        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+        <x:v>Gerringong / Werri Beach</x:v>
       </x:c>
       <x:c r="E152" t="str">
-        <x:v>最后采购</x:v>
+        <x:v>看海岸、草坡与小镇，沿海边短走</x:v>
       </x:c>
       <x:c r="F152" t="str">
-        <x:v>药妆、保健品、伴手礼</x:v>
+        <x:v>海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G152" t="str">
-        <x:v>只补漏买；保留 tax invoice 并核对 TRS 条件</x:v>
+        <x:v>14:00 是第一个时间闸门；无论停留状态如何，都按时转向 Kangaroo Valley。</x:v>
       </x:c>
       <x:c r="H152" t="str">
-        <x:v>qvb-map,chemist-warehouse-map</x:v>
+        <x:v>gerringong-map,d14-inland-return-map</x:v>
       </x:c>
     </x:row>
     <x:row r="153">
       <x:c r="A153" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B153" t="n">
-        <x:v>60</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C153" t="str">
-        <x:v>15:30–16:20</x:v>
+        <x:v>14:00–14:40</x:v>
       </x:c>
       <x:c r="D153" t="str">
-        <x:v>酒店</x:v>
+        <x:v>Werri Beach → Kangaroo Valley</x:v>
       </x:c>
       <x:c r="E153" t="str">
-        <x:v>整理 TRS 物品和返程行李</x:v>
+        <x:v>从海岸转入山谷道路，前往 Hampden Bridge</x:v>
       </x:c>
       <x:c r="F153" t="str">
-        <x:v>为 D16 机场退税做准备</x:v>
+        <x:v>从海边进入安静的绿色谷地</x:v>
       </x:c>
       <x:c r="G153" t="str">
-        <x:v>发票、商品、护照和支付卡集中整理；完成换装</x:v>
+        <x:v>弯道较多，保持舒服车距；不临时加入 Fitzroy Falls。</x:v>
       </x:c>
       <x:c r="H153" t="str">
-        <x:v>oaks-sydney-map,trs-official</x:v>
+        <x:v>d14-inland-return-map,hampden-bridge-map</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
       <x:c r="A154" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B154" t="n">
-        <x:v>70</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C154" t="str">
-        <x:v>16:40</x:v>
+        <x:v>14:40–15:25</x:v>
       </x:c>
       <x:c r="D154" t="str">
-        <x:v>酒店 → Circular Quay</x:v>
+        <x:v>Kangaroo Valley / Hampden Bridge</x:v>
       </x:c>
       <x:c r="E154" t="str">
-        <x:v>前往 Cafe Sydney</x:v>
+        <x:v>看历史悬索桥，并在村镇短走</x:v>
       </x:c>
       <x:c r="F154" t="str">
-        <x:v>避免迟到</x:v>
+        <x:v>砂岩桥塔与山谷小镇</x:v>
       </x:c>
       <x:c r="G154" t="str">
-        <x:v>Outdoor Terrace 晚上有风，带外套；17:15 左右开始餐厅签到</x:v>
+        <x:v>把停车、桥边观景与村镇散步合计控制在 45 分钟内。</x:v>
       </x:c>
       <x:c r="H154" t="str">
-        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+        <x:v>hampden-bridge-map,kangaroo-valley-map,d14-inland-return-map</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
       <x:c r="A155" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B155" t="n">
-        <x:v>80</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C155" t="str">
-        <x:v>17:30</x:v>
+        <x:v>15:25–15:30</x:v>
       </x:c>
       <x:c r="D155" t="str">
-        <x:v>Cafe Sydney</x:v>
+        <x:v>Kangaroo Valley</x:v>
       </x:c>
       <x:c r="E155" t="str">
-        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+        <x:v>完成上车与导航确认，正式返回悉尼</x:v>
       </x:c>
       <x:c r="F155" t="str">
-        <x:v>海港景观 + 澳洲最后一晚</x:v>
+        <x:v>第二个时间闸门</x:v>
       </x:c>
       <x:c r="G155" t="str">
-        <x:v>按预订时间入座；晚餐后回酒店做最终检查</x:v>
+        <x:v>15:30 前驶离袋鼠谷；不再增加沿途景点。</x:v>
       </x:c>
       <x:c r="H155" t="str">
-        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>d14-inland-return-map,sixt-sydney-city-map</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
       <x:c r="A156" t="str">
-        <x:v>d15</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B156" t="n">
-        <x:v>900</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C156" t="str">
-        <x:v>饮食</x:v>
+        <x:v>15:30–17:45</x:v>
       </x:c>
       <x:c r="D156" t="str">
-        <x:v>饮食安排</x:v>
+        <x:v>Kangaroo Valley → Sydney</x:v>
       </x:c>
       <x:c r="E156" t="str">
-        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>沿内陆主路与 M31 返回悉尼</x:v>
       </x:c>
       <x:c r="F156" t="str">
-        <x:v>当天餐食节奏</x:v>
+        <x:v>用较稳定的内陆路线收束环线</x:v>
       </x:c>
       <x:c r="G156" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
+        <x:v>途中按实时路况行驶；司机需要休息时，只在服务区做短停。</x:v>
       </x:c>
       <x:c r="H156" t="str">
-        <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+        <x:v>d14-inland-return-map,sixt-sydney-city-map</x:v>
       </x:c>
     </x:row>
     <x:row r="157">
       <x:c r="A157" t="str">
-        <x:v>d16</x:v>
+        <x:v>d14</x:v>
       </x:c>
       <x:c r="B157" t="n">
-        <x:v>10</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C157" t="str">
-        <x:v>上午</x:v>
+        <x:v>17:45–18:20</x:v>
       </x:c>
       <x:c r="D157" t="str">
-        <x:v>悉尼机场</x:v>
+        <x:v>Sydney / SIXT 门店附近</x:v>
       </x:c>
       <x:c r="E157" t="str">
-        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+        <x:v>按租车规则补满油，清点随身物品并拍下油表</x:v>
       </x:c>
       <x:c r="F157" t="str">
-        <x:v>满载而归</x:v>
+        <x:v>还车前完成最后检查</x:v>
       </x:c>
       <x:c r="G157" t="str">
-        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+        <x:v>加油站按当时位置搜索，避免为了指定品牌绕路。</x:v>
       </x:c>
       <x:c r="H157" t="str">
-        <x:v>sydney-airport-map,trs-official</x:v>
+        <x:v>sixt-sydney-city-map</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
       <x:c r="A158" t="str">
+        <x:v>d14</x:v>
+      </x:c>
+      <x:c r="B158" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>18:20–18:50</x:v>
+      </x:c>
+      <x:c r="D158" t="str">
+        <x:v>SIXT Sydney City</x:v>
+      </x:c>
+      <x:c r="E158" t="str">
+        <x:v>驶入指定还车区并完成 after-hours return</x:v>
+      </x:c>
+      <x:c r="F158" t="str">
+        <x:v>在 19:00 租期结束前交还车辆</x:v>
+      </x:c>
+      <x:c r="G158" t="str">
+        <x:v>按早上确认的车位停车、拍照并投递钥匙；18:50 前完成。</x:v>
+      </x:c>
+      <x:c r="H158" t="str">
+        <x:v>sixt-sydney-city-map,sixt-sydney-city-official,d14-south-coast-loop-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>d14</x:v>
+      </x:c>
+      <x:c r="B159" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E159" t="str">
+        <x:v>早餐：酒店附近 café；午餐：Kiama 简餐；晚餐：还车后在 CBD / 酒店附近简单吃</x:v>
+      </x:c>
+      <x:c r="F159" t="str">
+        <x:v>把时间留给海岸与安全返程</x:v>
+      </x:c>
+      <x:c r="G159" t="str">
+        <x:v>车里备水和零食；午餐控制在一小时内，晚餐不提前锁死。</x:v>
+      </x:c>
+      <x:c r="H159" t="str">
+        <x:v>kiama-map,kiama-hungry-monkey-map,oaks-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B160" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C160" t="str">
+        <x:v>08:30 左右</x:v>
+      </x:c>
+      <x:c r="D160" t="str">
+        <x:v>酒店</x:v>
+      </x:c>
+      <x:c r="E160" t="str">
+        <x:v>先回看 8/10 是否完成 Bondi，再结合天气与体力决定上午路线</x:v>
+      </x:c>
+      <x:c r="F160" t="str">
+        <x:v>告别日上午只完成一个方向</x:v>
+      </x:c>
+      <x:c r="G160" t="str">
+        <x:v>若 8/10 没去成 Bondi，今天优先补 Bondi并取消 Manly；若已经完成 Bondi，再从 Manly 或 CBD 中二选一。</x:v>
+      </x:c>
+      <x:c r="H160" t="str">
+        <x:v>oaks-sydney-map,d15-bondi-fallback-route-map,manly-ferry-map,qvb-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B161" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C161" t="str">
+        <x:v>Bondi 补位 · 09:00–12:30</x:v>
+      </x:c>
+      <x:c r="D161" t="str">
+        <x:v>Bondi Beach → Icebergs → Tamarama</x:v>
+      </x:c>
+      <x:c r="E161" t="str">
+        <x:v>补走 8/10 因天气未完成的 Bondi 短线</x:v>
+      </x:c>
+      <x:c r="F161" t="str">
+        <x:v>把悉尼海岸的缺口补完整</x:v>
+      </x:c>
+      <x:c r="G161" t="str">
+        <x:v>只在 8/10 未完成 Bondi 时使用；12:30 左右返程，Manly 不再安排。</x:v>
+      </x:c>
+      <x:c r="H161" t="str">
+        <x:v>d15-bondi-fallback-route-map,bondi-map,icebergs-map,tamarama-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B162" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C162" t="str">
+        <x:v>Manly 备选 · 09:00–12:30</x:v>
+      </x:c>
+      <x:c r="D162" t="str">
+        <x:v>Circular Quay → Manly</x:v>
+      </x:c>
+      <x:c r="E162" t="str">
+        <x:v>若 Bondi 已完成且天气、体力都好，搭 F1 Ferry 去 Manly 短走</x:v>
+      </x:c>
+      <x:c r="F162" t="str">
+        <x:v>渡轮本身就是一次海港巡游</x:v>
+      </x:c>
+      <x:c r="G162" t="str">
+        <x:v>只在 Bondi 已完成时选择；逛 The Corso 与海边后，12:30 左右准备返程。</x:v>
+      </x:c>
+      <x:c r="H162" t="str">
+        <x:v>circular-quay-map,manly-ferry-map,manly-beach-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B163" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C163" t="str">
+        <x:v>CBD 慢行 · 上午</x:v>
+      </x:c>
+      <x:c r="D163" t="str">
+        <x:v>CBD / 酒店附近</x:v>
+      </x:c>
+      <x:c r="E163" t="str">
+        <x:v>若不去海边，就慢早餐、喝咖啡并在市区轻松收尾</x:v>
+      </x:c>
+      <x:c r="F163" t="str">
+        <x:v>给最后一天留一点真正空白</x:v>
+      </x:c>
+      <x:c r="G163" t="str">
+        <x:v>上午不再临时加长线，午后仍按固定节奏采购和整理。</x:v>
+      </x:c>
+      <x:c r="H163" t="str">
+        <x:v>oaks-sydney-map,qvb-map,single-o-map,tobys-estate-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B164" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>12:30–13:30</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>Bondi / Manly → CBD</x:v>
+      </x:c>
+      <x:c r="E164" t="str">
+        <x:v>从上午路线返回市区</x:v>
+      </x:c>
+      <x:c r="F164" t="str">
+        <x:v>给最后采购与 TRS 留足余量</x:v>
+      </x:c>
+      <x:c r="G164" t="str">
+        <x:v>最晚 13:30 回到 CBD；若上午留在市区，可以直接开始采购。</x:v>
+      </x:c>
+      <x:c r="H164" t="str">
+        <x:v>d15-bondi-fallback-route-map,manly-ferry-map,qvb-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B165" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C165" t="str">
+        <x:v>13:30–15:15</x:v>
+      </x:c>
+      <x:c r="D165" t="str">
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+      </x:c>
+      <x:c r="E165" t="str">
+        <x:v>完成最后采购</x:v>
+      </x:c>
+      <x:c r="F165" t="str">
+        <x:v>药妆、保健品与伴手礼一次买齐</x:v>
+      </x:c>
+      <x:c r="G165" t="str">
+        <x:v>只补漏买；保留 tax invoice，并核对 TRS 商品与支付凭证。</x:v>
+      </x:c>
+      <x:c r="H165" t="str">
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B166" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C166" t="str">
+        <x:v>15:15–16:00</x:v>
+      </x:c>
+      <x:c r="D166" t="str">
+        <x:v>酒店</x:v>
+      </x:c>
+      <x:c r="E166" t="str">
+        <x:v>整理 TRS 物品、返程行李并换装</x:v>
+      </x:c>
+      <x:c r="F166" t="str">
+        <x:v>把 D16 机场手续提前准备好</x:v>
+      </x:c>
+      <x:c r="G166" t="str">
+        <x:v>发票、商品、护照和支付卡集中放好；16:00 前完成整理。</x:v>
+      </x:c>
+      <x:c r="H166" t="str">
+        <x:v>oaks-sydney-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B167" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C167" t="str">
+        <x:v>16:15–16:50</x:v>
+      </x:c>
+      <x:c r="D167" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E167" t="str">
+        <x:v>前往 Cafe Sydney 一带</x:v>
+      </x:c>
+      <x:c r="F167" t="str">
+        <x:v>给海港黄昏与签到留余量</x:v>
+      </x:c>
+      <x:c r="G167" t="str">
+        <x:v>Outdoor Terrace 晚上有风，外套随身；不要等到 17:00 后才出发。</x:v>
+      </x:c>
+      <x:c r="H167" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B168" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C168" t="str">
+        <x:v>16:50–17:15</x:v>
+      </x:c>
+      <x:c r="D168" t="str">
+        <x:v>Circular Quay / 海港边</x:v>
+      </x:c>
+      <x:c r="E168" t="str">
+        <x:v>在餐前看海港黄昏并拍照，随后到 Cafe Sydney 签到</x:v>
+      </x:c>
+      <x:c r="F168" t="str">
+        <x:v>最后一次看歌剧院与海港桥亮灯</x:v>
+      </x:c>
+      <x:c r="G168" t="str">
+        <x:v>17:15 左右进入餐厅签到，不为拍照压缩预订时间。</x:v>
+      </x:c>
+      <x:c r="H168" t="str">
+        <x:v>circular-quay-map,opera-house-map,cafe-sydney-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B169" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C169" t="str">
+        <x:v>17:30</x:v>
+      </x:c>
+      <x:c r="D169" t="str">
+        <x:v>Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="E169" t="str">
+        <x:v>Outdoor Terrace Dining 告别晚餐（已订）</x:v>
+      </x:c>
+      <x:c r="F169" t="str">
+        <x:v>海港景观与澳洲最后一晚</x:v>
+      </x:c>
+      <x:c r="G169" t="str">
+        <x:v>按预订时间入座；晚餐后回酒店做最终检查。</x:v>
+      </x:c>
+      <x:c r="H169" t="str">
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B170" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C170" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D170" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E170" t="str">
+        <x:v>早餐：按 Bondi / Manly / CBD 路线解决；午餐：海边 café 或 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="F170" t="str">
+        <x:v>当天餐食节奏</x:v>
+      </x:c>
+      <x:c r="G170" t="str">
+        <x:v>上午只选一条路线，13:30 前回 CBD；下午采购、整理 TRS，再去 Cafe Sydney。</x:v>
+      </x:c>
+      <x:c r="H170" t="str">
+        <x:v>bondi-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
         <x:v>d16</x:v>
       </x:c>
-      <x:c r="B158" t="n">
+      <x:c r="B171" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E171" t="str">
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
+      </x:c>
+      <x:c r="F171" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G171" t="str">
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H171" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B172" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C158" t="str">
+      <x:c r="C172" t="str">
         <x:v>饮食</x:v>
       </x:c>
-      <x:c r="D158" t="str">
+      <x:c r="D172" t="str">
         <x:v>饮食安排</x:v>
       </x:c>
-      <x:c r="E158" t="str">
+      <x:c r="E172" t="str">
         <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
-      <x:c r="F158" t="str">
+      <x:c r="F172" t="str">
         <x:v>返程日简单省心</x:v>
       </x:c>
-      <x:c r="G158" t="str">
+      <x:c r="G172" t="str">
         <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
-      <x:c r="H158"/>
+      <x:c r="H172"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6761,8 +7127,8 @@
       <x:c r="D41" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Curtain+Fig+Tree%2C+Fig+Tree+Road%2C+East+Barron+QLD+4883&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E41" t="str"/>
-      <x:c r="F41" t="str"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
       <x:c r="G41" t="str">
         <x:v>Google Maps · Fig Tree Road, East Barron</x:v>
       </x:c>
@@ -6818,8 +7184,8 @@
       <x:c r="D44" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Millaa+Millaa+Falls%2C+Falls+Road%2C+Millaa+Millaa+QLD+4886&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E44" t="str"/>
-      <x:c r="F44" t="str"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
       <x:c r="G44" t="str">
         <x:v>Google Maps · Falls Road, Millaa Millaa</x:v>
       </x:c>
@@ -7044,12 +7410,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Sea+Cliff+Bridge</x:v>
-      </x:c>
-      <x:c r="E56"/>
-      <x:c r="F56"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Sea+Cliff+Bridge%2C+Clifton+NSW+2515&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E56" t="str"/>
+      <x:c r="F56" t="str"/>
       <x:c r="G56" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Sea Cliff Bridge, Clifton</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -7063,12 +7429,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Kiama+Blowhole</x:v>
-      </x:c>
-      <x:c r="E57"/>
-      <x:c r="F57"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Kiama+Blowhole%2C+Blowhole+Point+Road%2C+Kiama+NSW+2533&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E57" t="str"/>
+      <x:c r="F57" t="str"/>
       <x:c r="G57" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Blowhole Point, Kiama</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -7614,12 +7980,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Bald+Hill+Lookout+Stanwell+Tops</x:v>
-      </x:c>
-      <x:c r="E86"/>
-      <x:c r="F86"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Bald+Hill+Lookout%2C+Otford+NSW+2508&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E86" t="str"/>
+      <x:c r="F86" t="str"/>
       <x:c r="G86" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Bald Hill Lookout, Otford</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -8370,12 +8736,12 @@
         <x:v>map</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Gerringong+Werri+Beach+NSW</x:v>
-      </x:c>
-      <x:c r="E126"/>
-      <x:c r="F126"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Werri+Beach%2C+Pacific+Avenue%2C+Gerringong+NSW+2534&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E126" t="str"/>
+      <x:c r="F126" t="str"/>
       <x:c r="G126" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Werri Beach, Gerringong</x:v>
       </x:c>
     </x:row>
     <x:row r="127" s="23" customFormat="1" ht="30" customHeight="1">
@@ -8459,18 +8825,18 @@
         <x:v>hampden-bridge-map</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Hampden Bridge, Kangaroo Valley</x:v>
+        <x:v>Hampden Bridge</x:v>
       </x:c>
       <x:c r="C131" t="str">
         <x:v>map</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Hampden+Bridge+Kangaroo+Valley+NSW</x:v>
-      </x:c>
-      <x:c r="E131"/>
-      <x:c r="F131"/>
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Hampden+Bridge%2C+Moss+Vale+Road%2C+Kangaroo+Valley+NSW+2577&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E131" t="str"/>
+      <x:c r="F131" t="str"/>
       <x:c r="G131" t="str">
-        <x:v>Google Maps</x:v>
+        <x:v>Google Maps · Moss Vale Road, Kangaroo Valley</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -9254,8 +9620,8 @@
       <x:c r="D172" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Cairns+QLD&amp;travelmode=driving&amp;waypoints=Kuranda+Village%7CMareeba+QLD%7CSkybury+Cafe+and+Roastery%7CLake+Eacham+Day+Use+Area%7CYungaburra+Village%7CCurtain+Fig+Tree%7CMillaa+Millaa+Public+Toilets%7CMillaa+Millaa+Falls</x:v>
       </x:c>
-      <x:c r="E172" t="str"/>
-      <x:c r="F172" t="str"/>
+      <x:c r="E172"/>
+      <x:c r="F172"/>
       <x:c r="G172" t="str">
         <x:v>Google Maps · Cairns → Kuranda → Mareeba → Skybury → Lake Eacham → Yungaburra → Curtain Fig → Millaa Millaa → Cairns</x:v>
       </x:c>
@@ -9311,8 +9677,8 @@
       <x:c r="D175" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Millaa+Millaa+Falls&amp;destination=Cairns+QLD&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E175" t="str"/>
-      <x:c r="F175" t="str"/>
+      <x:c r="E175"/>
+      <x:c r="F175"/>
       <x:c r="G175" t="str">
         <x:v>Google Maps · 返程前重新打开，按实时路况使用铺装主路</x:v>
       </x:c>
@@ -9349,8 +9715,8 @@
       <x:c r="D177" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Lake+Eacham+Day+Use+Area%2C+Lakes+Drive%2C+Lake+Eacham+QLD+4884&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E177" t="str"/>
-      <x:c r="F177" t="str"/>
+      <x:c r="E177"/>
+      <x:c r="F177"/>
       <x:c r="G177" t="str">
         <x:v>Google Maps · Lakes Drive, Lake Eacham</x:v>
       </x:c>
@@ -9387,8 +9753,8 @@
       <x:c r="D179" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Yungaburra+QLD+4884&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E179" t="str"/>
-      <x:c r="F179" t="str"/>
+      <x:c r="E179"/>
+      <x:c r="F179"/>
       <x:c r="G179" t="str">
         <x:v>Google Maps · Yungaburra Village</x:v>
       </x:c>
@@ -9482,8 +9848,8 @@
       <x:c r="D184" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Millaa+Millaa+Public+Toilets%2C+Main+Street%2C+Millaa+Millaa+QLD&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E184" t="str"/>
-      <x:c r="F184" t="str"/>
+      <x:c r="E184"/>
+      <x:c r="F184"/>
       <x:c r="G184" t="str">
         <x:v>Google Maps · 镇中心，Millaa Millaa Hotel 对面</x:v>
       </x:c>
@@ -9577,8 +9943,8 @@
       <x:c r="D189" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Cairns+QLD&amp;destination=Skybury+Cafe+and+Roastery%2C+136+Ivicevic+Road%2C+Paddys+Green+QLD+4880&amp;travelmode=driving&amp;waypoints=Kuranda+Village%7CMareeba+QLD</x:v>
       </x:c>
-      <x:c r="E189" t="str"/>
-      <x:c r="F189" t="str"/>
+      <x:c r="E189"/>
+      <x:c r="F189"/>
       <x:c r="G189" t="str">
         <x:v>Google Maps · 北上段，依次经过 Kuranda 与 Mareeba</x:v>
       </x:c>
@@ -9596,8 +9962,8 @@
       <x:c r="D190" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Skybury+Cafe+and+Roastery%2C+136+Ivicevic+Road%2C+Paddys+Green+QLD+4880&amp;destination=Millaa+Millaa+Falls&amp;travelmode=driving&amp;waypoints=Lake+Eacham+Day+Use+Area%7CYungaburra+Village%7CCurtain+Fig+Tree%7CMillaa+Millaa+Public+Toilets</x:v>
       </x:c>
-      <x:c r="E190" t="str"/>
-      <x:c r="F190" t="str"/>
+      <x:c r="E190"/>
+      <x:c r="F190"/>
       <x:c r="G190" t="str">
         <x:v>Google Maps · 高原段，依次经过火山湖、小镇、巨树与镇中心厕所</x:v>
       </x:c>
@@ -9615,8 +9981,8 @@
       <x:c r="D191" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Kuranda+Village%2C+Coondoo+Street%2C+Kuranda+QLD+4881&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E191" t="str"/>
-      <x:c r="F191" t="str"/>
+      <x:c r="E191"/>
+      <x:c r="F191"/>
       <x:c r="G191" t="str">
         <x:v>Google Maps · Coondoo Street, Kuranda</x:v>
       </x:c>
@@ -9634,8 +10000,8 @@
       <x:c r="D192" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Mareeba+QLD+4880&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E192" t="str"/>
-      <x:c r="F192" t="str"/>
+      <x:c r="E192"/>
+      <x:c r="F192"/>
       <x:c r="G192" t="str">
         <x:v>Google Maps · Mareeba 镇中心</x:v>
       </x:c>
@@ -9653,8 +10019,8 @@
       <x:c r="D193" t="str">
         <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Skybury+Cafe+and+Roastery%2C+136+Ivicevic+Road%2C+Paddys+Green+QLD+4880&amp;travelmode=driving</x:v>
       </x:c>
-      <x:c r="E193" t="str"/>
-      <x:c r="F193" t="str"/>
+      <x:c r="E193"/>
+      <x:c r="F193"/>
       <x:c r="G193" t="str">
         <x:v>Google Maps · 136 Ivicevic Road, Paddys Green QLD 4880</x:v>
       </x:c>
@@ -9672,10 +10038,238 @@
       <x:c r="D194" t="str">
         <x:v>https://skybury.com.au/</x:v>
       </x:c>
-      <x:c r="E194" t="str"/>
-      <x:c r="F194" t="str"/>
+      <x:c r="E194"/>
+      <x:c r="F194"/>
       <x:c r="G194" t="str">
         <x:v>Skybury · 周一至周五 09:00–16:00，公共假日关闭</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" t="str">
+        <x:v>d13-taronga-to-bondi-map</x:v>
+      </x:c>
+      <x:c r="B195" t="str">
+        <x:v>Taronga Zoo 正门 → Bondi Beach</x:v>
+      </x:c>
+      <x:c r="C195" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D195" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Taronga+Zoo+Sydney%2C+Bradleys+Head+Road%2C+Mosman+NSW+2088&amp;destination=Bondi+Beach%2C+NSW+2026&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E195" t="str"/>
+      <x:c r="F195" t="str"/>
+      <x:c r="G195" t="str">
+        <x:v>Google Maps · 天气好时从动物园正门直接前往 Bondi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" t="str">
+        <x:v>d15-bondi-fallback-route-map</x:v>
+      </x:c>
+      <x:c r="B196" t="str">
+        <x:v>酒店 → Bondi → Icebergs → Tamarama</x:v>
+      </x:c>
+      <x:c r="C196" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D196" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Oaks+Sydney+Goldsbrough+Suites%2C+243+Pyrmont+Street%2C+Darling+Harbour+NSW+2009&amp;destination=Tamarama+Beach%2C+NSW+2026&amp;travelmode=driving&amp;waypoints=Bondi+Beach%2C+NSW+2026%7CBondi+Icebergs%2C+1+Notts+Avenue%2C+Bondi+Beach+NSW+2026</x:v>
+      </x:c>
+      <x:c r="E196" t="str"/>
+      <x:c r="F196" t="str"/>
+      <x:c r="G196" t="str">
+        <x:v>Google Maps · 仅在 8/10 未完成 Bondi 时使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" t="str">
+        <x:v>sixt-sydney-city-map</x:v>
+      </x:c>
+      <x:c r="B197" t="str">
+        <x:v>SIXT Sydney City</x:v>
+      </x:c>
+      <x:c r="C197" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D197" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=SIXT+Car+Hire+Sydney+City%2C+Domain+Car+Park%2C+52+Sir+John+Young+Crescent%2C+Woolloomooloo+NSW+2011&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E197" t="str"/>
+      <x:c r="F197" t="str"/>
+      <x:c r="G197" t="str">
+        <x:v>Google Maps · Domain Car Park, 52 Sir John Young Crescent</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" t="str">
+        <x:v>sixt-sydney-city-official</x:v>
+      </x:c>
+      <x:c r="B198" t="str">
+        <x:v>SIXT Sydney City 门店</x:v>
+      </x:c>
+      <x:c r="C198" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D198" t="str">
+        <x:v>https://www.sixt.com.au/car-hire/au/sydney/sydney-city/</x:v>
+      </x:c>
+      <x:c r="E198" t="str"/>
+      <x:c r="F198" t="str"/>
+      <x:c r="G198" t="str">
+        <x:v>SIXT 官网 · 工作日 07:30–16:00，提供 24 小时还车</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" t="str">
+        <x:v>d14-hotel-to-sixt-map</x:v>
+      </x:c>
+      <x:c r="B199" t="str">
+        <x:v>酒店 → SIXT Sydney City</x:v>
+      </x:c>
+      <x:c r="C199" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D199" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Oaks+Sydney+Goldsbrough+Suites%2C+243+Pyrmont+Street%2C+Darling+Harbour+NSW+2009&amp;destination=SIXT+Car+Hire+Sydney+City%2C+Domain+Car+Park%2C+52+Sir+John+Young+Crescent%2C+Woolloomooloo+NSW+2011&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E199" t="str"/>
+      <x:c r="F199" t="str"/>
+      <x:c r="G199" t="str">
+        <x:v>Google Maps · 07:25 从酒店打车前往取车点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" t="str">
+        <x:v>d14-south-coast-loop-map</x:v>
+      </x:c>
+      <x:c r="B200" t="str">
+        <x:v>8/11 南海岸完整环线</x:v>
+      </x:c>
+      <x:c r="C200" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D200" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=SIXT+Car+Hire+Sydney+City%2C+Domain+Car+Park%2C+52+Sir+John+Young+Crescent%2C+Woolloomooloo+NSW+2011&amp;destination=SIXT+Car+Hire+Sydney+City%2C+Domain+Car+Park%2C+52+Sir+John+Young+Crescent%2C+Woolloomooloo+NSW+2011&amp;travelmode=driving&amp;waypoints=Bald+Hill+Lookout%2C+Otford+NSW%7CSea+Cliff+Bridge%2C+Clifton+NSW%7CKiama+Blowhole%2C+Kiama+NSW%7CWerri+Beach%2C+Gerringong+NSW%7CHampden+Bridge%2C+Kangaroo+Valley+NSW</x:v>
+      </x:c>
+      <x:c r="E200" t="str"/>
+      <x:c r="F200" t="str"/>
+      <x:c r="G200" t="str">
+        <x:v>Google Maps · SIXT → Bald Hill → Sea Cliff Bridge → Kiama → Werri Beach → Hampden Bridge → SIXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" t="str">
+        <x:v>d14-coastal-route-map</x:v>
+      </x:c>
+      <x:c r="B201" t="str">
+        <x:v>8/11 沿海去程</x:v>
+      </x:c>
+      <x:c r="C201" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D201" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=SIXT+Car+Hire+Sydney+City%2C+Domain+Car+Park%2C+52+Sir+John+Young+Crescent%2C+Woolloomooloo+NSW+2011&amp;destination=Werri+Beach%2C+Gerringong+NSW&amp;travelmode=driving&amp;waypoints=Bald+Hill+Lookout%2C+Otford+NSW%7CSea+Cliff+Bridge%2C+Clifton+NSW%7CKiama+Blowhole%2C+Kiama+NSW</x:v>
+      </x:c>
+      <x:c r="E201" t="str"/>
+      <x:c r="F201" t="str"/>
+      <x:c r="G201" t="str">
+        <x:v>Google Maps · SIXT → Bald Hill → Sea Cliff Bridge → Kiama → Werri Beach</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" t="str">
+        <x:v>d14-inland-return-map</x:v>
+      </x:c>
+      <x:c r="B202" t="str">
+        <x:v>8/11 袋鼠谷内陆返程</x:v>
+      </x:c>
+      <x:c r="C202" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D202" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Werri+Beach%2C+Gerringong+NSW&amp;destination=SIXT+Car+Hire+Sydney+City%2C+Domain+Car+Park%2C+52+Sir+John+Young+Crescent%2C+Woolloomooloo+NSW+2011&amp;travelmode=driving&amp;waypoints=Hampden+Bridge%2C+Kangaroo+Valley+NSW</x:v>
+      </x:c>
+      <x:c r="E202" t="str"/>
+      <x:c r="F202" t="str"/>
+      <x:c r="G202" t="str">
+        <x:v>Google Maps · Werri Beach → Hampden Bridge → SIXT Sydney City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" t="str">
+        <x:v>kiama-lighthouse-map</x:v>
+      </x:c>
+      <x:c r="B203" t="str">
+        <x:v>Kiama Lighthouse</x:v>
+      </x:c>
+      <x:c r="C203" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D203" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;destination=Kiama+Lighthouse%2C+Blowhole+Point+Road%2C+Kiama+NSW+2533&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E203" t="str"/>
+      <x:c r="F203" t="str"/>
+      <x:c r="G203" t="str">
+        <x:v>Google Maps · 与 Kiama Blowhole 同一区域</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" t="str">
+        <x:v>d11-harbour-walk-map</x:v>
+      </x:c>
+      <x:c r="B204" t="str">
+        <x:v>Barangaroo → The Rocks → Circular Quay</x:v>
+      </x:c>
+      <x:c r="C204" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D204" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Barangaroo+Reserve%2C+Hickson+Road%2C+Barangaroo+NSW+2000&amp;destination=Circular+Quay%2C+Sydney+NSW+2000&amp;travelmode=walking&amp;waypoints=The+Rocks%2C+Sydney+NSW+2000</x:v>
+      </x:c>
+      <x:c r="E204" t="str"/>
+      <x:c r="F204" t="str"/>
+      <x:c r="G204" t="str">
+        <x:v>Google Maps · D11 海港单向步行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" t="str">
+        <x:v>d12-hotel-to-mrs-map</x:v>
+      </x:c>
+      <x:c r="B205" t="str">
+        <x:v>酒店 → Mrs Macquarie's Chair</x:v>
+      </x:c>
+      <x:c r="C205" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D205" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Oaks+Sydney+Goldsbrough+Suites%2C+243+Pyrmont+Street%2C+Darling+Harbour+NSW+2009&amp;destination=Mrs+Macquarie%27s+Chair%2C+Mrs+Macquaries+Road%2C+Sydney+NSW+2000&amp;travelmode=driving</x:v>
+      </x:c>
+      <x:c r="E205" t="str"/>
+      <x:c r="F205" t="str"/>
+      <x:c r="G205" t="str">
+        <x:v>Google Maps · D12 清晨打车前往海港机位</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" t="str">
+        <x:v>d12-harbour-morning-walk-map</x:v>
+      </x:c>
+      <x:c r="B206" t="str">
+        <x:v>Mrs Macquarie's Chair → 植物园 → 歌剧院</x:v>
+      </x:c>
+      <x:c r="C206" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D206" t="str">
+        <x:v>https://www.google.com/maps/dir/?api=1&amp;origin=Mrs+Macquarie%27s+Chair%2C+Mrs+Macquaries+Road%2C+Sydney+NSW+2000&amp;destination=Sydney+Opera+House%2C+Bennelong+Point%2C+Sydney+NSW+2000&amp;travelmode=walking&amp;waypoints=Royal+Botanic+Garden+Sydney%2C+Mrs+Macquaries+Road%2C+Sydney+NSW+2000</x:v>
+      </x:c>
+      <x:c r="E206" t="str"/>
+      <x:c r="F206" t="str"/>
+      <x:c r="G206" t="str">
+        <x:v>Google Maps · D12 早晨单向步行</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9760,7 +10354,7 @@
         <x:v>约 ¥2,875</x:v>
       </x:c>
       <x:c r="D5" s="28" t="str">
-        <x:v>已确认大洋路租车 A$423.56、凯恩斯租车 A$279.51；预算另含悉尼南海岸租车、油费、停车、toll、机场接送、市内短途交通</x:v>
+        <x:v>已确认大洋路租车 A$423.56、凯恩斯租车 A$279.51，以及 8/11 SIXT Sydney City 08:00–19:00 南海岸租车；预算另含油费、停车、toll、机场接送与市内短途交通</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10032,10 +10626,10 @@
         <x:v>悉尼南海岸</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>Grand Pacific Drive / Sea Cliff Bridge / Kiama / Gerringong / Kangaroo Valley（可选）</x:v>
+        <x:v>Grand Pacific Drive / Sea Cliff Bridge / Kiama / Werri Beach / Kangaroo Valley</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
-        <x:v>路线已确定</x:v>
+        <x:v>已确认路线</x:v>
       </x:c>
       <x:c r="D9" s="28" t="str">
         <x:v>A$0 门票</x:v>
@@ -10044,7 +10638,7 @@
         <x:v>¥0</x:v>
       </x:c>
       <x:c r="F9" s="28" t="str">
-        <x:v>D13 使用；主要成本为一日租车、油费、toll 和停车，袋鼠谷按时间与体力决定</x:v>
+        <x:v>D14 使用；SIXT 08:00–19:00 已订，沿海去、内陆回；主要追加成本为油费、toll 与停车</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="23" customFormat="1" ht="15" customHeight="1">
@@ -10064,7 +10658,7 @@
         <x:v>¥0</x:v>
       </x:c>
       <x:c r="F10" s="28" t="str">
-        <x:v>餐饮另计，不放入门票活动</x:v>
+        <x:v>Bondi 先看 D13 天气；若 8/10 未完成，则 D15 上午补走并取消 Manly，餐饮另计</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="23" customFormat="1" ht="40" customHeight="1">
@@ -10084,7 +10678,7 @@
         <x:v>按实付计入</x:v>
       </x:c>
       <x:c r="F11" s="25" t="str">
-        <x:v>D14 使用；Circular Quay 往返使用公共 F2 Ferry，Opal / contactless 即可</x:v>
+        <x:v>D13 使用；Circular Quay 去程使用公共 F2 Ferry，下午从动物园正门直接转 Bondi 或回酒店</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -10494,162 +11088,124 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">临近决定</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D13 南海岸一日租车</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D13｜8/10，若选择 Grand Pacific Drive</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D2" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">等天气更明朗后再决定。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E2" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">天气晴、风不大时优先南海岸；若下雨或海边风大，改蓝山或悉尼市区。</x:t>
-        </x:is>
+      <x:c r="A2" s="28" t="str">
+        <x:v>已订</x:v>
+      </x:c>
+      <x:c r="B2" s="28" t="str">
+        <x:v>SIXT Sydney City 南海岸一日租车</x:v>
+      </x:c>
+      <x:c r="C2" s="28" t="str">
+        <x:v>D14｜8/11，08:00–19:00</x:v>
+      </x:c>
+      <x:c r="D2" s="28" t="str">
+        <x:v>沿海去、内陆回；不在 Wollongong 停留，不加 Fitzroy Falls。</x:v>
+      </x:c>
+      <x:c r="E2" s="28" t="str">
+        <x:v>Domain Car Park, 52 Sir John Young Crescent；18:50 前完成 after-hours return，取车时确认车位与钥匙投递。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">临近决定</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">蓝山 Scenic World / 一日团</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D13｜8/10，若选择蓝山</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">不早买不可退票。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">蓝山最怕雾和低云，临近天气好再买更稳。</x:t>
-        </x:is>
+      <x:c r="A3" s="28" t="str">
+        <x:v>已订</x:v>
+      </x:c>
+      <x:c r="B3" s="28" t="str">
+        <x:v>Puffing Billy + Sassafras 半日团</x:v>
+      </x:c>
+      <x:c r="C3" s="28" t="str">
+        <x:v>D2｜7/30</x:v>
+      </x:c>
+      <x:c r="D3" s="28" t="str">
+        <x:v>11:15 在 343 Russell Street 集合。</x:v>
+      </x:c>
+      <x:c r="E3" s="28" t="str">
+        <x:v>11:30–17:00 随团前往 Belgrave，乘坐 Puffing Billy，并游览 Lakeside 与 Sassafras；山里较凉，随身带防风外套。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="28" t="str">
+        <x:v>建议提前购买</x:v>
+      </x:c>
+      <x:c r="B4" s="28" t="str">
+        <x:v>Taronga Zoo Sydney 门票</x:v>
+      </x:c>
+      <x:c r="C4" s="28" t="str">
+        <x:v>D13｜8/10</x:v>
+      </x:c>
+      <x:c r="D4" s="28" t="str">
+        <x:v>上午游园；下午 Bondi 视天气决定。</x:v>
+      </x:c>
+      <x:c r="E4" s="28" t="str">
+        <x:v>F2 渡轮与动物园门票分开；若下午天气好，从动物园正门直接打车去 Bondi。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="28" t="str">
+        <x:v>灵活餐饮</x:v>
+      </x:c>
+      <x:c r="B5" s="28" t="str">
+        <x:v>Prawn Star / Hello Auntie / Sydney Fish Market 等 food moments</x:v>
+      </x:c>
+      <x:c r="C5" s="28" t="str">
+        <x:v>D7 / D10 / D12 / D13</x:v>
+      </x:c>
+      <x:c r="D5" s="28" t="str">
+        <x:v>餐饮点多数不提前锁死。</x:v>
+      </x:c>
+      <x:c r="E5" s="28" t="str">
+        <x:v>Prawn Star 可看是否需要订位；Hello Auntie 为 D12 晚餐备选；Sydney Fish Market 自由活动；Totti's Bondi 已订 D13 17:30。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="28" t="str">
         <x:v>已订</x:v>
       </x:c>
-      <x:c r="B4" s="28" t="str">
-        <x:v>Puffing Billy + Sassafras 半日团</x:v>
-      </x:c>
-      <x:c r="C4" s="28" t="str">
-        <x:v>D2｜7/30</x:v>
-      </x:c>
-      <x:c r="D4" s="28" t="str">
-        <x:v>11:15 在 343 Russell Street 集合。</x:v>
-      </x:c>
-      <x:c r="E4" s="28" t="str">
-        <x:v>11:30–17:00 随团前往 Belgrave，乘坐 Puffing Billy，并游览 Lakeside 与 Sassafras；山里较凉，随身带防风外套。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">建议提前购买</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Taronga Zoo Sydney 门票</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D15｜8/12</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">官网线上价低于现场价；确定行程后购买。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">动物园冬季 09:30 开门；F2 渡轮与动物园门票分开，出发前查看当天班次。</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">灵活餐饮</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prawn Star / Hello Auntie / Sydney Fish Market 等 food moments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D7 / D10 / D12 / D14</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">餐饮点多数不提前锁死。</x:t>
-        </x:is>
+      <x:c r="B6" s="28" t="str">
+        <x:v>Totti's Bondi 晚餐</x:v>
+      </x:c>
+      <x:c r="C6" s="28" t="str">
+        <x:v>D13｜8/10，17:30</x:v>
+      </x:c>
+      <x:c r="D6" s="28" t="str">
+        <x:v>无论下午是否完成 Bondi，都按预订时间用餐。</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str">
-        <x:v>Prawn Star 可看是否需要订位；Hello Auntie 为 D12 晚餐备选；Sydney Fish Market 自由活动；Icebergs / Bondi Bistro 因 Totti's 已订降级为备选；Lune Croissanterie 看排队和路线。</x:v>
+        <x:v>餐厅位于 Bondi Road；若从酒店出发，预留叫车与晚高峰时间。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="28" t="n"/>
-      <x:c r="B7" s="28" t="n"/>
-      <x:c r="C7" s="28" t="n"/>
-      <x:c r="D7" s="28" t="n"/>
-      <x:c r="E7" s="28" t="n"/>
+      <x:c r="A7" s="28"/>
+      <x:c r="B7" s="28"/>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="28" t="n"/>
-      <x:c r="B8" s="28" t="n"/>
-      <x:c r="C8" s="28" t="n"/>
-      <x:c r="D8" s="28" t="n"/>
-      <x:c r="E8" s="28" t="n"/>
+      <x:c r="A8" s="28"/>
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="28" t="n"/>
-      <x:c r="B9" s="28" t="n"/>
-      <x:c r="C9" s="28" t="n"/>
-      <x:c r="D9" s="28" t="n"/>
-      <x:c r="E9" s="28" t="n"/>
+      <x:c r="A9" s="28"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="28" t="n"/>
-      <x:c r="B10" s="28" t="n"/>
-      <x:c r="C10" s="28" t="n"/>
-      <x:c r="D10" s="28" t="n"/>
-      <x:c r="E10" s="28" t="n"/>
+      <x:c r="A10" s="28"/>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="28" t="n"/>
-      <x:c r="B11" s="28" t="n"/>
-      <x:c r="C11" s="28" t="n"/>
-      <x:c r="D11" s="28" t="n"/>
-      <x:c r="E11" s="28" t="n"/>
+      <x:c r="A11" s="28"/>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10857,88 +11413,93 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>D11 悉尼</x:v>
+        <x:v>D11 悉尼抵达 + 海港黄昏</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>café / A.P Bakery（可选）</x:v>
+        <x:v>机场 / 飞机简餐</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>飞机/机场 / mezze feast</x:v>
+        <x:v>Darling Harbour 就近简餐</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>The Rocks pub</x:v>
+        <x:v>The Rocks / Circular Quay</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
-      </x:c>
+        <x:v>午后先在酒店休息，15:00 后从 Barangaroo 单向走到 Circular Quay，先看日落再吃晚餐。</x:v>
+      </x:c>
+      <x:c r="F12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>D12 悉尼</x:v>
+        <x:v>D12 海港晨光 + 歌剧院 + QVB</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>bills / Toby's Estate</x:v>
+        <x:v>酒店附近 café</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>The Rocks Markets / Circular Quay 简餐</x:v>
+        <x:v>Circular Quay / CBD 简餐</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>Hello Auntie</x:v>
+        <x:v>Hello Auntie / 酒店附近</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
-      </x:c>
+        <x:v>清晨先走 Mrs Macquarie's Chair 与植物园，09:30 中文导览已订；下午集中在 QVB / Westfield。</x:v>
+      </x:c>
+      <x:c r="F13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>D13 南海岸</x:v>
+        <x:v>D13 Taronga + Bondi</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>café</x:v>
+        <x:v>CBD café</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Kiama Hungry Monkey / Kiama 简餐</x:v>
+        <x:v>Taronga Zoo 轻食</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>回城后 CBD / 酒店附近简餐</x:v>
+        <x:v>Totti's Bondi 17:30（已订）</x:v>
       </x:c>
       <x:c r="E14" t="str">
-        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
-      </x:c>
+        <x:v>下午按天气决定 Bondi 或回酒店休息；无论哪条路线，都按 17:30 的预订前往 Totti's。</x:v>
+      </x:c>
+      <x:c r="F14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>D14 Taronga + Bondi</x:v>
+        <x:v>D14 南海岸环线</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>CBD café</x:v>
+        <x:v>酒店附近 café</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>Taronga Zoo 轻食 / Circular Quay 简餐</x:v>
+        <x:v>Kiama 简餐</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>Totti's Bondi 18:30（已订）</x:v>
+        <x:v>还车后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
-      </x:c>
+        <x:v>14:00 离开 Werri Beach，15:30 离开 Kangaroo Valley；午餐控制在一小时内。</x:v>
+      </x:c>
+      <x:c r="F15"/>
     </x:row>
     <x:row r="16" s="23" customFormat="1" ht="40" customHeight="1">
       <x:c r="A16" s="25" t="str">
-        <x:v>D15 Manly 弹性 + 告别</x:v>
+        <x:v>D15 Bondi 补位 / Manly 备选 + 告别</x:v>
       </x:c>
       <x:c r="B16" s="25" t="str">
-        <x:v>café / Single O / Toby's Estate</x:v>
+        <x:v>按 Bondi / Manly / CBD 路线解决</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
-        <x:v>若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐</x:v>
+        <x:v>海边 café / CBD 简餐</x:v>
       </x:c>
       <x:c r="D16" s="25" t="str">
         <x:v>Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
       </x:c>
       <x:c r="E16" s="25" t="str">
-        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
-      </x:c>
+        <x:v>若 8/10 未完成 Bondi，上午优先补走并取消 Manly；13:30 前回 CBD，下午采购、整理 TRS。</x:v>
+      </x:c>
+      <x:c r="F16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">

</xml_diff>